<commit_message>
feat(display): window modes (windowed/borderless/exclusive), settings v8, narrow-room centring, hold-to-skip
D91/I-054: Settings Window row, default borderless, tests force windowed. DISP-14: settings_version 8 maps fit_screen to window_mode.
DISP-10: rm_floor6_5 drawn centred, nothing outside the room shown. D48/I-055: hold confirm ~1 s skips cutscenes and camera pans.

Co-Authored-By: Claude Sonnet <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datafiles/localization/game_text.xlsx
+++ b/datafiles/localization/game_text.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C678"/>
+  <dimension ref="A1:C684"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -11949,6 +11949,108 @@
         </is>
       </c>
     </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>settings.row.window_mode</t>
+        </is>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>Window</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>창 모드</t>
+        </is>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>settings.value.window_windowed</t>
+        </is>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>Windowed</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>창</t>
+        </is>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>settings.value.window_borderless</t>
+        </is>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>Borderless</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>테두리 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>settings.value.window_exclusive</t>
+        </is>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>Exclusive</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>전체 화면</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>settings.value.auto</t>
+        </is>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>자동</t>
+        </is>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>ui.skip_hold</t>
+        </is>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>Hold to skip</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>길게 눌러 건너뛰기</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C678"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(ui): shared menu framework (D95-D98, D100, D101) + title and settings pilot
One data-driven menu component in scr_menu.gml: wrap-around cursor that skips greyed items, hold-to-scroll (300 ms then
accelerating, time based), a menu stack where Back goes up one level, cursor remembered per menu id, mouse hover/click/
right-click/wheel, 120 ms panel slide+fade, gliding highlight, bobbing marker, soft blips, in-code 4-colour pixel frame,
details panel, speaker name tab, tabs header. Title menu, difficulty panel and the settings screen (also used by the
pause menu) now run on it; the old per-screen code is gone. Settings gain text speed, screen shake and QTE assist
(settings_version 9). Korean uses Galmuri9/11 at whole multiples of their native size. Test_Suite_UI (204 checks), smoke
drives title, settings, difficulty and pause settings through the real input, 6 new -shots (73 total).

Co-Authored-By: Claude Sonnet <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datafiles/localization/game_text.xlsx
+++ b/datafiles/localization/game_text.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C684"/>
+  <dimension ref="A1:C707"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -6930,7 +6930,7 @@
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>뒤쪽에</t>
+          <t>뒤로</t>
         </is>
       </c>
     </row>
@@ -10483,7 +10483,7 @@
       </c>
       <c r="C592" t="inlineStr">
         <is>
-          <t>적용하다</t>
+          <t>적용</t>
         </is>
       </c>
     </row>
@@ -10500,7 +10500,7 @@
       </c>
       <c r="C593" t="inlineStr">
         <is>
-          <t>뒤쪽에</t>
+          <t>뒤로</t>
         </is>
       </c>
     </row>
@@ -12048,6 +12048,397 @@
       <c r="C684" t="inlineStr">
         <is>
           <t>길게 눌러 건너뛰기</t>
+        </is>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>settings.row.text_speed</t>
+        </is>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>Text speed</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>글자 속도</t>
+        </is>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" t="inlineStr">
+        <is>
+          <t>settings.row.shake</t>
+        </is>
+      </c>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>Screen shake</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>화면 흔들림</t>
+        </is>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" t="inlineStr">
+        <is>
+          <t>settings.row.qte_assist</t>
+        </is>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>QTE assist</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr">
+        <is>
+          <t>QTE 보조</t>
+        </is>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" t="inlineStr">
+        <is>
+          <t>settings.value.speed_slow</t>
+        </is>
+      </c>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>Slow</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr">
+        <is>
+          <t>느리게</t>
+        </is>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" t="inlineStr">
+        <is>
+          <t>settings.value.speed_normal</t>
+        </is>
+      </c>
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="C689" t="inlineStr">
+        <is>
+          <t>보통</t>
+        </is>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" t="inlineStr">
+        <is>
+          <t>settings.value.speed_fast</t>
+        </is>
+      </c>
+      <c r="B690" t="inlineStr">
+        <is>
+          <t>Fast</t>
+        </is>
+      </c>
+      <c r="C690" t="inlineStr">
+        <is>
+          <t>빠르게</t>
+        </is>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" t="inlineStr">
+        <is>
+          <t>settings.value.on</t>
+        </is>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>On</t>
+        </is>
+      </c>
+      <c r="C691" t="inlineStr">
+        <is>
+          <t>켜짐</t>
+        </is>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" t="inlineStr">
+        <is>
+          <t>settings.value.off</t>
+        </is>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="C692" t="inlineStr">
+        <is>
+          <t>꺼짐</t>
+        </is>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" t="inlineStr">
+        <is>
+          <t>settings.line.cps</t>
+        </is>
+      </c>
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>Characters per second</t>
+        </is>
+      </c>
+      <c r="C693" t="inlineStr">
+        <is>
+          <t>초당 글자 수</t>
+        </is>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" t="inlineStr">
+        <is>
+          <t>settings.line.monitor</t>
+        </is>
+      </c>
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>Monitor</t>
+        </is>
+      </c>
+      <c r="C694" t="inlineStr">
+        <is>
+          <t>모니터</t>
+        </is>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" t="inlineStr">
+        <is>
+          <t>settings.line.window_size</t>
+        </is>
+      </c>
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>Window size</t>
+        </is>
+      </c>
+      <c r="C695" t="inlineStr">
+        <is>
+          <t>창 크기</t>
+        </is>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" t="inlineStr">
+        <is>
+          <t>settings.help.vol_ui</t>
+        </is>
+      </c>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>How loud menu clicks and other interface sounds are.</t>
+        </is>
+      </c>
+      <c r="C696" t="inlineStr">
+        <is>
+          <t>메뉴 소리와 인터페이스 효과음의 크기입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" t="inlineStr">
+        <is>
+          <t>settings.help.vol_sfx</t>
+        </is>
+      </c>
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>How loud hits, footsteps and other game sounds are.</t>
+        </is>
+      </c>
+      <c r="C697" t="inlineStr">
+        <is>
+          <t>타격음, 발소리 등 게임 효과음의 크기입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" t="inlineStr">
+        <is>
+          <t>settings.help.vol_bgm</t>
+        </is>
+      </c>
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>How loud the music is.</t>
+        </is>
+      </c>
+      <c r="C698" t="inlineStr">
+        <is>
+          <t>배경 음악의 크기입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" t="inlineStr">
+        <is>
+          <t>settings.help.text_speed</t>
+        </is>
+      </c>
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>How fast dialogue text appears.</t>
+        </is>
+      </c>
+      <c r="C699" t="inlineStr">
+        <is>
+          <t>대사가 나타나는 속도입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" t="inlineStr">
+        <is>
+          <t>settings.help.shake</t>
+        </is>
+      </c>
+      <c r="B700" t="inlineStr">
+        <is>
+          <t>Turns the screen shake on hits on or off.</t>
+        </is>
+      </c>
+      <c r="C700" t="inlineStr">
+        <is>
+          <t>공격을 받을 때 화면이 흔들리는 효과를 켜거나 끕니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" t="inlineStr">
+        <is>
+          <t>settings.help.qte_assist</t>
+        </is>
+      </c>
+      <c r="B701" t="inlineStr">
+        <is>
+          <t>Planned: more forgiving timing on button prompts.</t>
+        </is>
+      </c>
+      <c r="C701" t="inlineStr">
+        <is>
+          <t>예정: 버튼 입력 타이밍 판정을 더 너그럽게 합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" t="inlineStr">
+        <is>
+          <t>settings.help.window</t>
+        </is>
+      </c>
+      <c r="B702" t="inlineStr">
+        <is>
+          <t>Windowed, borderless fullscreen, or exclusive fullscreen.</t>
+        </is>
+      </c>
+      <c r="C702" t="inlineStr">
+        <is>
+          <t>창 모드, 테두리 없는 전체 화면, 전용 전체 화면 중에서 고릅니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" t="inlineStr">
+        <is>
+          <t>settings.help.scale</t>
+        </is>
+      </c>
+      <c r="B703" t="inlineStr">
+        <is>
+          <t>How many times the picture is enlarged in a window. Only used when windowed.</t>
+        </is>
+      </c>
+      <c r="C703" t="inlineStr">
+        <is>
+          <t>창 모드에서 화면을 몇 배로 키울지 정합니다. 창 모드에서만 쓰입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" t="inlineStr">
+        <is>
+          <t>settings.help.language</t>
+        </is>
+      </c>
+      <c r="B704" t="inlineStr">
+        <is>
+          <t>Language of all text in the game.</t>
+        </is>
+      </c>
+      <c r="C704" t="inlineStr">
+        <is>
+          <t>게임의 모든 글자 언어입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" t="inlineStr">
+        <is>
+          <t>settings.help.apply</t>
+        </is>
+      </c>
+      <c r="B705" t="inlineStr">
+        <is>
+          <t>Saves your changes and applies them now. Back leaves without saving.</t>
+        </is>
+      </c>
+      <c r="C705" t="inlineStr">
+        <is>
+          <t>변경 사항을 저장하고 지금 적용합니다. 뒤로 가면 저장하지 않습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" t="inlineStr">
+        <is>
+          <t>settings.lang.korean</t>
+        </is>
+      </c>
+      <c r="B706" t="inlineStr">
+        <is>
+          <t>Korean</t>
+        </is>
+      </c>
+      <c r="C706" t="inlineStr">
+        <is>
+          <t>한국어</t>
+        </is>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" t="inlineStr">
+        <is>
+          <t>settings.lang.english</t>
+        </is>
+      </c>
+      <c r="B707" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="C707" t="inlineStr">
+        <is>
+          <t>English</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(status): poison stacks, burn tick + DEF -25%, bleed per action, Foresight reveal + wider Perfect zones, data-driven descriptions (packet B2)
D78: Poison hurts its stacks then loses one (max 10, reapply adds); Burning is a fixed
tick (0.3 x caster MAG, min 2) for 2 turns, no stacking, DEF x0.75; Bleeding hurts only
when its owner acts, stacks to 3, lasts 3 turns; the three coexist (exclusions removed).
Defence bar only shortens or reduces (D21, D59). D79/D24: Foresight lasts 3 turns, shows
the enemy's next action (Battle_EnemyNextActionPreview, "You foresee:" log line) and
widens every Perfect zone x1.5; always_hit removed. BUG-17: Curse rolls its chance per
status and logs only what landed. BUG-16: skill status turns are the real numbers;
Status_Describe / Status_DisplayList give the UI plain text and counters from the data.
Vectors, Test_Suite_StatusRules, bot v=6 (battles A and B), spec section 10, R-066/R-067.

Co-Authored-By: Claude Sonnet <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datafiles/localization/game_text.xlsx
+++ b/datafiles/localization/game_text.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C664"/>
+  <dimension ref="A1:C686"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -11711,6 +11711,380 @@
         </is>
       </c>
     </row>
+    <row r="665">
+      <c r="A665" t="inlineStr">
+        <is>
+          <t>status.desc.poison.data</t>
+        </is>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>Lose {tick} HP each turn, then 1 stack fades ({stacks} stacks, max {max}).{mods}</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>매 턴 {tick} HP를 잃고, 중첩이 1 줄어듭니다 ({stacks}중첩, 최대 {max}).{mods}</t>
+        </is>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="inlineStr">
+        <is>
+          <t>status.desc.poison</t>
+        </is>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>Lose HP equal to its stacks each turn, then 1 stack fades. Stacks up to {max}.{mods}</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>매 턴 중첩 수만큼 HP를 잃고, 중첩이 1 줄어듭니다. 최대 {max}중첩.{mods}</t>
+        </is>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="inlineStr">
+        <is>
+          <t>status.desc.bleed.data</t>
+        </is>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>Lose {tick} HP each time you act ({stacks} stacks, max {max}), for {turns} more turns.{mods}</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>행동할 때마다 {tick} HP를 잃습니다 ({stacks}중첩, 최대 {max}). {turns}턴 더 지속.{mods}</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="inlineStr">
+        <is>
+          <t>status.desc.bleed</t>
+        </is>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>Lose {tick} HP per stack each time you act. Stacks up to {max}, lasts {dur} turns.{mods}</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>행동할 때마다 중첩당 {tick} HP를 잃습니다. 최대 {max}중첩, {dur}턴 지속.{mods}</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>status.desc.burn.data</t>
+        </is>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>Lose {tick} HP each turn for {turns} more turns.{mods}</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>매 턴 {tick} HP를 잃습니다. {turns}턴 더 지속.{mods}</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr">
+        <is>
+          <t>status.desc.burn</t>
+        </is>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>Lose a fixed amount of HP (it grows with the caster's MAG) each turn for {dur} turns. Does not stack.{mods}</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>매 턴 정해진 HP(시전자의 MAG에 비례)를 {dur}턴 동안 잃습니다. 중첩되지 않습니다.{mods}</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>status.desc.status_stun</t>
+        </is>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>Cannot act.</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>행동할 수 없습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>status.desc.status_guard</t>
+        </is>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>Blocks the next incoming hit.</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>다음에 받는 공격을 막습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr">
+        <is>
+          <t>status.desc.status_dmg_up</t>
+        </is>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>Next attack deals {mult} times the damage.</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>다음 공격이 {mult}배의 피해를 줍니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>status.desc.status_evasion</t>
+        </is>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>Dodges the next incoming attack.</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>다음에 받는 공격을 피합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>status.desc.status_crit_up</t>
+        </is>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>Critical chance +{pct}%.</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>치명타 확률 +{pct}%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>status.desc.status_hit_up</t>
+        </is>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>For {turns} turns: you see the enemy's next move and every Perfect zone is {pct}% wider.</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>{turns}턴 동안 적의 다음 행동이 보이고 모든 퍼펙트 구간이 {pct}% 넓어집니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>status.desc.status_meditation</t>
+        </is>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>Recover {lo}-{hi} MP each turn.</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>매 턴 MP를 {lo}-{hi} 회복합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>status.desc.status_solidify</t>
+        </is>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>Takes {pct}% less damage from the next hit.</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>다음 공격에서 받는 피해가 {pct}% 줄어듭니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>status.desc.status_bloodthirsty</t>
+        </is>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>Until hit: take {take}% less, deal {deal}% more damage.</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>맞을 때까지: 받는 피해 {take}% 감소, 주는 피해 {deal}% 증가.</t>
+        </is>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>status.desc.status_blessing</t>
+        </is>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>Next incoming hit deals {pct}% less damage.</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>다음에 받는 공격의 피해가 {pct}% 줄어듭니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>status.desc.status_sunder</t>
+        </is>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>Lose defence.{mods}</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>방어력이 떨어집니다.{mods}</t>
+        </is>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>combat.msg.status_tick_enemy</t>
+        </is>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>{status} hurts {enemy} for {dmg}.</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>{status} 때문에 {enemy}가 {dmg}의 피해를 입었습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>combat.msg.multi_status_none</t>
+        </is>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>Nothing took hold.</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>아무 효과도 없었습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>combat.msg.foresee</t>
+        </is>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>You foresee: {action}</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>예견: {action}</t>
+        </is>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>combat.foresee.attack</t>
+        </is>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>a plain attack</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>일반 공격</t>
+        </is>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" t="inlineStr">
+        <is>
+          <t>combat.foresee.stunned</t>
+        </is>
+      </c>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>nothing, it is stunned</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>기절해서 아무것도 못 합니다</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C678"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(combat): turn timeline (SPD gauges, next-5 strip), stun push-back + Steadfast, stagger meter + BREAK, floating damage numbers (B3: D19 D74 D75 D79 D92)
Replaces the alternating/initiative flow with Turn_Next; removes the stun-gives-extra-actions exploit (S1). Foresight preview now rides on the strip
(the log line is gone). New: spec section 11, reference + vectors, Test_Suite_Turns, bot_turns, B3 shots, EN+KO strings.

Co-Authored-By: Claude Sonnet <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datafiles/localization/game_text.xlsx
+++ b/datafiles/localization/game_text.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C731"/>
+  <dimension ref="A1:C737"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -12212,12 +12212,12 @@
       </c>
       <c r="B694" t="inlineStr">
         <is>
-          <t>Cannot act.</t>
+          <t>Pushed back on the turn bar. Then Steadfast: cannot be stunned for 2 turns.</t>
         </is>
       </c>
       <c r="C694" t="inlineStr">
         <is>
-          <t>행동할 수 없습니다.</t>
+          <t>차례가 뒤로 밀립니다. 그 뒤 2턴 동안은 기절하지 않습니다.</t>
         </is>
       </c>
     </row>
@@ -12847,6 +12847,108 @@
       <c r="C731" t="inlineStr">
         <is>
           <t>이전 버전의 저장 파일은 이 버전에서 불러올 수 없습니다. 파일은 그대로 두었습니다. 새 도전을 시작하세요.</t>
+        </is>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" t="inlineStr">
+        <is>
+          <t>combat.msg.pushed_back</t>
+        </is>
+      </c>
+      <c r="B732" t="inlineStr">
+        <is>
+          <t>{name} is pushed back!</t>
+        </is>
+      </c>
+      <c r="C732" t="inlineStr">
+        <is>
+          <t>{name}의 차례가 뒤로 밀렸습니다!</t>
+        </is>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" t="inlineStr">
+        <is>
+          <t>combat.msg.pushed_back_you</t>
+        </is>
+      </c>
+      <c r="B733" t="inlineStr">
+        <is>
+          <t>You are pushed back!</t>
+        </is>
+      </c>
+      <c r="C733" t="inlineStr">
+        <is>
+          <t>당신의 차례가 뒤로 밀렸습니다!</t>
+        </is>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" t="inlineStr">
+        <is>
+          <t>combat.msg.steadfast</t>
+        </is>
+      </c>
+      <c r="B734" t="inlineStr">
+        <is>
+          <t>{name} is Steadfast!</t>
+        </is>
+      </c>
+      <c r="C734" t="inlineStr">
+        <is>
+          <t>{name}은(는) 버티고 있습니다!</t>
+        </is>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" t="inlineStr">
+        <is>
+          <t>combat.msg.steadfast_you</t>
+        </is>
+      </c>
+      <c r="B735" t="inlineStr">
+        <is>
+          <t>You are Steadfast!</t>
+        </is>
+      </c>
+      <c r="C735" t="inlineStr">
+        <is>
+          <t>당신은 버티고 있습니다!</t>
+        </is>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" t="inlineStr">
+        <is>
+          <t>combat.msg.break</t>
+        </is>
+      </c>
+      <c r="B736" t="inlineStr">
+        <is>
+          <t>BREAK! {name} takes +50% damage!</t>
+        </is>
+      </c>
+      <c r="C736" t="inlineStr">
+        <is>
+          <t>브레이크! {name}이(가) 받는 피해 +50%!</t>
+        </is>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" t="inlineStr">
+        <is>
+          <t>battle.hud.break</t>
+        </is>
+      </c>
+      <c r="B737" t="inlineStr">
+        <is>
+          <t>BREAK!</t>
+        </is>
+      </c>
+      <c r="C737" t="inlineStr">
+        <is>
+          <t>브레이크!</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(cards): 1-of-3 card picks, upgrades, passives, class chest, level-up stat point (packet C2)
Cards (D18, D81-D83): 14 skill cards, 14 upgrades, 19 passives (7 shared, 3 per class, 3 Nobody), 3 fallbacks.
Card_OfferGenerate is pure: weighted by kind, new-skill quota, pity after 2 offers without an upgrade, decline
memory, same seed = same offers (run "cards" stream; pity state saved in the run save). Max 3 skills: a 4th asks
which to replace. Chests (D73, fixes I-057): the first class or skill chest of a run gives the class choice
(Nobody locked until a first win, D83), later ones a pick. Level-up (D76, D81): free stat point prompt, then a pick.
Screens on the shared UI framework (class, stat, replace, 3-card pick). Skill books removed (D18).
Tests: Test_Suite_Cards (140 assertions), smoke steps 133-141, 8 new shots; text EN + KO draft.

Co-Authored-By: Claude Sonnet <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datafiles/localization/game_text.xlsx
+++ b/datafiles/localization/game_text.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C731"/>
+  <dimension ref="A1:C837"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -12850,6 +12850,1808 @@
         </is>
       </c>
     </row>
+    <row r="732">
+      <c r="A732" t="inlineStr">
+        <is>
+          <t>card.lbl.arrows</t>
+        </is>
+      </c>
+      <c r="B732" t="inlineStr">
+        <is>
+          <t>Arrows</t>
+        </is>
+      </c>
+      <c r="C732" t="inlineStr">
+        <is>
+          <t>화살표</t>
+        </is>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" t="inlineStr">
+        <is>
+          <t>card.lbl.power</t>
+        </is>
+      </c>
+      <c r="B733" t="inlineStr">
+        <is>
+          <t>Power</t>
+        </is>
+      </c>
+      <c r="C733" t="inlineStr">
+        <is>
+          <t>위력</t>
+        </is>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" t="inlineStr">
+        <is>
+          <t>card.lbl.mp</t>
+        </is>
+      </c>
+      <c r="B734" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+      <c r="C734" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" t="inlineStr">
+        <is>
+          <t>card.lbl.chance</t>
+        </is>
+      </c>
+      <c r="B735" t="inlineStr">
+        <is>
+          <t>Chance</t>
+        </is>
+      </c>
+      <c r="C735" t="inlineStr">
+        <is>
+          <t>확률</t>
+        </is>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" t="inlineStr">
+        <is>
+          <t>card.lbl.turns</t>
+        </is>
+      </c>
+      <c r="B736" t="inlineStr">
+        <is>
+          <t>Turns</t>
+        </is>
+      </c>
+      <c r="C736" t="inlineStr">
+        <is>
+          <t>턴</t>
+        </is>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" t="inlineStr">
+        <is>
+          <t>card.lbl.stacks</t>
+        </is>
+      </c>
+      <c r="B737" t="inlineStr">
+        <is>
+          <t>Stacks</t>
+        </is>
+      </c>
+      <c r="C737" t="inlineStr">
+        <is>
+          <t>중첩</t>
+        </is>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" t="inlineStr">
+        <is>
+          <t>card.lbl.atk</t>
+        </is>
+      </c>
+      <c r="B738" t="inlineStr">
+        <is>
+          <t>ATK</t>
+        </is>
+      </c>
+      <c r="C738" t="inlineStr">
+        <is>
+          <t>ATK</t>
+        </is>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" t="inlineStr">
+        <is>
+          <t>card.lbl.def</t>
+        </is>
+      </c>
+      <c r="B739" t="inlineStr">
+        <is>
+          <t>DEF</t>
+        </is>
+      </c>
+      <c r="C739" t="inlineStr">
+        <is>
+          <t>DEF</t>
+        </is>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" t="inlineStr">
+        <is>
+          <t>card.lbl.spd</t>
+        </is>
+      </c>
+      <c r="B740" t="inlineStr">
+        <is>
+          <t>SPD</t>
+        </is>
+      </c>
+      <c r="C740" t="inlineStr">
+        <is>
+          <t>SPD</t>
+        </is>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" t="inlineStr">
+        <is>
+          <t>card.lbl.mag</t>
+        </is>
+      </c>
+      <c r="B741" t="inlineStr">
+        <is>
+          <t>MAG</t>
+        </is>
+      </c>
+      <c r="C741" t="inlineStr">
+        <is>
+          <t>MAG</t>
+        </is>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" t="inlineStr">
+        <is>
+          <t>card.lbl.main_stat</t>
+        </is>
+      </c>
+      <c r="B742" t="inlineStr">
+        <is>
+          <t>Main stat</t>
+        </is>
+      </c>
+      <c r="C742" t="inlineStr">
+        <is>
+          <t>주력 능력치</t>
+        </is>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" t="inlineStr">
+        <is>
+          <t>card.lbl.poison_stacks</t>
+        </is>
+      </c>
+      <c r="B743" t="inlineStr">
+        <is>
+          <t>Poison stacks</t>
+        </is>
+      </c>
+      <c r="C743" t="inlineStr">
+        <is>
+          <t>독 중첩</t>
+        </is>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" t="inlineStr">
+        <is>
+          <t>card.lbl.after_fight</t>
+        </is>
+      </c>
+      <c r="B744" t="inlineStr">
+        <is>
+          <t>After fight</t>
+        </is>
+      </c>
+      <c r="C744" t="inlineStr">
+        <is>
+          <t>전투 후</t>
+        </is>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" t="inlineStr">
+        <is>
+          <t>card.lbl.potion_find</t>
+        </is>
+      </c>
+      <c r="B745" t="inlineStr">
+        <is>
+          <t>Potion find</t>
+        </is>
+      </c>
+      <c r="C745" t="inlineStr">
+        <is>
+          <t>물약 발견</t>
+        </is>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" t="inlineStr">
+        <is>
+          <t>card.lbl.perfect</t>
+        </is>
+      </c>
+      <c r="B746" t="inlineStr">
+        <is>
+          <t>Perfect zone</t>
+        </is>
+      </c>
+      <c r="C746" t="inlineStr">
+        <is>
+          <t>퍼펙트 구간</t>
+        </is>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" t="inlineStr">
+        <is>
+          <t>card.lbl.gold</t>
+        </is>
+      </c>
+      <c r="B747" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="C747" t="inlineStr">
+        <is>
+          <t>골드</t>
+        </is>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" t="inlineStr">
+        <is>
+          <t>card.lbl.each_turn</t>
+        </is>
+      </c>
+      <c r="B748" t="inlineStr">
+        <is>
+          <t>Each turn</t>
+        </is>
+      </c>
+      <c r="C748" t="inlineStr">
+        <is>
+          <t>매 턴</t>
+        </is>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" t="inlineStr">
+        <is>
+          <t>card.lbl.potions</t>
+        </is>
+      </c>
+      <c r="B749" t="inlineStr">
+        <is>
+          <t>Potions</t>
+        </is>
+      </c>
+      <c r="C749" t="inlineStr">
+        <is>
+          <t>물약</t>
+        </is>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" t="inlineStr">
+        <is>
+          <t>card.lbl.guard</t>
+        </is>
+      </c>
+      <c r="B750" t="inlineStr">
+        <is>
+          <t>Guard</t>
+        </is>
+      </c>
+      <c r="C750" t="inlineStr">
+        <is>
+          <t>방어</t>
+        </is>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" t="inlineStr">
+        <is>
+          <t>card.lbl.skill_power</t>
+        </is>
+      </c>
+      <c r="B751" t="inlineStr">
+        <is>
+          <t>Skill power</t>
+        </is>
+      </c>
+      <c r="C751" t="inlineStr">
+        <is>
+          <t>스킬 위력</t>
+        </is>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" t="inlineStr">
+        <is>
+          <t>card.lbl.skill_mp</t>
+        </is>
+      </c>
+      <c r="B752" t="inlineStr">
+        <is>
+          <t>Skill MP</t>
+        </is>
+      </c>
+      <c r="C752" t="inlineStr">
+        <is>
+          <t>스킬 MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" t="inlineStr">
+        <is>
+          <t>card.lbl.status_turns</t>
+        </is>
+      </c>
+      <c r="B753" t="inlineStr">
+        <is>
+          <t>Status turns</t>
+        </is>
+      </c>
+      <c r="C753" t="inlineStr">
+        <is>
+          <t>상태 턴</t>
+        </is>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" t="inlineStr">
+        <is>
+          <t>card.lbl.potion_mp</t>
+        </is>
+      </c>
+      <c r="B754" t="inlineStr">
+        <is>
+          <t>Potion MP</t>
+        </is>
+      </c>
+      <c r="C754" t="inlineStr">
+        <is>
+          <t>물약 MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" t="inlineStr">
+        <is>
+          <t>card.lbl.restores</t>
+        </is>
+      </c>
+      <c r="B755" t="inlineStr">
+        <is>
+          <t>Restores</t>
+        </is>
+      </c>
+      <c r="C755" t="inlineStr">
+        <is>
+          <t>회복량</t>
+        </is>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" t="inlineStr">
+        <is>
+          <t>card.lbl.skills</t>
+        </is>
+      </c>
+      <c r="B756" t="inlineStr">
+        <is>
+          <t>Skills</t>
+        </is>
+      </c>
+      <c r="C756" t="inlineStr">
+        <is>
+          <t>스킬</t>
+        </is>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" t="inlineStr">
+        <is>
+          <t>card.mp_short</t>
+        </is>
+      </c>
+      <c r="B757" t="inlineStr">
+        <is>
+          <t>{mp} MP</t>
+        </is>
+      </c>
+      <c r="C757" t="inlineStr">
+        <is>
+          <t>{mp} MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" t="inlineStr">
+        <is>
+          <t>card.val.hp</t>
+        </is>
+      </c>
+      <c r="B758" t="inlineStr">
+        <is>
+          <t>+{n} HP</t>
+        </is>
+      </c>
+      <c r="C758" t="inlineStr">
+        <is>
+          <t>HP +{n}</t>
+        </is>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" t="inlineStr">
+        <is>
+          <t>card.val.mp</t>
+        </is>
+      </c>
+      <c r="B759" t="inlineStr">
+        <is>
+          <t>+{n} MP</t>
+        </is>
+      </c>
+      <c r="C759" t="inlineStr">
+        <is>
+          <t>MP +{n}</t>
+        </is>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" t="inlineStr">
+        <is>
+          <t>card.val.turns</t>
+        </is>
+      </c>
+      <c r="B760" t="inlineStr">
+        <is>
+          <t>+{n} turns</t>
+        </is>
+      </c>
+      <c r="C760" t="inlineStr">
+        <is>
+          <t>+{n}턴</t>
+        </is>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" t="inlineStr">
+        <is>
+          <t>card.val.restores</t>
+        </is>
+      </c>
+      <c r="B761" t="inlineStr">
+        <is>
+          <t>{pct} HP, MP</t>
+        </is>
+      </c>
+      <c r="C761" t="inlineStr">
+        <is>
+          <t>HP, MP {pct}</t>
+        </is>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" t="inlineStr">
+        <is>
+          <t>card.skill.buff</t>
+        </is>
+      </c>
+      <c r="B762" t="inlineStr">
+        <is>
+          <t>Gain {status} for {turns} turns.</t>
+        </is>
+      </c>
+      <c r="C762" t="inlineStr">
+        <is>
+          <t>{status} 효과를 {turns}턴 동안 얻는다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" t="inlineStr">
+        <is>
+          <t>card.skill.hit</t>
+        </is>
+      </c>
+      <c r="B763" t="inlineStr">
+        <is>
+          <t>Strike for {power} power.</t>
+        </is>
+      </c>
+      <c r="C763" t="inlineStr">
+        <is>
+          <t>위력 {power}로 공격한다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" t="inlineStr">
+        <is>
+          <t>card.skill.hit_status</t>
+        </is>
+      </c>
+      <c r="B764" t="inlineStr">
+        <is>
+          <t>{chance}% to inflict {status}.</t>
+        </is>
+      </c>
+      <c r="C764" t="inlineStr">
+        <is>
+          <t>{chance}% 확률로 {status} 부여.</t>
+        </is>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" t="inlineStr">
+        <is>
+          <t>card.skill.hits</t>
+        </is>
+      </c>
+      <c r="B765" t="inlineStr">
+        <is>
+          <t>Strike {hits} times for {power} power each.</t>
+        </is>
+      </c>
+      <c r="C765" t="inlineStr">
+        <is>
+          <t>{hits}번 공격한다. 한 번에 위력 {power}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" t="inlineStr">
+        <is>
+          <t>card.skill.other</t>
+        </is>
+      </c>
+      <c r="B766" t="inlineStr">
+        <is>
+          <t>A special technique.</t>
+        </is>
+      </c>
+      <c r="C766" t="inlineStr">
+        <is>
+          <t>특수한 기술.</t>
+        </is>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" t="inlineStr">
+        <is>
+          <t>card.tag.boon</t>
+        </is>
+      </c>
+      <c r="B767" t="inlineStr">
+        <is>
+          <t>Boon</t>
+        </is>
+      </c>
+      <c r="C767" t="inlineStr">
+        <is>
+          <t>은총</t>
+        </is>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" t="inlineStr">
+        <is>
+          <t>card.tag.class_passive</t>
+        </is>
+      </c>
+      <c r="B768" t="inlineStr">
+        <is>
+          <t>Class passive</t>
+        </is>
+      </c>
+      <c r="C768" t="inlineStr">
+        <is>
+          <t>직업 패시브</t>
+        </is>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" t="inlineStr">
+        <is>
+          <t>card.tag.passive</t>
+        </is>
+      </c>
+      <c r="B769" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="C769" t="inlineStr">
+        <is>
+          <t>패시브</t>
+        </is>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" t="inlineStr">
+        <is>
+          <t>card.tag.skill</t>
+        </is>
+      </c>
+      <c r="B770" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="C770" t="inlineStr">
+        <is>
+          <t>스킬</t>
+        </is>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" t="inlineStr">
+        <is>
+          <t>card.tag.upgrade</t>
+        </is>
+      </c>
+      <c r="B771" t="inlineStr">
+        <is>
+          <t>Upgrade</t>
+        </is>
+      </c>
+      <c r="C771" t="inlineStr">
+        <is>
+          <t>강화</t>
+        </is>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" t="inlineStr">
+        <is>
+          <t>cards.pick.hint</t>
+        </is>
+      </c>
+      <c r="B772" t="inlineStr">
+        <is>
+          <t>Left / Right to choose, confirm to take it</t>
+        </is>
+      </c>
+      <c r="C772" t="inlineStr">
+        <is>
+          <t>좌/우로 고르고, 확인으로 받는다</t>
+        </is>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" t="inlineStr">
+        <is>
+          <t>cards.pick.left</t>
+        </is>
+      </c>
+      <c r="B773" t="inlineStr">
+        <is>
+          <t>({n} picks left)</t>
+        </is>
+      </c>
+      <c r="C773" t="inlineStr">
+        <is>
+          <t>(남은 선택 {n}번)</t>
+        </is>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" t="inlineStr">
+        <is>
+          <t>cards.pick.skip</t>
+        </is>
+      </c>
+      <c r="B774" t="inlineStr">
+        <is>
+          <t>Skip: +{gold} gold</t>
+        </is>
+      </c>
+      <c r="C774" t="inlineStr">
+        <is>
+          <t>건너뛰기: +{gold} 골드</t>
+        </is>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" t="inlineStr">
+        <is>
+          <t>cards.pick.title</t>
+        </is>
+      </c>
+      <c r="B775" t="inlineStr">
+        <is>
+          <t>Choose a card</t>
+        </is>
+      </c>
+      <c r="C775" t="inlineStr">
+        <is>
+          <t>카드를 고르세요</t>
+        </is>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" t="inlineStr">
+        <is>
+          <t>cards.replace.keep</t>
+        </is>
+      </c>
+      <c r="B776" t="inlineStr">
+        <is>
+          <t>Keep my skills</t>
+        </is>
+      </c>
+      <c r="C776" t="inlineStr">
+        <is>
+          <t>스킬 유지</t>
+        </is>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" t="inlineStr">
+        <is>
+          <t>cards.replace.lose</t>
+        </is>
+      </c>
+      <c r="B777" t="inlineStr">
+        <is>
+          <t>Gives up: {line}</t>
+        </is>
+      </c>
+      <c r="C777" t="inlineStr">
+        <is>
+          <t>잃는 것: {line}</t>
+        </is>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" t="inlineStr">
+        <is>
+          <t>cards.replace.keep_help</t>
+        </is>
+      </c>
+      <c r="B778" t="inlineStr">
+        <is>
+          <t>Go back to the cards and choose again.</t>
+        </is>
+      </c>
+      <c r="C778" t="inlineStr">
+        <is>
+          <t>카드 화면으로 돌아가 다시 고릅니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" t="inlineStr">
+        <is>
+          <t>cards.replace.title</t>
+        </is>
+      </c>
+      <c r="B779" t="inlineStr">
+        <is>
+          <t>Learn {skill}: replace which?</t>
+        </is>
+      </c>
+      <c r="C779" t="inlineStr">
+        <is>
+          <t>{skill} 배우기: 무엇을 바꿀까요?</t>
+        </is>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" t="inlineStr">
+        <is>
+          <t>cards.stat.after</t>
+        </is>
+      </c>
+      <c r="B780" t="inlineStr">
+        <is>
+          <t>After</t>
+        </is>
+      </c>
+      <c r="C780" t="inlineStr">
+        <is>
+          <t>이후</t>
+        </is>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" t="inlineStr">
+        <is>
+          <t>cards.stat.now</t>
+        </is>
+      </c>
+      <c r="B781" t="inlineStr">
+        <is>
+          <t>Now</t>
+        </is>
+      </c>
+      <c r="C781" t="inlineStr">
+        <is>
+          <t>현재</t>
+        </is>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" t="inlineStr">
+        <is>
+          <t>cards.stat.title</t>
+        </is>
+      </c>
+      <c r="B782" t="inlineStr">
+        <is>
+          <t>Level {lvl}: place 1 point</t>
+        </is>
+      </c>
+      <c r="C782" t="inlineStr">
+        <is>
+          <t>레벨 {lvl}: 포인트 1개 배분</t>
+        </is>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" t="inlineStr">
+        <is>
+          <t>class.lbl.five</t>
+        </is>
+      </c>
+      <c r="B783" t="inlineStr">
+        <is>
+          <t>5 to find</t>
+        </is>
+      </c>
+      <c r="C783" t="inlineStr">
+        <is>
+          <t>5개 발견 가능</t>
+        </is>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" t="inlineStr">
+        <is>
+          <t>class.lbl.none</t>
+        </is>
+      </c>
+      <c r="B784" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="C784" t="inlineStr">
+        <is>
+          <t>없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" t="inlineStr">
+        <is>
+          <t>class.line.archer</t>
+        </is>
+      </c>
+      <c r="B785" t="inlineStr">
+        <is>
+          <t>Fast and sharp. High speed, poison and double shots to find.</t>
+        </is>
+      </c>
+      <c r="C785" t="inlineStr">
+        <is>
+          <t>빠르고 날카롭다. 높은 속도, 독과 연속 사격을 찾아보자.</t>
+        </is>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" t="inlineStr">
+        <is>
+          <t>class.line.knight</t>
+        </is>
+      </c>
+      <c r="B786" t="inlineStr">
+        <is>
+          <t>A sturdy fighter. Strong attack and defence, five skills to find.</t>
+        </is>
+      </c>
+      <c r="C786" t="inlineStr">
+        <is>
+          <t>듬직한 전사. 강한 공격과 방어, 찾아야 할 스킬 5개.</t>
+        </is>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" t="inlineStr">
+        <is>
+          <t>class.line.mage</t>
+        </is>
+      </c>
+      <c r="B787" t="inlineStr">
+        <is>
+          <t>A spell caster. Great magic and mana, five spells to find.</t>
+        </is>
+      </c>
+      <c r="C787" t="inlineStr">
+        <is>
+          <t>주문 시전자. 뛰어난 마법과 마나, 찾아야 할 주문 5개.</t>
+        </is>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" t="inlineStr">
+        <is>
+          <t>class.line.nobody</t>
+        </is>
+      </c>
+      <c r="B788" t="inlineStr">
+        <is>
+          <t>No skills at all. Fight with your blade, your passives and your items.</t>
+        </is>
+      </c>
+      <c r="C788" t="inlineStr">
+        <is>
+          <t>스킬이 전혀 없다. 칼, 패시브, 아이템으로 싸운다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" t="inlineStr">
+        <is>
+          <t>class.nobody.locked</t>
+        </is>
+      </c>
+      <c r="B789" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+      <c r="C789" t="inlineStr">
+        <is>
+          <t>잠김</t>
+        </is>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" t="inlineStr">
+        <is>
+          <t>class.nobody.locked_hint</t>
+        </is>
+      </c>
+      <c r="B790" t="inlineStr">
+        <is>
+          <t>Win a run to unlock this path.</t>
+        </is>
+      </c>
+      <c r="C790" t="inlineStr">
+        <is>
+          <t>한 번 승리하면 이 길이 열립니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" t="inlineStr">
+        <is>
+          <t>class.select.become</t>
+        </is>
+      </c>
+      <c r="B791" t="inlineStr">
+        <is>
+          <t>Become {cls}?</t>
+        </is>
+      </c>
+      <c r="C791" t="inlineStr">
+        <is>
+          <t>{cls}(이)가 될까요?</t>
+        </is>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" t="inlineStr">
+        <is>
+          <t>menu.common.yes</t>
+        </is>
+      </c>
+      <c r="B792" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C792" t="inlineStr">
+        <is>
+          <t>예</t>
+        </is>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" t="inlineStr">
+        <is>
+          <t>menu.common.no</t>
+        </is>
+      </c>
+      <c r="B793" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C793" t="inlineStr">
+        <is>
+          <t>아니오</t>
+        </is>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" t="inlineStr">
+        <is>
+          <t>card.pas.quick_feet.name</t>
+        </is>
+      </c>
+      <c r="B794" t="inlineStr">
+        <is>
+          <t>Quick Feet</t>
+        </is>
+      </c>
+      <c r="C794" t="inlineStr">
+        <is>
+          <t>빠른 발</t>
+        </is>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" t="inlineStr">
+        <is>
+          <t>card.pas.quick_feet.line</t>
+        </is>
+      </c>
+      <c r="B795" t="inlineStr">
+        <is>
+          <t>Light on your feet: +{n} SPD for good.</t>
+        </is>
+      </c>
+      <c r="C795" t="inlineStr">
+        <is>
+          <t>가벼운 발걸음: 영구히 SPD +{n}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" t="inlineStr">
+        <is>
+          <t>card.pas.venom_coat.name</t>
+        </is>
+      </c>
+      <c r="B796" t="inlineStr">
+        <is>
+          <t>Venom Coat</t>
+        </is>
+      </c>
+      <c r="C796" t="inlineStr">
+        <is>
+          <t>독 바르기</t>
+        </is>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" t="inlineStr">
+        <is>
+          <t>card.pas.venom_coat.line</t>
+        </is>
+      </c>
+      <c r="B797" t="inlineStr">
+        <is>
+          <t>Poison you apply lands {n} extra stack.</t>
+        </is>
+      </c>
+      <c r="C797" t="inlineStr">
+        <is>
+          <t>내가 거는 독이 {n}중첩 더 쌓인다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" t="inlineStr">
+        <is>
+          <t>card.pas.field_medic.name</t>
+        </is>
+      </c>
+      <c r="B798" t="inlineStr">
+        <is>
+          <t>Field Medic</t>
+        </is>
+      </c>
+      <c r="C798" t="inlineStr">
+        <is>
+          <t>야전 의무병</t>
+        </is>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" t="inlineStr">
+        <is>
+          <t>card.pas.field_medic.line</t>
+        </is>
+      </c>
+      <c r="B799" t="inlineStr">
+        <is>
+          <t>Heal {n} HP after each fight you win.</t>
+        </is>
+      </c>
+      <c r="C799" t="inlineStr">
+        <is>
+          <t>전투에서 이길 때마다 HP를 {n} 회복한다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" t="inlineStr">
+        <is>
+          <t>card.pas.steady_hands.name</t>
+        </is>
+      </c>
+      <c r="B800" t="inlineStr">
+        <is>
+          <t>Steady Hands</t>
+        </is>
+      </c>
+      <c r="C800" t="inlineStr">
+        <is>
+          <t>흔들림 없는 손</t>
+        </is>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" t="inlineStr">
+        <is>
+          <t>card.pas.steady_hands.line</t>
+        </is>
+      </c>
+      <c r="B801" t="inlineStr">
+        <is>
+          <t>Perfect zones are {n}% wider.</t>
+        </is>
+      </c>
+      <c r="C801" t="inlineStr">
+        <is>
+          <t>퍼펙트 구간이 {n}% 넓어진다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" t="inlineStr">
+        <is>
+          <t>card.pas.coin_sense.name</t>
+        </is>
+      </c>
+      <c r="B802" t="inlineStr">
+        <is>
+          <t>Coin Sense</t>
+        </is>
+      </c>
+      <c r="C802" t="inlineStr">
+        <is>
+          <t>돈 냄새</t>
+        </is>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" t="inlineStr">
+        <is>
+          <t>card.pas.coin_sense.line</t>
+        </is>
+      </c>
+      <c r="B803" t="inlineStr">
+        <is>
+          <t>Find {n}% more gold.</t>
+        </is>
+      </c>
+      <c r="C803" t="inlineStr">
+        <is>
+          <t>골드를 {n}% 더 얻는다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" t="inlineStr">
+        <is>
+          <t>card.pas.mana_spring.name</t>
+        </is>
+      </c>
+      <c r="B804" t="inlineStr">
+        <is>
+          <t>Mana Spring</t>
+        </is>
+      </c>
+      <c r="C804" t="inlineStr">
+        <is>
+          <t>마나의 샘</t>
+        </is>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" t="inlineStr">
+        <is>
+          <t>card.pas.mana_spring.line</t>
+        </is>
+      </c>
+      <c r="B805" t="inlineStr">
+        <is>
+          <t>Regain {n} MP at the start of each of your turns.</t>
+        </is>
+      </c>
+      <c r="C805" t="inlineStr">
+        <is>
+          <t>내 턴이 시작될 때마다 MP를 {n} 회복한다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" t="inlineStr">
+        <is>
+          <t>card.pas.potion_lore.name</t>
+        </is>
+      </c>
+      <c r="B806" t="inlineStr">
+        <is>
+          <t>Potion Lore</t>
+        </is>
+      </c>
+      <c r="C806" t="inlineStr">
+        <is>
+          <t>물약 지식</t>
+        </is>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" t="inlineStr">
+        <is>
+          <t>card.pas.potion_lore.line</t>
+        </is>
+      </c>
+      <c r="B807" t="inlineStr">
+        <is>
+          <t>Potions work {n}% better.</t>
+        </is>
+      </c>
+      <c r="C807" t="inlineStr">
+        <is>
+          <t>물약의 효과가 {n}% 커진다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" t="inlineStr">
+        <is>
+          <t>card.pas.k_iron_hide.name</t>
+        </is>
+      </c>
+      <c r="B808" t="inlineStr">
+        <is>
+          <t>Iron Hide</t>
+        </is>
+      </c>
+      <c r="C808" t="inlineStr">
+        <is>
+          <t>강철 가죽</t>
+        </is>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" t="inlineStr">
+        <is>
+          <t>card.pas.k_iron_hide.line</t>
+        </is>
+      </c>
+      <c r="B809" t="inlineStr">
+        <is>
+          <t>Thick armour sense: +{n} DEF for good.</t>
+        </is>
+      </c>
+      <c r="C809" t="inlineStr">
+        <is>
+          <t>단단한 감각: 영구히 DEF +{n}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" t="inlineStr">
+        <is>
+          <t>card.pas.k_bulwark.name</t>
+        </is>
+      </c>
+      <c r="B810" t="inlineStr">
+        <is>
+          <t>Bulwark</t>
+        </is>
+      </c>
+      <c r="C810" t="inlineStr">
+        <is>
+          <t>방벽</t>
+        </is>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" t="inlineStr">
+        <is>
+          <t>card.pas.k_bulwark.line</t>
+        </is>
+      </c>
+      <c r="B811" t="inlineStr">
+        <is>
+          <t>Guard on yourself lasts {n} turns longer.</t>
+        </is>
+      </c>
+      <c r="C811" t="inlineStr">
+        <is>
+          <t>나에게 건 방어 효과가 {n}턴 더 오래간다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" t="inlineStr">
+        <is>
+          <t>card.pas.k_heavy_hands.name</t>
+        </is>
+      </c>
+      <c r="B812" t="inlineStr">
+        <is>
+          <t>Heavy Hands</t>
+        </is>
+      </c>
+      <c r="C812" t="inlineStr">
+        <is>
+          <t>묵직한 손</t>
+        </is>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" t="inlineStr">
+        <is>
+          <t>card.pas.k_heavy_hands.line</t>
+        </is>
+      </c>
+      <c r="B813" t="inlineStr">
+        <is>
+          <t>A harder swing: +{n} ATK for good.</t>
+        </is>
+      </c>
+      <c r="C813" t="inlineStr">
+        <is>
+          <t>더 묵직한 일격: 영구히 ATK +{n}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" t="inlineStr">
+        <is>
+          <t>card.pas.a_fleet_foot.name</t>
+        </is>
+      </c>
+      <c r="B814" t="inlineStr">
+        <is>
+          <t>Fleet Foot</t>
+        </is>
+      </c>
+      <c r="C814" t="inlineStr">
+        <is>
+          <t>날랜 발</t>
+        </is>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" t="inlineStr">
+        <is>
+          <t>card.pas.a_fleet_foot.line</t>
+        </is>
+      </c>
+      <c r="B815" t="inlineStr">
+        <is>
+          <t>Quicker than the wind: +{n} SPD for good.</t>
+        </is>
+      </c>
+      <c r="C815" t="inlineStr">
+        <is>
+          <t>바람보다 빠르게: 영구히 SPD +{n}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" t="inlineStr">
+        <is>
+          <t>card.pas.a_barbed.name</t>
+        </is>
+      </c>
+      <c r="B816" t="inlineStr">
+        <is>
+          <t>Barbed Arrows</t>
+        </is>
+      </c>
+      <c r="C816" t="inlineStr">
+        <is>
+          <t>가시 화살</t>
+        </is>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" t="inlineStr">
+        <is>
+          <t>card.pas.a_barbed.line</t>
+        </is>
+      </c>
+      <c r="B817" t="inlineStr">
+        <is>
+          <t>Your damage skills hit for {n} more power.</t>
+        </is>
+      </c>
+      <c r="C817" t="inlineStr">
+        <is>
+          <t>내 공격 스킬의 위력이 {n} 높아진다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" t="inlineStr">
+        <is>
+          <t>card.pas.a_second_wind.name</t>
+        </is>
+      </c>
+      <c r="B818" t="inlineStr">
+        <is>
+          <t>Second Wind</t>
+        </is>
+      </c>
+      <c r="C818" t="inlineStr">
+        <is>
+          <t>두 번째 숨</t>
+        </is>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" t="inlineStr">
+        <is>
+          <t>card.pas.a_second_wind.line</t>
+        </is>
+      </c>
+      <c r="B819" t="inlineStr">
+        <is>
+          <t>Regain {n} MP after each fight you win.</t>
+        </is>
+      </c>
+      <c r="C819" t="inlineStr">
+        <is>
+          <t>전투에서 이길 때마다 MP를 {n} 회복한다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" t="inlineStr">
+        <is>
+          <t>card.pas.m_arcane_well.name</t>
+        </is>
+      </c>
+      <c r="B820" t="inlineStr">
+        <is>
+          <t>Arcane Well</t>
+        </is>
+      </c>
+      <c r="C820" t="inlineStr">
+        <is>
+          <t>비전의 샘</t>
+        </is>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" t="inlineStr">
+        <is>
+          <t>card.pas.m_arcane_well.line</t>
+        </is>
+      </c>
+      <c r="B821" t="inlineStr">
+        <is>
+          <t>A deeper well: +{n} MAG for good.</t>
+        </is>
+      </c>
+      <c r="C821" t="inlineStr">
+        <is>
+          <t>더 깊은 샘: 영구히 MAG +{n}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" t="inlineStr">
+        <is>
+          <t>card.pas.m_spellweave.name</t>
+        </is>
+      </c>
+      <c r="B822" t="inlineStr">
+        <is>
+          <t>Spellweave</t>
+        </is>
+      </c>
+      <c r="C822" t="inlineStr">
+        <is>
+          <t>주문 엮기</t>
+        </is>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" t="inlineStr">
+        <is>
+          <t>card.pas.m_spellweave.line</t>
+        </is>
+      </c>
+      <c r="B823" t="inlineStr">
+        <is>
+          <t>Your skills cost {n} MP less (never below 1).</t>
+        </is>
+      </c>
+      <c r="C823" t="inlineStr">
+        <is>
+          <t>스킬의 MP 소모가 {n} 줄어든다 (최소 1).</t>
+        </is>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" t="inlineStr">
+        <is>
+          <t>card.pas.m_cold_focus.name</t>
+        </is>
+      </c>
+      <c r="B824" t="inlineStr">
+        <is>
+          <t>Cold Focus</t>
+        </is>
+      </c>
+      <c r="C824" t="inlineStr">
+        <is>
+          <t>차가운 집중</t>
+        </is>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" t="inlineStr">
+        <is>
+          <t>card.pas.m_cold_focus.line</t>
+        </is>
+      </c>
+      <c r="B825" t="inlineStr">
+        <is>
+          <t>Statuses you inflict last {n} turn longer.</t>
+        </is>
+      </c>
+      <c r="C825" t="inlineStr">
+        <is>
+          <t>내가 거는 상태 이상이 {n}턴 더 오래간다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" t="inlineStr">
+        <is>
+          <t>card.pas.n_tonic.name</t>
+        </is>
+      </c>
+      <c r="B826" t="inlineStr">
+        <is>
+          <t>Tonic Blend</t>
+        </is>
+      </c>
+      <c r="C826" t="inlineStr">
+        <is>
+          <t>강장제 배합</t>
+        </is>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" t="inlineStr">
+        <is>
+          <t>card.pas.n_tonic.line</t>
+        </is>
+      </c>
+      <c r="B827" t="inlineStr">
+        <is>
+          <t>Healing potions also restore {n} MP.</t>
+        </is>
+      </c>
+      <c r="C827" t="inlineStr">
+        <is>
+          <t>회복 물약이 MP도 {n} 회복시킨다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" t="inlineStr">
+        <is>
+          <t>card.pas.n_apothecary.name</t>
+        </is>
+      </c>
+      <c r="B828" t="inlineStr">
+        <is>
+          <t>Apothecary</t>
+        </is>
+      </c>
+      <c r="C828" t="inlineStr">
+        <is>
+          <t>약제사</t>
+        </is>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" t="inlineStr">
+        <is>
+          <t>card.pas.n_apothecary.line</t>
+        </is>
+      </c>
+      <c r="B829" t="inlineStr">
+        <is>
+          <t>Potions work {n}% better.</t>
+        </is>
+      </c>
+      <c r="C829" t="inlineStr">
+        <is>
+          <t>물약의 효과가 {n}% 커진다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" t="inlineStr">
+        <is>
+          <t>card.pas.n_scrounger.name</t>
+        </is>
+      </c>
+      <c r="B830" t="inlineStr">
+        <is>
+          <t>Scrounger</t>
+        </is>
+      </c>
+      <c r="C830" t="inlineStr">
+        <is>
+          <t>주워 모으는 자</t>
+        </is>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" t="inlineStr">
+        <is>
+          <t>card.pas.n_scrounger.line</t>
+        </is>
+      </c>
+      <c r="B831" t="inlineStr">
+        <is>
+          <t>{n}% chance to find a potion after each fight you win.</t>
+        </is>
+      </c>
+      <c r="C831" t="inlineStr">
+        <is>
+          <t>전투에서 이길 때마다 {n}% 확률로 물약을 줍는다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" t="inlineStr">
+        <is>
+          <t>card.fb.rest.name</t>
+        </is>
+      </c>
+      <c r="B832" t="inlineStr">
+        <is>
+          <t>Second Breath</t>
+        </is>
+      </c>
+      <c r="C832" t="inlineStr">
+        <is>
+          <t>숨 고르기</t>
+        </is>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" t="inlineStr">
+        <is>
+          <t>card.fb.rest.line</t>
+        </is>
+      </c>
+      <c r="B833" t="inlineStr">
+        <is>
+          <t>Restore {n}% of your HP and MP now.</t>
+        </is>
+      </c>
+      <c r="C833" t="inlineStr">
+        <is>
+          <t>지금 HP와 MP를 {n}% 회복한다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" t="inlineStr">
+        <is>
+          <t>card.fb.gold.name</t>
+        </is>
+      </c>
+      <c r="B834" t="inlineStr">
+        <is>
+          <t>Coin Purse</t>
+        </is>
+      </c>
+      <c r="C834" t="inlineStr">
+        <is>
+          <t>동전 주머니</t>
+        </is>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" t="inlineStr">
+        <is>
+          <t>card.fb.gold.line</t>
+        </is>
+      </c>
+      <c r="B835" t="inlineStr">
+        <is>
+          <t>Take {n} gold.</t>
+        </is>
+      </c>
+      <c r="C835" t="inlineStr">
+        <is>
+          <t>골드 {n}을 얻는다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" t="inlineStr">
+        <is>
+          <t>card.fb.focus.name</t>
+        </is>
+      </c>
+      <c r="B836" t="inlineStr">
+        <is>
+          <t>Whetstone</t>
+        </is>
+      </c>
+      <c r="C836" t="inlineStr">
+        <is>
+          <t>숫돌</t>
+        </is>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" t="inlineStr">
+        <is>
+          <t>card.fb.focus.line</t>
+        </is>
+      </c>
+      <c r="B837" t="inlineStr">
+        <is>
+          <t>Your main stat grows by {n} for good.</t>
+        </is>
+      </c>
+      <c r="C837" t="inlineStr">
+        <is>
+          <t>주력 능력치가 영구히 {n} 오른다.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C678"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(story): death scene with tiered lines, wake line, boss banner, lore notes, closing text and credits (packet C5)
Co-Authored-By: Claude Sonnet <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datafiles/localization/game_text.xlsx
+++ b/datafiles/localization/game_text.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C731"/>
+  <dimension ref="A1:C812"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -3117,12 +3117,12 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>This was around 2 months of development, and I'm glad you were able to get through our prototype story.</t>
+          <t>We're glad you made it all the way to the end.</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>이 게임은 약 2개월 동안 개발되었고, 여러분이 우리의 프로토타입 스토리를 끝까지 플레이해 주셔서 정말 기쁩니다.</t>
+          <t>끝까지 함께해 주셔서 정말 기쁩니다.</t>
         </is>
       </c>
     </row>
@@ -12847,6 +12847,1383 @@
       <c r="C731" t="inlineStr">
         <is>
           <t>이전 버전의 저장 파일은 이 버전에서 불러올 수 없습니다. 파일은 그대로 두었습니다. 새 도전을 시작하세요.</t>
+        </is>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" t="inlineStr">
+        <is>
+          <t>death.t1.0</t>
+        </is>
+      </c>
+      <c r="B732" t="inlineStr">
+        <is>
+          <t>The dark takes you. Quietly.</t>
+        </is>
+      </c>
+      <c r="C732" t="inlineStr">
+        <is>
+          <t>어둠이 당신을 조용히 데려간다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" t="inlineStr">
+        <is>
+          <t>death.t1.1</t>
+        </is>
+      </c>
+      <c r="B733" t="inlineStr">
+        <is>
+          <t>So this is how it ends.</t>
+        </is>
+      </c>
+      <c r="C733" t="inlineStr">
+        <is>
+          <t>결국 이렇게 끝나는구나.</t>
+        </is>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" t="inlineStr">
+        <is>
+          <t>death.t1.2</t>
+        </is>
+      </c>
+      <c r="B734" t="inlineStr">
+        <is>
+          <t>The floor gives way beneath you.</t>
+        </is>
+      </c>
+      <c r="C734" t="inlineStr">
+        <is>
+          <t>발밑의 바닥이 꺼진다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" t="inlineStr">
+        <is>
+          <t>death.t2.0</t>
+        </is>
+      </c>
+      <c r="B735" t="inlineStr">
+        <is>
+          <t>You were sure that was the end.</t>
+        </is>
+      </c>
+      <c r="C735" t="inlineStr">
+        <is>
+          <t>분명 이게 끝이라고 생각했다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" t="inlineStr">
+        <is>
+          <t>death.t2.1</t>
+        </is>
+      </c>
+      <c r="B736" t="inlineStr">
+        <is>
+          <t>The tunnel is not finished with you.</t>
+        </is>
+      </c>
+      <c r="C736" t="inlineStr">
+        <is>
+          <t>터널은 아직 당신을 놓아주지 않는다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" t="inlineStr">
+        <is>
+          <t>death.t2.2</t>
+        </is>
+      </c>
+      <c r="B737" t="inlineStr">
+        <is>
+          <t>Cold stone. A fall. Again.</t>
+        </is>
+      </c>
+      <c r="C737" t="inlineStr">
+        <is>
+          <t>차가운 돌. 추락. 또다시.</t>
+        </is>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" t="inlineStr">
+        <is>
+          <t>death.t3.0</t>
+        </is>
+      </c>
+      <c r="B738" t="inlineStr">
+        <is>
+          <t>You know this fall by heart now.</t>
+        </is>
+      </c>
+      <c r="C738" t="inlineStr">
+        <is>
+          <t>이 추락은 이제 눈 감고도 안다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" t="inlineStr">
+        <is>
+          <t>death.t3.1</t>
+        </is>
+      </c>
+      <c r="B739" t="inlineStr">
+        <is>
+          <t>How many times has it been?</t>
+        </is>
+      </c>
+      <c r="C739" t="inlineStr">
+        <is>
+          <t>벌써 몇 번째일까?</t>
+        </is>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" t="inlineStr">
+        <is>
+          <t>death.t3.2</t>
+        </is>
+      </c>
+      <c r="B740" t="inlineStr">
+        <is>
+          <t>Dying is starting to feel like routine.</t>
+        </is>
+      </c>
+      <c r="C740" t="inlineStr">
+        <is>
+          <t>죽는 일이 일상처럼 느껴지기 시작한다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" t="inlineStr">
+        <is>
+          <t>death.t4.0</t>
+        </is>
+      </c>
+      <c r="B741" t="inlineStr">
+        <is>
+          <t>You stopped counting. The walls didn't.</t>
+        </is>
+      </c>
+      <c r="C741" t="inlineStr">
+        <is>
+          <t>세는 건 그만뒀다. 벽은 아니었다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" t="inlineStr">
+        <is>
+          <t>death.t4.1</t>
+        </is>
+      </c>
+      <c r="B742" t="inlineStr">
+        <is>
+          <t>{killer}. You don't even flinch anymore.</t>
+        </is>
+      </c>
+      <c r="C742" t="inlineStr">
+        <is>
+          <t>{killer}. 이제 놀라지도 않는다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" t="inlineStr">
+        <is>
+          <t>death.t4.2</t>
+        </is>
+      </c>
+      <c r="B743" t="inlineStr">
+        <is>
+          <t>Nobody is coming. Nobody ever did.</t>
+        </is>
+      </c>
+      <c r="C743" t="inlineStr">
+        <is>
+          <t>아무도 오지 않는다. 한 번도 온 적 없다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" t="inlineStr">
+        <is>
+          <t>death.t5.0</t>
+        </is>
+      </c>
+      <c r="B744" t="inlineStr">
+        <is>
+          <t>Even wanting to leave has gone quiet.</t>
+        </is>
+      </c>
+      <c r="C744" t="inlineStr">
+        <is>
+          <t>떠나고 싶다는 마음마저 조용해졌다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" t="inlineStr">
+        <is>
+          <t>death.t5.1</t>
+        </is>
+      </c>
+      <c r="B745" t="inlineStr">
+        <is>
+          <t>{killer}. Of course it was.</t>
+        </is>
+      </c>
+      <c r="C745" t="inlineStr">
+        <is>
+          <t>{killer}. 역시 그랬다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" t="inlineStr">
+        <is>
+          <t>death.t5.2</t>
+        </is>
+      </c>
+      <c r="B746" t="inlineStr">
+        <is>
+          <t>Down here, at least, you know what to expect.</t>
+        </is>
+      </c>
+      <c r="C746" t="inlineStr">
+        <is>
+          <t>적어도 여기서는 무엇이 올지 안다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" t="inlineStr">
+        <is>
+          <t>death.killer.enemy_slime</t>
+        </is>
+      </c>
+      <c r="B747" t="inlineStr">
+        <is>
+          <t>A slime. You were beaten by a slime.</t>
+        </is>
+      </c>
+      <c r="C747" t="inlineStr">
+        <is>
+          <t>고작 더러운 것에게 당했다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" t="inlineStr">
+        <is>
+          <t>death.killer.enemy_direwolf</t>
+        </is>
+      </c>
+      <c r="B748" t="inlineStr">
+        <is>
+          <t>The wolf was faster than your fear.</t>
+        </is>
+      </c>
+      <c r="C748" t="inlineStr">
+        <is>
+          <t>늑대는 당신의 두려움보다 빨랐다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" t="inlineStr">
+        <is>
+          <t>death.killer.enemy_ghostsword</t>
+        </is>
+      </c>
+      <c r="B749" t="inlineStr">
+        <is>
+          <t>A blade with no hand to hold it.</t>
+        </is>
+      </c>
+      <c r="C749" t="inlineStr">
+        <is>
+          <t>손도 없이 휘둘러지는 검.</t>
+        </is>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" t="inlineStr">
+        <is>
+          <t>death.killer.enemy_spider</t>
+        </is>
+      </c>
+      <c r="B750" t="inlineStr">
+        <is>
+          <t>Eight eyes. The last thing you saw.</t>
+        </is>
+      </c>
+      <c r="C750" t="inlineStr">
+        <is>
+          <t>여덟 개의 눈. 마지막으로 본 것.</t>
+        </is>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" t="inlineStr">
+        <is>
+          <t>death.killer.enemy_madwhisp</t>
+        </is>
+      </c>
+      <c r="B751" t="inlineStr">
+        <is>
+          <t>The glow led you here. It always does.</t>
+        </is>
+      </c>
+      <c r="C751" t="inlineStr">
+        <is>
+          <t>그 빛이 여기까지 이끌었다. 언제나 그렇다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" t="inlineStr">
+        <is>
+          <t>death.killer.enemy_snake</t>
+        </is>
+      </c>
+      <c r="B752" t="inlineStr">
+        <is>
+          <t>A hiss. Then nothing.</t>
+        </is>
+      </c>
+      <c r="C752" t="inlineStr">
+        <is>
+          <t>쉬익. 그리고 아무것도 없다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" t="inlineStr">
+        <is>
+          <t>death.killer.enemy_killer_plant</t>
+        </is>
+      </c>
+      <c r="B753" t="inlineStr">
+        <is>
+          <t>Even the plants here want you gone.</t>
+        </is>
+      </c>
+      <c r="C753" t="inlineStr">
+        <is>
+          <t>여기선 식물조차 당신을 죽이려 든다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" t="inlineStr">
+        <is>
+          <t>death.killer.enemy_stranger</t>
+        </is>
+      </c>
+      <c r="B754" t="inlineStr">
+        <is>
+          <t>The stranger smiled the whole time.</t>
+        </is>
+      </c>
+      <c r="C754" t="inlineStr">
+        <is>
+          <t>낯선 이는 내내 웃고 있었다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" t="inlineStr">
+        <is>
+          <t>death.killer.enemy_mini_boss</t>
+        </is>
+      </c>
+      <c r="B755" t="inlineStr">
+        <is>
+          <t>{killer} did not even slow down.</t>
+        </is>
+      </c>
+      <c r="C755" t="inlineStr">
+        <is>
+          <t>{killer}은(는) 속도조차 늦추지 않았다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" t="inlineStr">
+        <is>
+          <t>death.killer.enemy_final_boss</t>
+        </is>
+      </c>
+      <c r="B756" t="inlineStr">
+        <is>
+          <t>The choir sings. You were its last note.</t>
+        </is>
+      </c>
+      <c r="C756" t="inlineStr">
+        <is>
+          <t>성가대가 노래한다. 당신은 그 마지막 음이었다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" t="inlineStr">
+        <is>
+          <t>death.killer.status_poison</t>
+        </is>
+      </c>
+      <c r="B757" t="inlineStr">
+        <is>
+          <t>The poison finished what the fight began.</t>
+        </is>
+      </c>
+      <c r="C757" t="inlineStr">
+        <is>
+          <t>독이 싸움이 남긴 일을 끝냈다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" t="inlineStr">
+        <is>
+          <t>death.killer.status_burn</t>
+        </is>
+      </c>
+      <c r="B758" t="inlineStr">
+        <is>
+          <t>The fire was warm, at least.</t>
+        </is>
+      </c>
+      <c r="C758" t="inlineStr">
+        <is>
+          <t>적어도 불은 따뜻했다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" t="inlineStr">
+        <is>
+          <t>death.killer.status_bleed</t>
+        </is>
+      </c>
+      <c r="B759" t="inlineStr">
+        <is>
+          <t>You bled out, counting the drops.</t>
+        </is>
+      </c>
+      <c r="C759" t="inlineStr">
+        <is>
+          <t>방울을 세며 피를 흘렸다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" t="inlineStr">
+        <is>
+          <t>death.killer.abandoned</t>
+        </is>
+      </c>
+      <c r="B760" t="inlineStr">
+        <is>
+          <t>You let go. The tunnel did not mind.</t>
+        </is>
+      </c>
+      <c r="C760" t="inlineStr">
+        <is>
+          <t>당신은 손을 놓았다. 터널은 개의치 않았다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" t="inlineStr">
+        <is>
+          <t>death.killer.unknown_name</t>
+        </is>
+      </c>
+      <c r="B761" t="inlineStr">
+        <is>
+          <t>Something</t>
+        </is>
+      </c>
+      <c r="C761" t="inlineStr">
+        <is>
+          <t>무언가</t>
+        </is>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" t="inlineStr">
+        <is>
+          <t>wake.t1</t>
+        </is>
+      </c>
+      <c r="B762" t="inlineStr">
+        <is>
+          <t>You wake where you first fell. Alive.</t>
+        </is>
+      </c>
+      <c r="C762" t="inlineStr">
+        <is>
+          <t>처음 떨어진 곳에서 눈을 뜬다. 살아 있다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" t="inlineStr">
+        <is>
+          <t>wake.t2</t>
+        </is>
+      </c>
+      <c r="B763" t="inlineStr">
+        <is>
+          <t>The same stone. The same cold. You wake again.</t>
+        </is>
+      </c>
+      <c r="C763" t="inlineStr">
+        <is>
+          <t>같은 돌바닥. 같은 냉기. 다시 눈을 뜬다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" t="inlineStr">
+        <is>
+          <t>wake.t3</t>
+        </is>
+      </c>
+      <c r="B764" t="inlineStr">
+        <is>
+          <t>You wake at the entrance. It almost feels like home.</t>
+        </is>
+      </c>
+      <c r="C764" t="inlineStr">
+        <is>
+          <t>입구에서 눈을 뜬다. 어쩐지 집처럼 느껴진다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" t="inlineStr">
+        <is>
+          <t>wake.t4</t>
+        </is>
+      </c>
+      <c r="B765" t="inlineStr">
+        <is>
+          <t>You wake. You no longer ask why.</t>
+        </is>
+      </c>
+      <c r="C765" t="inlineStr">
+        <is>
+          <t>눈을 뜬다. 더는 이유를 묻지 않는다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" t="inlineStr">
+        <is>
+          <t>runflow.sum.floor</t>
+        </is>
+      </c>
+      <c r="B766" t="inlineStr">
+        <is>
+          <t>Floor reached</t>
+        </is>
+      </c>
+      <c r="C766" t="inlineStr">
+        <is>
+          <t>도달한 층</t>
+        </is>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" t="inlineStr">
+        <is>
+          <t>runflow.sum.class</t>
+        </is>
+      </c>
+      <c r="B767" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="C767" t="inlineStr">
+        <is>
+          <t>직업</t>
+        </is>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" t="inlineStr">
+        <is>
+          <t>runflow.sum.level</t>
+        </is>
+      </c>
+      <c r="B768" t="inlineStr">
+        <is>
+          <t>Level</t>
+        </is>
+      </c>
+      <c r="C768" t="inlineStr">
+        <is>
+          <t>레벨</t>
+        </is>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" t="inlineStr">
+        <is>
+          <t>runflow.sum.kills</t>
+        </is>
+      </c>
+      <c r="B769" t="inlineStr">
+        <is>
+          <t>Foes beaten</t>
+        </is>
+      </c>
+      <c r="C769" t="inlineStr">
+        <is>
+          <t>쓰러뜨린 적</t>
+        </is>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" t="inlineStr">
+        <is>
+          <t>runflow.sum.falls</t>
+        </is>
+      </c>
+      <c r="B770" t="inlineStr">
+        <is>
+          <t>Falls so far</t>
+        </is>
+      </c>
+      <c r="C770" t="inlineStr">
+        <is>
+          <t>지금까지 추락</t>
+        </is>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" t="inlineStr">
+        <is>
+          <t>note.map_page.title</t>
+        </is>
+      </c>
+      <c r="B771" t="inlineStr">
+        <is>
+          <t>Torn survey page</t>
+        </is>
+      </c>
+      <c r="C771" t="inlineStr">
+        <is>
+          <t>찢어진 측량 기록</t>
+        </is>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" t="inlineStr">
+        <is>
+          <t>note.map_page.0</t>
+        </is>
+      </c>
+      <c r="B772" t="inlineStr">
+        <is>
+          <t>A page torn from a survey book. Your handwriting.</t>
+        </is>
+      </c>
+      <c r="C772" t="inlineStr">
+        <is>
+          <t>측량 수첩에서 뜯긴 한 장. 당신의 필체다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" t="inlineStr">
+        <is>
+          <t>note.map_page.1</t>
+        </is>
+      </c>
+      <c r="B773" t="inlineStr">
+        <is>
+          <t>"No tunnel here. Not on any map I ever drew."</t>
+        </is>
+      </c>
+      <c r="C773" t="inlineStr">
+        <is>
+          <t>"이곳에 터널은 없다. 내가 그린 어떤 지도에도."</t>
+        </is>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" t="inlineStr">
+        <is>
+          <t>note.map_page.2</t>
+        </is>
+      </c>
+      <c r="B774" t="inlineStr">
+        <is>
+          <t>The ink still looks wet. You don't remember writing it.</t>
+        </is>
+      </c>
+      <c r="C774" t="inlineStr">
+        <is>
+          <t>잉크가 아직 젖어 있다. 쓴 기억은 없다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" t="inlineStr">
+        <is>
+          <t>note.wall_breath.title</t>
+        </is>
+      </c>
+      <c r="B775" t="inlineStr">
+        <is>
+          <t>Wall scratches</t>
+        </is>
+      </c>
+      <c r="C775" t="inlineStr">
+        <is>
+          <t>벽의 긁힌 자국</t>
+        </is>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" t="inlineStr">
+        <is>
+          <t>note.wall_breath.0</t>
+        </is>
+      </c>
+      <c r="B776" t="inlineStr">
+        <is>
+          <t>Scratched deep into the stone, slowly and carefully:</t>
+        </is>
+      </c>
+      <c r="C776" t="inlineStr">
+        <is>
+          <t>돌에 깊고 신중하게 새겨져 있다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" t="inlineStr">
+        <is>
+          <t>note.wall_breath.1</t>
+        </is>
+      </c>
+      <c r="B777" t="inlineStr">
+        <is>
+          <t>"It breathes. Hold still and you can feel it."</t>
+        </is>
+      </c>
+      <c r="C777" t="inlineStr">
+        <is>
+          <t>"숨을 쉰다. 가만히 있으면 느껴진다."</t>
+        </is>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" t="inlineStr">
+        <is>
+          <t>note.wall_breath.2</t>
+        </is>
+      </c>
+      <c r="B778" t="inlineStr">
+        <is>
+          <t>"Every step goes deeper. None of them go back."</t>
+        </is>
+      </c>
+      <c r="C778" t="inlineStr">
+        <is>
+          <t>"한 걸음마다 더 깊어진다. 돌아가는 길은 없다."</t>
+        </is>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" t="inlineStr">
+        <is>
+          <t>note.lost_others.title</t>
+        </is>
+      </c>
+      <c r="B779" t="inlineStr">
+        <is>
+          <t>Unfinished letter</t>
+        </is>
+      </c>
+      <c r="C779" t="inlineStr">
+        <is>
+          <t>쓰다 만 편지</t>
+        </is>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" t="inlineStr">
+        <is>
+          <t>note.lost_others.0</t>
+        </is>
+      </c>
+      <c r="B780" t="inlineStr">
+        <is>
+          <t>A letter that stops in the middle of a sentence.</t>
+        </is>
+      </c>
+      <c r="C780" t="inlineStr">
+        <is>
+          <t>문장 중간에서 끊긴 편지.</t>
+        </is>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" t="inlineStr">
+        <is>
+          <t>note.lost_others.1</t>
+        </is>
+      </c>
+      <c r="B781" t="inlineStr">
+        <is>
+          <t>"The others went ahead. Or I did. I can't tell anymore."</t>
+        </is>
+      </c>
+      <c r="C781" t="inlineStr">
+        <is>
+          <t>"다른 이들이 먼저 갔다. 아니면 내가. 이제 모르겠다."</t>
+        </is>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" t="inlineStr">
+        <is>
+          <t>note.lost_others.2</t>
+        </is>
+      </c>
+      <c r="B782" t="inlineStr">
+        <is>
+          <t>"I keep calling for them. Only the walls answer."</t>
+        </is>
+      </c>
+      <c r="C782" t="inlineStr">
+        <is>
+          <t>"계속 불러보지만 벽만 대답한다."</t>
+        </is>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" t="inlineStr">
+        <is>
+          <t>note.carved_arrow.title</t>
+        </is>
+      </c>
+      <c r="B783" t="inlineStr">
+        <is>
+          <t>Carved arrow</t>
+        </is>
+      </c>
+      <c r="C783" t="inlineStr">
+        <is>
+          <t>새겨진 화살표</t>
+        </is>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" t="inlineStr">
+        <is>
+          <t>note.carved_arrow.0</t>
+        </is>
+      </c>
+      <c r="B784" t="inlineStr">
+        <is>
+          <t>An arrow is carved here, pointing up.</t>
+        </is>
+      </c>
+      <c r="C784" t="inlineStr">
+        <is>
+          <t>위쪽을 가리키는 화살표가 새겨져 있다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" t="inlineStr">
+        <is>
+          <t>note.carved_arrow.1</t>
+        </is>
+      </c>
+      <c r="B785" t="inlineStr">
+        <is>
+          <t>Someone crossed it out. Beneath it, one word:</t>
+        </is>
+      </c>
+      <c r="C785" t="inlineStr">
+        <is>
+          <t>누군가 그 위에 줄을 긋고, 아래에 한 단어를 남겼다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" t="inlineStr">
+        <is>
+          <t>note.carved_arrow.2</t>
+        </is>
+      </c>
+      <c r="B786" t="inlineStr">
+        <is>
+          <t>"Don't."</t>
+        </is>
+      </c>
+      <c r="C786" t="inlineStr">
+        <is>
+          <t>"가지 마."</t>
+        </is>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" t="inlineStr">
+        <is>
+          <t>note.three_marks.title</t>
+        </is>
+      </c>
+      <c r="B787" t="inlineStr">
+        <is>
+          <t>Three marks</t>
+        </is>
+      </c>
+      <c r="C787" t="inlineStr">
+        <is>
+          <t>세 줄의 흔적</t>
+        </is>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" t="inlineStr">
+        <is>
+          <t>note.three_marks.0</t>
+        </is>
+      </c>
+      <c r="B788" t="inlineStr">
+        <is>
+          <t>Three short scratches in the stone.</t>
+        </is>
+      </c>
+      <c r="C788" t="inlineStr">
+        <is>
+          <t>돌에 짧은 긁힘이 세 개 있다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" t="inlineStr">
+        <is>
+          <t>note.three_marks.1</t>
+        </is>
+      </c>
+      <c r="B789" t="inlineStr">
+        <is>
+          <t>You made these. You don't remember making them.</t>
+        </is>
+      </c>
+      <c r="C789" t="inlineStr">
+        <is>
+          <t>당신이 새긴 것이다. 새긴 기억은 없다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" t="inlineStr">
+        <is>
+          <t>note.mapmaker_scrap.title</t>
+        </is>
+      </c>
+      <c r="B790" t="inlineStr">
+        <is>
+          <t>Mapmaker's scrap</t>
+        </is>
+      </c>
+      <c r="C790" t="inlineStr">
+        <is>
+          <t>지도 제작자의 쪽지</t>
+        </is>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" t="inlineStr">
+        <is>
+          <t>note.mapmaker_scrap.0</t>
+        </is>
+      </c>
+      <c r="B791" t="inlineStr">
+        <is>
+          <t>A scrap of paper in your own hand:</t>
+        </is>
+      </c>
+      <c r="C791" t="inlineStr">
+        <is>
+          <t>당신의 필체로 쓰인 쪽지.</t>
+        </is>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" t="inlineStr">
+        <is>
+          <t>note.mapmaker_scrap.1</t>
+        </is>
+      </c>
+      <c r="B792" t="inlineStr">
+        <is>
+          <t>"The fall was no accident. It wanted a mapmaker."</t>
+        </is>
+      </c>
+      <c r="C792" t="inlineStr">
+        <is>
+          <t>"추락은 사고가 아니었다. 터널은 지도 제작자를 원했다."</t>
+        </is>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" t="inlineStr">
+        <is>
+          <t>note.mapmaker_scrap.2</t>
+        </is>
+      </c>
+      <c r="B793" t="inlineStr">
+        <is>
+          <t>"Someone who would map it, and come back to map it again."</t>
+        </is>
+      </c>
+      <c r="C793" t="inlineStr">
+        <is>
+          <t>"그리고 돌아와서 다시 지도를 그릴 사람을."</t>
+        </is>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" t="inlineStr">
+        <is>
+          <t>note.six_marks.title</t>
+        </is>
+      </c>
+      <c r="B794" t="inlineStr">
+        <is>
+          <t>Six marks</t>
+        </is>
+      </c>
+      <c r="C794" t="inlineStr">
+        <is>
+          <t>여섯 줄의 흔적</t>
+        </is>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" t="inlineStr">
+        <is>
+          <t>note.six_marks.0</t>
+        </is>
+      </c>
+      <c r="B795" t="inlineStr">
+        <is>
+          <t>Six scratches in a row, tidy as a ledger.</t>
+        </is>
+      </c>
+      <c r="C795" t="inlineStr">
+        <is>
+          <t>장부처럼 가지런한 긁힘 여섯 개.</t>
+        </is>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" t="inlineStr">
+        <is>
+          <t>note.six_marks.1</t>
+        </is>
+      </c>
+      <c r="B796" t="inlineStr">
+        <is>
+          <t>Beside them, in a shakier hand: "Stop counting."</t>
+        </is>
+      </c>
+      <c r="C796" t="inlineStr">
+        <is>
+          <t>그 옆에 떨리는 필체로: "세지 마."</t>
+        </is>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" t="inlineStr">
+        <is>
+          <t>note.six_marks.2</t>
+        </is>
+      </c>
+      <c r="B797" t="inlineStr">
+        <is>
+          <t>"It only counts you back."</t>
+        </is>
+      </c>
+      <c r="C797" t="inlineStr">
+        <is>
+          <t>"세면, 터널도 너를 센다."</t>
+        </is>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" t="inlineStr">
+        <is>
+          <t>note.wall_of_marks.title</t>
+        </is>
+      </c>
+      <c r="B798" t="inlineStr">
+        <is>
+          <t>A wall of marks</t>
+        </is>
+      </c>
+      <c r="C798" t="inlineStr">
+        <is>
+          <t>흔적으로 가득한 벽</t>
+        </is>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" t="inlineStr">
+        <is>
+          <t>note.wall_of_marks.0</t>
+        </is>
+      </c>
+      <c r="B799" t="inlineStr">
+        <is>
+          <t>Ten scratches. Then more, far older than yours.</t>
+        </is>
+      </c>
+      <c r="C799" t="inlineStr">
+        <is>
+          <t>긁힘 열 개. 그 너머로 훨씬 오래된 자국들.</t>
+        </is>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" t="inlineStr">
+        <is>
+          <t>note.wall_of_marks.1</t>
+        </is>
+      </c>
+      <c r="B800" t="inlineStr">
+        <is>
+          <t>Some are in other hands.</t>
+        </is>
+      </c>
+      <c r="C800" t="inlineStr">
+        <is>
+          <t>일부는 다른 사람의 손길이다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" t="inlineStr">
+        <is>
+          <t>note.wall_of_marks.2</t>
+        </is>
+      </c>
+      <c r="B801" t="inlineStr">
+        <is>
+          <t>You are not the first to wake down here.</t>
+        </is>
+      </c>
+      <c r="C801" t="inlineStr">
+        <is>
+          <t>여기서 눈을 뜬 사람은 당신이 처음이 아니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" t="inlineStr">
+        <is>
+          <t>credits.title</t>
+        </is>
+      </c>
+      <c r="B802" t="inlineStr">
+        <is>
+          <t>NO HOPE</t>
+        </is>
+      </c>
+      <c r="C802" t="inlineStr">
+        <is>
+          <t>NO HOPE</t>
+        </is>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" t="inlineStr">
+        <is>
+          <t>credits.game_by</t>
+        </is>
+      </c>
+      <c r="B803" t="inlineStr">
+        <is>
+          <t>Game and art by PaleRook</t>
+        </is>
+      </c>
+      <c r="C803" t="inlineStr">
+        <is>
+          <t>게임과 그림: PaleRook</t>
+        </is>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" t="inlineStr">
+        <is>
+          <t>credits.fonts</t>
+        </is>
+      </c>
+      <c r="B804" t="inlineStr">
+        <is>
+          <t>Fonts</t>
+        </is>
+      </c>
+      <c r="C804" t="inlineStr">
+        <is>
+          <t>글꼴</t>
+        </is>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" t="inlineStr">
+        <is>
+          <t>credits.font_galmuri</t>
+        </is>
+      </c>
+      <c r="B805" t="inlineStr">
+        <is>
+          <t>Galmuri by Lee Minseo (OFL-1.1)</t>
+        </is>
+      </c>
+      <c r="C805" t="inlineStr">
+        <is>
+          <t>Galmuri - Lee Minseo (OFL-1.1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" t="inlineStr">
+        <is>
+          <t>credits.font_pixel</t>
+        </is>
+      </c>
+      <c r="B806" t="inlineStr">
+        <is>
+          <t>Retro Gaming pixel font</t>
+        </is>
+      </c>
+      <c r="C806" t="inlineStr">
+        <is>
+          <t>Retro Gaming 픽셀 글꼴</t>
+        </is>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" t="inlineStr">
+        <is>
+          <t>credits.tools</t>
+        </is>
+      </c>
+      <c r="B807" t="inlineStr">
+        <is>
+          <t>Tools</t>
+        </is>
+      </c>
+      <c r="C807" t="inlineStr">
+        <is>
+          <t>도구</t>
+        </is>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" t="inlineStr">
+        <is>
+          <t>credits.tool_gamemaker</t>
+        </is>
+      </c>
+      <c r="B808" t="inlineStr">
+        <is>
+          <t>Made with GameMaker</t>
+        </is>
+      </c>
+      <c r="C808" t="inlineStr">
+        <is>
+          <t>GameMaker로 제작</t>
+        </is>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" t="inlineStr">
+        <is>
+          <t>credits.sounds</t>
+        </is>
+      </c>
+      <c r="B809" t="inlineStr">
+        <is>
+          <t>Sound and music</t>
+        </is>
+      </c>
+      <c r="C809" t="inlineStr">
+        <is>
+          <t>효과음과 음악</t>
+        </is>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" t="inlineStr">
+        <is>
+          <t>credits.creator</t>
+        </is>
+      </c>
+      <c r="B810" t="inlineStr">
+        <is>
+          <t>creator: {name}</t>
+        </is>
+      </c>
+      <c r="C810" t="inlineStr">
+        <is>
+          <t>제작자: {name}</t>
+        </is>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" t="inlineStr">
+        <is>
+          <t>credits.thanks</t>
+        </is>
+      </c>
+      <c r="B811" t="inlineStr">
+        <is>
+          <t>Thank you for playing.</t>
+        </is>
+      </c>
+      <c r="C811" t="inlineStr">
+        <is>
+          <t>플레이해 주셔서 감사합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" t="inlineStr">
+        <is>
+          <t>credits.by</t>
+        </is>
+      </c>
+      <c r="B812" t="inlineStr">
+        <is>
+          <t>by PaleRook</t>
+        </is>
+      </c>
+      <c r="C812" t="inlineStr">
+        <is>
+          <t>PaleRook 제작</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(combat): data-driven enemy AI, telegraphed big attacks with BREAK counterplay, boss phases (B4: D7 D59 D68 D75 D79 D80)
Every enemy has a brain (priority rules + weighted default + boss phases) decided by the pure EnemyAI_Choose on the combat stream.
Heavy moves are announced one turn (log, banner, "!" on the strip, Foresight shows it); a BREAK during the wind-up cancels the attack.
Palehorn and the Pale Choirbeast get two phases (+SPD/+ATK, new rule lists, banners); Rampage and Fury double actions are gone.
New skills Regrow, Snuff, Gore, Pale Hymn. Spec section 12, Test_Suite_EnemyAI, bot_ai_*, B4 shots (140-148), EN+KO strings.

Co-Authored-By: Claude Sonnet <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datafiles/localization/game_text.xlsx
+++ b/datafiles/localization/game_text.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C737"/>
+  <dimension ref="A1:C753"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -12952,6 +12952,278 @@
         </is>
       </c>
     </row>
+    <row r="738">
+      <c r="A738" t="inlineStr">
+        <is>
+          <t>combat.msg.windup.skill_vine_trap</t>
+        </is>
+      </c>
+      <c r="B738" t="inlineStr">
+        <is>
+          <t>{enemy} coils its vines!</t>
+        </is>
+      </c>
+      <c r="C738" t="inlineStr">
+        <is>
+          <t>{enemy}이(가) 덩굴을 감아 올립니다!</t>
+        </is>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" t="inlineStr">
+        <is>
+          <t>combat.msg.windup.skill_ghost_cut</t>
+        </is>
+      </c>
+      <c r="B739" t="inlineStr">
+        <is>
+          <t>{enemy} raises its blade!</t>
+        </is>
+      </c>
+      <c r="C739" t="inlineStr">
+        <is>
+          <t>{enemy}이(가) 칼날을 치켜듭니다!</t>
+        </is>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" t="inlineStr">
+        <is>
+          <t>combat.msg.windup.skill_ramming</t>
+        </is>
+      </c>
+      <c r="B740" t="inlineStr">
+        <is>
+          <t>{enemy} lowers its horns!</t>
+        </is>
+      </c>
+      <c r="C740" t="inlineStr">
+        <is>
+          <t>{enemy}이(가) 뿔을 낮춥니다!</t>
+        </is>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" t="inlineStr">
+        <is>
+          <t>combat.msg.windup.skill_pale_hymn</t>
+        </is>
+      </c>
+      <c r="B741" t="inlineStr">
+        <is>
+          <t>{enemy} draws a deep breath!</t>
+        </is>
+      </c>
+      <c r="C741" t="inlineStr">
+        <is>
+          <t>{enemy}이(가) 숨을 크게 들이쉽니다!</t>
+        </is>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" t="inlineStr">
+        <is>
+          <t>combat.msg.phase.mini_boss.1</t>
+        </is>
+      </c>
+      <c r="B742" t="inlineStr">
+        <is>
+          <t>{enemy} paws the ground, snorting!</t>
+        </is>
+      </c>
+      <c r="C742" t="inlineStr">
+        <is>
+          <t>{enemy}이(가) 콧김을 내뿜으며 땅을 긁습니다!</t>
+        </is>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" t="inlineStr">
+        <is>
+          <t>combat.msg.phase.mini_boss.2</t>
+        </is>
+      </c>
+      <c r="B743" t="inlineStr">
+        <is>
+          <t>{enemy} bellows in a blind rage!</t>
+        </is>
+      </c>
+      <c r="C743" t="inlineStr">
+        <is>
+          <t>{enemy}이(가) 분노에 눈이 멀어 포효합니다!</t>
+        </is>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" t="inlineStr">
+        <is>
+          <t>combat.msg.phase.final_boss.1</t>
+        </is>
+      </c>
+      <c r="B744" t="inlineStr">
+        <is>
+          <t>{enemy} sings a second voice!</t>
+        </is>
+      </c>
+      <c r="C744" t="inlineStr">
+        <is>
+          <t>{enemy}이(가) 두 번째 목소리로 노래합니다!</t>
+        </is>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" t="inlineStr">
+        <is>
+          <t>combat.msg.phase.final_boss.2</t>
+        </is>
+      </c>
+      <c r="B745" t="inlineStr">
+        <is>
+          <t>{enemy} howls in fury!</t>
+        </is>
+      </c>
+      <c r="C745" t="inlineStr">
+        <is>
+          <t>{enemy}이(가) 격노하여 울부짖습니다!</t>
+        </is>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" t="inlineStr">
+        <is>
+          <t>combat.msg.windup_broken</t>
+        </is>
+      </c>
+      <c r="B746" t="inlineStr">
+        <is>
+          <t>{enemy}'s {skill} is broken off!</t>
+        </is>
+      </c>
+      <c r="C746" t="inlineStr">
+        <is>
+          <t>{enemy}의 {skill}이(가) 끊겼습니다!</t>
+        </is>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" t="inlineStr">
+        <is>
+          <t>combat.foresee.windup</t>
+        </is>
+      </c>
+      <c r="B747" t="inlineStr">
+        <is>
+          <t>winding up {skill}</t>
+        </is>
+      </c>
+      <c r="C747" t="inlineStr">
+        <is>
+          <t>{skill}을(를) 준비 중</t>
+        </is>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" t="inlineStr">
+        <is>
+          <t>skill.name.skill_regrow</t>
+        </is>
+      </c>
+      <c r="B748" t="inlineStr">
+        <is>
+          <t>Regrow</t>
+        </is>
+      </c>
+      <c r="C748" t="inlineStr">
+        <is>
+          <t>재생</t>
+        </is>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" t="inlineStr">
+        <is>
+          <t>skill.name.skill_snuff</t>
+        </is>
+      </c>
+      <c r="B749" t="inlineStr">
+        <is>
+          <t>Snuff</t>
+        </is>
+      </c>
+      <c r="C749" t="inlineStr">
+        <is>
+          <t>꺼뜨리기</t>
+        </is>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" t="inlineStr">
+        <is>
+          <t>skill.name.skill_gore</t>
+        </is>
+      </c>
+      <c r="B750" t="inlineStr">
+        <is>
+          <t>Gore</t>
+        </is>
+      </c>
+      <c r="C750" t="inlineStr">
+        <is>
+          <t>뿔치기</t>
+        </is>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" t="inlineStr">
+        <is>
+          <t>skill.name.skill_pale_hymn</t>
+        </is>
+      </c>
+      <c r="B751" t="inlineStr">
+        <is>
+          <t>Pale Hymn</t>
+        </is>
+      </c>
+      <c r="C751" t="inlineStr">
+        <is>
+          <t>창백한 찬가</t>
+        </is>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" t="inlineStr">
+        <is>
+          <t>combat.msg.skill.use.skill_regrow</t>
+        </is>
+      </c>
+      <c r="B752" t="inlineStr">
+        <is>
+          <t>It regrows its wounds!</t>
+        </is>
+      </c>
+      <c r="C752" t="inlineStr">
+        <is>
+          <t>상처가 아물어 갑니다!</t>
+        </is>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" t="inlineStr">
+        <is>
+          <t>combat.msg.skill.use.skill_snuff</t>
+        </is>
+      </c>
+      <c r="B753" t="inlineStr">
+        <is>
+          <t>Your enchantments are snuffed out!</t>
+        </is>
+      </c>
+      <c r="C753" t="inlineStr">
+        <is>
+          <t>당신의 강화 효과가 꺼졌습니다!</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C678"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(economy): gold, merchant shop, throwables, accessory slot, elites, per-run shuffles (packet C3: D23 D33 D84 D85 D86 D92)
Gold per fight (10 + 2 x level, x1.2 rank 2, x3 boss, x2 elite, +-25%), kept in the run and lost with it; merchant (obj_npc placed in code) after floors 2/5/8 with a seeded stock, buy / sell and a details panel; four throwables thrown through the sliding bar (Nobody x1.5, carries 8); accessory slot (items 40-46); elites (15% of map enemies, one of five modifiers, pulsing outline, ELITE tag, double gold, a guaranteed card pick); per-run enemy pools, spots and chest contents derived from the seed.

Test_Suite_Economy (about 240 assertions), smoke steps 142-146, bot v=8, shots +11, 91 EN+KO text rows.

Co-Authored-By: Claude Sonnet <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datafiles/localization/game_text.xlsx
+++ b/datafiles/localization/game_text.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C846"/>
+  <dimension ref="A1:C937"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -14805,6 +14805,1553 @@
         </is>
       </c>
     </row>
+    <row r="847">
+      <c r="A847" t="inlineStr">
+        <is>
+          <t>elite.tag</t>
+        </is>
+      </c>
+      <c r="B847" t="inlineStr">
+        <is>
+          <t>ELITE</t>
+        </is>
+      </c>
+      <c r="C847" t="inlineStr">
+        <is>
+          <t>정예</t>
+        </is>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" t="inlineStr">
+        <is>
+          <t>item.msg.throw_in_battle</t>
+        </is>
+      </c>
+      <c r="B848" t="inlineStr">
+        <is>
+          <t>Throw it at an enemy in battle.</t>
+        </is>
+      </c>
+      <c r="C848" t="inlineStr">
+        <is>
+          <t>전투 중 적에게 던지세요.</t>
+        </is>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" t="inlineStr">
+        <is>
+          <t>throw.msg.damage</t>
+        </is>
+      </c>
+      <c r="B849" t="inlineStr">
+        <is>
+          <t>{dmg} damage.</t>
+        </is>
+      </c>
+      <c r="C849" t="inlineStr">
+        <is>
+          <t>{dmg}의 피해.</t>
+        </is>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" t="inlineStr">
+        <is>
+          <t>throw.msg.burn</t>
+        </is>
+      </c>
+      <c r="B850" t="inlineStr">
+        <is>
+          <t>It burns for {n} a turn.</t>
+        </is>
+      </c>
+      <c r="C850" t="inlineStr">
+        <is>
+          <t>매 턴 {n}의 화상을 입습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" t="inlineStr">
+        <is>
+          <t>throw.msg.poison</t>
+        </is>
+      </c>
+      <c r="B851" t="inlineStr">
+        <is>
+          <t>{n} stacks of poison.</t>
+        </is>
+      </c>
+      <c r="C851" t="inlineStr">
+        <is>
+          <t>독 {n}중첩.</t>
+        </is>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" t="inlineStr">
+        <is>
+          <t>throw.msg.evade</t>
+        </is>
+      </c>
+      <c r="B852" t="inlineStr">
+        <is>
+          <t>You will dodge the next attack.</t>
+        </is>
+      </c>
+      <c r="C852" t="inlineStr">
+        <is>
+          <t>다음 공격을 피합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" t="inlineStr">
+        <is>
+          <t>throw.msg.escape</t>
+        </is>
+      </c>
+      <c r="B853" t="inlineStr">
+        <is>
+          <t>You slip away in the smoke!</t>
+        </is>
+      </c>
+      <c r="C853" t="inlineStr">
+        <is>
+          <t>연기 속으로 빠져나갔습니다!</t>
+        </is>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" t="inlineStr">
+        <is>
+          <t>throw.msg.thrown</t>
+        </is>
+      </c>
+      <c r="B854" t="inlineStr">
+        <is>
+          <t>You throw the {item}!</t>
+        </is>
+      </c>
+      <c r="C854" t="inlineStr">
+        <is>
+          <t>{item}을(를) 던졌다!</t>
+        </is>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" t="inlineStr">
+        <is>
+          <t>item.sent.30</t>
+        </is>
+      </c>
+      <c r="B855" t="inlineStr">
+        <is>
+          <t>Throw it for {power} power of damage; it burns for {turns} turns. Costs your turn.</t>
+        </is>
+      </c>
+      <c r="C855" t="inlineStr">
+        <is>
+          <t>위력 {power}의 피해를 주고 {turns}턴 동안 불탑니다. 턴을 소모합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" t="inlineStr">
+        <is>
+          <t>item.sent.31</t>
+        </is>
+      </c>
+      <c r="B856" t="inlineStr">
+        <is>
+          <t>Throw it to poison the enemy with {n} stacks. Costs your turn.</t>
+        </is>
+      </c>
+      <c r="C856" t="inlineStr">
+        <is>
+          <t>적을 독 {n}중첩으로 중독시킵니다. 턴을 소모합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" t="inlineStr">
+        <is>
+          <t>item.sent.32</t>
+        </is>
+      </c>
+      <c r="B857" t="inlineStr">
+        <is>
+          <t>Throw it for {power} power of damage and a stun that pushes the enemy back. Costs your turn.</t>
+        </is>
+      </c>
+      <c r="C857" t="inlineStr">
+        <is>
+          <t>위력 {power}의 피해를 주고 기절시켜 적을 뒤로 밉니다. 턴을 소모합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" t="inlineStr">
+        <is>
+          <t>item.sent.33</t>
+        </is>
+      </c>
+      <c r="B858" t="inlineStr">
+        <is>
+          <t>Throw it to dodge the next attack ({turns} turns); a Perfect throw lets you slip away. Costs your turn.</t>
+        </is>
+      </c>
+      <c r="C858" t="inlineStr">
+        <is>
+          <t>다음 공격을 피합니다({turns}턴). 완벽하게 던지면 도망칩니다. 턴을 소모합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" t="inlineStr">
+        <is>
+          <t>item.sent.throw</t>
+        </is>
+      </c>
+      <c r="B859" t="inlineStr">
+        <is>
+          <t>Throw it at the enemy. Costs your turn.</t>
+        </is>
+      </c>
+      <c r="C859" t="inlineStr">
+        <is>
+          <t>적에게 던집니다. 턴을 소모합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="860">
+      <c r="A860" t="inlineStr">
+        <is>
+          <t>item.sent.accessory_stat</t>
+        </is>
+      </c>
+      <c r="B860" t="inlineStr">
+        <is>
+          <t>Wear it for {bonus}.</t>
+        </is>
+      </c>
+      <c r="C860" t="inlineStr">
+        <is>
+          <t>착용하면 {bonus}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="861">
+      <c r="A861" t="inlineStr">
+        <is>
+          <t>item.sent.accessory_passive</t>
+        </is>
+      </c>
+      <c r="B861" t="inlineStr">
+        <is>
+          <t>Wear it: {line}.</t>
+        </is>
+      </c>
+      <c r="C861" t="inlineStr">
+        <is>
+          <t>착용: {line}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="862">
+      <c r="A862" t="inlineStr">
+        <is>
+          <t>item.sent.accessory</t>
+        </is>
+      </c>
+      <c r="B862" t="inlineStr">
+        <is>
+          <t>A ring or charm worn in the accessory slot.</t>
+        </is>
+      </c>
+      <c r="C862" t="inlineStr">
+        <is>
+          <t>장신구 칸에 착용하는 반지나 부적입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" t="inlineStr">
+        <is>
+          <t>item.sent.heal</t>
+        </is>
+      </c>
+      <c r="B863" t="inlineStr">
+        <is>
+          <t>Restores {min} to {max} HP.</t>
+        </is>
+      </c>
+      <c r="C863" t="inlineStr">
+        <is>
+          <t>HP를 {min}에서 {max}만큼 회복합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" t="inlineStr">
+        <is>
+          <t>item.sent.mp</t>
+        </is>
+      </c>
+      <c r="B864" t="inlineStr">
+        <is>
+          <t>Restores {min} to {max} MP.</t>
+        </is>
+      </c>
+      <c r="C864" t="inlineStr">
+        <is>
+          <t>MP를 {min}에서 {max}만큼 회복합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" t="inlineStr">
+        <is>
+          <t>item.sent.cure</t>
+        </is>
+      </c>
+      <c r="B865" t="inlineStr">
+        <is>
+          <t>Cures {status}.</t>
+        </is>
+      </c>
+      <c r="C865" t="inlineStr">
+        <is>
+          <t>{status}을(를) 치료합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="866">
+      <c r="A866" t="inlineStr">
+        <is>
+          <t>item.sent.weapon</t>
+        </is>
+      </c>
+      <c r="B866" t="inlineStr">
+        <is>
+          <t>A weapon with {power} power.</t>
+        </is>
+      </c>
+      <c r="C866" t="inlineStr">
+        <is>
+          <t>위력 {power}의 무기입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" t="inlineStr">
+        <is>
+          <t>item.sent.armor</t>
+        </is>
+      </c>
+      <c r="B867" t="inlineStr">
+        <is>
+          <t>Armor: {bonus}.</t>
+        </is>
+      </c>
+      <c r="C867" t="inlineStr">
+        <is>
+          <t>방어구: {bonus}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" t="inlineStr">
+        <is>
+          <t>shop.lbl.power</t>
+        </is>
+      </c>
+      <c r="B868" t="inlineStr">
+        <is>
+          <t>Power</t>
+        </is>
+      </c>
+      <c r="C868" t="inlineStr">
+        <is>
+          <t>위력</t>
+        </is>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" t="inlineStr">
+        <is>
+          <t>shop.lbl.burn</t>
+        </is>
+      </c>
+      <c r="B869" t="inlineStr">
+        <is>
+          <t>Burn</t>
+        </is>
+      </c>
+      <c r="C869" t="inlineStr">
+        <is>
+          <t>화상</t>
+        </is>
+      </c>
+    </row>
+    <row r="870">
+      <c r="A870" t="inlineStr">
+        <is>
+          <t>shop.lbl.poison</t>
+        </is>
+      </c>
+      <c r="B870" t="inlineStr">
+        <is>
+          <t>Poison</t>
+        </is>
+      </c>
+      <c r="C870" t="inlineStr">
+        <is>
+          <t>독</t>
+        </is>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" t="inlineStr">
+        <is>
+          <t>shop.lbl.stun</t>
+        </is>
+      </c>
+      <c r="B871" t="inlineStr">
+        <is>
+          <t>Stun</t>
+        </is>
+      </c>
+      <c r="C871" t="inlineStr">
+        <is>
+          <t>기절</t>
+        </is>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" t="inlineStr">
+        <is>
+          <t>shop.val.pushback</t>
+        </is>
+      </c>
+      <c r="B872" t="inlineStr">
+        <is>
+          <t>Push back</t>
+        </is>
+      </c>
+      <c r="C872" t="inlineStr">
+        <is>
+          <t>뒤로 밀기</t>
+        </is>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" t="inlineStr">
+        <is>
+          <t>shop.lbl.evade</t>
+        </is>
+      </c>
+      <c r="B873" t="inlineStr">
+        <is>
+          <t>Dodge</t>
+        </is>
+      </c>
+      <c r="C873" t="inlineStr">
+        <is>
+          <t>회피</t>
+        </is>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" t="inlineStr">
+        <is>
+          <t>shop.val.turns</t>
+        </is>
+      </c>
+      <c r="B874" t="inlineStr">
+        <is>
+          <t>{n} turns</t>
+        </is>
+      </c>
+      <c r="C874" t="inlineStr">
+        <is>
+          <t>{n}턴</t>
+        </is>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" t="inlineStr">
+        <is>
+          <t>shop.lbl.perfect</t>
+        </is>
+      </c>
+      <c r="B875" t="inlineStr">
+        <is>
+          <t>Perfect</t>
+        </is>
+      </c>
+      <c r="C875" t="inlineStr">
+        <is>
+          <t>완벽</t>
+        </is>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" t="inlineStr">
+        <is>
+          <t>shop.val.escape</t>
+        </is>
+      </c>
+      <c r="B876" t="inlineStr">
+        <is>
+          <t>Escape</t>
+        </is>
+      </c>
+      <c r="C876" t="inlineStr">
+        <is>
+          <t>도망</t>
+        </is>
+      </c>
+    </row>
+    <row r="877">
+      <c r="A877" t="inlineStr">
+        <is>
+          <t>shop.lbl.nobody</t>
+        </is>
+      </c>
+      <c r="B877" t="inlineStr">
+        <is>
+          <t>Nobody</t>
+        </is>
+      </c>
+      <c r="C877" t="inlineStr">
+        <is>
+          <t>무명</t>
+        </is>
+      </c>
+    </row>
+    <row r="878">
+      <c r="A878" t="inlineStr">
+        <is>
+          <t>shop.lbl.carry</t>
+        </is>
+      </c>
+      <c r="B878" t="inlineStr">
+        <is>
+          <t>Carry up to</t>
+        </is>
+      </c>
+      <c r="C878" t="inlineStr">
+        <is>
+          <t>최대 소지</t>
+        </is>
+      </c>
+    </row>
+    <row r="879">
+      <c r="A879" t="inlineStr">
+        <is>
+          <t>shop.lbl.damage_taken</t>
+        </is>
+      </c>
+      <c r="B879" t="inlineStr">
+        <is>
+          <t>Damage taken</t>
+        </is>
+      </c>
+      <c r="C879" t="inlineStr">
+        <is>
+          <t>받는 피해</t>
+        </is>
+      </c>
+    </row>
+    <row r="880">
+      <c r="A880" t="inlineStr">
+        <is>
+          <t>shop.lbl.mp</t>
+        </is>
+      </c>
+      <c r="B880" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+      <c r="C880" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="881">
+      <c r="A881" t="inlineStr">
+        <is>
+          <t>shop.val.mp_every</t>
+        </is>
+      </c>
+      <c r="B881" t="inlineStr">
+        <is>
+          <t>+{n} every {k} turns</t>
+        </is>
+      </c>
+      <c r="C881" t="inlineStr">
+        <is>
+          <t>+{n} ({k}턴마다)</t>
+        </is>
+      </c>
+    </row>
+    <row r="882">
+      <c r="A882" t="inlineStr">
+        <is>
+          <t>shop.lbl.gold</t>
+        </is>
+      </c>
+      <c r="B882" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="C882" t="inlineStr">
+        <is>
+          <t>골드</t>
+        </is>
+      </c>
+    </row>
+    <row r="883">
+      <c r="A883" t="inlineStr">
+        <is>
+          <t>shop.lbl.hp</t>
+        </is>
+      </c>
+      <c r="B883" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="C883" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+    </row>
+    <row r="884">
+      <c r="A884" t="inlineStr">
+        <is>
+          <t>shop.lbl.cures</t>
+        </is>
+      </c>
+      <c r="B884" t="inlineStr">
+        <is>
+          <t>Cures</t>
+        </is>
+      </c>
+      <c r="C884" t="inlineStr">
+        <is>
+          <t>치료</t>
+        </is>
+      </c>
+    </row>
+    <row r="885">
+      <c r="A885" t="inlineStr">
+        <is>
+          <t>shop.lbl.stat</t>
+        </is>
+      </c>
+      <c r="B885" t="inlineStr">
+        <is>
+          <t>Uses</t>
+        </is>
+      </c>
+      <c r="C885" t="inlineStr">
+        <is>
+          <t>능력치</t>
+        </is>
+      </c>
+    </row>
+    <row r="886">
+      <c r="A886" t="inlineStr">
+        <is>
+          <t>shop.lbl.bonus</t>
+        </is>
+      </c>
+      <c r="B886" t="inlineStr">
+        <is>
+          <t>Bonus</t>
+        </is>
+      </c>
+      <c r="C886" t="inlineStr">
+        <is>
+          <t>보너스</t>
+        </is>
+      </c>
+    </row>
+    <row r="887">
+      <c r="A887" t="inlineStr">
+        <is>
+          <t>combat.msg.gold_gain</t>
+        </is>
+      </c>
+      <c r="B887" t="inlineStr">
+        <is>
+          <t>(+{gold} gold)</t>
+        </is>
+      </c>
+      <c r="C887" t="inlineStr">
+        <is>
+          <t>(+{gold} 골드)</t>
+        </is>
+      </c>
+    </row>
+    <row r="888">
+      <c r="A888" t="inlineStr">
+        <is>
+          <t>merchant.name</t>
+        </is>
+      </c>
+      <c r="B888" t="inlineStr">
+        <is>
+          <t>Merchant</t>
+        </is>
+      </c>
+      <c r="C888" t="inlineStr">
+        <is>
+          <t>상인</t>
+        </is>
+      </c>
+    </row>
+    <row r="889">
+      <c r="A889" t="inlineStr">
+        <is>
+          <t>elite.name.armored</t>
+        </is>
+      </c>
+      <c r="B889" t="inlineStr">
+        <is>
+          <t>Armored</t>
+        </is>
+      </c>
+      <c r="C889" t="inlineStr">
+        <is>
+          <t>철갑</t>
+        </is>
+      </c>
+    </row>
+    <row r="890">
+      <c r="A890" t="inlineStr">
+        <is>
+          <t>elite.name.venomous</t>
+        </is>
+      </c>
+      <c r="B890" t="inlineStr">
+        <is>
+          <t>Venomous</t>
+        </is>
+      </c>
+      <c r="C890" t="inlineStr">
+        <is>
+          <t>맹독</t>
+        </is>
+      </c>
+    </row>
+    <row r="891">
+      <c r="A891" t="inlineStr">
+        <is>
+          <t>elite.name.swift</t>
+        </is>
+      </c>
+      <c r="B891" t="inlineStr">
+        <is>
+          <t>Swift</t>
+        </is>
+      </c>
+      <c r="C891" t="inlineStr">
+        <is>
+          <t>신속</t>
+        </is>
+      </c>
+    </row>
+    <row r="892">
+      <c r="A892" t="inlineStr">
+        <is>
+          <t>elite.name.brutal</t>
+        </is>
+      </c>
+      <c r="B892" t="inlineStr">
+        <is>
+          <t>Brutal</t>
+        </is>
+      </c>
+      <c r="C892" t="inlineStr">
+        <is>
+          <t>흉포</t>
+        </is>
+      </c>
+    </row>
+    <row r="893">
+      <c r="A893" t="inlineStr">
+        <is>
+          <t>elite.name.regenerating</t>
+        </is>
+      </c>
+      <c r="B893" t="inlineStr">
+        <is>
+          <t>Regenerating</t>
+        </is>
+      </c>
+      <c r="C893" t="inlineStr">
+        <is>
+          <t>재생</t>
+        </is>
+      </c>
+    </row>
+    <row r="894">
+      <c r="A894" t="inlineStr">
+        <is>
+          <t>elite.line.armored</t>
+        </is>
+      </c>
+      <c r="B894" t="inlineStr">
+        <is>
+          <t>Armored: +{n} DEF.</t>
+        </is>
+      </c>
+      <c r="C894" t="inlineStr">
+        <is>
+          <t>철갑: 방어 +{n}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="895">
+      <c r="A895" t="inlineStr">
+        <is>
+          <t>elite.line.venomous</t>
+        </is>
+      </c>
+      <c r="B895" t="inlineStr">
+        <is>
+          <t>Venomous: its hits poison you for {n} stacks.</t>
+        </is>
+      </c>
+      <c r="C895" t="inlineStr">
+        <is>
+          <t>맹독: 공격이 {n}중첩의 독을 겁니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="896">
+      <c r="A896" t="inlineStr">
+        <is>
+          <t>elite.line.swift</t>
+        </is>
+      </c>
+      <c r="B896" t="inlineStr">
+        <is>
+          <t>Swift: +{n} SPD.</t>
+        </is>
+      </c>
+      <c r="C896" t="inlineStr">
+        <is>
+          <t>신속: 속도 +{n}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="897">
+      <c r="A897" t="inlineStr">
+        <is>
+          <t>elite.line.brutal</t>
+        </is>
+      </c>
+      <c r="B897" t="inlineStr">
+        <is>
+          <t>Brutal: +{n} ATK.</t>
+        </is>
+      </c>
+      <c r="C897" t="inlineStr">
+        <is>
+          <t>흉포: 공격 +{n}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="898">
+      <c r="A898" t="inlineStr">
+        <is>
+          <t>elite.line.regenerating</t>
+        </is>
+      </c>
+      <c r="B898" t="inlineStr">
+        <is>
+          <t>Regenerating: heals {pct}% of its HP each turn.</t>
+        </is>
+      </c>
+      <c r="C898" t="inlineStr">
+        <is>
+          <t>재생: 매 턴 HP의 {pct}%를 회복합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="899">
+      <c r="A899" t="inlineStr">
+        <is>
+          <t>menu.tooltip.item.type.accessory</t>
+        </is>
+      </c>
+      <c r="B899" t="inlineStr">
+        <is>
+          <t>Accessory</t>
+        </is>
+      </c>
+      <c r="C899" t="inlineStr">
+        <is>
+          <t>장신구</t>
+        </is>
+      </c>
+    </row>
+    <row r="900">
+      <c r="A900" t="inlineStr">
+        <is>
+          <t>menu.gold</t>
+        </is>
+      </c>
+      <c r="B900" t="inlineStr">
+        <is>
+          <t>Gold: {n}</t>
+        </is>
+      </c>
+      <c r="C900" t="inlineStr">
+        <is>
+          <t>골드: {n}</t>
+        </is>
+      </c>
+    </row>
+    <row r="901">
+      <c r="A901" t="inlineStr">
+        <is>
+          <t>shop.sold_out</t>
+        </is>
+      </c>
+      <c r="B901" t="inlineStr">
+        <is>
+          <t>Sold out</t>
+        </is>
+      </c>
+      <c r="C901" t="inlineStr">
+        <is>
+          <t>품절</t>
+        </is>
+      </c>
+    </row>
+    <row r="902">
+      <c r="A902" t="inlineStr">
+        <is>
+          <t>shop.lbl.have</t>
+        </is>
+      </c>
+      <c r="B902" t="inlineStr">
+        <is>
+          <t>You have</t>
+        </is>
+      </c>
+      <c r="C902" t="inlineStr">
+        <is>
+          <t>보유</t>
+        </is>
+      </c>
+    </row>
+    <row r="903">
+      <c r="A903" t="inlineStr">
+        <is>
+          <t>shop.lbl.in_stock</t>
+        </is>
+      </c>
+      <c r="B903" t="inlineStr">
+        <is>
+          <t>In stock</t>
+        </is>
+      </c>
+      <c r="C903" t="inlineStr">
+        <is>
+          <t>재고</t>
+        </is>
+      </c>
+    </row>
+    <row r="904">
+      <c r="A904" t="inlineStr">
+        <is>
+          <t>shop.lbl.sells_for</t>
+        </is>
+      </c>
+      <c r="B904" t="inlineStr">
+        <is>
+          <t>Sells for</t>
+        </is>
+      </c>
+      <c r="C904" t="inlineStr">
+        <is>
+          <t>판매가</t>
+        </is>
+      </c>
+    </row>
+    <row r="905">
+      <c r="A905" t="inlineStr">
+        <is>
+          <t>shop.worn</t>
+        </is>
+      </c>
+      <c r="B905" t="inlineStr">
+        <is>
+          <t>Worn</t>
+        </is>
+      </c>
+      <c r="C905" t="inlineStr">
+        <is>
+          <t>착용 중</t>
+        </is>
+      </c>
+    </row>
+    <row r="906">
+      <c r="A906" t="inlineStr">
+        <is>
+          <t>shop.nothing_to_sell</t>
+        </is>
+      </c>
+      <c r="B906" t="inlineStr">
+        <is>
+          <t>Nothing to sell</t>
+        </is>
+      </c>
+      <c r="C906" t="inlineStr">
+        <is>
+          <t>팔 것이 없습니다</t>
+        </is>
+      </c>
+    </row>
+    <row r="907">
+      <c r="A907" t="inlineStr">
+        <is>
+          <t>shop.gold</t>
+        </is>
+      </c>
+      <c r="B907" t="inlineStr">
+        <is>
+          <t>Gold {n}</t>
+        </is>
+      </c>
+      <c r="C907" t="inlineStr">
+        <is>
+          <t>골드 {n}</t>
+        </is>
+      </c>
+    </row>
+    <row r="908">
+      <c r="A908" t="inlineStr">
+        <is>
+          <t>shop.buy</t>
+        </is>
+      </c>
+      <c r="B908" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="C908" t="inlineStr">
+        <is>
+          <t>구매</t>
+        </is>
+      </c>
+    </row>
+    <row r="909">
+      <c r="A909" t="inlineStr">
+        <is>
+          <t>shop.sell</t>
+        </is>
+      </c>
+      <c r="B909" t="inlineStr">
+        <is>
+          <t>Sell</t>
+        </is>
+      </c>
+      <c r="C909" t="inlineStr">
+        <is>
+          <t>판매</t>
+        </is>
+      </c>
+    </row>
+    <row r="910">
+      <c r="A910" t="inlineStr">
+        <is>
+          <t>shop.leave</t>
+        </is>
+      </c>
+      <c r="B910" t="inlineStr">
+        <is>
+          <t>Leave</t>
+        </is>
+      </c>
+      <c r="C910" t="inlineStr">
+        <is>
+          <t>나가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="911">
+      <c r="A911" t="inlineStr">
+        <is>
+          <t>shop.title</t>
+        </is>
+      </c>
+      <c r="B911" t="inlineStr">
+        <is>
+          <t>Merchant</t>
+        </is>
+      </c>
+      <c r="C911" t="inlineStr">
+        <is>
+          <t>상인</t>
+        </is>
+      </c>
+    </row>
+    <row r="912">
+      <c r="A912" t="inlineStr">
+        <is>
+          <t>shop.msg.gold</t>
+        </is>
+      </c>
+      <c r="B912" t="inlineStr">
+        <is>
+          <t>Not enough gold.</t>
+        </is>
+      </c>
+      <c r="C912" t="inlineStr">
+        <is>
+          <t>골드가 부족합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="913">
+      <c r="A913" t="inlineStr">
+        <is>
+          <t>shop.msg.sold_out</t>
+        </is>
+      </c>
+      <c r="B913" t="inlineStr">
+        <is>
+          <t>Sold out.</t>
+        </is>
+      </c>
+      <c r="C913" t="inlineStr">
+        <is>
+          <t>품절입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="914">
+      <c r="A914" t="inlineStr">
+        <is>
+          <t>shop.msg.full</t>
+        </is>
+      </c>
+      <c r="B914" t="inlineStr">
+        <is>
+          <t>You cannot carry more of those.</t>
+        </is>
+      </c>
+      <c r="C914" t="inlineStr">
+        <is>
+          <t>더 이상 가질 수 없습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="915">
+      <c r="A915" t="inlineStr">
+        <is>
+          <t>shop.msg.owned</t>
+        </is>
+      </c>
+      <c r="B915" t="inlineStr">
+        <is>
+          <t>You already have that.</t>
+        </is>
+      </c>
+      <c r="C915" t="inlineStr">
+        <is>
+          <t>이미 가지고 있습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="916">
+      <c r="A916" t="inlineStr">
+        <is>
+          <t>shop.msg.slots</t>
+        </is>
+      </c>
+      <c r="B916" t="inlineStr">
+        <is>
+          <t>All your skill slots are full.</t>
+        </is>
+      </c>
+      <c r="C916" t="inlineStr">
+        <is>
+          <t>스킬 칸이 가득 찼습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="917">
+      <c r="A917" t="inlineStr">
+        <is>
+          <t>shop.msg.equipped</t>
+        </is>
+      </c>
+      <c r="B917" t="inlineStr">
+        <is>
+          <t>Take it off first.</t>
+        </is>
+      </c>
+      <c r="C917" t="inlineStr">
+        <is>
+          <t>먼저 벗으세요.</t>
+        </is>
+      </c>
+    </row>
+    <row r="918">
+      <c r="A918" t="inlineStr">
+        <is>
+          <t>shop.msg.cant</t>
+        </is>
+      </c>
+      <c r="B918" t="inlineStr">
+        <is>
+          <t>Cannot do that.</t>
+        </is>
+      </c>
+      <c r="C918" t="inlineStr">
+        <is>
+          <t>할 수 없습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="919">
+      <c r="A919" t="inlineStr">
+        <is>
+          <t>shop.msg.bought</t>
+        </is>
+      </c>
+      <c r="B919" t="inlineStr">
+        <is>
+          <t>Bought {name} for {price}.</t>
+        </is>
+      </c>
+      <c r="C919" t="inlineStr">
+        <is>
+          <t>{name}을(를) {price}에 샀습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="920">
+      <c r="A920" t="inlineStr">
+        <is>
+          <t>shop.msg.sold</t>
+        </is>
+      </c>
+      <c r="B920" t="inlineStr">
+        <is>
+          <t>Sold {name} for {price}.</t>
+        </is>
+      </c>
+      <c r="C920" t="inlineStr">
+        <is>
+          <t>{name}을(를) {price}에 팔았습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="921">
+      <c r="A921" t="inlineStr">
+        <is>
+          <t>item.name.30</t>
+        </is>
+      </c>
+      <c r="B921" t="inlineStr">
+        <is>
+          <t>Firebomb</t>
+        </is>
+      </c>
+      <c r="C921" t="inlineStr">
+        <is>
+          <t>화염병</t>
+        </is>
+      </c>
+    </row>
+    <row r="922">
+      <c r="A922" t="inlineStr">
+        <is>
+          <t>item.name.31</t>
+        </is>
+      </c>
+      <c r="B922" t="inlineStr">
+        <is>
+          <t>Poison Pot</t>
+        </is>
+      </c>
+      <c r="C922" t="inlineStr">
+        <is>
+          <t>독 항아리</t>
+        </is>
+      </c>
+    </row>
+    <row r="923">
+      <c r="A923" t="inlineStr">
+        <is>
+          <t>item.name.32</t>
+        </is>
+      </c>
+      <c r="B923" t="inlineStr">
+        <is>
+          <t>Ice Flask</t>
+        </is>
+      </c>
+      <c r="C923" t="inlineStr">
+        <is>
+          <t>얼음 병</t>
+        </is>
+      </c>
+    </row>
+    <row r="924">
+      <c r="A924" t="inlineStr">
+        <is>
+          <t>item.name.33</t>
+        </is>
+      </c>
+      <c r="B924" t="inlineStr">
+        <is>
+          <t>Smoke Bomb</t>
+        </is>
+      </c>
+      <c r="C924" t="inlineStr">
+        <is>
+          <t>연막탄</t>
+        </is>
+      </c>
+    </row>
+    <row r="925">
+      <c r="A925" t="inlineStr">
+        <is>
+          <t>item.name.40</t>
+        </is>
+      </c>
+      <c r="B925" t="inlineStr">
+        <is>
+          <t>Copper Ring</t>
+        </is>
+      </c>
+      <c r="C925" t="inlineStr">
+        <is>
+          <t>구리 반지</t>
+        </is>
+      </c>
+    </row>
+    <row r="926">
+      <c r="A926" t="inlineStr">
+        <is>
+          <t>item.name.41</t>
+        </is>
+      </c>
+      <c r="B926" t="inlineStr">
+        <is>
+          <t>Guard Ring</t>
+        </is>
+      </c>
+      <c r="C926" t="inlineStr">
+        <is>
+          <t>수호 반지</t>
+        </is>
+      </c>
+    </row>
+    <row r="927">
+      <c r="A927" t="inlineStr">
+        <is>
+          <t>item.name.42</t>
+        </is>
+      </c>
+      <c r="B927" t="inlineStr">
+        <is>
+          <t>Swift Charm</t>
+        </is>
+      </c>
+      <c r="C927" t="inlineStr">
+        <is>
+          <t>신속의 부적</t>
+        </is>
+      </c>
+    </row>
+    <row r="928">
+      <c r="A928" t="inlineStr">
+        <is>
+          <t>item.name.43</t>
+        </is>
+      </c>
+      <c r="B928" t="inlineStr">
+        <is>
+          <t>Sage Charm</t>
+        </is>
+      </c>
+      <c r="C928" t="inlineStr">
+        <is>
+          <t>현자의 부적</t>
+        </is>
+      </c>
+    </row>
+    <row r="929">
+      <c r="A929" t="inlineStr">
+        <is>
+          <t>item.name.44</t>
+        </is>
+      </c>
+      <c r="B929" t="inlineStr">
+        <is>
+          <t>Stone Charm</t>
+        </is>
+      </c>
+      <c r="C929" t="inlineStr">
+        <is>
+          <t>돌 부적</t>
+        </is>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930" t="inlineStr">
+        <is>
+          <t>item.name.45</t>
+        </is>
+      </c>
+      <c r="B930" t="inlineStr">
+        <is>
+          <t>Spring Ring</t>
+        </is>
+      </c>
+      <c r="C930" t="inlineStr">
+        <is>
+          <t>샘물 반지</t>
+        </is>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931" t="inlineStr">
+        <is>
+          <t>item.name.46</t>
+        </is>
+      </c>
+      <c r="B931" t="inlineStr">
+        <is>
+          <t>Lucky Charm</t>
+        </is>
+      </c>
+      <c r="C931" t="inlineStr">
+        <is>
+          <t>행운의 부적</t>
+        </is>
+      </c>
+    </row>
+    <row r="932">
+      <c r="A932" t="inlineStr">
+        <is>
+          <t>item.passive.name.44</t>
+        </is>
+      </c>
+      <c r="B932" t="inlineStr">
+        <is>
+          <t>Hardened</t>
+        </is>
+      </c>
+      <c r="C932" t="inlineStr">
+        <is>
+          <t>단단함</t>
+        </is>
+      </c>
+    </row>
+    <row r="933">
+      <c r="A933" t="inlineStr">
+        <is>
+          <t>item.passive.desc.44</t>
+        </is>
+      </c>
+      <c r="B933" t="inlineStr">
+        <is>
+          <t>Take 10% less damage</t>
+        </is>
+      </c>
+      <c r="C933" t="inlineStr">
+        <is>
+          <t>받는 피해 10% 감소</t>
+        </is>
+      </c>
+    </row>
+    <row r="934">
+      <c r="A934" t="inlineStr">
+        <is>
+          <t>item.passive.name.45</t>
+        </is>
+      </c>
+      <c r="B934" t="inlineStr">
+        <is>
+          <t>Spring</t>
+        </is>
+      </c>
+      <c r="C934" t="inlineStr">
+        <is>
+          <t>샘물</t>
+        </is>
+      </c>
+    </row>
+    <row r="935">
+      <c r="A935" t="inlineStr">
+        <is>
+          <t>item.passive.desc.45</t>
+        </is>
+      </c>
+      <c r="B935" t="inlineStr">
+        <is>
+          <t>+1 MP every 3 turns</t>
+        </is>
+      </c>
+      <c r="C935" t="inlineStr">
+        <is>
+          <t>3턴마다 MP +1</t>
+        </is>
+      </c>
+    </row>
+    <row r="936">
+      <c r="A936" t="inlineStr">
+        <is>
+          <t>item.passive.name.46</t>
+        </is>
+      </c>
+      <c r="B936" t="inlineStr">
+        <is>
+          <t>Lucky</t>
+        </is>
+      </c>
+      <c r="C936" t="inlineStr">
+        <is>
+          <t>행운</t>
+        </is>
+      </c>
+    </row>
+    <row r="937">
+      <c r="A937" t="inlineStr">
+        <is>
+          <t>item.passive.desc.46</t>
+        </is>
+      </c>
+      <c r="B937" t="inlineStr">
+        <is>
+          <t>Find 15% more gold</t>
+        </is>
+      </c>
+      <c r="C937" t="inlineStr">
+        <is>
+          <t>골드를 15% 더 얻음</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C678"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(c4): QTE assist, beds as rest sites, tutorial pop-ups + Help, key rebinding, device-aware button prompts (D35 D45 D47 D49 D92 D95)
Pure suites Assist/Binds/Prompt/Tutorial/Bed, smoke 161-168, bot v=9, shots 161-169.

Co-Authored-By: Claude Sonnet <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datafiles/localization/game_text.xlsx
+++ b/datafiles/localization/game_text.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C927"/>
+  <dimension ref="A1:C991"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>뒤쪽에</t>
+          <t>뒤로</t>
         </is>
       </c>
     </row>
@@ -11991,12 +11991,12 @@
       </c>
       <c r="B681" t="inlineStr">
         <is>
-          <t>Planned: more forgiving timing on button prompts.</t>
+          <t>Wider bar zones and more time on arrow skills.</t>
         </is>
       </c>
       <c r="C681" t="inlineStr">
         <is>
-          <t>예정: 버튼 입력 타이밍 판정을 더 너그럽게 합니다.</t>
+          <t>막대 판정 구간이 넓어지고 화살표 기술의 시간이 늘어납니다.</t>
         </is>
       </c>
     </row>
@@ -13657,12 +13657,12 @@
       </c>
       <c r="B779" t="inlineStr">
         <is>
-          <t>Left / Right to choose, confirm to take it</t>
+          <t>{left}{right} Choose   {confirm} Take</t>
         </is>
       </c>
       <c r="C779" t="inlineStr">
         <is>
-          <t>좌/우로 고르고, 확인으로 받는다</t>
+          <t>{left}{right} 고르기   {confirm} 받기</t>
         </is>
       </c>
     </row>
@@ -16179,6 +16179,1094 @@
       <c r="C927" t="inlineStr">
         <is>
           <t>PaleRook 제작</t>
+        </is>
+      </c>
+    </row>
+    <row r="928">
+      <c r="A928" t="inlineStr">
+        <is>
+          <t>tutorial.timeline.title</t>
+        </is>
+      </c>
+      <c r="B928" t="inlineStr">
+        <is>
+          <t>Turn order</t>
+        </is>
+      </c>
+      <c r="C928" t="inlineStr">
+        <is>
+          <t>턴 순서</t>
+        </is>
+      </c>
+    </row>
+    <row r="929">
+      <c r="A929" t="inlineStr">
+        <is>
+          <t>tutorial.timeline.body</t>
+        </is>
+      </c>
+      <c r="B929" t="inlineStr">
+        <is>
+          <t>The strip at the top shows who acts next. Faster fighters act more often, and some skills push an enemy back a turn.</t>
+        </is>
+      </c>
+      <c r="C929" t="inlineStr">
+        <is>
+          <t>위쪽 띠는 다음에 행동할 상대를 보여 줍니다. 빠른 쪽이 더 자주 행동하고, 어떤 기술은 적을 한 턴 뒤로 밀어냅니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930" t="inlineStr">
+        <is>
+          <t>tutorial.bar.title</t>
+        </is>
+      </c>
+      <c r="B930" t="inlineStr">
+        <is>
+          <t>The sliding bar</t>
+        </is>
+      </c>
+      <c r="C930" t="inlineStr">
+        <is>
+          <t>움직이는 막대</t>
+        </is>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931" t="inlineStr">
+        <is>
+          <t>tutorial.bar.body</t>
+        </is>
+      </c>
+      <c r="B931" t="inlineStr">
+        <is>
+          <t>A cursor slides along the bar. Press {confirm} when it is over the bright zone. The closer to the middle, the harder you hit.</t>
+        </is>
+      </c>
+      <c r="C931" t="inlineStr">
+        <is>
+          <t>커서가 막대를 따라 움직입니다. 밝은 구간 위에 왔을 때 {confirm}을(를) 누르세요. 가운데에 가까울수록 더 세게 때립니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="932">
+      <c r="A932" t="inlineStr">
+        <is>
+          <t>tutorial.arrows.title</t>
+        </is>
+      </c>
+      <c r="B932" t="inlineStr">
+        <is>
+          <t>Arrow skills</t>
+        </is>
+      </c>
+      <c r="C932" t="inlineStr">
+        <is>
+          <t>화살표 기술</t>
+        </is>
+      </c>
+    </row>
+    <row r="933">
+      <c r="A933" t="inlineStr">
+        <is>
+          <t>tutorial.arrows.body</t>
+        </is>
+      </c>
+      <c r="B933" t="inlineStr">
+        <is>
+          <t>Skills show a row of arrows. Press {up}{down}{left}{right} in that order before the time bar runs out. A wrong press costs time.</t>
+        </is>
+      </c>
+      <c r="C933" t="inlineStr">
+        <is>
+          <t>기술을 쓰면 화살표 줄이 나옵니다. 시간 막대가 다 줄기 전에 {up}{down}{left}{right}으로 순서대로 누르세요. 틀리면 시간이 깎입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="934">
+      <c r="A934" t="inlineStr">
+        <is>
+          <t>tutorial.defence.title</t>
+        </is>
+      </c>
+      <c r="B934" t="inlineStr">
+        <is>
+          <t>Defending</t>
+        </is>
+      </c>
+      <c r="C934" t="inlineStr">
+        <is>
+          <t>막기</t>
+        </is>
+      </c>
+    </row>
+    <row r="935">
+      <c r="A935" t="inlineStr">
+        <is>
+          <t>tutorial.defence.body</t>
+        </is>
+      </c>
+      <c r="B935" t="inlineStr">
+        <is>
+          <t>When an enemy winds up a big attack, a bar appears. Press {confirm} on the bright zone to take less damage and shake off its effects.</t>
+        </is>
+      </c>
+      <c r="C935" t="inlineStr">
+        <is>
+          <t>적이 큰 공격을 준비하면 막대가 나타납니다. 밝은 구간에서 {confirm}을(를) 누르면 피해가 줄고 부가 효과도 털어냅니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="936">
+      <c r="A936" t="inlineStr">
+        <is>
+          <t>tutorial.stagger.title</t>
+        </is>
+      </c>
+      <c r="B936" t="inlineStr">
+        <is>
+          <t>Stagger and BREAK</t>
+        </is>
+      </c>
+      <c r="C936" t="inlineStr">
+        <is>
+          <t>경직과 BREAK</t>
+        </is>
+      </c>
+    </row>
+    <row r="937">
+      <c r="A937" t="inlineStr">
+        <is>
+          <t>tutorial.stagger.body</t>
+        </is>
+      </c>
+      <c r="B937" t="inlineStr">
+        <is>
+          <t>Good hits fill the enemy's stagger meter. When it is full the enemy is BROKEN: it loses a turn and takes +50% damage.</t>
+        </is>
+      </c>
+      <c r="C937" t="inlineStr">
+        <is>
+          <t>좋은 공격은 적의 경직 게이지를 채웁니다. 가득 차면 적이 BREAK 상태가 되어 한 턴을 잃고 피해를 50% 더 받습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="938">
+      <c r="A938" t="inlineStr">
+        <is>
+          <t>tutorial.cards.title</t>
+        </is>
+      </c>
+      <c r="B938" t="inlineStr">
+        <is>
+          <t>Cards</t>
+        </is>
+      </c>
+      <c r="C938" t="inlineStr">
+        <is>
+          <t>카드</t>
+        </is>
+      </c>
+    </row>
+    <row r="939">
+      <c r="A939" t="inlineStr">
+        <is>
+          <t>tutorial.cards.body</t>
+        </is>
+      </c>
+      <c r="B939" t="inlineStr">
+        <is>
+          <t>Level-ups and skill chests offer 3 cards: a new skill, an upgrade or a passive. Take one, or skip for a little gold.</t>
+        </is>
+      </c>
+      <c r="C939" t="inlineStr">
+        <is>
+          <t>레벨업과 기술 상자는 카드 3장을 보여 줍니다. 새 기술, 강화, 패시브 중 하나를 고르거나, 건너뛰고 약간의 골드를 받으세요.</t>
+        </is>
+      </c>
+    </row>
+    <row r="940">
+      <c r="A940" t="inlineStr">
+        <is>
+          <t>tutorial.shop.title</t>
+        </is>
+      </c>
+      <c r="B940" t="inlineStr">
+        <is>
+          <t>The shop</t>
+        </is>
+      </c>
+      <c r="C940" t="inlineStr">
+        <is>
+          <t>상점</t>
+        </is>
+      </c>
+    </row>
+    <row r="941">
+      <c r="A941" t="inlineStr">
+        <is>
+          <t>tutorial.shop.body</t>
+        </is>
+      </c>
+      <c r="B941" t="inlineStr">
+        <is>
+          <t>The merchant sells potions and gear. Gold is kept for the whole run, and the stock changes with every run.</t>
+        </is>
+      </c>
+      <c r="C941" t="inlineStr">
+        <is>
+          <t>상인은 물약과 장비를 팝니다. 골드는 한 번의 도전 동안 유지되고, 상품은 도전마다 바뀝니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="942">
+      <c r="A942" t="inlineStr">
+        <is>
+          <t>tutorial.throwables.title</t>
+        </is>
+      </c>
+      <c r="B942" t="inlineStr">
+        <is>
+          <t>Throwables</t>
+        </is>
+      </c>
+      <c r="C942" t="inlineStr">
+        <is>
+          <t>투척 도구</t>
+        </is>
+      </c>
+    </row>
+    <row r="943">
+      <c r="A943" t="inlineStr">
+        <is>
+          <t>tutorial.throwables.body</t>
+        </is>
+      </c>
+      <c r="B943" t="inlineStr">
+        <is>
+          <t>Throwable items hurt an enemy straight from the item menu. Each one is used up when thrown, so save them for hard fights.</t>
+        </is>
+      </c>
+      <c r="C943" t="inlineStr">
+        <is>
+          <t>투척 도구는 아이템 메뉴에서 바로 적에게 피해를 줍니다. 던지면 사라지니 어려운 싸움을 위해 아껴 두세요.</t>
+        </is>
+      </c>
+    </row>
+    <row r="944">
+      <c r="A944" t="inlineStr">
+        <is>
+          <t>tutorial.bed.title</t>
+        </is>
+      </c>
+      <c r="B944" t="inlineStr">
+        <is>
+          <t>Beds</t>
+        </is>
+      </c>
+      <c r="C944" t="inlineStr">
+        <is>
+          <t>침대</t>
+        </is>
+      </c>
+    </row>
+    <row r="945">
+      <c r="A945" t="inlineStr">
+        <is>
+          <t>tutorial.bed.body</t>
+        </is>
+      </c>
+      <c r="B945" t="inlineStr">
+        <is>
+          <t>Each bed can be used once per run. Rest to restore all your HP and MP, or use it to upgrade one of your skills.</t>
+        </is>
+      </c>
+      <c r="C945" t="inlineStr">
+        <is>
+          <t>침대는 도전마다 한 번씩만 쓸 수 있습니다. 쉬어서 HP와 MP를 모두 채우거나, 기술 하나를 강화하세요.</t>
+        </is>
+      </c>
+    </row>
+    <row r="946">
+      <c r="A946" t="inlineStr">
+        <is>
+          <t>tutorial.elite.title</t>
+        </is>
+      </c>
+      <c r="B946" t="inlineStr">
+        <is>
+          <t>Elites</t>
+        </is>
+      </c>
+      <c r="C946" t="inlineStr">
+        <is>
+          <t>정예</t>
+        </is>
+      </c>
+    </row>
+    <row r="947">
+      <c r="A947" t="inlineStr">
+        <is>
+          <t>tutorial.elite.body</t>
+        </is>
+      </c>
+      <c r="B947" t="inlineStr">
+        <is>
+          <t>Marked enemies are Elites. They are tougher than normal ones, but their rewards are better.</t>
+        </is>
+      </c>
+      <c r="C947" t="inlineStr">
+        <is>
+          <t>표시가 붙은 적은 정예입니다. 일반 적보다 강하지만 보상이 더 좋습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="948">
+      <c r="A948" t="inlineStr">
+        <is>
+          <t>tutorial.status.title</t>
+        </is>
+      </c>
+      <c r="B948" t="inlineStr">
+        <is>
+          <t>Statuses</t>
+        </is>
+      </c>
+      <c r="C948" t="inlineStr">
+        <is>
+          <t>상태 이상</t>
+        </is>
+      </c>
+    </row>
+    <row r="949">
+      <c r="A949" t="inlineStr">
+        <is>
+          <t>tutorial.status.body</t>
+        </is>
+      </c>
+      <c r="B949" t="inlineStr">
+        <is>
+          <t>Poison, Burning, Bleeding and Stun last a few turns. The icons under a name show which ones a fighter has.</t>
+        </is>
+      </c>
+      <c r="C949" t="inlineStr">
+        <is>
+          <t>독, 화상, 출혈, 기절은 몇 턴 동안 이어집니다. 이름 아래 아이콘이 걸려 있는 상태를 보여 줍니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="950">
+      <c r="A950" t="inlineStr">
+        <is>
+          <t>tutorial.footer</t>
+        </is>
+      </c>
+      <c r="B950" t="inlineStr">
+        <is>
+          <t>{confirm} Continue</t>
+        </is>
+      </c>
+      <c r="C950" t="inlineStr">
+        <is>
+          <t>{confirm} 계속</t>
+        </is>
+      </c>
+    </row>
+    <row r="951">
+      <c r="A951" t="inlineStr">
+        <is>
+          <t>tutorial.more</t>
+        </is>
+      </c>
+      <c r="B951" t="inlineStr">
+        <is>
+          <t>+{n} more</t>
+        </is>
+      </c>
+      <c r="C951" t="inlineStr">
+        <is>
+          <t>+{n}개 더</t>
+        </is>
+      </c>
+    </row>
+    <row r="952">
+      <c r="A952" t="inlineStr">
+        <is>
+          <t>help.title</t>
+        </is>
+      </c>
+      <c r="B952" t="inlineStr">
+        <is>
+          <t>Help</t>
+        </is>
+      </c>
+      <c r="C952" t="inlineStr">
+        <is>
+          <t>도움말</t>
+        </is>
+      </c>
+    </row>
+    <row r="953">
+      <c r="A953" t="inlineStr">
+        <is>
+          <t>pause.option.help</t>
+        </is>
+      </c>
+      <c r="B953" t="inlineStr">
+        <is>
+          <t>Help</t>
+        </is>
+      </c>
+      <c r="C953" t="inlineStr">
+        <is>
+          <t>도움말</t>
+        </is>
+      </c>
+    </row>
+    <row r="954">
+      <c r="A954" t="inlineStr">
+        <is>
+          <t>bed.title</t>
+        </is>
+      </c>
+      <c r="B954" t="inlineStr">
+        <is>
+          <t>Bed</t>
+        </is>
+      </c>
+      <c r="C954" t="inlineStr">
+        <is>
+          <t>침대</t>
+        </is>
+      </c>
+    </row>
+    <row r="955">
+      <c r="A955" t="inlineStr">
+        <is>
+          <t>bed.option.heal</t>
+        </is>
+      </c>
+      <c r="B955" t="inlineStr">
+        <is>
+          <t>Rest</t>
+        </is>
+      </c>
+      <c r="C955" t="inlineStr">
+        <is>
+          <t>쉬기</t>
+        </is>
+      </c>
+    </row>
+    <row r="956">
+      <c r="A956" t="inlineStr">
+        <is>
+          <t>bed.option.upgrade</t>
+        </is>
+      </c>
+      <c r="B956" t="inlineStr">
+        <is>
+          <t>Upgrade a skill</t>
+        </is>
+      </c>
+      <c r="C956" t="inlineStr">
+        <is>
+          <t>기술 강화</t>
+        </is>
+      </c>
+    </row>
+    <row r="957">
+      <c r="A957" t="inlineStr">
+        <is>
+          <t>bed.option.leave</t>
+        </is>
+      </c>
+      <c r="B957" t="inlineStr">
+        <is>
+          <t>Leave</t>
+        </is>
+      </c>
+      <c r="C957" t="inlineStr">
+        <is>
+          <t>떠나기</t>
+        </is>
+      </c>
+    </row>
+    <row r="958">
+      <c r="A958" t="inlineStr">
+        <is>
+          <t>bed.help.heal</t>
+        </is>
+      </c>
+      <c r="B958" t="inlineStr">
+        <is>
+          <t>Sleep a while and wake with all your HP and MP.</t>
+        </is>
+      </c>
+      <c r="C958" t="inlineStr">
+        <is>
+          <t>잠시 자고 나면 HP와 MP가 가득 찹니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="959">
+      <c r="A959" t="inlineStr">
+        <is>
+          <t>bed.help.upgrade</t>
+        </is>
+      </c>
+      <c r="B959" t="inlineStr">
+        <is>
+          <t>Think over one of your skills and make it better for good.</t>
+        </is>
+      </c>
+      <c r="C959" t="inlineStr">
+        <is>
+          <t>기술 하나를 곰곰이 되짚어 영구히 더 강하게 만듭니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="960">
+      <c r="A960" t="inlineStr">
+        <is>
+          <t>bed.help.upgrade_none</t>
+        </is>
+      </c>
+      <c r="B960" t="inlineStr">
+        <is>
+          <t>None of your skills can be upgraded any more.</t>
+        </is>
+      </c>
+      <c r="C960" t="inlineStr">
+        <is>
+          <t>더 강화할 수 있는 기술이 없습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="961">
+      <c r="A961" t="inlineStr">
+        <is>
+          <t>bed.help.leave</t>
+        </is>
+      </c>
+      <c r="B961" t="inlineStr">
+        <is>
+          <t>Walk away. The bed stays free for later.</t>
+        </is>
+      </c>
+      <c r="C961" t="inlineStr">
+        <is>
+          <t>그냥 떠납니다. 침대는 나중을 위해 비어 있습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="962">
+      <c r="A962" t="inlineStr">
+        <is>
+          <t>bed.help.back</t>
+        </is>
+      </c>
+      <c r="B962" t="inlineStr">
+        <is>
+          <t>Go back without choosing.</t>
+        </is>
+      </c>
+      <c r="C962" t="inlineStr">
+        <is>
+          <t>고르지 않고 돌아갑니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="963">
+      <c r="A963" t="inlineStr">
+        <is>
+          <t>bed.lbl.hp</t>
+        </is>
+      </c>
+      <c r="B963" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="C963" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+    </row>
+    <row r="964">
+      <c r="A964" t="inlineStr">
+        <is>
+          <t>bed.lbl.mp</t>
+        </is>
+      </c>
+      <c r="B964" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+      <c r="C964" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="965">
+      <c r="A965" t="inlineStr">
+        <is>
+          <t>bed.upgrade_title</t>
+        </is>
+      </c>
+      <c r="B965" t="inlineStr">
+        <is>
+          <t>Upgrade which skill?</t>
+        </is>
+      </c>
+      <c r="C965" t="inlineStr">
+        <is>
+          <t>어떤 기술을 강화할까요?</t>
+        </is>
+      </c>
+    </row>
+    <row r="966">
+      <c r="A966" t="inlineStr">
+        <is>
+          <t>bed.used</t>
+        </is>
+      </c>
+      <c r="B966" t="inlineStr">
+        <is>
+          <t>You have rested here already. The bed is still warm.</t>
+        </is>
+      </c>
+      <c r="C966" t="inlineStr">
+        <is>
+          <t>이미 여기서 쉬었습니다. 침대는 아직 따뜻합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="967">
+      <c r="A967" t="inlineStr">
+        <is>
+          <t>bed.msg.heal</t>
+        </is>
+      </c>
+      <c r="B967" t="inlineStr">
+        <is>
+          <t>You sleep a while. HP and MP are full again.</t>
+        </is>
+      </c>
+      <c r="C967" t="inlineStr">
+        <is>
+          <t>잠시 잠들었습니다. HP와 MP가 다시 가득 찼습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="968">
+      <c r="A968" t="inlineStr">
+        <is>
+          <t>bed.msg.upgrade</t>
+        </is>
+      </c>
+      <c r="B968" t="inlineStr">
+        <is>
+          <t>{skill} is better now.</t>
+        </is>
+      </c>
+      <c r="C968" t="inlineStr">
+        <is>
+          <t>{skill}이(가) 더 강해졌습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="969">
+      <c r="A969" t="inlineStr">
+        <is>
+          <t>settings.row.controls</t>
+        </is>
+      </c>
+      <c r="B969" t="inlineStr">
+        <is>
+          <t>Controls</t>
+        </is>
+      </c>
+      <c r="C969" t="inlineStr">
+        <is>
+          <t>조작</t>
+        </is>
+      </c>
+    </row>
+    <row r="970">
+      <c r="A970" t="inlineStr">
+        <is>
+          <t>settings.help.controls</t>
+        </is>
+      </c>
+      <c r="B970" t="inlineStr">
+        <is>
+          <t>Change the keyboard keys. The controller stays as it is.</t>
+        </is>
+      </c>
+      <c r="C970" t="inlineStr">
+        <is>
+          <t>키보드 키를 바꿉니다. 컨트롤러는 그대로입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="971">
+      <c r="A971" t="inlineStr">
+        <is>
+          <t>controls.title</t>
+        </is>
+      </c>
+      <c r="B971" t="inlineStr">
+        <is>
+          <t>Controls</t>
+        </is>
+      </c>
+      <c r="C971" t="inlineStr">
+        <is>
+          <t>조작</t>
+        </is>
+      </c>
+    </row>
+    <row r="972">
+      <c r="A972" t="inlineStr">
+        <is>
+          <t>controls.row.confirm</t>
+        </is>
+      </c>
+      <c r="B972" t="inlineStr">
+        <is>
+          <t>Confirm</t>
+        </is>
+      </c>
+      <c r="C972" t="inlineStr">
+        <is>
+          <t>확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="973">
+      <c r="A973" t="inlineStr">
+        <is>
+          <t>controls.row.back</t>
+        </is>
+      </c>
+      <c r="B973" t="inlineStr">
+        <is>
+          <t>Back</t>
+        </is>
+      </c>
+      <c r="C973" t="inlineStr">
+        <is>
+          <t>뒤로</t>
+        </is>
+      </c>
+    </row>
+    <row r="974">
+      <c r="A974" t="inlineStr">
+        <is>
+          <t>controls.row.up</t>
+        </is>
+      </c>
+      <c r="B974" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="C974" t="inlineStr">
+        <is>
+          <t>위</t>
+        </is>
+      </c>
+    </row>
+    <row r="975">
+      <c r="A975" t="inlineStr">
+        <is>
+          <t>controls.row.down</t>
+        </is>
+      </c>
+      <c r="B975" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="C975" t="inlineStr">
+        <is>
+          <t>아래</t>
+        </is>
+      </c>
+    </row>
+    <row r="976">
+      <c r="A976" t="inlineStr">
+        <is>
+          <t>controls.row.left</t>
+        </is>
+      </c>
+      <c r="B976" t="inlineStr">
+        <is>
+          <t>Left</t>
+        </is>
+      </c>
+      <c r="C976" t="inlineStr">
+        <is>
+          <t>왼쪽</t>
+        </is>
+      </c>
+    </row>
+    <row r="977">
+      <c r="A977" t="inlineStr">
+        <is>
+          <t>controls.row.right</t>
+        </is>
+      </c>
+      <c r="B977" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="C977" t="inlineStr">
+        <is>
+          <t>오른쪽</t>
+        </is>
+      </c>
+    </row>
+    <row r="978">
+      <c r="A978" t="inlineStr">
+        <is>
+          <t>controls.row.run</t>
+        </is>
+      </c>
+      <c r="B978" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="C978" t="inlineStr">
+        <is>
+          <t>달리기</t>
+        </is>
+      </c>
+    </row>
+    <row r="979">
+      <c r="A979" t="inlineStr">
+        <is>
+          <t>controls.row.tab_prev</t>
+        </is>
+      </c>
+      <c r="B979" t="inlineStr">
+        <is>
+          <t>Previous tab</t>
+        </is>
+      </c>
+      <c r="C979" t="inlineStr">
+        <is>
+          <t>이전 탭</t>
+        </is>
+      </c>
+    </row>
+    <row r="980">
+      <c r="A980" t="inlineStr">
+        <is>
+          <t>controls.row.tab_next</t>
+        </is>
+      </c>
+      <c r="B980" t="inlineStr">
+        <is>
+          <t>Next tab</t>
+        </is>
+      </c>
+      <c r="C980" t="inlineStr">
+        <is>
+          <t>다음 탭</t>
+        </is>
+      </c>
+    </row>
+    <row r="981">
+      <c r="A981" t="inlineStr">
+        <is>
+          <t>controls.row.interact</t>
+        </is>
+      </c>
+      <c r="B981" t="inlineStr">
+        <is>
+          <t>Interact</t>
+        </is>
+      </c>
+      <c r="C981" t="inlineStr">
+        <is>
+          <t>상호작용</t>
+        </is>
+      </c>
+    </row>
+    <row r="982">
+      <c r="A982" t="inlineStr">
+        <is>
+          <t>controls.reset</t>
+        </is>
+      </c>
+      <c r="B982" t="inlineStr">
+        <is>
+          <t>Reset to defaults</t>
+        </is>
+      </c>
+      <c r="C982" t="inlineStr">
+        <is>
+          <t>기본값으로</t>
+        </is>
+      </c>
+    </row>
+    <row r="983">
+      <c r="A983" t="inlineStr">
+        <is>
+          <t>controls.press_key</t>
+        </is>
+      </c>
+      <c r="B983" t="inlineStr">
+        <is>
+          <t>Press a key...</t>
+        </is>
+      </c>
+      <c r="C983" t="inlineStr">
+        <is>
+          <t>키를 누르세요...</t>
+        </is>
+      </c>
+    </row>
+    <row r="984">
+      <c r="A984" t="inlineStr">
+        <is>
+          <t>controls.help.row</t>
+        </is>
+      </c>
+      <c r="B984" t="inlineStr">
+        <is>
+          <t>Confirm, then press the new key. If another action already uses it, the two swap. Esc cancels.</t>
+        </is>
+      </c>
+      <c r="C984" t="inlineStr">
+        <is>
+          <t>확인을 누른 뒤 새 키를 누르세요. 다른 동작이 이미 쓰는 키면 둘이 서로 바뀝니다. Esc로 취소합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="985">
+      <c r="A985" t="inlineStr">
+        <is>
+          <t>controls.help.reset</t>
+        </is>
+      </c>
+      <c r="B985" t="inlineStr">
+        <is>
+          <t>Puts every keyboard key back to how it was. The controller is never changed.</t>
+        </is>
+      </c>
+      <c r="C985" t="inlineStr">
+        <is>
+          <t>키보드 키를 모두 처음대로 되돌립니다. 컨트롤러는 바뀌지 않습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="986">
+      <c r="A986" t="inlineStr">
+        <is>
+          <t>controls.waiting</t>
+        </is>
+      </c>
+      <c r="B986" t="inlineStr">
+        <is>
+          <t>Press the new key for {action}. Esc cancels.</t>
+        </is>
+      </c>
+      <c r="C986" t="inlineStr">
+        <is>
+          <t>{action}에 쓸 새 키를 누르세요. Esc로 취소합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="987">
+      <c r="A987" t="inlineStr">
+        <is>
+          <t>controls.set</t>
+        </is>
+      </c>
+      <c r="B987" t="inlineStr">
+        <is>
+          <t>Key changed. Apply saves it.</t>
+        </is>
+      </c>
+      <c r="C987" t="inlineStr">
+        <is>
+          <t>키가 바뀌었습니다. 적용을 누르면 저장됩니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="988">
+      <c r="A988" t="inlineStr">
+        <is>
+          <t>controls.swapped</t>
+        </is>
+      </c>
+      <c r="B988" t="inlineStr">
+        <is>
+          <t>{other} had that key, so the two swapped.</t>
+        </is>
+      </c>
+      <c r="C988" t="inlineStr">
+        <is>
+          <t>{other}이(가) 그 키를 쓰고 있어 서로 바꿨습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="989">
+      <c r="A989" t="inlineStr">
+        <is>
+          <t>controls.reserved</t>
+        </is>
+      </c>
+      <c r="B989" t="inlineStr">
+        <is>
+          <t>That key is reserved.</t>
+        </is>
+      </c>
+      <c r="C989" t="inlineStr">
+        <is>
+          <t>그 키는 따로 쓰이고 있습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="990">
+      <c r="A990" t="inlineStr">
+        <is>
+          <t>controls.unusable</t>
+        </is>
+      </c>
+      <c r="B990" t="inlineStr">
+        <is>
+          <t>That key cannot be used.</t>
+        </is>
+      </c>
+      <c r="C990" t="inlineStr">
+        <is>
+          <t>그 키는 쓸 수 없습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="991">
+      <c r="A991" t="inlineStr">
+        <is>
+          <t>controls.reset_done</t>
+        </is>
+      </c>
+      <c r="B991" t="inlineStr">
+        <is>
+          <t>Keys are back to the defaults. Apply saves them.</t>
+        </is>
+      </c>
+      <c r="C991" t="inlineStr">
+        <is>
+          <t>키가 기본값으로 돌아갔습니다. 적용을 누르면 저장됩니다.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(ui): battle HUD and dialogue box on the shared framework, Guard command, I-066 plain moves have no defence bar, I-065 verdict (D1a: D89 D95-D101)
Battle: turn strip plate, enemy plate with HP / stagger / status chips, player panel, command menu (Attack Skill Item Guard Run), skill and item lists with icon, MP, details from the data and the arrows, log plate (I-067). Dialogue: frame, name tab, typewriter, arrow, choices above the box. I-065 was a scenario artifact (max HP is derived at every battle start): scenarios use global.scn.boost, bot v=10 plays a levelled Knight through a fight. Old battle draw code and the old HUD removed. C5 note carved_arrow moved out of rm_floor8's only corridor; smoke checks every door stays reachable.

Co-Authored-By: Claude Sonnet <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datafiles/localization/game_text.xlsx
+++ b/datafiles/localization/game_text.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C943"/>
+  <dimension ref="A1:C961"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -504,7 +504,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>목</t>
+          <t>아이템</t>
         </is>
       </c>
     </row>
@@ -521,7 +521,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>달리다</t>
+          <t>도망</t>
         </is>
       </c>
     </row>
@@ -538,7 +538,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>기능</t>
+          <t>기술</t>
         </is>
       </c>
     </row>
@@ -16451,6 +16451,312 @@
       <c r="C943" t="inlineStr">
         <is>
           <t>당신의 강화 효과가 꺼졌습니다!</t>
+        </is>
+      </c>
+    </row>
+    <row r="944">
+      <c r="A944" t="inlineStr">
+        <is>
+          <t>battle.action.guard</t>
+        </is>
+      </c>
+      <c r="B944" t="inlineStr">
+        <is>
+          <t>GUARD</t>
+        </is>
+      </c>
+      <c r="C944" t="inlineStr">
+        <is>
+          <t>방어</t>
+        </is>
+      </c>
+    </row>
+    <row r="945">
+      <c r="A945" t="inlineStr">
+        <is>
+          <t>battle.hud.hp</t>
+        </is>
+      </c>
+      <c r="B945" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="C945" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+    </row>
+    <row r="946">
+      <c r="A946" t="inlineStr">
+        <is>
+          <t>battle.hud.mp</t>
+        </is>
+      </c>
+      <c r="B946" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+      <c r="C946" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="947">
+      <c r="A947" t="inlineStr">
+        <is>
+          <t>battle.hud.level</t>
+        </is>
+      </c>
+      <c r="B947" t="inlineStr">
+        <is>
+          <t>Lv {n}</t>
+        </is>
+      </c>
+      <c r="C947" t="inlineStr">
+        <is>
+          <t>Lv {n}</t>
+        </is>
+      </c>
+    </row>
+    <row r="948">
+      <c r="A948" t="inlineStr">
+        <is>
+          <t>battle.menu.mp</t>
+        </is>
+      </c>
+      <c r="B948" t="inlineStr">
+        <is>
+          <t>{mp} MP</t>
+        </is>
+      </c>
+      <c r="C948" t="inlineStr">
+        <is>
+          <t>{mp} MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="949">
+      <c r="A949" t="inlineStr">
+        <is>
+          <t>battle.det.hits</t>
+        </is>
+      </c>
+      <c r="B949" t="inlineStr">
+        <is>
+          <t>Hits</t>
+        </is>
+      </c>
+      <c r="C949" t="inlineStr">
+        <is>
+          <t>타수</t>
+        </is>
+      </c>
+    </row>
+    <row r="950">
+      <c r="A950" t="inlineStr">
+        <is>
+          <t>battle.det.hp</t>
+        </is>
+      </c>
+      <c r="B950" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="C950" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+    </row>
+    <row r="951">
+      <c r="A951" t="inlineStr">
+        <is>
+          <t>battle.det.mp</t>
+        </is>
+      </c>
+      <c r="B951" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+      <c r="C951" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="952">
+      <c r="A952" t="inlineStr">
+        <is>
+          <t>battle.item.other</t>
+        </is>
+      </c>
+      <c r="B952" t="inlineStr">
+        <is>
+          <t>A useful item.</t>
+        </is>
+      </c>
+      <c r="C952" t="inlineStr">
+        <is>
+          <t>쓸모 있는 물건입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="953">
+      <c r="A953" t="inlineStr">
+        <is>
+          <t>battle.item.heal</t>
+        </is>
+      </c>
+      <c r="B953" t="inlineStr">
+        <is>
+          <t>Restores your HP.</t>
+        </is>
+      </c>
+      <c r="C953" t="inlineStr">
+        <is>
+          <t>HP를 회복합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="954">
+      <c r="A954" t="inlineStr">
+        <is>
+          <t>battle.item.mp</t>
+        </is>
+      </c>
+      <c r="B954" t="inlineStr">
+        <is>
+          <t>Restores your MP.</t>
+        </is>
+      </c>
+      <c r="C954" t="inlineStr">
+        <is>
+          <t>MP를 회복합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="955">
+      <c r="A955" t="inlineStr">
+        <is>
+          <t>battle.item.cure</t>
+        </is>
+      </c>
+      <c r="B955" t="inlineStr">
+        <is>
+          <t>Cures {status}.</t>
+        </is>
+      </c>
+      <c r="C955" t="inlineStr">
+        <is>
+          <t>{status} 상태를 치료합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="956">
+      <c r="A956" t="inlineStr">
+        <is>
+          <t>battle.chip.steadfast</t>
+        </is>
+      </c>
+      <c r="B956" t="inlineStr">
+        <is>
+          <t>Steadfast</t>
+        </is>
+      </c>
+      <c r="C956" t="inlineStr">
+        <is>
+          <t>버티기</t>
+        </is>
+      </c>
+    </row>
+    <row r="957">
+      <c r="A957" t="inlineStr">
+        <is>
+          <t>battle.chip.steadfast.line</t>
+        </is>
+      </c>
+      <c r="B957" t="inlineStr">
+        <is>
+          <t>Cannot be stunned.</t>
+        </is>
+      </c>
+      <c r="C957" t="inlineStr">
+        <is>
+          <t>기절하지 않습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="958">
+      <c r="A958" t="inlineStr">
+        <is>
+          <t>battle.chip.break.line</t>
+        </is>
+      </c>
+      <c r="B958" t="inlineStr">
+        <is>
+          <t>Takes +50% damage until its next turn.</t>
+        </is>
+      </c>
+      <c r="C958" t="inlineStr">
+        <is>
+          <t>다음 차례까지 받는 피해가 50% 늘어납니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="959">
+      <c r="A959" t="inlineStr">
+        <is>
+          <t>combat.msg.guard</t>
+        </is>
+      </c>
+      <c r="B959" t="inlineStr">
+        <is>
+          <t>You brace yourself.</t>
+        </is>
+      </c>
+      <c r="C959" t="inlineStr">
+        <is>
+          <t>당신은 몸을 웅크립니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="960">
+      <c r="A960" t="inlineStr">
+        <is>
+          <t>status.name.status_brace</t>
+        </is>
+      </c>
+      <c r="B960" t="inlineStr">
+        <is>
+          <t>Braced</t>
+        </is>
+      </c>
+      <c r="C960" t="inlineStr">
+        <is>
+          <t>방어 태세</t>
+        </is>
+      </c>
+    </row>
+    <row r="961">
+      <c r="A961" t="inlineStr">
+        <is>
+          <t>status.desc.status_brace</t>
+        </is>
+      </c>
+      <c r="B961" t="inlineStr">
+        <is>
+          <t>Braced for the next hit: it deals {pct}% less damage.</t>
+        </is>
+      </c>
+      <c r="C961" t="inlineStr">
+        <is>
+          <t>다음 공격에 대비합니다. 피해가 {pct}% 줄어듭니다.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(ui): Tab menu, pause menu and Codex on the framework, D115 white text, merchant lines, text rows (D1b: D88-D90, D92, D95-D100, D107, D115)
Co-Authored-By: Claude Sonnet <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datafiles/localization/game_text.xlsx
+++ b/datafiles/localization/game_text.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C927"/>
+  <dimension ref="A1:C1018"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -8302,12 +8302,12 @@
       </c>
       <c r="B464" t="inlineStr">
         <is>
-          <t>Characters per second</t>
+          <t>Chars per sec</t>
         </is>
       </c>
       <c r="C464" t="inlineStr">
         <is>
-          <t>초당 글자 수</t>
+          <t>초당 글자</t>
         </is>
       </c>
     </row>
@@ -16179,6 +16179,1553 @@
       <c r="C927" t="inlineStr">
         <is>
           <t>속박 사격이 적을 기절시켰습니다!</t>
+        </is>
+      </c>
+    </row>
+    <row r="928">
+      <c r="A928" t="inlineStr">
+        <is>
+          <t>pause.help.abandon</t>
+        </is>
+      </c>
+      <c r="B928" t="inlineStr">
+        <is>
+          <t>Ends this run now. It counts as a death, but you keep the echo.</t>
+        </is>
+      </c>
+      <c r="C928" t="inlineStr">
+        <is>
+          <t>지금 도전을 끝냅니다. 죽음으로 기록되지만 메아리는 그대로 가져갑니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="929">
+      <c r="A929" t="inlineStr">
+        <is>
+          <t>pause.help.abandon_armed</t>
+        </is>
+      </c>
+      <c r="B929" t="inlineStr">
+        <is>
+          <t>Confirm once more to end this run now. Back or another row cancels.</t>
+        </is>
+      </c>
+      <c r="C929" t="inlineStr">
+        <is>
+          <t>한 번 더 확인하면 지금 도전이 끝납니다. 뒤로 가기나 다른 항목을 고르면 취소됩니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930" t="inlineStr">
+        <is>
+          <t>pause.help.help</t>
+        </is>
+      </c>
+      <c r="B930" t="inlineStr">
+        <is>
+          <t>Every hint the game has: the ones you have seen and the ones still to come.</t>
+        </is>
+      </c>
+      <c r="C930" t="inlineStr">
+        <is>
+          <t>게임이 알려 주는 모든 도움말입니다. 본 것도, 앞으로 볼 것도 있습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931" t="inlineStr">
+        <is>
+          <t>pause.help.quit</t>
+        </is>
+      </c>
+      <c r="B931" t="inlineStr">
+        <is>
+          <t>Saves the run and goes to the title. Continue picks it up again.</t>
+        </is>
+      </c>
+      <c r="C931" t="inlineStr">
+        <is>
+          <t>도전을 저장하고 타이틀로 갑니다. 이어하기로 다시 시작할 수 있습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="932">
+      <c r="A932" t="inlineStr">
+        <is>
+          <t>pause.help.resume</t>
+        </is>
+      </c>
+      <c r="B932" t="inlineStr">
+        <is>
+          <t>Back to the game.</t>
+        </is>
+      </c>
+      <c r="C932" t="inlineStr">
+        <is>
+          <t>게임으로 돌아갑니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="933">
+      <c r="A933" t="inlineStr">
+        <is>
+          <t>pause.help.settings</t>
+        </is>
+      </c>
+      <c r="B933" t="inlineStr">
+        <is>
+          <t>Sound, text, window, language and keys.</t>
+        </is>
+      </c>
+      <c r="C933" t="inlineStr">
+        <is>
+          <t>소리, 글자, 창, 언어, 키를 바꿉니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="934">
+      <c r="A934" t="inlineStr">
+        <is>
+          <t>pause.option.quit</t>
+        </is>
+      </c>
+      <c r="B934" t="inlineStr">
+        <is>
+          <t>Quit to title</t>
+        </is>
+      </c>
+      <c r="C934" t="inlineStr">
+        <is>
+          <t>타이틀로 나가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="935">
+      <c r="A935" t="inlineStr">
+        <is>
+          <t>pause.title</t>
+        </is>
+      </c>
+      <c r="B935" t="inlineStr">
+        <is>
+          <t>Paused</t>
+        </is>
+      </c>
+      <c r="C935" t="inlineStr">
+        <is>
+          <t>일시 정지</t>
+        </is>
+      </c>
+    </row>
+    <row r="936">
+      <c r="A936" t="inlineStr">
+        <is>
+          <t>tab.bestiary.attack</t>
+        </is>
+      </c>
+      <c r="B936" t="inlineStr">
+        <is>
+          <t>Attack</t>
+        </is>
+      </c>
+      <c r="C936" t="inlineStr">
+        <is>
+          <t>공격</t>
+        </is>
+      </c>
+    </row>
+    <row r="937">
+      <c r="A937" t="inlineStr">
+        <is>
+          <t>tab.bestiary.boss</t>
+        </is>
+      </c>
+      <c r="B937" t="inlineStr">
+        <is>
+          <t>A boss.</t>
+        </is>
+      </c>
+      <c r="C937" t="inlineStr">
+        <is>
+          <t>보스입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="938">
+      <c r="A938" t="inlineStr">
+        <is>
+          <t>tab.bestiary.moves</t>
+        </is>
+      </c>
+      <c r="B938" t="inlineStr">
+        <is>
+          <t>Moves: {list}.</t>
+        </is>
+      </c>
+      <c r="C938" t="inlineStr">
+        <is>
+          <t>행동: {list}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="939">
+      <c r="A939" t="inlineStr">
+        <is>
+          <t>tab.bestiary.unknown</t>
+        </is>
+      </c>
+      <c r="B939" t="inlineStr">
+        <is>
+          <t>You have not met this one yet.</t>
+        </is>
+      </c>
+      <c r="C939" t="inlineStr">
+        <is>
+          <t>아직 만난 적 없는 적입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="940">
+      <c r="A940" t="inlineStr">
+        <is>
+          <t>tab.codex</t>
+        </is>
+      </c>
+      <c r="B940" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="C940" t="inlineStr">
+        <is>
+          <t>도감</t>
+        </is>
+      </c>
+    </row>
+    <row r="941">
+      <c r="A941" t="inlineStr">
+        <is>
+          <t>tab.codex.bestiary</t>
+        </is>
+      </c>
+      <c r="B941" t="inlineStr">
+        <is>
+          <t>Bestiary</t>
+        </is>
+      </c>
+      <c r="C941" t="inlineStr">
+        <is>
+          <t>적 도감</t>
+        </is>
+      </c>
+    </row>
+    <row r="942">
+      <c r="A942" t="inlineStr">
+        <is>
+          <t>tab.codex.bestiary_help</t>
+        </is>
+      </c>
+      <c r="B942" t="inlineStr">
+        <is>
+          <t>The enemies you have met: their numbers and their moves.</t>
+        </is>
+      </c>
+      <c r="C942" t="inlineStr">
+        <is>
+          <t>만난 적들의 능력치와 행동입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="943">
+      <c r="A943" t="inlineStr">
+        <is>
+          <t>tab.codex.bestiary_title</t>
+        </is>
+      </c>
+      <c r="B943" t="inlineStr">
+        <is>
+          <t>Bestiary {n}/{max}</t>
+        </is>
+      </c>
+      <c r="C943" t="inlineStr">
+        <is>
+          <t>적 도감 {n}/{max}</t>
+        </is>
+      </c>
+    </row>
+    <row r="944">
+      <c r="A944" t="inlineStr">
+        <is>
+          <t>tab.codex.history</t>
+        </is>
+      </c>
+      <c r="B944" t="inlineStr">
+        <is>
+          <t>Run history</t>
+        </is>
+      </c>
+      <c r="C944" t="inlineStr">
+        <is>
+          <t>도전 기록</t>
+        </is>
+      </c>
+    </row>
+    <row r="945">
+      <c r="A945" t="inlineStr">
+        <is>
+          <t>tab.codex.history_help</t>
+        </is>
+      </c>
+      <c r="B945" t="inlineStr">
+        <is>
+          <t>Every run you have finished, newest first.</t>
+        </is>
+      </c>
+      <c r="C945" t="inlineStr">
+        <is>
+          <t>끝낸 도전이 최근 순서로 나옵니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="946">
+      <c r="A946" t="inlineStr">
+        <is>
+          <t>tab.codex.notes</t>
+        </is>
+      </c>
+      <c r="B946" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="C946" t="inlineStr">
+        <is>
+          <t>쪽지</t>
+        </is>
+      </c>
+    </row>
+    <row r="947">
+      <c r="A947" t="inlineStr">
+        <is>
+          <t>tab.codex.notes_help</t>
+        </is>
+      </c>
+      <c r="B947" t="inlineStr">
+        <is>
+          <t>The notes you have read in the tunnel.</t>
+        </is>
+      </c>
+      <c r="C947" t="inlineStr">
+        <is>
+          <t>터널에서 읽은 쪽지입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="948">
+      <c r="A948" t="inlineStr">
+        <is>
+          <t>tab.codex.notes_title</t>
+        </is>
+      </c>
+      <c r="B948" t="inlineStr">
+        <is>
+          <t>Notes {n}/{max}</t>
+        </is>
+      </c>
+      <c r="C948" t="inlineStr">
+        <is>
+          <t>쪽지 {n}/{max}</t>
+        </is>
+      </c>
+    </row>
+    <row r="949">
+      <c r="A949" t="inlineStr">
+        <is>
+          <t>tab.codex.unlocks</t>
+        </is>
+      </c>
+      <c r="B949" t="inlineStr">
+        <is>
+          <t>Unlocks</t>
+        </is>
+      </c>
+      <c r="C949" t="inlineStr">
+        <is>
+          <t>해금</t>
+        </is>
+      </c>
+    </row>
+    <row r="950">
+      <c r="A950" t="inlineStr">
+        <is>
+          <t>tab.codex.unlocks_help</t>
+        </is>
+      </c>
+      <c r="B950" t="inlineStr">
+        <is>
+          <t>What winning has opened up for later runs.</t>
+        </is>
+      </c>
+      <c r="C950" t="inlineStr">
+        <is>
+          <t>승리로 이후 도전에 열린 것들입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="951">
+      <c r="A951" t="inlineStr">
+        <is>
+          <t>tab.gear</t>
+        </is>
+      </c>
+      <c r="B951" t="inlineStr">
+        <is>
+          <t>Gear</t>
+        </is>
+      </c>
+      <c r="C951" t="inlineStr">
+        <is>
+          <t>장비</t>
+        </is>
+      </c>
+    </row>
+    <row r="952">
+      <c r="A952" t="inlineStr">
+        <is>
+          <t>tab.gear.bag</t>
+        </is>
+      </c>
+      <c r="B952" t="inlineStr">
+        <is>
+          <t>Bag</t>
+        </is>
+      </c>
+      <c r="C952" t="inlineStr">
+        <is>
+          <t>가방</t>
+        </is>
+      </c>
+    </row>
+    <row r="953">
+      <c r="A953" t="inlineStr">
+        <is>
+          <t>tab.gear.empty</t>
+        </is>
+      </c>
+      <c r="B953" t="inlineStr">
+        <is>
+          <t>Nothing worn</t>
+        </is>
+      </c>
+      <c r="C953" t="inlineStr">
+        <is>
+          <t>착용 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="954">
+      <c r="A954" t="inlineStr">
+        <is>
+          <t>tab.gear.empty_help</t>
+        </is>
+      </c>
+      <c r="B954" t="inlineStr">
+        <is>
+          <t>Nothing is worn in this slot.</t>
+        </is>
+      </c>
+      <c r="C954" t="inlineStr">
+        <is>
+          <t>이 칸에는 아무것도 착용하지 않았습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="955">
+      <c r="A955" t="inlineStr">
+        <is>
+          <t>tab.gear.no_accessory</t>
+        </is>
+      </c>
+      <c r="B955" t="inlineStr">
+        <is>
+          <t>No accessory</t>
+        </is>
+      </c>
+      <c r="C955" t="inlineStr">
+        <is>
+          <t>장신구 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="956">
+      <c r="A956" t="inlineStr">
+        <is>
+          <t>tab.gear.no_armor</t>
+        </is>
+      </c>
+      <c r="B956" t="inlineStr">
+        <is>
+          <t>No armor</t>
+        </is>
+      </c>
+      <c r="C956" t="inlineStr">
+        <is>
+          <t>방어구 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="957">
+      <c r="A957" t="inlineStr">
+        <is>
+          <t>tab.gear.no_weapon</t>
+        </is>
+      </c>
+      <c r="B957" t="inlineStr">
+        <is>
+          <t>No weapon</t>
+        </is>
+      </c>
+      <c r="C957" t="inlineStr">
+        <is>
+          <t>무기 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="958">
+      <c r="A958" t="inlineStr">
+        <is>
+          <t>tab.gear.replaces</t>
+        </is>
+      </c>
+      <c r="B958" t="inlineStr">
+        <is>
+          <t>Replaces {item}.</t>
+        </is>
+      </c>
+      <c r="C958" t="inlineStr">
+        <is>
+          <t>{item}을(를) 대체합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="959">
+      <c r="A959" t="inlineStr">
+        <is>
+          <t>tab.gear.worn</t>
+        </is>
+      </c>
+      <c r="B959" t="inlineStr">
+        <is>
+          <t>Worn</t>
+        </is>
+      </c>
+      <c r="C959" t="inlineStr">
+        <is>
+          <t>착용 중</t>
+        </is>
+      </c>
+    </row>
+    <row r="960">
+      <c r="A960" t="inlineStr">
+        <is>
+          <t>tab.hint.back</t>
+        </is>
+      </c>
+      <c r="B960" t="inlineStr">
+        <is>
+          <t>{back} Back</t>
+        </is>
+      </c>
+      <c r="C960" t="inlineStr">
+        <is>
+          <t>{back} 뒤로</t>
+        </is>
+      </c>
+    </row>
+    <row r="961">
+      <c r="A961" t="inlineStr">
+        <is>
+          <t>tab.hint.change</t>
+        </is>
+      </c>
+      <c r="B961" t="inlineStr">
+        <is>
+          <t>{left}{right} Change</t>
+        </is>
+      </c>
+      <c r="C961" t="inlineStr">
+        <is>
+          <t>{left}{right} 변경</t>
+        </is>
+      </c>
+    </row>
+    <row r="962">
+      <c r="A962" t="inlineStr">
+        <is>
+          <t>tab.hint.close</t>
+        </is>
+      </c>
+      <c r="B962" t="inlineStr">
+        <is>
+          <t>{back} Close</t>
+        </is>
+      </c>
+      <c r="C962" t="inlineStr">
+        <is>
+          <t>{back} 닫기</t>
+        </is>
+      </c>
+    </row>
+    <row r="963">
+      <c r="A963" t="inlineStr">
+        <is>
+          <t>tab.hint.equip</t>
+        </is>
+      </c>
+      <c r="B963" t="inlineStr">
+        <is>
+          <t>{confirm} Equip</t>
+        </is>
+      </c>
+      <c r="C963" t="inlineStr">
+        <is>
+          <t>{confirm} 착용</t>
+        </is>
+      </c>
+    </row>
+    <row r="964">
+      <c r="A964" t="inlineStr">
+        <is>
+          <t>tab.hint.open</t>
+        </is>
+      </c>
+      <c r="B964" t="inlineStr">
+        <is>
+          <t>{confirm} Open</t>
+        </is>
+      </c>
+      <c r="C964" t="inlineStr">
+        <is>
+          <t>{confirm} 열기</t>
+        </is>
+      </c>
+    </row>
+    <row r="965">
+      <c r="A965" t="inlineStr">
+        <is>
+          <t>tab.hint.select</t>
+        </is>
+      </c>
+      <c r="B965" t="inlineStr">
+        <is>
+          <t>{confirm} Select</t>
+        </is>
+      </c>
+      <c r="C965" t="inlineStr">
+        <is>
+          <t>{confirm} 선택</t>
+        </is>
+      </c>
+    </row>
+    <row r="966">
+      <c r="A966" t="inlineStr">
+        <is>
+          <t>tab.hint.takeoff</t>
+        </is>
+      </c>
+      <c r="B966" t="inlineStr">
+        <is>
+          <t>{confirm} Take off</t>
+        </is>
+      </c>
+      <c r="C966" t="inlineStr">
+        <is>
+          <t>{confirm} 해제</t>
+        </is>
+      </c>
+    </row>
+    <row r="967">
+      <c r="A967" t="inlineStr">
+        <is>
+          <t>tab.hint.use</t>
+        </is>
+      </c>
+      <c r="B967" t="inlineStr">
+        <is>
+          <t>{confirm} Use</t>
+        </is>
+      </c>
+      <c r="C967" t="inlineStr">
+        <is>
+          <t>{confirm} 사용</t>
+        </is>
+      </c>
+    </row>
+    <row r="968">
+      <c r="A968" t="inlineStr">
+        <is>
+          <t>tab.hist.abandoned</t>
+        </is>
+      </c>
+      <c r="B968" t="inlineStr">
+        <is>
+          <t>You gave this run up on floor {n}.</t>
+        </is>
+      </c>
+      <c r="C968" t="inlineStr">
+        <is>
+          <t>{n}층에서 도전을 포기했습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="969">
+      <c r="A969" t="inlineStr">
+        <is>
+          <t>tab.hist.died</t>
+        </is>
+      </c>
+      <c r="B969" t="inlineStr">
+        <is>
+          <t>You fell on floor {n}.</t>
+        </is>
+      </c>
+      <c r="C969" t="inlineStr">
+        <is>
+          <t>{n}층에서 쓰러졌습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="970">
+      <c r="A970" t="inlineStr">
+        <is>
+          <t>tab.hist.died_to</t>
+        </is>
+      </c>
+      <c r="B970" t="inlineStr">
+        <is>
+          <t>Floor {n}: felled by {name}.</t>
+        </is>
+      </c>
+      <c r="C970" t="inlineStr">
+        <is>
+          <t>{n}층: {name}에게 쓰러졌습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="971">
+      <c r="A971" t="inlineStr">
+        <is>
+          <t>tab.hist.row</t>
+        </is>
+      </c>
+      <c r="B971" t="inlineStr">
+        <is>
+          <t>{cls} Lv {n}</t>
+        </is>
+      </c>
+      <c r="C971" t="inlineStr">
+        <is>
+          <t>{cls} Lv {n}</t>
+        </is>
+      </c>
+    </row>
+    <row r="972">
+      <c r="A972" t="inlineStr">
+        <is>
+          <t>tab.hist.won</t>
+        </is>
+      </c>
+      <c r="B972" t="inlineStr">
+        <is>
+          <t>You climbed out of the tunnel.</t>
+        </is>
+      </c>
+      <c r="C972" t="inlineStr">
+        <is>
+          <t>터널을 빠져나왔습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="973">
+      <c r="A973" t="inlineStr">
+        <is>
+          <t>tab.items</t>
+        </is>
+      </c>
+      <c r="B973" t="inlineStr">
+        <is>
+          <t>Items</t>
+        </is>
+      </c>
+      <c r="C973" t="inlineStr">
+        <is>
+          <t>아이템</t>
+        </is>
+      </c>
+    </row>
+    <row r="974">
+      <c r="A974" t="inlineStr">
+        <is>
+          <t>tab.items.key</t>
+        </is>
+      </c>
+      <c r="B974" t="inlineStr">
+        <is>
+          <t>An item you keep for the way ahead.</t>
+        </is>
+      </c>
+      <c r="C974" t="inlineStr">
+        <is>
+          <t>앞으로의 길을 위해 간직하는 아이템입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="975">
+      <c r="A975" t="inlineStr">
+        <is>
+          <t>tab.items.none</t>
+        </is>
+      </c>
+      <c r="B975" t="inlineStr">
+        <is>
+          <t>Nothing in your bag</t>
+        </is>
+      </c>
+      <c r="C975" t="inlineStr">
+        <is>
+          <t>소지품이 없습니다</t>
+        </is>
+      </c>
+    </row>
+    <row r="976">
+      <c r="A976" t="inlineStr">
+        <is>
+          <t>tab.items.none_help</t>
+        </is>
+      </c>
+      <c r="B976" t="inlineStr">
+        <is>
+          <t>Potions, throwables and keys you find show up here.</t>
+        </is>
+      </c>
+      <c r="C976" t="inlineStr">
+        <is>
+          <t>찾은 물약, 투척 아이템, 열쇠가 여기에 나옵니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="977">
+      <c r="A977" t="inlineStr">
+        <is>
+          <t>tab.lbl.base</t>
+        </is>
+      </c>
+      <c r="B977" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C977" t="inlineStr">
+        <is>
+          <t>기본</t>
+        </is>
+      </c>
+    </row>
+    <row r="978">
+      <c r="A978" t="inlineStr">
+        <is>
+          <t>tab.lbl.best_floor</t>
+        </is>
+      </c>
+      <c r="B978" t="inlineStr">
+        <is>
+          <t>Best floor</t>
+        </is>
+      </c>
+      <c r="C978" t="inlineStr">
+        <is>
+          <t>최고 층</t>
+        </is>
+      </c>
+    </row>
+    <row r="979">
+      <c r="A979" t="inlineStr">
+        <is>
+          <t>tab.lbl.effects</t>
+        </is>
+      </c>
+      <c r="B979" t="inlineStr">
+        <is>
+          <t>Effects</t>
+        </is>
+      </c>
+      <c r="C979" t="inlineStr">
+        <is>
+          <t>효과</t>
+        </is>
+      </c>
+    </row>
+    <row r="980">
+      <c r="A980" t="inlineStr">
+        <is>
+          <t>tab.lbl.elite</t>
+        </is>
+      </c>
+      <c r="B980" t="inlineStr">
+        <is>
+          <t>Elite</t>
+        </is>
+      </c>
+      <c r="C980" t="inlineStr">
+        <is>
+          <t>정예</t>
+        </is>
+      </c>
+    </row>
+    <row r="981">
+      <c r="A981" t="inlineStr">
+        <is>
+          <t>tab.lbl.falls</t>
+        </is>
+      </c>
+      <c r="B981" t="inlineStr">
+        <is>
+          <t>Falls</t>
+        </is>
+      </c>
+      <c r="C981" t="inlineStr">
+        <is>
+          <t>추락</t>
+        </is>
+      </c>
+    </row>
+    <row r="982">
+      <c r="A982" t="inlineStr">
+        <is>
+          <t>tab.lbl.floor</t>
+        </is>
+      </c>
+      <c r="B982" t="inlineStr">
+        <is>
+          <t>Floor</t>
+        </is>
+      </c>
+      <c r="C982" t="inlineStr">
+        <is>
+          <t>층</t>
+        </is>
+      </c>
+    </row>
+    <row r="983">
+      <c r="A983" t="inlineStr">
+        <is>
+          <t>tab.lbl.gear</t>
+        </is>
+      </c>
+      <c r="B983" t="inlineStr">
+        <is>
+          <t>Gear</t>
+        </is>
+      </c>
+      <c r="C983" t="inlineStr">
+        <is>
+          <t>장비</t>
+        </is>
+      </c>
+    </row>
+    <row r="984">
+      <c r="A984" t="inlineStr">
+        <is>
+          <t>tab.lbl.gold</t>
+        </is>
+      </c>
+      <c r="B984" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="C984" t="inlineStr">
+        <is>
+          <t>골드</t>
+        </is>
+      </c>
+    </row>
+    <row r="985">
+      <c r="A985" t="inlineStr">
+        <is>
+          <t>tab.lbl.hp</t>
+        </is>
+      </c>
+      <c r="B985" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="C985" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+    </row>
+    <row r="986">
+      <c r="A986" t="inlineStr">
+        <is>
+          <t>tab.lbl.kills</t>
+        </is>
+      </c>
+      <c r="B986" t="inlineStr">
+        <is>
+          <t>Foes beaten</t>
+        </is>
+      </c>
+      <c r="C986" t="inlineStr">
+        <is>
+          <t>처치한 적</t>
+        </is>
+      </c>
+    </row>
+    <row r="987">
+      <c r="A987" t="inlineStr">
+        <is>
+          <t>tab.lbl.level</t>
+        </is>
+      </c>
+      <c r="B987" t="inlineStr">
+        <is>
+          <t>Level</t>
+        </is>
+      </c>
+      <c r="C987" t="inlineStr">
+        <is>
+          <t>레벨</t>
+        </is>
+      </c>
+    </row>
+    <row r="988">
+      <c r="A988" t="inlineStr">
+        <is>
+          <t>tab.lbl.met</t>
+        </is>
+      </c>
+      <c r="B988" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="C988" t="inlineStr">
+        <is>
+          <t>만난 횟수</t>
+        </is>
+      </c>
+    </row>
+    <row r="989">
+      <c r="A989" t="inlineStr">
+        <is>
+          <t>tab.lbl.seed</t>
+        </is>
+      </c>
+      <c r="B989" t="inlineStr">
+        <is>
+          <t>Seed</t>
+        </is>
+      </c>
+      <c r="C989" t="inlineStr">
+        <is>
+          <t>시드</t>
+        </is>
+      </c>
+    </row>
+    <row r="990">
+      <c r="A990" t="inlineStr">
+        <is>
+          <t>tab.lbl.seed_small</t>
+        </is>
+      </c>
+      <c r="B990" t="inlineStr">
+        <is>
+          <t>Seed {n}</t>
+        </is>
+      </c>
+      <c r="C990" t="inlineStr">
+        <is>
+          <t>시드 {n}</t>
+        </is>
+      </c>
+    </row>
+    <row r="991">
+      <c r="A991" t="inlineStr">
+        <is>
+          <t>tab.lbl.total</t>
+        </is>
+      </c>
+      <c r="B991" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C991" t="inlineStr">
+        <is>
+          <t>합계</t>
+        </is>
+      </c>
+    </row>
+    <row r="992">
+      <c r="A992" t="inlineStr">
+        <is>
+          <t>tab.lbl.upgrade</t>
+        </is>
+      </c>
+      <c r="B992" t="inlineStr">
+        <is>
+          <t>Upgrade</t>
+        </is>
+      </c>
+      <c r="C992" t="inlineStr">
+        <is>
+          <t>강화</t>
+        </is>
+      </c>
+    </row>
+    <row r="993">
+      <c r="A993" t="inlineStr">
+        <is>
+          <t>tab.lbl.wins</t>
+        </is>
+      </c>
+      <c r="B993" t="inlineStr">
+        <is>
+          <t>Wins</t>
+        </is>
+      </c>
+      <c r="C993" t="inlineStr">
+        <is>
+          <t>승리</t>
+        </is>
+      </c>
+    </row>
+    <row r="994">
+      <c r="A994" t="inlineStr">
+        <is>
+          <t>tab.lbl.xp</t>
+        </is>
+      </c>
+      <c r="B994" t="inlineStr">
+        <is>
+          <t>XP</t>
+        </is>
+      </c>
+      <c r="C994" t="inlineStr">
+        <is>
+          <t>경험치</t>
+        </is>
+      </c>
+    </row>
+    <row r="995">
+      <c r="A995" t="inlineStr">
+        <is>
+          <t>tab.notes.unknown</t>
+        </is>
+      </c>
+      <c r="B995" t="inlineStr">
+        <is>
+          <t>A note you have not found yet. Look at the walls.</t>
+        </is>
+      </c>
+      <c r="C995" t="inlineStr">
+        <is>
+          <t>아직 찾지 못한 쪽지입니다. 벽을 살펴보세요.</t>
+        </is>
+      </c>
+    </row>
+    <row r="996">
+      <c r="A996" t="inlineStr">
+        <is>
+          <t>tab.settings</t>
+        </is>
+      </c>
+      <c r="B996" t="inlineStr">
+        <is>
+          <t>Settings</t>
+        </is>
+      </c>
+      <c r="C996" t="inlineStr">
+        <is>
+          <t>설정</t>
+        </is>
+      </c>
+    </row>
+    <row r="997">
+      <c r="A997" t="inlineStr">
+        <is>
+          <t>tab.skills</t>
+        </is>
+      </c>
+      <c r="B997" t="inlineStr">
+        <is>
+          <t>Skills</t>
+        </is>
+      </c>
+      <c r="C997" t="inlineStr">
+        <is>
+          <t>스킬</t>
+        </is>
+      </c>
+    </row>
+    <row r="998">
+      <c r="A998" t="inlineStr">
+        <is>
+          <t>tab.skills.none</t>
+        </is>
+      </c>
+      <c r="B998" t="inlineStr">
+        <is>
+          <t>No skills yet</t>
+        </is>
+      </c>
+      <c r="C998" t="inlineStr">
+        <is>
+          <t>스킬 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="999">
+      <c r="A999" t="inlineStr">
+        <is>
+          <t>tab.skills.none_help</t>
+        </is>
+      </c>
+      <c r="B999" t="inlineStr">
+        <is>
+          <t>Cards and chests teach skills. They appear here with the arrows to press.</t>
+        </is>
+      </c>
+      <c r="C999" t="inlineStr">
+        <is>
+          <t>카드와 상자에서 스킬을 얻습니다. 누를 화살표와 함께 여기에 나옵니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1000">
+      <c r="A1000" t="inlineStr">
+        <is>
+          <t>tab.skills.passives</t>
+        </is>
+      </c>
+      <c r="B1000" t="inlineStr">
+        <is>
+          <t>Passives</t>
+        </is>
+      </c>
+      <c r="C1000" t="inlineStr">
+        <is>
+          <t>패시브</t>
+        </is>
+      </c>
+    </row>
+    <row r="1001">
+      <c r="A1001" t="inlineStr">
+        <is>
+          <t>tab.status</t>
+        </is>
+      </c>
+      <c r="B1001" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="C1001" t="inlineStr">
+        <is>
+          <t>상태</t>
+        </is>
+      </c>
+    </row>
+    <row r="1002">
+      <c r="A1002" t="inlineStr">
+        <is>
+          <t>tab.title.codex</t>
+        </is>
+      </c>
+      <c r="B1002" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="C1002" t="inlineStr">
+        <is>
+          <t>도감</t>
+        </is>
+      </c>
+    </row>
+    <row r="1003">
+      <c r="A1003" t="inlineStr">
+        <is>
+          <t>tab.title.gear</t>
+        </is>
+      </c>
+      <c r="B1003" t="inlineStr">
+        <is>
+          <t>Gear</t>
+        </is>
+      </c>
+      <c r="C1003" t="inlineStr">
+        <is>
+          <t>장비</t>
+        </is>
+      </c>
+    </row>
+    <row r="1004">
+      <c r="A1004" t="inlineStr">
+        <is>
+          <t>tab.title.items</t>
+        </is>
+      </c>
+      <c r="B1004" t="inlineStr">
+        <is>
+          <t>Items</t>
+        </is>
+      </c>
+      <c r="C1004" t="inlineStr">
+        <is>
+          <t>아이템</t>
+        </is>
+      </c>
+    </row>
+    <row r="1005">
+      <c r="A1005" t="inlineStr">
+        <is>
+          <t>tab.title.skills</t>
+        </is>
+      </c>
+      <c r="B1005" t="inlineStr">
+        <is>
+          <t>Skills {n}/{max}</t>
+        </is>
+      </c>
+      <c r="C1005" t="inlineStr">
+        <is>
+          <t>스킬 {n}/{max}</t>
+        </is>
+      </c>
+    </row>
+    <row r="1006">
+      <c r="A1006" t="inlineStr">
+        <is>
+          <t>tab.title.status</t>
+        </is>
+      </c>
+      <c r="B1006" t="inlineStr">
+        <is>
+          <t>Stats</t>
+        </is>
+      </c>
+      <c r="C1006" t="inlineStr">
+        <is>
+          <t>능력치</t>
+        </is>
+      </c>
+    </row>
+    <row r="1007">
+      <c r="A1007" t="inlineStr">
+        <is>
+          <t>tab.unlock.nobody</t>
+        </is>
+      </c>
+      <c r="B1007" t="inlineStr">
+        <is>
+          <t>Nobody</t>
+        </is>
+      </c>
+      <c r="C1007" t="inlineStr">
+        <is>
+          <t>무명</t>
+        </is>
+      </c>
+    </row>
+    <row r="1008">
+      <c r="A1008" t="inlineStr">
+        <is>
+          <t>tab.unlock.nobody_off</t>
+        </is>
+      </c>
+      <c r="B1008" t="inlineStr">
+        <is>
+          <t>Win a run to unlock a fighter with no class.</t>
+        </is>
+      </c>
+      <c r="C1008" t="inlineStr">
+        <is>
+          <t>승리하면 직업이 없는 전사가 해금됩니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1009">
+      <c r="A1009" t="inlineStr">
+        <is>
+          <t>tab.unlock.nobody_on</t>
+        </is>
+      </c>
+      <c r="B1009" t="inlineStr">
+        <is>
+          <t>A fighter with no class. Throws {m}x as hard and carries {cap} of each throwable.</t>
+        </is>
+      </c>
+      <c r="C1009" t="inlineStr">
+        <is>
+          <t>직업이 없는 전사입니다. 투척 아이템을 {m}배 강하게 던지고 종류마다 {cap}개를 가질 수 있습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1010">
+      <c r="A1010" t="inlineStr">
+        <is>
+          <t>tab.val.abandoned</t>
+        </is>
+      </c>
+      <c r="B1010" t="inlineStr">
+        <is>
+          <t>Gave up</t>
+        </is>
+      </c>
+      <c r="C1010" t="inlineStr">
+        <is>
+          <t>포기</t>
+        </is>
+      </c>
+    </row>
+    <row r="1011">
+      <c r="A1011" t="inlineStr">
+        <is>
+          <t>tab.val.applied</t>
+        </is>
+      </c>
+      <c r="B1011" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="C1011" t="inlineStr">
+        <is>
+          <t>적용됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="1012">
+      <c r="A1012" t="inlineStr">
+        <is>
+          <t>tab.val.floor</t>
+        </is>
+      </c>
+      <c r="B1012" t="inlineStr">
+        <is>
+          <t>Floor {n}</t>
+        </is>
+      </c>
+      <c r="C1012" t="inlineStr">
+        <is>
+          <t>{n}층</t>
+        </is>
+      </c>
+    </row>
+    <row r="1013">
+      <c r="A1013" t="inlineStr">
+        <is>
+          <t>tab.val.locked</t>
+        </is>
+      </c>
+      <c r="B1013" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+      <c r="C1013" t="inlineStr">
+        <is>
+          <t>잠김</t>
+        </is>
+      </c>
+    </row>
+    <row r="1014">
+      <c r="A1014" t="inlineStr">
+        <is>
+          <t>tab.val.max</t>
+        </is>
+      </c>
+      <c r="B1014" t="inlineStr">
+        <is>
+          <t>MAX</t>
+        </is>
+      </c>
+      <c r="C1014" t="inlineStr">
+        <is>
+          <t>최대</t>
+        </is>
+      </c>
+    </row>
+    <row r="1015">
+      <c r="A1015" t="inlineStr">
+        <is>
+          <t>tab.val.none</t>
+        </is>
+      </c>
+      <c r="B1015" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="C1015" t="inlineStr">
+        <is>
+          <t>없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="1016">
+      <c r="A1016" t="inlineStr">
+        <is>
+          <t>tab.val.seen</t>
+        </is>
+      </c>
+      <c r="B1016" t="inlineStr">
+        <is>
+          <t>Seen</t>
+        </is>
+      </c>
+      <c r="C1016" t="inlineStr">
+        <is>
+          <t>목격</t>
+        </is>
+      </c>
+    </row>
+    <row r="1017">
+      <c r="A1017" t="inlineStr">
+        <is>
+          <t>tab.val.unlocked</t>
+        </is>
+      </c>
+      <c r="B1017" t="inlineStr">
+        <is>
+          <t>Unlocked</t>
+        </is>
+      </c>
+      <c r="C1017" t="inlineStr">
+        <is>
+          <t>해금됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="1018">
+      <c r="A1018" t="inlineStr">
+        <is>
+          <t>tab.val.won</t>
+        </is>
+      </c>
+      <c r="B1018" t="inlineStr">
+        <is>
+          <t>Won</t>
+        </is>
+      </c>
+      <c r="C1018" t="inlineStr">
+        <is>
+          <t>승리</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(ui): pause on focus loss, flee % on RUN, crit odds in plain words (D122, D124)
- Focus_ShouldPause / Focus_Step (scr_menu): window unfocused -> pause menu (battle variant in a fight), music lowered to 25% through BGM_Duck and restored exactly on focus
- PauseMenu_Items/Open(_in_battle): Abandon run and Quit to title off in a battle
- Battle_RunPct, Battle_CmdItems(_bc): RUN row shows the flee chance, "no" for bosses; the battle controller draws the pause menu over its HUD
- Take Aim status line from Crit_BagSize ("1 in every 4 hits is a critical.")
- Loc rows + KO draft; smoke steps 200-205, shots 200-203 (gate expects 169 shots)

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datafiles/localization/game_text.xlsx
+++ b/datafiles/localization/game_text.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1018"/>
+  <dimension ref="A1:C1021"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -8727,12 +8727,12 @@
       </c>
       <c r="B489" t="inlineStr">
         <is>
-          <t>Critical chance +{pct}%.</t>
+          <t>1 in every {n} hits is a critical.</t>
         </is>
       </c>
       <c r="C489" t="inlineStr">
         <is>
-          <t>치명타 확률 +{pct}%.</t>
+          <t>{n}번 공격마다 1번은 치명타입니다.</t>
         </is>
       </c>
     </row>
@@ -17726,6 +17726,57 @@
       <c r="C1018" t="inlineStr">
         <is>
           <t>승리</t>
+        </is>
+      </c>
+    </row>
+    <row r="1019">
+      <c r="A1019" t="inlineStr">
+        <is>
+          <t>status.desc.status_crit_up_many</t>
+        </is>
+      </c>
+      <c r="B1019" t="inlineStr">
+        <is>
+          <t>In every {n} hits, {reds} are criticals.</t>
+        </is>
+      </c>
+      <c r="C1019" t="inlineStr">
+        <is>
+          <t>{n}번 공격 중 {reds}번은 치명타입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1020">
+      <c r="A1020" t="inlineStr">
+        <is>
+          <t>battle.action.run_no</t>
+        </is>
+      </c>
+      <c r="B1020" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="C1020" t="inlineStr">
+        <is>
+          <t>불가</t>
+        </is>
+      </c>
+    </row>
+    <row r="1021">
+      <c r="A1021" t="inlineStr">
+        <is>
+          <t>pause.help.in_battle</t>
+        </is>
+      </c>
+      <c r="B1021" t="inlineStr">
+        <is>
+          <t>Not available during a battle.</t>
+        </is>
+      </c>
+      <c r="C1021" t="inlineStr">
+        <is>
+          <t>전투 중에는 사용할 수 없습니다.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(run): the first class chest cannot be skipped — two lines and a step back at the exit (D127)
Floor 1's exit refuses a player who has not chosen a class: the step into the
exit is undone, the two lines play, then the player steps one tile away from
the exit through the normal movement code. Repeats until the class is chosen.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datafiles/localization/game_text.xlsx
+++ b/datafiles/localization/game_text.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1021"/>
+  <dimension ref="A1:C1023"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -17780,6 +17780,40 @@
         </is>
       </c>
     </row>
+    <row r="1022">
+      <c r="A1022" t="inlineStr">
+        <is>
+          <t>dialogue.sys_class_chest_guard.0</t>
+        </is>
+      </c>
+      <c r="B1022" t="inlineStr">
+        <is>
+          <t>Wait, there was a chest back there. I think I should open it...</t>
+        </is>
+      </c>
+      <c r="C1022" t="inlineStr">
+        <is>
+          <t>잠깐, 저 뒤에 상자가 있었어. 열어 봐야겠어...</t>
+        </is>
+      </c>
+    </row>
+    <row r="1023">
+      <c r="A1023" t="inlineStr">
+        <is>
+          <t>dialogue.sys_class_chest_guard.1</t>
+        </is>
+      </c>
+      <c r="B1023" t="inlineStr">
+        <is>
+          <t>...there might be something I can use to protect myself.</t>
+        </is>
+      </c>
+      <c r="C1023" t="inlineStr">
+        <is>
+          <t>...나를 지킬 만한 뭔가가 들어 있을지도 몰라.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C678"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(input): controller rumble on Perfect, BREAK, big hits and death, with a Settings toggle (D136)
Rumble_* in scr_input: the events are read from state, not called from combat code
(Perfect freeze edge, enemy broken edge, HP drop >= 25% max HP or a heavy move's defence
bar ending with damage, HP reaching 0). Only the last-used pad, never with keyboard/mouse
as last device; stops on pause, focus loss, room change and game end. New Rumble row in
Settings (On by default), saved as a rumble field (no settings_version bump: a file
without it loads On). Smoke steps 360-379 chained onto the end; settings shot added.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datafiles/localization/game_text.xlsx
+++ b/datafiles/localization/game_text.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1027"/>
+  <dimension ref="A1:C1029"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -17882,6 +17882,40 @@
         </is>
       </c>
     </row>
+    <row r="1028">
+      <c r="A1028" t="inlineStr">
+        <is>
+          <t>settings.row.rumble</t>
+        </is>
+      </c>
+      <c r="B1028" t="inlineStr">
+        <is>
+          <t>Rumble</t>
+        </is>
+      </c>
+      <c r="C1028" t="inlineStr">
+        <is>
+          <t>진동</t>
+        </is>
+      </c>
+    </row>
+    <row r="1029">
+      <c r="A1029" t="inlineStr">
+        <is>
+          <t>settings.help.rumble</t>
+        </is>
+      </c>
+      <c r="B1029" t="inlineStr">
+        <is>
+          <t>Short controller vibration on Perfect hits, BREAK, big hits and defeat.</t>
+        </is>
+      </c>
+      <c r="C1029" t="inlineStr">
+        <is>
+          <t>완벽한 공격, 브레이크, 큰 피해, 쓰러질 때 컨트롤러가 짧게 진동합니다.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C678"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
wip(g9): run stats (D137) implemented; bot run and final look at the 800x720 summary shot left
Done: RunStats_* (scr_room_state), hooks in scr_combat, run save/restore, history entry, summary rows, Codex rows (Level and Gold lines dropped from the Runs details to fit 800x720), loc rows, smoke 440-447, shots 460-466 (Shots = 192). Runtests 4187/0, smoke 695/0, shots 495/0 (the last shots run was after the Codex change; smoke and runtests were run before it). Not done: -Only bot, re-run of fast/smoke after the Codex line change, opening shot_runstats_summary_800x720.png.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datafiles/localization/game_text.xlsx
+++ b/datafiles/localization/game_text.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1030"/>
+  <dimension ref="A1:C1036"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -17933,6 +17933,108 @@
         </is>
       </c>
     </row>
+    <row r="1031">
+      <c r="A1031" t="inlineStr">
+        <is>
+          <t>stat.perfect</t>
+        </is>
+      </c>
+      <c r="B1031" t="inlineStr">
+        <is>
+          <t>Perfect rate</t>
+        </is>
+      </c>
+      <c r="C1031" t="inlineStr">
+        <is>
+          <t>퍼펙트 비율</t>
+        </is>
+      </c>
+    </row>
+    <row r="1032">
+      <c r="A1032" t="inlineStr">
+        <is>
+          <t>stat.crits</t>
+        </is>
+      </c>
+      <c r="B1032" t="inlineStr">
+        <is>
+          <t>Crits landed</t>
+        </is>
+      </c>
+      <c r="C1032" t="inlineStr">
+        <is>
+          <t>치명타 횟수</t>
+        </is>
+      </c>
+    </row>
+    <row r="1033">
+      <c r="A1033" t="inlineStr">
+        <is>
+          <t>stat.dmg_dealt</t>
+        </is>
+      </c>
+      <c r="B1033" t="inlineStr">
+        <is>
+          <t>Damage dealt</t>
+        </is>
+      </c>
+      <c r="C1033" t="inlineStr">
+        <is>
+          <t>준 피해</t>
+        </is>
+      </c>
+    </row>
+    <row r="1034">
+      <c r="A1034" t="inlineStr">
+        <is>
+          <t>stat.dmg_taken</t>
+        </is>
+      </c>
+      <c r="B1034" t="inlineStr">
+        <is>
+          <t>Damage taken</t>
+        </is>
+      </c>
+      <c r="C1034" t="inlineStr">
+        <is>
+          <t>받은 피해</t>
+        </is>
+      </c>
+    </row>
+    <row r="1035">
+      <c r="A1035" t="inlineStr">
+        <is>
+          <t>stat.fights_won</t>
+        </is>
+      </c>
+      <c r="B1035" t="inlineStr">
+        <is>
+          <t>Fights won</t>
+        </is>
+      </c>
+      <c r="C1035" t="inlineStr">
+        <is>
+          <t>승리한 전투</t>
+        </is>
+      </c>
+    </row>
+    <row r="1036">
+      <c r="A1036" t="inlineStr">
+        <is>
+          <t>stat.time</t>
+        </is>
+      </c>
+      <c r="B1036" t="inlineStr">
+        <is>
+          <t>Run time</t>
+        </is>
+      </c>
+      <c r="C1036" t="inlineStr">
+        <is>
+          <t>플레이 시간</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C678"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(levelup): show the class growth on the level-up screen, free point may go to Max HP +3 / Max MP +2, victory text drops the auto gains (D143)
LevelUp_GrowthText, Cards_FreePointOptions, Level_ApplyResourcePoint; hp_bonus/mp_bonus on the character feed RecomputeResources (a respec refunds them with the points). layout.note draws one line under a menu title. Smoke steps 520-523 and shots 540-543 (shots count 195 -> 198).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datafiles/localization/game_text.xlsx
+++ b/datafiles/localization/game_text.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1036"/>
+  <dimension ref="A1:C1042"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -18035,6 +18035,108 @@
         </is>
       </c>
     </row>
+    <row r="1037">
+      <c r="A1037" t="inlineStr">
+        <is>
+          <t>levelup.gain</t>
+        </is>
+      </c>
+      <c r="B1037" t="inlineStr">
+        <is>
+          <t>{stat} +{n}</t>
+        </is>
+      </c>
+      <c r="C1037" t="inlineStr">
+        <is>
+          <t>{stat} +{n}</t>
+        </is>
+      </c>
+    </row>
+    <row r="1038">
+      <c r="A1038" t="inlineStr">
+        <is>
+          <t>levelup.growth</t>
+        </is>
+      </c>
+      <c r="B1038" t="inlineStr">
+        <is>
+          <t>{name} growth: {gains}</t>
+        </is>
+      </c>
+      <c r="C1038" t="inlineStr">
+        <is>
+          <t>{name} 성장: {gains}</t>
+        </is>
+      </c>
+    </row>
+    <row r="1039">
+      <c r="A1039" t="inlineStr">
+        <is>
+          <t>cards.stat.maxhp</t>
+        </is>
+      </c>
+      <c r="B1039" t="inlineStr">
+        <is>
+          <t>Max HP +{n}</t>
+        </is>
+      </c>
+      <c r="C1039" t="inlineStr">
+        <is>
+          <t>최대 HP +{n}</t>
+        </is>
+      </c>
+    </row>
+    <row r="1040">
+      <c r="A1040" t="inlineStr">
+        <is>
+          <t>cards.stat.maxmp</t>
+        </is>
+      </c>
+      <c r="B1040" t="inlineStr">
+        <is>
+          <t>Max MP +{n}</t>
+        </is>
+      </c>
+      <c r="C1040" t="inlineStr">
+        <is>
+          <t>최대 MP +{n}</t>
+        </is>
+      </c>
+    </row>
+    <row r="1041">
+      <c r="A1041" t="inlineStr">
+        <is>
+          <t>cards.stat.maxhp.desc</t>
+        </is>
+      </c>
+      <c r="B1041" t="inlineStr">
+        <is>
+          <t>Raises your max HP by {n} and heals {n} HP.</t>
+        </is>
+      </c>
+      <c r="C1041" t="inlineStr">
+        <is>
+          <t>최대 HP가 {n} 오르고 HP를 {n} 회복합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1042">
+      <c r="A1042" t="inlineStr">
+        <is>
+          <t>cards.stat.maxmp.desc</t>
+        </is>
+      </c>
+      <c r="B1042" t="inlineStr">
+        <is>
+          <t>Raises your max MP by {n} and restores {n} MP.</t>
+        </is>
+      </c>
+      <c r="C1042" t="inlineStr">
+        <is>
+          <t>최대 MP가 {n} 오르고 MP를 {n} 회복합니다.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C678"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(title): seed pick on New Game (Random default / Enter seed), number entry for keyboard and pad, seed on Status tab and run summary (D152)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datafiles/localization/game_text.xlsx
+++ b/datafiles/localization/game_text.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1036"/>
+  <dimension ref="A1:C1045"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -17244,12 +17244,12 @@
       </c>
       <c r="B990" t="inlineStr">
         <is>
-          <t>Seed {n}</t>
+          <t>Seed: {n}</t>
         </is>
       </c>
       <c r="C990" t="inlineStr">
         <is>
-          <t>시드 {n}</t>
+          <t>시드: {n}</t>
         </is>
       </c>
     </row>
@@ -18032,6 +18032,159 @@
       <c r="C1036" t="inlineStr">
         <is>
           <t>x2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1037">
+      <c r="A1037" t="inlineStr">
+        <is>
+          <t>seed.choice.title</t>
+        </is>
+      </c>
+      <c r="B1037" t="inlineStr">
+        <is>
+          <t>Choose a seed</t>
+        </is>
+      </c>
+      <c r="C1037" t="inlineStr">
+        <is>
+          <t>시드 선택</t>
+        </is>
+      </c>
+    </row>
+    <row r="1038">
+      <c r="A1038" t="inlineStr">
+        <is>
+          <t>seed.choice.random</t>
+        </is>
+      </c>
+      <c r="B1038" t="inlineStr">
+        <is>
+          <t>Random seed</t>
+        </is>
+      </c>
+      <c r="C1038" t="inlineStr">
+        <is>
+          <t>무작위 시드</t>
+        </is>
+      </c>
+    </row>
+    <row r="1039">
+      <c r="A1039" t="inlineStr">
+        <is>
+          <t>seed.choice.enter</t>
+        </is>
+      </c>
+      <c r="B1039" t="inlineStr">
+        <is>
+          <t>Enter seed</t>
+        </is>
+      </c>
+      <c r="C1039" t="inlineStr">
+        <is>
+          <t>시드 입력</t>
+        </is>
+      </c>
+    </row>
+    <row r="1040">
+      <c r="A1040" t="inlineStr">
+        <is>
+          <t>seed.entry.title</t>
+        </is>
+      </c>
+      <c r="B1040" t="inlineStr">
+        <is>
+          <t>Enter seed</t>
+        </is>
+      </c>
+      <c r="C1040" t="inlineStr">
+        <is>
+          <t>시드 입력</t>
+        </is>
+      </c>
+    </row>
+    <row r="1041">
+      <c r="A1041" t="inlineStr">
+        <is>
+          <t>seed.entry.info</t>
+        </is>
+      </c>
+      <c r="B1041" t="inlineStr">
+        <is>
+          <t>Up to 9 digits. Same seed, same run.</t>
+        </is>
+      </c>
+      <c r="C1041" t="inlineStr">
+        <is>
+          <t>최대 9자리. 같은 시드, 같은 모험.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1042">
+      <c r="A1042" t="inlineStr">
+        <is>
+          <t>seed.entry.need</t>
+        </is>
+      </c>
+      <c r="B1042" t="inlineStr">
+        <is>
+          <t>Enter a seed above zero.</t>
+        </is>
+      </c>
+      <c r="C1042" t="inlineStr">
+        <is>
+          <t>0보다 큰 시드를 입력하세요.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1043">
+      <c r="A1043" t="inlineStr">
+        <is>
+          <t>seed.entry.hint</t>
+        </is>
+      </c>
+      <c r="B1043" t="inlineStr">
+        <is>
+          <t>{up}{down} Digit   {left}{right} Move</t>
+        </is>
+      </c>
+      <c r="C1043" t="inlineStr">
+        <is>
+          <t>{up}{down} 숫자   {left}{right} 이동</t>
+        </is>
+      </c>
+    </row>
+    <row r="1044">
+      <c r="A1044" t="inlineStr">
+        <is>
+          <t>seed.entry.hint2</t>
+        </is>
+      </c>
+      <c r="B1044" t="inlineStr">
+        <is>
+          <t>{confirm} Start</t>
+        </is>
+      </c>
+      <c r="C1044" t="inlineStr">
+        <is>
+          <t>{confirm} 시작</t>
+        </is>
+      </c>
+    </row>
+    <row r="1045">
+      <c r="A1045" t="inlineStr">
+        <is>
+          <t>seed.entry.hint3</t>
+        </is>
+      </c>
+      <c r="B1045" t="inlineStr">
+        <is>
+          <t>{back} Back   {tab_prev} Delete</t>
+        </is>
+      </c>
+      <c r="C1045" t="inlineStr">
+        <is>
+          <t>{back} 뒤로   {tab_prev} 지우기</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(notes): notes are picked up by stepping on them, never block, stay gone, read in a Codex reader (D147)
A note is no longer an obj_interactable: it is an entry of Notes_Live, so it blocks neither the
player nor the enemies' grid. Stepping onto it records it in the profile, takes it off the map,
shows a 'Note found' notice and a rising page. A note found in any run never spawns again.
The Codex Notes page says 'Notes found x/8'; a found note opens a scrolling reader.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datafiles/localization/game_text.xlsx
+++ b/datafiles/localization/game_text.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1042"/>
+  <dimension ref="A1:C1045"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -16513,12 +16513,12 @@
       </c>
       <c r="B947" t="inlineStr">
         <is>
-          <t>The notes you have read in the tunnel.</t>
+          <t>The notes you have found in the tunnel.</t>
         </is>
       </c>
       <c r="C947" t="inlineStr">
         <is>
-          <t>터널에서 읽은 쪽지입니다.</t>
+          <t>터널에서 찾은 쪽지입니다.</t>
         </is>
       </c>
     </row>
@@ -16530,12 +16530,12 @@
       </c>
       <c r="B948" t="inlineStr">
         <is>
-          <t>Notes {n}/{max}</t>
+          <t>Notes found {n}/{max}</t>
         </is>
       </c>
       <c r="C948" t="inlineStr">
         <is>
-          <t>쪽지 {n}/{max}</t>
+          <t>찾은 쪽지 {n}/{max}</t>
         </is>
       </c>
     </row>
@@ -18134,6 +18134,57 @@
       <c r="C1042" t="inlineStr">
         <is>
           <t>{confirm} 유지   {back} 되돌리기</t>
+        </is>
+      </c>
+    </row>
+    <row r="1043">
+      <c r="A1043" t="inlineStr">
+        <is>
+          <t>tab.hint.read</t>
+        </is>
+      </c>
+      <c r="B1043" t="inlineStr">
+        <is>
+          <t>{confirm} Read</t>
+        </is>
+      </c>
+      <c r="C1043" t="inlineStr">
+        <is>
+          <t>{confirm} 읽기</t>
+        </is>
+      </c>
+    </row>
+    <row r="1044">
+      <c r="A1044" t="inlineStr">
+        <is>
+          <t>tab.hint.scroll</t>
+        </is>
+      </c>
+      <c r="B1044" t="inlineStr">
+        <is>
+          <t>{up}{down} Scroll</t>
+        </is>
+      </c>
+      <c r="C1044" t="inlineStr">
+        <is>
+          <t>{up}{down} 넘기기</t>
+        </is>
+      </c>
+    </row>
+    <row r="1045">
+      <c r="A1045" t="inlineStr">
+        <is>
+          <t>note.found</t>
+        </is>
+      </c>
+      <c r="B1045" t="inlineStr">
+        <is>
+          <t>Note found: {title}</t>
+        </is>
+      </c>
+      <c r="C1045" t="inlineStr">
+        <is>
+          <t>쪽지를 찾았다: {title}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(text): one markup for terms, accents and buttons; device-aware prompts with arrows and d-pad; one battle prompt line (D149, D156)
[t] terms in the bright green, [a] the one gold accent, [k:action] a button by last device, in the dialogue box, cards, tooltips,
tutorials and hints; width and wrap count glyph widths; typewriter counts visible characters. English and Korean strings marked.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datafiles/localization/game_text.xlsx
+++ b/datafiles/localization/game_text.xlsx
@@ -2964,12 +2964,12 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Received {item} x{qty}.</t>
+          <t>Received [a]{item}[/a] x{qty}.</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>{item} x{qty}을(를) 받았습니다.</t>
+          <t>[a]{item}[/a] x{qty}을(를) 받았습니다.</t>
         </is>
       </c>
     </row>
@@ -4885,12 +4885,12 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>A Weak press counts as OK (once per turn)</t>
+          <t>A [t]Weak[/t] press counts as [t]OK[/t] (once per turn)</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>약함 판정이 무난으로 처리됩니다 (턴당 1회)</t>
+          <t>[t]약함[/t] 판정이 [t]무난[/t]으로 처리됩니다 (턴당 1회)</t>
         </is>
       </c>
     </row>
@@ -4902,12 +4902,12 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>First hit: -1 DEF for 2 turns</t>
+          <t>First hit: -1 [t]DEF[/t] for 2 turns</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>첫 타격: 2턴 동안 DEF -1</t>
+          <t>첫 타격: 2턴 동안 [t]DEF[/t] -1</t>
         </is>
       </c>
     </row>
@@ -4970,12 +4970,12 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>+1 MP every 2 turns, +1 physical damage taken</t>
+          <t>+1 [t]MP[/t] every 2 turns, +1 physical damage taken</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>2턴마다 MP +1, 받는 물리 피해 +1</t>
+          <t>2턴마다 [t]MP[/t] +1, 받는 물리 피해 +1</t>
         </is>
       </c>
     </row>
@@ -5004,12 +5004,12 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>Reflects the first status (costs 1 MP)</t>
+          <t>Reflects the first status (costs 1 [t]MP[/t])</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>첫 상태 이상을 반사 (MP 1 소모)</t>
+          <t>첫 상태 이상을 반사 ([t]MP[/t] 1 소모)</t>
         </is>
       </c>
     </row>
@@ -5021,12 +5021,12 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>+35% damage to foes below 35% HP</t>
+          <t>+35% damage to foes below 35% [t]HP[/t]</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>HP 35% 미만 적에게 피해 +35%</t>
+          <t>[t]HP[/t] 35% 미만 적에게 피해 +35%</t>
         </is>
       </c>
     </row>
@@ -5038,12 +5038,12 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>A Good press counts as Perfect (once per turn)</t>
+          <t>A [t]Good[/t] press counts as [a]Perfect[/a] (once per turn)</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>좋음 판정이 완벽으로 처리됩니다 (턴당 1회)</t>
+          <t>[t]좋음[/t] 판정이 [a]완벽[/a]으로 처리됩니다 (턴당 1회)</t>
         </is>
       </c>
     </row>
@@ -5055,12 +5055,12 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>Good or Perfect: may Stun (3-turn cooldown)</t>
+          <t>[t]Good[/t] or [a]Perfect[/a]: may [t]Stun[/t] (3-turn cooldown)</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>좋음 이상: 기절시킬 수 있음 (재사용 3턴)</t>
+          <t>[t]좋음[/t] 또는 [a]완벽[/a]: [t]기절[/t]시킬 수 있음 (재사용 3턴)</t>
         </is>
       </c>
     </row>
@@ -5089,12 +5089,12 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>+1 MP every 2 turns</t>
+          <t>+1 [t]MP[/t] every 2 turns</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>2턴마다 MP +1</t>
+          <t>2턴마다 [t]MP[/t] +1</t>
         </is>
       </c>
     </row>
@@ -5123,12 +5123,12 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>+25% skill damage, Perfect +1 MP</t>
+          <t>+25% skill damage, [a]Perfect[/a] +1 [t]MP[/t]</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>스킬 피해 +25%, 완벽 판정 시 MP +1</t>
+          <t>스킬 피해 +25%, [a]완벽[/a] 판정 시 [t]MP[/t] +1</t>
         </is>
       </c>
     </row>
@@ -6500,12 +6500,12 @@
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>Increases spell damage and max MP.</t>
+          <t>Increases spell damage and max [t]MP[/t].</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>마법 피해와 최대 MP를 늘립니다.</t>
+          <t>마법 피해와 최대 [t]MP[/t]를 늘립니다.</t>
         </is>
       </c>
     </row>
@@ -6517,12 +6517,12 @@
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>Increases physical damage (basic attacks and ATK skills).</t>
+          <t>Increases physical damage (basic attacks and [t]ATK[/t] skills).</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>물리 피해(기본 공격과 ATK 스킬)를 늘립니다.</t>
+          <t>물리 피해(기본 공격과 [t]ATK[/t] 스킬)를 늘립니다.</t>
         </is>
       </c>
     </row>
@@ -8557,12 +8557,12 @@
       </c>
       <c r="B479" t="inlineStr">
         <is>
-          <t>Lose {tick} HP each turn, then 1 stack fades ({stacks} stacks, max {max}).{mods}</t>
+          <t>Lose {tick} [t]HP[/t] each turn, then 1 stack fades ({stacks} stacks, max {max}).{mods}</t>
         </is>
       </c>
       <c r="C479" t="inlineStr">
         <is>
-          <t>매 턴 {tick} HP를 잃고, 중첩이 1 줄어듭니다 ({stacks}중첩, 최대 {max}).{mods}</t>
+          <t>매 턴 {tick} [t]HP[/t]를 잃고, 중첩이 1 줄어듭니다 ({stacks}중첩, 최대 {max}).{mods}</t>
         </is>
       </c>
     </row>
@@ -8574,12 +8574,12 @@
       </c>
       <c r="B480" t="inlineStr">
         <is>
-          <t>Lose HP equal to its stacks each turn, then 1 stack fades. Stacks up to {max}.{mods}</t>
+          <t>Lose [t]HP[/t] equal to its stacks each turn, then 1 stack fades. Stacks up to {max}.{mods}</t>
         </is>
       </c>
       <c r="C480" t="inlineStr">
         <is>
-          <t>매 턴 중첩 수만큼 HP를 잃고, 중첩이 1 줄어듭니다. 최대 {max}중첩.{mods}</t>
+          <t>매 턴 중첩 수만큼 [t]HP[/t]를 잃고, 중첩이 1 줄어듭니다. 최대 {max}중첩.{mods}</t>
         </is>
       </c>
     </row>
@@ -8591,12 +8591,12 @@
       </c>
       <c r="B481" t="inlineStr">
         <is>
-          <t>Lose {tick} HP each time you act ({stacks} stacks, max {max}), for {turns} more turns.{mods}</t>
+          <t>Lose {tick} [t]HP[/t] each time you act ({stacks} stacks, max {max}), for {turns} more turns.{mods}</t>
         </is>
       </c>
       <c r="C481" t="inlineStr">
         <is>
-          <t>행동할 때마다 {tick} HP를 잃습니다 ({stacks}중첩, 최대 {max}). {turns}턴 더 지속.{mods}</t>
+          <t>행동할 때마다 {tick} [t]HP[/t]를 잃습니다 ({stacks}중첩, 최대 {max}). {turns}턴 더 지속.{mods}</t>
         </is>
       </c>
     </row>
@@ -8608,12 +8608,12 @@
       </c>
       <c r="B482" t="inlineStr">
         <is>
-          <t>Lose {tick} HP per stack each time you act. Stacks up to {max}, lasts {dur} turns.{mods}</t>
+          <t>Lose {tick} [t]HP[/t] per stack each time you act. Stacks up to {max}, lasts {dur} turns.{mods}</t>
         </is>
       </c>
       <c r="C482" t="inlineStr">
         <is>
-          <t>행동할 때마다 중첩당 {tick} HP를 잃습니다. 최대 {max}중첩, {dur}턴 지속.{mods}</t>
+          <t>행동할 때마다 중첩당 {tick} [t]HP[/t]를 잃습니다. 최대 {max}중첩, {dur}턴 지속.{mods}</t>
         </is>
       </c>
     </row>
@@ -8625,12 +8625,12 @@
       </c>
       <c r="B483" t="inlineStr">
         <is>
-          <t>Lose {tick} HP each turn for {turns} more turns.{mods}</t>
+          <t>Lose {tick} [t]HP[/t] each turn for {turns} more turns.{mods}</t>
         </is>
       </c>
       <c r="C483" t="inlineStr">
         <is>
-          <t>매 턴 {tick} HP를 잃습니다. {turns}턴 더 지속.{mods}</t>
+          <t>매 턴 {tick} [t]HP[/t]를 잃습니다. {turns}턴 더 지속.{mods}</t>
         </is>
       </c>
     </row>
@@ -8642,12 +8642,12 @@
       </c>
       <c r="B484" t="inlineStr">
         <is>
-          <t>Lose a fixed amount of HP (it grows with the caster's MAG) each turn for {dur} turns. Does not stack.{mods}</t>
+          <t>Lose a fixed amount of [t]HP[/t] (it grows with the caster's [t]MAG[/t]) each turn for {dur} turns. Does not stack.{mods}</t>
         </is>
       </c>
       <c r="C484" t="inlineStr">
         <is>
-          <t>매 턴 정해진 HP(시전자의 MAG에 비례)를 {dur}턴 동안 잃습니다. 중첩되지 않습니다.{mods}</t>
+          <t>매 턴 정해진 [t]HP[/t](시전자의 [t]MAG[/t]에 비례)를 {dur}턴 동안 잃습니다. 중첩되지 않습니다.{mods}</t>
         </is>
       </c>
     </row>
@@ -8659,12 +8659,12 @@
       </c>
       <c r="B485" t="inlineStr">
         <is>
-          <t>Pushed back on the turn bar. Then Steadfast: cannot be stunned for 2 turns.</t>
+          <t>Pushed back on the turn bar. Then [t]Steadfast[/t]: cannot be stunned for 2 turns.</t>
         </is>
       </c>
       <c r="C485" t="inlineStr">
         <is>
-          <t>차례가 뒤로 밀립니다. 이후 2턴간 버티기 상태가 되어 기절하지 않습니다.</t>
+          <t>차례가 뒤로 밀립니다. 이후 2턴간 [t]버티기[/t] 상태가 되어 [t]기절[/t]하지 않습니다.</t>
         </is>
       </c>
     </row>
@@ -8744,12 +8744,12 @@
       </c>
       <c r="B490" t="inlineStr">
         <is>
-          <t>For {turns} turns: you see the enemy's next move and every Perfect zone is {pct}% wider.</t>
+          <t>For {turns} turns: you see the enemy's next move and every [a]Perfect[/a] zone is {pct}% wider.</t>
         </is>
       </c>
       <c r="C490" t="inlineStr">
         <is>
-          <t>{turns}턴 동안 적의 다음 행동이 보이고 모든 완벽 구간이 {pct}% 넓어집니다.</t>
+          <t>{turns}턴 동안 적의 다음 행동이 보이고 모든 [a]완벽[/a] 구간이 {pct}% 넓어집니다.</t>
         </is>
       </c>
     </row>
@@ -8761,12 +8761,12 @@
       </c>
       <c r="B491" t="inlineStr">
         <is>
-          <t>Recover {n} MP each turn.</t>
+          <t>Recover {n} [t]MP[/t] each turn.</t>
         </is>
       </c>
       <c r="C491" t="inlineStr">
         <is>
-          <t>매 턴 MP를 {n} 회복합니다.</t>
+          <t>매 턴 [t]MP[/t]를 {n} 회복합니다.</t>
         </is>
       </c>
     </row>
@@ -9152,12 +9152,12 @@
       </c>
       <c r="B514" t="inlineStr">
         <is>
-          <t>Press confirm to go on</t>
+          <t>Press [k:confirm] to go on</t>
         </is>
       </c>
       <c r="C514" t="inlineStr">
         <is>
-          <t>확인을 눌러 계속</t>
+          <t>[k:confirm]을(를) 눌러 계속</t>
         </is>
       </c>
     </row>
@@ -9169,12 +9169,12 @@
       </c>
       <c r="B515" t="inlineStr">
         <is>
-          <t>Up / Down to choose, confirm to take it</t>
+          <t>[k:up][k:down] Choose   [k:confirm] Take it</t>
         </is>
       </c>
       <c r="C515" t="inlineStr">
         <is>
-          <t>위/아래로 선택, 확인으로 가져가기</t>
+          <t>[k:up][k:down] 고르기   [k:confirm] 가져가기</t>
         </is>
       </c>
     </row>
@@ -9934,12 +9934,12 @@
       </c>
       <c r="B560" t="inlineStr">
         <is>
-          <t>Gain {status} for {turns} turns.</t>
+          <t>Gain [t]{status}[/t] for {turns} turns.</t>
         </is>
       </c>
       <c r="C560" t="inlineStr">
         <is>
-          <t>{status} 효과를 {turns}턴 동안 얻는다.</t>
+          <t>[t]{status}[/t] 효과를 {turns}턴 동안 얻는다.</t>
         </is>
       </c>
     </row>
@@ -9968,12 +9968,12 @@
       </c>
       <c r="B562" t="inlineStr">
         <is>
-          <t>{chance}% to inflict {status}.</t>
+          <t>{chance}% to inflict [t]{status}[/t].</t>
         </is>
       </c>
       <c r="C562" t="inlineStr">
         <is>
-          <t>{chance}% 확률로 {status} 부여.</t>
+          <t>{chance}% 확률로 [t]{status}[/t] 부여.</t>
         </is>
       </c>
     </row>
@@ -10104,12 +10104,12 @@
       </c>
       <c r="B570" t="inlineStr">
         <is>
-          <t>{left}{right} Choose   {confirm} Take</t>
+          <t>[k:left][k:right] Choose   [k:confirm] Take</t>
         </is>
       </c>
       <c r="C570" t="inlineStr">
         <is>
-          <t>{left}{right} 고르기   {confirm} 받기</t>
+          <t>[k:left][k:right] 고르기   [k:confirm] 받기</t>
         </is>
       </c>
     </row>
@@ -10330,7 +10330,7 @@
       </c>
       <c r="C583" t="inlineStr">
         <is>
-          <t>빠르고 날카롭다. 높은 속도, 독과 연속 사격을 찾아보자.</t>
+          <t>빠르고 날카롭다. 높은 속도, [t]독[/t]과 연속 사격을 찾아보자.</t>
         </is>
       </c>
     </row>
@@ -10359,12 +10359,12 @@
       </c>
       <c r="B585" t="inlineStr">
         <is>
-          <t>A spell caster. Great magic and MP, five skills to find.</t>
+          <t>A spell caster. Great magic and [t]MP[/t], five skills to find.</t>
         </is>
       </c>
       <c r="C585" t="inlineStr">
         <is>
-          <t>주문 시전자. 뛰어난 마법과 MP, 찾아야 할 스킬 5개.</t>
+          <t>주문 시전자. 뛰어난 마법과 [t]MP[/t], 찾아야 할 스킬 5개.</t>
         </is>
       </c>
     </row>
@@ -10495,12 +10495,12 @@
       </c>
       <c r="B593" t="inlineStr">
         <is>
-          <t>Light on your feet: +{n} SPD for good.</t>
+          <t>Light on your feet: +{n} [t]SPD[/t] for good.</t>
         </is>
       </c>
       <c r="C593" t="inlineStr">
         <is>
-          <t>가벼운 발걸음: 영구히 SPD +{n}.</t>
+          <t>가벼운 발걸음: 영구히 [t]SPD[/t] +{n}.</t>
         </is>
       </c>
     </row>
@@ -10529,12 +10529,12 @@
       </c>
       <c r="B595" t="inlineStr">
         <is>
-          <t>Poison you apply adds {n} extra stack.</t>
+          <t>[t]Poison[/t] you apply adds {n} extra stack.</t>
         </is>
       </c>
       <c r="C595" t="inlineStr">
         <is>
-          <t>내가 거는 독이 {n}중첩 더 쌓인다.</t>
+          <t>내가 거는 [t]독[/t]이 {n}중첩 더 쌓인다.</t>
         </is>
       </c>
     </row>
@@ -10563,12 +10563,12 @@
       </c>
       <c r="B597" t="inlineStr">
         <is>
-          <t>Restore {n} HP after each fight you win.</t>
+          <t>Restore {n} [t]HP[/t] after each fight you win.</t>
         </is>
       </c>
       <c r="C597" t="inlineStr">
         <is>
-          <t>전투에서 이길 때마다 HP를 {n} 회복한다.</t>
+          <t>전투에서 이길 때마다 [t]HP[/t]를 {n} 회복한다.</t>
         </is>
       </c>
     </row>
@@ -10597,12 +10597,12 @@
       </c>
       <c r="B599" t="inlineStr">
         <is>
-          <t>Perfect zones are {n}% wider.</t>
+          <t>[a]Perfect[/a] zones are {n}% wider.</t>
         </is>
       </c>
       <c r="C599" t="inlineStr">
         <is>
-          <t>완벽 구간이 {n}% 넓어진다.</t>
+          <t>[a]완벽[/a] 구간이 {n}% 넓어진다.</t>
         </is>
       </c>
     </row>
@@ -10665,12 +10665,12 @@
       </c>
       <c r="B603" t="inlineStr">
         <is>
-          <t>Regain {n} MP at the start of each of your turns.</t>
+          <t>Regain {n} [t]MP[/t] at the start of each of your turns.</t>
         </is>
       </c>
       <c r="C603" t="inlineStr">
         <is>
-          <t>내 턴이 시작될 때마다 MP를 {n} 회복한다.</t>
+          <t>내 턴이 시작될 때마다 [t]MP[/t]를 {n} 회복한다.</t>
         </is>
       </c>
     </row>
@@ -10733,12 +10733,12 @@
       </c>
       <c r="B607" t="inlineStr">
         <is>
-          <t>Enemies start each fight with {n} stagger.</t>
+          <t>Enemies start each fight with {n} [t]stagger[/t].</t>
         </is>
       </c>
       <c r="C607" t="inlineStr">
         <is>
-          <t>전투가 시작될 때 적의 경직이 {n} 쌓여 있다.</t>
+          <t>전투가 시작될 때 적의 [t]경직[/t]이 {n} 쌓여 있다.</t>
         </is>
       </c>
     </row>
@@ -10767,12 +10767,12 @@
       </c>
       <c r="B609" t="inlineStr">
         <is>
-          <t>Thicker hide: +{n} DEF for good.</t>
+          <t>Thicker hide: +{n} [t]DEF[/t] for good.</t>
         </is>
       </c>
       <c r="C609" t="inlineStr">
         <is>
-          <t>두꺼운 가죽: 영구히 DEF +{n}.</t>
+          <t>두꺼운 가죽: 영구히 [t]DEF[/t] +{n}.</t>
         </is>
       </c>
     </row>
@@ -10801,7 +10801,7 @@
       </c>
       <c r="B611" t="inlineStr">
         <is>
-          <t>Guard on yourself lasts {n} turns longer.</t>
+          <t>[t]Guard[/t] on yourself lasts {n} turns longer.</t>
         </is>
       </c>
       <c r="C611" t="inlineStr">
@@ -10835,12 +10835,12 @@
       </c>
       <c r="B613" t="inlineStr">
         <is>
-          <t>A harder swing: +{n} ATK for good.</t>
+          <t>A harder swing: +{n} [t]ATK[/t] for good.</t>
         </is>
       </c>
       <c r="C613" t="inlineStr">
         <is>
-          <t>더 묵직한 일격: 영구히 ATK +{n}.</t>
+          <t>더 묵직한 일격: 영구히 [t]ATK[/t] +{n}.</t>
         </is>
       </c>
     </row>
@@ -10869,12 +10869,12 @@
       </c>
       <c r="B615" t="inlineStr">
         <is>
-          <t>Quicker than the wind: +{n} SPD for good.</t>
+          <t>Quicker than the wind: +{n} [t]SPD[/t] for good.</t>
         </is>
       </c>
       <c r="C615" t="inlineStr">
         <is>
-          <t>바람보다 빠르게: 영구히 SPD +{n}.</t>
+          <t>바람보다 빠르게: 영구히 [t]SPD[/t] +{n}.</t>
         </is>
       </c>
     </row>
@@ -10937,12 +10937,12 @@
       </c>
       <c r="B619" t="inlineStr">
         <is>
-          <t>Regain {n} MP after each fight you win.</t>
+          <t>Regain {n} [t]MP[/t] after each fight you win.</t>
         </is>
       </c>
       <c r="C619" t="inlineStr">
         <is>
-          <t>전투에서 이길 때마다 MP를 {n} 회복한다.</t>
+          <t>전투에서 이길 때마다 [t]MP[/t]를 {n} 회복한다.</t>
         </is>
       </c>
     </row>
@@ -10971,12 +10971,12 @@
       </c>
       <c r="B621" t="inlineStr">
         <is>
-          <t>A deeper well: +{n} MAG for good.</t>
+          <t>A deeper well: +{n} [t]MAG[/t] for good.</t>
         </is>
       </c>
       <c r="C621" t="inlineStr">
         <is>
-          <t>더 깊은 샘: 영구히 MAG +{n}.</t>
+          <t>더 깊은 샘: 영구히 [t]MAG[/t] +{n}.</t>
         </is>
       </c>
     </row>
@@ -11005,12 +11005,12 @@
       </c>
       <c r="B623" t="inlineStr">
         <is>
-          <t>Your skills cost {n} MP less (never below 1).</t>
+          <t>Your skills cost {n} [t]MP[/t] less (never below 1).</t>
         </is>
       </c>
       <c r="C623" t="inlineStr">
         <is>
-          <t>스킬의 MP 소모가 {n} 줄어든다 (최소 1).</t>
+          <t>스킬의 [t]MP[/t] 소모가 {n} 줄어든다 (최소 1).</t>
         </is>
       </c>
     </row>
@@ -11073,12 +11073,12 @@
       </c>
       <c r="B627" t="inlineStr">
         <is>
-          <t>Healing potions also restore {n} MP.</t>
+          <t>Healing potions also restore {n} [t]MP[/t].</t>
         </is>
       </c>
       <c r="C627" t="inlineStr">
         <is>
-          <t>회복 물약이 MP도 {n} 회복시킨다.</t>
+          <t>회복 물약이 [t]MP[/t]도 {n} 회복시킨다.</t>
         </is>
       </c>
     </row>
@@ -11175,12 +11175,12 @@
       </c>
       <c r="B633" t="inlineStr">
         <is>
-          <t>Restore {n}% of your HP and MP now.</t>
+          <t>Restore {n}% of your [t]HP[/t] and [t]MP[/t] now.</t>
         </is>
       </c>
       <c r="C633" t="inlineStr">
         <is>
-          <t>지금 HP와 MP를 {n}% 회복한다.</t>
+          <t>지금 [t]HP[/t]와 [t]MP[/t]를 {n}% 회복한다.</t>
         </is>
       </c>
     </row>
@@ -13067,7 +13067,7 @@
       </c>
       <c r="C744" t="inlineStr">
         <is>
-          <t>적에게 독 {n}중첩을 겁니다. 턴을 소모합니다.</t>
+          <t>적에게 [t]독[/t] {n}중첩을 겁니다. 턴을 소모합니다.</t>
         </is>
       </c>
     </row>
@@ -13084,7 +13084,7 @@
       </c>
       <c r="C745" t="inlineStr">
         <is>
-          <t>위력 {power}의 피해를 주고 기절시켜 적을 뒤로 밉니다. 턴을 소모합니다.</t>
+          <t>위력 {power}의 피해를 주고 [t]기절[/t]시켜 적을 뒤로 밉니다. 턴을 소모합니다.</t>
         </is>
       </c>
     </row>
@@ -13096,12 +13096,12 @@
       </c>
       <c r="B746" t="inlineStr">
         <is>
-          <t>Throw it to dodge the next attack ({turns} turns); a Perfect throw lets you slip away. Costs your turn.</t>
+          <t>Throw it to dodge the next attack ({turns} turns); a [a]Perfect[/a] throw lets you slip away. Costs your turn.</t>
         </is>
       </c>
       <c r="C746" t="inlineStr">
         <is>
-          <t>다음 공격을 피합니다({turns}턴). 완벽하게 던지면 도망칩니다. 턴을 소모합니다.</t>
+          <t>다음 공격을 피합니다({turns}턴). [a]완벽[/a]하게 던지면 도망칩니다. 턴을 소모합니다.</t>
         </is>
       </c>
     </row>
@@ -13181,12 +13181,12 @@
       </c>
       <c r="B751" t="inlineStr">
         <is>
-          <t>Restores {n} HP.</t>
+          <t>Restores {n} [t]HP[/t].</t>
         </is>
       </c>
       <c r="C751" t="inlineStr">
         <is>
-          <t>HP를 {n}만큼 회복합니다.</t>
+          <t>[t]HP[/t]를 {n}만큼 회복합니다.</t>
         </is>
       </c>
     </row>
@@ -13198,12 +13198,12 @@
       </c>
       <c r="B752" t="inlineStr">
         <is>
-          <t>Restores {n} MP.</t>
+          <t>Restores {n} [t]MP[/t].</t>
         </is>
       </c>
       <c r="C752" t="inlineStr">
         <is>
-          <t>MP를 {n}만큼 회복합니다.</t>
+          <t>[t]MP[/t]를 {n}만큼 회복합니다.</t>
         </is>
       </c>
     </row>
@@ -14405,12 +14405,12 @@
       </c>
       <c r="B823" t="inlineStr">
         <is>
-          <t>+1 MP every 3 turns</t>
+          <t>+1 [t]MP[/t] every 3 turns</t>
         </is>
       </c>
       <c r="C823" t="inlineStr">
         <is>
-          <t>3턴마다 MP +1</t>
+          <t>3턴마다 [t]MP[/t] +1</t>
         </is>
       </c>
     </row>
@@ -14507,12 +14507,12 @@
       </c>
       <c r="B829" t="inlineStr">
         <is>
-          <t>A cursor slides along the bar. Press {confirm} when it is over the bright zone. The closer to the middle, the harder you hit.</t>
+          <t>A cursor slides along the bar. Press [k:confirm] when it is over the bright zone. The closer to the middle, the harder you hit.</t>
         </is>
       </c>
       <c r="C829" t="inlineStr">
         <is>
-          <t>커서가 막대를 따라 움직입니다. 밝은 구간 위에 왔을 때 {confirm}을(를) 누르세요. 가운데에 가까울수록 더 세게 때립니다.</t>
+          <t>커서가 막대를 따라 움직입니다. 밝은 구간 위에 왔을 때 [k:confirm]을(를) 누르세요. 가운데에 가까울수록 더 세게 때립니다.</t>
         </is>
       </c>
     </row>
@@ -14541,12 +14541,12 @@
       </c>
       <c r="B831" t="inlineStr">
         <is>
-          <t>Skills show a row of arrows. Press {up}{down}{left}{right} in that order before the time bar runs out. A wrong press costs time.</t>
+          <t>Skills show a row of arrows. Press [k:up][k:down][k:left][k:right] in that order before the time bar runs out. A wrong press costs time.</t>
         </is>
       </c>
       <c r="C831" t="inlineStr">
         <is>
-          <t>스킬을 쓰면 화살표 줄이 나옵니다. 시간 막대가 다 줄기 전에 {up}{down}{left}{right}으로 순서대로 누르세요. 틀리면 시간이 깎입니다.</t>
+          <t>스킬을 쓰면 화살표 줄이 나옵니다. 시간 막대가 다 줄기 전에 [k:up][k:down][k:left][k:right]으로 순서대로 누르세요. 틀리면 시간이 깎입니다.</t>
         </is>
       </c>
     </row>
@@ -14575,12 +14575,12 @@
       </c>
       <c r="B833" t="inlineStr">
         <is>
-          <t>When an enemy winds up a big attack, a bar appears. Press {confirm} on the bright zone to take less damage and shake off its effects.</t>
+          <t>When an enemy winds up a big attack, a bar appears. Press [k:confirm] on the bright zone to take less damage and shake off its effects.</t>
         </is>
       </c>
       <c r="C833" t="inlineStr">
         <is>
-          <t>적이 큰 공격을 준비하면 막대가 나타납니다. 밝은 구간에서 {confirm}을(를) 누르면 피해가 줄고 부가 효과도 털어냅니다.</t>
+          <t>적이 큰 공격을 준비하면 막대가 나타납니다. 밝은 구간에서 [k:confirm]을(를) 누르면 피해가 줄고 부가 효과도 털어냅니다.</t>
         </is>
       </c>
     </row>
@@ -14609,12 +14609,12 @@
       </c>
       <c r="B835" t="inlineStr">
         <is>
-          <t>Good hits fill the enemy's stagger meter. When it is full the enemy goes into BREAK: it loses a turn and takes +50% damage.</t>
+          <t>[t]Good[/t] hits fill the enemy's [t]stagger[/t] meter. When it is full the enemy goes into [a]BREAK[/a]: it loses a turn and takes +50% damage.</t>
         </is>
       </c>
       <c r="C835" t="inlineStr">
         <is>
-          <t>좋은 공격은 적의 경직 게이지를 채웁니다. 가득 차면 적이 브레이크 상태가 되어 한 턴을 잃고 피해를 50% 더 받습니다.</t>
+          <t>좋은 공격은 적의 [t]경직[/t] 게이지를 채웁니다. 가득 차면 적이 [a]브레이크[/a] 상태가 되어 한 턴을 잃고 피해를 50% 더 받습니다.</t>
         </is>
       </c>
     </row>
@@ -14745,12 +14745,12 @@
       </c>
       <c r="B843" t="inlineStr">
         <is>
-          <t>Each bed can be used once per run. Rest to restore all your HP and MP, or use it to upgrade one of your skills.</t>
+          <t>Each bed can be used once per run. Rest to restore all your [t]HP[/t] and [t]MP[/t], or use it to upgrade one of your skills.</t>
         </is>
       </c>
       <c r="C843" t="inlineStr">
         <is>
-          <t>침대는 도전마다 한 번씩만 쓸 수 있습니다. 쉬어서 HP와 MP를 모두 채우거나, 스킬 하나를 강화하세요.</t>
+          <t>침대는 도전마다 한 번씩만 쓸 수 있습니다. 쉬어서 [t]HP[/t]와 [t]MP[/t]를 모두 채우거나, 스킬 하나를 강화하세요.</t>
         </is>
       </c>
     </row>
@@ -14779,12 +14779,12 @@
       </c>
       <c r="B845" t="inlineStr">
         <is>
-          <t>Marked enemies are Elites. They are tougher than normal ones, but their rewards are better.</t>
+          <t>Marked enemies are [t]Elites[/t]. They are tougher than normal ones, but their rewards are better.</t>
         </is>
       </c>
       <c r="C845" t="inlineStr">
         <is>
-          <t>표시가 붙은 적은 정예입니다. 일반 적보다 강하지만 보상이 더 좋습니다.</t>
+          <t>표시가 붙은 적은 [t]정예[/t]입니다. 일반 적보다 강하지만 보상이 더 좋습니다.</t>
         </is>
       </c>
     </row>
@@ -14813,12 +14813,12 @@
       </c>
       <c r="B847" t="inlineStr">
         <is>
-          <t>Poison, Burn, Bleed and Stun last a few turns. The icons under a name show which ones a fighter has.</t>
+          <t>[t]Poison[/t], [t]Burn[/t], [t]Bleed[/t] and [t]Stun[/t] last a few turns. The icons under a name show which ones a fighter has.</t>
         </is>
       </c>
       <c r="C847" t="inlineStr">
         <is>
-          <t>독, 화상, 출혈, 기절은 몇 턴 동안 이어집니다. 이름 아래 아이콘이 걸려 있는 상태를 보여 줍니다.</t>
+          <t>[t]독[/t], [t]화상[/t], [t]출혈[/t], [t]기절[/t]은 몇 턴 동안 이어집니다. 이름 아래 아이콘이 걸려 있는 상태를 보여 줍니다.</t>
         </is>
       </c>
     </row>
@@ -14830,12 +14830,12 @@
       </c>
       <c r="B848" t="inlineStr">
         <is>
-          <t>{confirm} Continue</t>
+          <t>[k:confirm] Continue</t>
         </is>
       </c>
       <c r="C848" t="inlineStr">
         <is>
-          <t>{confirm} 계속</t>
+          <t>[k:confirm] 계속</t>
         </is>
       </c>
     </row>
@@ -15697,12 +15697,12 @@
       </c>
       <c r="B899" t="inlineStr">
         <is>
-          <t>Restores your HP.</t>
+          <t>Restores your [t]HP[/t].</t>
         </is>
       </c>
       <c r="C899" t="inlineStr">
         <is>
-          <t>HP를 회복합니다.</t>
+          <t>[t]HP[/t]를 회복합니다.</t>
         </is>
       </c>
     </row>
@@ -15714,12 +15714,12 @@
       </c>
       <c r="B900" t="inlineStr">
         <is>
-          <t>Restores your MP.</t>
+          <t>Restores your [t]MP[/t].</t>
         </is>
       </c>
       <c r="C900" t="inlineStr">
         <is>
-          <t>MP를 회복합니다.</t>
+          <t>[t]MP[/t]를 회복합니다.</t>
         </is>
       </c>
     </row>
@@ -15731,12 +15731,12 @@
       </c>
       <c r="B901" t="inlineStr">
         <is>
-          <t>Cures {status}.</t>
+          <t>Cures [t]{status}[/t].</t>
         </is>
       </c>
       <c r="C901" t="inlineStr">
         <is>
-          <t>{status} 상태를 치료합니다.</t>
+          <t>[t]{status}[/t] 상태를 치료합니다.</t>
         </is>
       </c>
     </row>
@@ -15770,7 +15770,7 @@
       </c>
       <c r="C903" t="inlineStr">
         <is>
-          <t>기절하지 않습니다.</t>
+          <t>[t]기절[/t]하지 않습니다.</t>
         </is>
       </c>
     </row>
@@ -15850,12 +15850,12 @@
       </c>
       <c r="B908" t="inlineStr">
         <is>
-          <t>{confirm} Choose   {back} Back</t>
+          <t>[k:confirm] Choose</t>
         </is>
       </c>
       <c r="C908" t="inlineStr">
         <is>
-          <t>{confirm} 선택   {back} 뒤로</t>
+          <t>[k:confirm] 선택</t>
         </is>
       </c>
     </row>
@@ -16734,12 +16734,12 @@
       </c>
       <c r="B960" t="inlineStr">
         <is>
-          <t>{back} Back</t>
+          <t>[k:back] Back</t>
         </is>
       </c>
       <c r="C960" t="inlineStr">
         <is>
-          <t>{back} 뒤로</t>
+          <t>[k:back] 뒤로</t>
         </is>
       </c>
     </row>
@@ -16751,12 +16751,12 @@
       </c>
       <c r="B961" t="inlineStr">
         <is>
-          <t>{left}{right} Change</t>
+          <t>[k:left][k:right] Change</t>
         </is>
       </c>
       <c r="C961" t="inlineStr">
         <is>
-          <t>{left}{right} 변경</t>
+          <t>[k:left][k:right] 변경</t>
         </is>
       </c>
     </row>
@@ -16768,12 +16768,12 @@
       </c>
       <c r="B962" t="inlineStr">
         <is>
-          <t>{back} Close</t>
+          <t>[k:back] Close</t>
         </is>
       </c>
       <c r="C962" t="inlineStr">
         <is>
-          <t>{back} 닫기</t>
+          <t>[k:back] 닫기</t>
         </is>
       </c>
     </row>
@@ -16785,12 +16785,12 @@
       </c>
       <c r="B963" t="inlineStr">
         <is>
-          <t>{confirm} Equip</t>
+          <t>[k:confirm] Equip</t>
         </is>
       </c>
       <c r="C963" t="inlineStr">
         <is>
-          <t>{confirm} 착용</t>
+          <t>[k:confirm] 착용</t>
         </is>
       </c>
     </row>
@@ -16802,12 +16802,12 @@
       </c>
       <c r="B964" t="inlineStr">
         <is>
-          <t>{confirm} Open</t>
+          <t>[k:confirm] Open</t>
         </is>
       </c>
       <c r="C964" t="inlineStr">
         <is>
-          <t>{confirm} 열기</t>
+          <t>[k:confirm] 열기</t>
         </is>
       </c>
     </row>
@@ -16819,12 +16819,12 @@
       </c>
       <c r="B965" t="inlineStr">
         <is>
-          <t>{confirm} Select</t>
+          <t>[k:confirm] Select</t>
         </is>
       </c>
       <c r="C965" t="inlineStr">
         <is>
-          <t>{confirm} 선택</t>
+          <t>[k:confirm] 선택</t>
         </is>
       </c>
     </row>
@@ -16836,12 +16836,12 @@
       </c>
       <c r="B966" t="inlineStr">
         <is>
-          <t>{confirm} Take off</t>
+          <t>[k:confirm] Take off</t>
         </is>
       </c>
       <c r="C966" t="inlineStr">
         <is>
-          <t>{confirm} 해제</t>
+          <t>[k:confirm] 해제</t>
         </is>
       </c>
     </row>
@@ -16853,12 +16853,12 @@
       </c>
       <c r="B967" t="inlineStr">
         <is>
-          <t>{confirm} Use</t>
+          <t>[k:confirm] Use</t>
         </is>
       </c>
       <c r="C967" t="inlineStr">
         <is>
-          <t>{confirm} 사용</t>
+          <t>[k:confirm] 사용</t>
         </is>
       </c>
     </row>
@@ -18213,12 +18213,12 @@
       </c>
       <c r="B1047" t="inlineStr">
         <is>
-          <t>Raises your max HP by {n} and heals {n} HP.</t>
+          <t>Raises your max [t]HP[/t] by {n} and heals {n} [t]HP[/t].</t>
         </is>
       </c>
       <c r="C1047" t="inlineStr">
         <is>
-          <t>최대 HP가 {n} 오르고 HP를 {n} 회복합니다.</t>
+          <t>최대 [t]HP[/t]가 {n} 오르고 [t]HP[/t]를 {n} 회복합니다.</t>
         </is>
       </c>
     </row>
@@ -18230,12 +18230,12 @@
       </c>
       <c r="B1048" t="inlineStr">
         <is>
-          <t>Raises your max MP by {n} and restores {n} MP.</t>
+          <t>Raises your max [t]MP[/t] by {n} and restores {n} [t]MP[/t].</t>
         </is>
       </c>
       <c r="C1048" t="inlineStr">
         <is>
-          <t>최대 MP가 {n} 오르고 MP를 {n} 회복합니다.</t>
+          <t>최대 [t]MP[/t]가 {n} 오르고 [t]MP[/t]를 {n} 회복합니다.</t>
         </is>
       </c>
     </row>
@@ -18332,12 +18332,12 @@
       </c>
       <c r="B1054" t="inlineStr">
         <is>
-          <t>{confirm} Keep   {back} Revert</t>
+          <t>[k:confirm] Keep   [k:back] Revert</t>
         </is>
       </c>
       <c r="C1054" t="inlineStr">
         <is>
-          <t>{confirm} 유지   {back} 되돌리기</t>
+          <t>[k:confirm] 유지   [k:back] 되돌리기</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(ui): status labels under every chip with the full sentence on highlight, distinct XP bar, Equipped header, Help Stats & terms page, bed and item refusals (D150, D156)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datafiles/localization/game_text.xlsx
+++ b/datafiles/localization/game_text.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1054"/>
+  <dimension ref="A1:C1094"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -13895,7 +13895,7 @@
       </c>
       <c r="B793" t="inlineStr">
         <is>
-          <t>Worn</t>
+          <t>Equipped</t>
         </is>
       </c>
       <c r="C793" t="inlineStr">
@@ -16615,7 +16615,7 @@
       </c>
       <c r="B953" t="inlineStr">
         <is>
-          <t>Nothing worn</t>
+          <t>Nothing equipped</t>
         </is>
       </c>
       <c r="C953" t="inlineStr">
@@ -16632,7 +16632,7 @@
       </c>
       <c r="B954" t="inlineStr">
         <is>
-          <t>Nothing is worn in this slot.</t>
+          <t>Nothing is equipped in this slot.</t>
         </is>
       </c>
       <c r="C954" t="inlineStr">
@@ -16717,7 +16717,7 @@
       </c>
       <c r="B959" t="inlineStr">
         <is>
-          <t>Worn</t>
+          <t>Equipped</t>
         </is>
       </c>
       <c r="C959" t="inlineStr">
@@ -18338,6 +18338,686 @@
       <c r="C1054" t="inlineStr">
         <is>
           <t>{confirm} 유지   {back} 되돌리기</t>
+        </is>
+      </c>
+    </row>
+    <row r="1055">
+      <c r="A1055" t="inlineStr">
+        <is>
+          <t>status.short.status_poison</t>
+        </is>
+      </c>
+      <c r="B1055" t="inlineStr">
+        <is>
+          <t>PSN</t>
+        </is>
+      </c>
+      <c r="C1055" t="inlineStr">
+        <is>
+          <t>독</t>
+        </is>
+      </c>
+    </row>
+    <row r="1056">
+      <c r="A1056" t="inlineStr">
+        <is>
+          <t>status.short.status_bleed</t>
+        </is>
+      </c>
+      <c r="B1056" t="inlineStr">
+        <is>
+          <t>BLD</t>
+        </is>
+      </c>
+      <c r="C1056" t="inlineStr">
+        <is>
+          <t>출혈</t>
+        </is>
+      </c>
+    </row>
+    <row r="1057">
+      <c r="A1057" t="inlineStr">
+        <is>
+          <t>status.short.status_burn</t>
+        </is>
+      </c>
+      <c r="B1057" t="inlineStr">
+        <is>
+          <t>BRN</t>
+        </is>
+      </c>
+      <c r="C1057" t="inlineStr">
+        <is>
+          <t>화상</t>
+        </is>
+      </c>
+    </row>
+    <row r="1058">
+      <c r="A1058" t="inlineStr">
+        <is>
+          <t>status.short.status_stun</t>
+        </is>
+      </c>
+      <c r="B1058" t="inlineStr">
+        <is>
+          <t>STN</t>
+        </is>
+      </c>
+      <c r="C1058" t="inlineStr">
+        <is>
+          <t>기절</t>
+        </is>
+      </c>
+    </row>
+    <row r="1059">
+      <c r="A1059" t="inlineStr">
+        <is>
+          <t>status.short.status_guard</t>
+        </is>
+      </c>
+      <c r="B1059" t="inlineStr">
+        <is>
+          <t>GRD</t>
+        </is>
+      </c>
+      <c r="C1059" t="inlineStr">
+        <is>
+          <t>방어</t>
+        </is>
+      </c>
+    </row>
+    <row r="1060">
+      <c r="A1060" t="inlineStr">
+        <is>
+          <t>status.short.status_dmg_up</t>
+        </is>
+      </c>
+      <c r="B1060" t="inlineStr">
+        <is>
+          <t>REV</t>
+        </is>
+      </c>
+      <c r="C1060" t="inlineStr">
+        <is>
+          <t>기세</t>
+        </is>
+      </c>
+    </row>
+    <row r="1061">
+      <c r="A1061" t="inlineStr">
+        <is>
+          <t>status.short.status_evasion</t>
+        </is>
+      </c>
+      <c r="B1061" t="inlineStr">
+        <is>
+          <t>EVA</t>
+        </is>
+      </c>
+      <c r="C1061" t="inlineStr">
+        <is>
+          <t>회피</t>
+        </is>
+      </c>
+    </row>
+    <row r="1062">
+      <c r="A1062" t="inlineStr">
+        <is>
+          <t>status.short.status_crit_up</t>
+        </is>
+      </c>
+      <c r="B1062" t="inlineStr">
+        <is>
+          <t>AIM</t>
+        </is>
+      </c>
+      <c r="C1062" t="inlineStr">
+        <is>
+          <t>조준</t>
+        </is>
+      </c>
+    </row>
+    <row r="1063">
+      <c r="A1063" t="inlineStr">
+        <is>
+          <t>status.short.status_hit_up</t>
+        </is>
+      </c>
+      <c r="B1063" t="inlineStr">
+        <is>
+          <t>FORE</t>
+        </is>
+      </c>
+      <c r="C1063" t="inlineStr">
+        <is>
+          <t>선견</t>
+        </is>
+      </c>
+    </row>
+    <row r="1064">
+      <c r="A1064" t="inlineStr">
+        <is>
+          <t>status.short.status_meditation</t>
+        </is>
+      </c>
+      <c r="B1064" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="C1064" t="inlineStr">
+        <is>
+          <t>명상</t>
+        </is>
+      </c>
+    </row>
+    <row r="1065">
+      <c r="A1065" t="inlineStr">
+        <is>
+          <t>status.short.status_solidify</t>
+        </is>
+      </c>
+      <c r="B1065" t="inlineStr">
+        <is>
+          <t>Solid</t>
+        </is>
+      </c>
+      <c r="C1065" t="inlineStr">
+        <is>
+          <t>굳힘</t>
+        </is>
+      </c>
+    </row>
+    <row r="1066">
+      <c r="A1066" t="inlineStr">
+        <is>
+          <t>status.short.status_bloodthirsty</t>
+        </is>
+      </c>
+      <c r="B1066" t="inlineStr">
+        <is>
+          <t>Thirst</t>
+        </is>
+      </c>
+      <c r="C1066" t="inlineStr">
+        <is>
+          <t>갈증</t>
+        </is>
+      </c>
+    </row>
+    <row r="1067">
+      <c r="A1067" t="inlineStr">
+        <is>
+          <t>status.short.status_blessing</t>
+        </is>
+      </c>
+      <c r="B1067" t="inlineStr">
+        <is>
+          <t>Bless</t>
+        </is>
+      </c>
+      <c r="C1067" t="inlineStr">
+        <is>
+          <t>축복</t>
+        </is>
+      </c>
+    </row>
+    <row r="1068">
+      <c r="A1068" t="inlineStr">
+        <is>
+          <t>status.short.status_sunder</t>
+        </is>
+      </c>
+      <c r="B1068" t="inlineStr">
+        <is>
+          <t>Sunder</t>
+        </is>
+      </c>
+      <c r="C1068" t="inlineStr">
+        <is>
+          <t>분쇄</t>
+        </is>
+      </c>
+    </row>
+    <row r="1069">
+      <c r="A1069" t="inlineStr">
+        <is>
+          <t>status.short.status_brace</t>
+        </is>
+      </c>
+      <c r="B1069" t="inlineStr">
+        <is>
+          <t>Brace</t>
+        </is>
+      </c>
+      <c r="C1069" t="inlineStr">
+        <is>
+          <t>태세</t>
+        </is>
+      </c>
+    </row>
+    <row r="1070">
+      <c r="A1070" t="inlineStr">
+        <is>
+          <t>battle.chip.steadfast.short</t>
+        </is>
+      </c>
+      <c r="B1070" t="inlineStr">
+        <is>
+          <t>Steady</t>
+        </is>
+      </c>
+      <c r="C1070" t="inlineStr">
+        <is>
+          <t>버티기</t>
+        </is>
+      </c>
+    </row>
+    <row r="1071">
+      <c r="A1071" t="inlineStr">
+        <is>
+          <t>battle.chip.break.short</t>
+        </is>
+      </c>
+      <c r="B1071" t="inlineStr">
+        <is>
+          <t>BREAK</t>
+        </is>
+      </c>
+      <c r="C1071" t="inlineStr">
+        <is>
+          <t>브레이크</t>
+        </is>
+      </c>
+    </row>
+    <row r="1072">
+      <c r="A1072" t="inlineStr">
+        <is>
+          <t>status.turns_left</t>
+        </is>
+      </c>
+      <c r="B1072" t="inlineStr">
+        <is>
+          <t>{turns} turns left.</t>
+        </is>
+      </c>
+      <c r="C1072" t="inlineStr">
+        <is>
+          <t>{turns}턴 남았습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1073">
+      <c r="A1073" t="inlineStr">
+        <is>
+          <t>status.turn_left</t>
+        </is>
+      </c>
+      <c r="B1073" t="inlineStr">
+        <is>
+          <t>1 turn left.</t>
+        </is>
+      </c>
+      <c r="C1073" t="inlineStr">
+        <is>
+          <t>1턴 남았습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1074">
+      <c r="A1074" t="inlineStr">
+        <is>
+          <t>bed.msg.rested</t>
+        </is>
+      </c>
+      <c r="B1074" t="inlineStr">
+        <is>
+          <t>You are already rested.</t>
+        </is>
+      </c>
+      <c r="C1074" t="inlineStr">
+        <is>
+          <t>이미 충분히 쉬었습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1075">
+      <c r="A1075" t="inlineStr">
+        <is>
+          <t>bed.msg.nothing_to_upgrade</t>
+        </is>
+      </c>
+      <c r="B1075" t="inlineStr">
+        <is>
+          <t>Nothing to upgrade there.</t>
+        </is>
+      </c>
+      <c r="C1075" t="inlineStr">
+        <is>
+          <t>강화할 수 있는 것이 없습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1076">
+      <c r="A1076" t="inlineStr">
+        <is>
+          <t>bed.help.heal_rested</t>
+        </is>
+      </c>
+      <c r="B1076" t="inlineStr">
+        <is>
+          <t>You are already rested. Come back when HP or MP is missing.</t>
+        </is>
+      </c>
+      <c r="C1076" t="inlineStr">
+        <is>
+          <t>이미 충분히 쉬었습니다. HP나 MP가 줄었을 때 다시 오세요.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1077">
+      <c r="A1077" t="inlineStr">
+        <is>
+          <t>item.msg.nothing_happens</t>
+        </is>
+      </c>
+      <c r="B1077" t="inlineStr">
+        <is>
+          <t>Nothing happens.</t>
+        </is>
+      </c>
+      <c r="C1077" t="inlineStr">
+        <is>
+          <t>아무 일도 일어나지 않았습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1078">
+      <c r="A1078" t="inlineStr">
+        <is>
+          <t>help.stats.title</t>
+        </is>
+      </c>
+      <c r="B1078" t="inlineStr">
+        <is>
+          <t>Stats &amp; terms</t>
+        </is>
+      </c>
+      <c r="C1078" t="inlineStr">
+        <is>
+          <t>능력치와 용어</t>
+        </is>
+      </c>
+    </row>
+    <row r="1079">
+      <c r="A1079" t="inlineStr">
+        <is>
+          <t>help.stats.help</t>
+        </is>
+      </c>
+      <c r="B1079" t="inlineStr">
+        <is>
+          <t>What Power, ATK, DEF, MAG, SPD, Crit, the grades, BREAK and every status mean.</t>
+        </is>
+      </c>
+      <c r="C1079" t="inlineStr">
+        <is>
+          <t>위력, ATK, DEF, MAG, SPD, 치명타, 등급, 브레이크와 모든 상태 이상의 뜻입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1080">
+      <c r="A1080" t="inlineStr">
+        <is>
+          <t>help.term.crit</t>
+        </is>
+      </c>
+      <c r="B1080" t="inlineStr">
+        <is>
+          <t>Crit</t>
+        </is>
+      </c>
+      <c r="C1080" t="inlineStr">
+        <is>
+          <t>치명타</t>
+        </is>
+      </c>
+    </row>
+    <row r="1081">
+      <c r="A1081" t="inlineStr">
+        <is>
+          <t>help.term.good</t>
+        </is>
+      </c>
+      <c r="B1081" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="C1081" t="inlineStr">
+        <is>
+          <t>좋음</t>
+        </is>
+      </c>
+    </row>
+    <row r="1082">
+      <c r="A1082" t="inlineStr">
+        <is>
+          <t>help.term.ok</t>
+        </is>
+      </c>
+      <c r="B1082" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="C1082" t="inlineStr">
+        <is>
+          <t>무난</t>
+        </is>
+      </c>
+    </row>
+    <row r="1083">
+      <c r="A1083" t="inlineStr">
+        <is>
+          <t>help.term.weak</t>
+        </is>
+      </c>
+      <c r="B1083" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="C1083" t="inlineStr">
+        <is>
+          <t>약함</t>
+        </is>
+      </c>
+    </row>
+    <row r="1084">
+      <c r="A1084" t="inlineStr">
+        <is>
+          <t>help.term.break</t>
+        </is>
+      </c>
+      <c r="B1084" t="inlineStr">
+        <is>
+          <t>BREAK</t>
+        </is>
+      </c>
+      <c r="C1084" t="inlineStr">
+        <is>
+          <t>브레이크</t>
+        </is>
+      </c>
+    </row>
+    <row r="1085">
+      <c r="A1085" t="inlineStr">
+        <is>
+          <t>help.line.power</t>
+        </is>
+      </c>
+      <c r="B1085" t="inlineStr">
+        <is>
+          <t>How hard a weapon or skill hits. More Power means more damage.</t>
+        </is>
+      </c>
+      <c r="C1085" t="inlineStr">
+        <is>
+          <t>무기나 스킬의 타격 세기입니다. 위력이 높을수록 피해가 커집니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1086">
+      <c r="A1086" t="inlineStr">
+        <is>
+          <t>help.line.hp</t>
+        </is>
+      </c>
+      <c r="B1086" t="inlineStr">
+        <is>
+          <t>Health. At 0 HP you fall.</t>
+        </is>
+      </c>
+      <c r="C1086" t="inlineStr">
+        <is>
+          <t>체력입니다. HP가 0이 되면 쓰러집니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1087">
+      <c r="A1087" t="inlineStr">
+        <is>
+          <t>help.line.mp</t>
+        </is>
+      </c>
+      <c r="B1087" t="inlineStr">
+        <is>
+          <t>Magic points. Skills spend them; potions and rest restore them.</t>
+        </is>
+      </c>
+      <c r="C1087" t="inlineStr">
+        <is>
+          <t>스킬을 쓰면 줄어드는 마력입니다. 물약과 휴식으로 회복합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1088">
+      <c r="A1088" t="inlineStr">
+        <is>
+          <t>help.line.crit</t>
+        </is>
+      </c>
+      <c r="B1088" t="inlineStr">
+        <is>
+          <t>A critical hit deals {mult} times the damage. Take Aim and some gear raise the odds.</t>
+        </is>
+      </c>
+      <c r="C1088" t="inlineStr">
+        <is>
+          <t>치명타는 피해를 {mult}배로 줍니다. 조준과 일부 장비가 확률을 높입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1089">
+      <c r="A1089" t="inlineStr">
+        <is>
+          <t>help.line.perfect</t>
+        </is>
+      </c>
+      <c r="B1089" t="inlineStr">
+        <is>
+          <t>Press in the bright zone of the bar for +{pct}% damage.</t>
+        </is>
+      </c>
+      <c r="C1089" t="inlineStr">
+        <is>
+          <t>막대의 밝은 구간에서 누르면 피해가 {pct}% 늘어납니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1090">
+      <c r="A1090" t="inlineStr">
+        <is>
+          <t>help.line.good</t>
+        </is>
+      </c>
+      <c r="B1090" t="inlineStr">
+        <is>
+          <t>Press near the middle for +{pct}% damage.</t>
+        </is>
+      </c>
+      <c r="C1090" t="inlineStr">
+        <is>
+          <t>가운데 근처에서 누르면 피해가 {pct}% 늘어납니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1091">
+      <c r="A1091" t="inlineStr">
+        <is>
+          <t>help.line.ok</t>
+        </is>
+      </c>
+      <c r="B1091" t="inlineStr">
+        <is>
+          <t>Press on the bar but off the middle for normal damage.</t>
+        </is>
+      </c>
+      <c r="C1091" t="inlineStr">
+        <is>
+          <t>막대 위에서 가운데를 벗어나 누르면 보통 피해를 줍니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1092">
+      <c r="A1092" t="inlineStr">
+        <is>
+          <t>help.line.weak</t>
+        </is>
+      </c>
+      <c r="B1092" t="inlineStr">
+        <is>
+          <t>Miss the zone and the hit deals {pct}% less damage.</t>
+        </is>
+      </c>
+      <c r="C1092" t="inlineStr">
+        <is>
+          <t>구간을 놓치면 피해가 {pct}% 줄어듭니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1093">
+      <c r="A1093" t="inlineStr">
+        <is>
+          <t>help.line.break</t>
+        </is>
+      </c>
+      <c r="B1093" t="inlineStr">
+        <is>
+          <t>Good hits fill the stagger meter. When it is full the enemy loses a turn and takes +{pct}% damage.</t>
+        </is>
+      </c>
+      <c r="C1093" t="inlineStr">
+        <is>
+          <t>좋은 공격은 경직 게이지를 채웁니다. 가득 차면 적이 한 턴을 잃고 피해를 {pct}% 더 받습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1094">
+      <c r="A1094" t="inlineStr">
+        <is>
+          <t>help.line.elite</t>
+        </is>
+      </c>
+      <c r="B1094" t="inlineStr">
+        <is>
+          <t>A marked, tougher enemy with a special trait. Its rewards are better.</t>
+        </is>
+      </c>
+      <c r="C1094" t="inlineStr">
+        <is>
+          <t>표시가 붙은 더 강한 적으로, 특별한 특성이 있습니다. 보상이 더 좋습니다.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Merge h12a-choices: small flavour choices at the merchant, the Stranger, a note and the wake line (D154) - WIP integration
Notes: H7 (D147) picks a note up without a dialogue, so the note's question (written for the old read-on-pickup) has no place yet;
Note_ReadLines / Note_RunChoice are kept for the follow-up that asks it in the Codex reader. Steps 890-909 / 910-913, shots 274.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datafiles/localization/game_text.xlsx
+++ b/datafiles/localization/game_text.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1111"/>
+  <dimension ref="A1:C1151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -19310,6 +19310,686 @@
         </is>
       </c>
     </row>
+    <row r="1112">
+      <c r="A1112" t="inlineStr">
+        <is>
+          <t>choice.stranger.ask.0</t>
+        </is>
+      </c>
+      <c r="B1112" t="inlineStr">
+        <is>
+          <t>There you are.</t>
+        </is>
+      </c>
+      <c r="C1112" t="inlineStr">
+        <is>
+          <t>거기 있었군.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1113">
+      <c r="A1113" t="inlineStr">
+        <is>
+          <t>choice.stranger.ask.1</t>
+        </is>
+      </c>
+      <c r="B1113" t="inlineStr">
+        <is>
+          <t>Do you remember me?</t>
+        </is>
+      </c>
+      <c r="C1113" t="inlineStr">
+        <is>
+          <t>나를 기억해?</t>
+        </is>
+      </c>
+    </row>
+    <row r="1114">
+      <c r="A1114" t="inlineStr">
+        <is>
+          <t>choice.stranger.label.0</t>
+        </is>
+      </c>
+      <c r="B1114" t="inlineStr">
+        <is>
+          <t>Should I?</t>
+        </is>
+      </c>
+      <c r="C1114" t="inlineStr">
+        <is>
+          <t>기억해야 해?</t>
+        </is>
+      </c>
+    </row>
+    <row r="1115">
+      <c r="A1115" t="inlineStr">
+        <is>
+          <t>choice.stranger.label.1</t>
+        </is>
+      </c>
+      <c r="B1115" t="inlineStr">
+        <is>
+          <t>Back off.</t>
+        </is>
+      </c>
+      <c r="C1115" t="inlineStr">
+        <is>
+          <t>저리 가.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1116">
+      <c r="A1116" t="inlineStr">
+        <is>
+          <t>choice.stranger.reply1.0</t>
+        </is>
+      </c>
+      <c r="B1116" t="inlineStr">
+        <is>
+          <t>Not yet.</t>
+        </is>
+      </c>
+      <c r="C1116" t="inlineStr">
+        <is>
+          <t>아직은 아니야.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1117">
+      <c r="A1117" t="inlineStr">
+        <is>
+          <t>choice.stranger.reply1.1</t>
+        </is>
+      </c>
+      <c r="B1117" t="inlineStr">
+        <is>
+          <t>Ask again when the tunnel has had you a few more times.</t>
+        </is>
+      </c>
+      <c r="C1117" t="inlineStr">
+        <is>
+          <t>터널이 널 몇 번 더 삼키면 다시 물어봐.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1118">
+      <c r="A1118" t="inlineStr">
+        <is>
+          <t>choice.stranger.reply2.0</t>
+        </is>
+      </c>
+      <c r="B1118" t="inlineStr">
+        <is>
+          <t>Ha. Fair.</t>
+        </is>
+      </c>
+      <c r="C1118" t="inlineStr">
+        <is>
+          <t>하하, 그렇겠지.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1119">
+      <c r="A1119" t="inlineStr">
+        <is>
+          <t>choice.stranger.reply2.1</t>
+        </is>
+      </c>
+      <c r="B1119" t="inlineStr">
+        <is>
+          <t>Nobody does, at first.</t>
+        </is>
+      </c>
+      <c r="C1119" t="inlineStr">
+        <is>
+          <t>처음엔 다들 그래.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1120">
+      <c r="A1120" t="inlineStr">
+        <is>
+          <t>choice.stranger.again1.0</t>
+        </is>
+      </c>
+      <c r="B1120" t="inlineStr">
+        <is>
+          <t>Still asking if you should?</t>
+        </is>
+      </c>
+      <c r="C1120" t="inlineStr">
+        <is>
+          <t>아직도 기억해야 하는지 묻는군?</t>
+        </is>
+      </c>
+    </row>
+    <row r="1121">
+      <c r="A1121" t="inlineStr">
+        <is>
+          <t>choice.stranger.again1.1</t>
+        </is>
+      </c>
+      <c r="B1121" t="inlineStr">
+        <is>
+          <t>You'll know me when you stop asking.</t>
+        </is>
+      </c>
+      <c r="C1121" t="inlineStr">
+        <is>
+          <t>묻기를 그만두면 알게 될 거야.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1122">
+      <c r="A1122" t="inlineStr">
+        <is>
+          <t>choice.stranger.again2.0</t>
+        </is>
+      </c>
+      <c r="B1122" t="inlineStr">
+        <is>
+          <t>Still telling me to back off?</t>
+        </is>
+      </c>
+      <c r="C1122" t="inlineStr">
+        <is>
+          <t>아직도 저리 가라고 하는군?</t>
+        </is>
+      </c>
+    </row>
+    <row r="1123">
+      <c r="A1123" t="inlineStr">
+        <is>
+          <t>choice.stranger.again2.1</t>
+        </is>
+      </c>
+      <c r="B1123" t="inlineStr">
+        <is>
+          <t>I'm patient. I've had practice.</t>
+        </is>
+      </c>
+      <c r="C1123" t="inlineStr">
+        <is>
+          <t>난 참을성이 있어. 연습을 많이 했거든.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1124">
+      <c r="A1124" t="inlineStr">
+        <is>
+          <t>choice.merchant.ask.0</t>
+        </is>
+      </c>
+      <c r="B1124" t="inlineStr">
+        <is>
+          <t>Tell me, friend.</t>
+        </is>
+      </c>
+      <c r="C1124" t="inlineStr">
+        <is>
+          <t>말해 봐, 친구.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1125">
+      <c r="A1125" t="inlineStr">
+        <is>
+          <t>choice.merchant.ask.1</t>
+        </is>
+      </c>
+      <c r="B1125" t="inlineStr">
+        <is>
+          <t>Looking for a way out, or something to buy?</t>
+        </is>
+      </c>
+      <c r="C1125" t="inlineStr">
+        <is>
+          <t>나갈 길을 찾는 거야, 아니면 살 게 있는 거야?</t>
+        </is>
+      </c>
+    </row>
+    <row r="1126">
+      <c r="A1126" t="inlineStr">
+        <is>
+          <t>choice.merchant.label.0</t>
+        </is>
+      </c>
+      <c r="B1126" t="inlineStr">
+        <is>
+          <t>A way out.</t>
+        </is>
+      </c>
+      <c r="C1126" t="inlineStr">
+        <is>
+          <t>나갈 길.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1127">
+      <c r="A1127" t="inlineStr">
+        <is>
+          <t>choice.merchant.label.1</t>
+        </is>
+      </c>
+      <c r="B1127" t="inlineStr">
+        <is>
+          <t>Something to buy.</t>
+        </is>
+      </c>
+      <c r="C1127" t="inlineStr">
+        <is>
+          <t>살 물건.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1128">
+      <c r="A1128" t="inlineStr">
+        <is>
+          <t>choice.merchant.reply1.0</t>
+        </is>
+      </c>
+      <c r="B1128" t="inlineStr">
+        <is>
+          <t>Ha. They all say that.</t>
+        </is>
+      </c>
+      <c r="C1128" t="inlineStr">
+        <is>
+          <t>하하, 다들 그렇게 말하지.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1129">
+      <c r="A1129" t="inlineStr">
+        <is>
+          <t>choice.merchant.reply1.1</t>
+        </is>
+      </c>
+      <c r="B1129" t="inlineStr">
+        <is>
+          <t>Shop first. Hope walks better with a full pack.</t>
+        </is>
+      </c>
+      <c r="C1129" t="inlineStr">
+        <is>
+          <t>일단 사. 짐이 든든해야 희망도 잘 걷거든.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1130">
+      <c r="A1130" t="inlineStr">
+        <is>
+          <t>choice.merchant.reply2.0</t>
+        </is>
+      </c>
+      <c r="B1130" t="inlineStr">
+        <is>
+          <t>Good. Buying I understand.</t>
+        </is>
+      </c>
+      <c r="C1130" t="inlineStr">
+        <is>
+          <t>좋아. 장사라면 내가 잘 알지.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1131">
+      <c r="A1131" t="inlineStr">
+        <is>
+          <t>choice.merchant.reply2.1</t>
+        </is>
+      </c>
+      <c r="B1131" t="inlineStr">
+        <is>
+          <t>Asking after exits gets people killed.</t>
+        </is>
+      </c>
+      <c r="C1131" t="inlineStr">
+        <is>
+          <t>출구를 캐묻다 죽은 사람이 한둘이 아니야.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1132">
+      <c r="A1132" t="inlineStr">
+        <is>
+          <t>choice.merchant.again1.0</t>
+        </is>
+      </c>
+      <c r="B1132" t="inlineStr">
+        <is>
+          <t>Found your way out yet? No? Then buy something.</t>
+        </is>
+      </c>
+      <c r="C1132" t="inlineStr">
+        <is>
+          <t>나갈 길은 찾았어? 아직이면 뭐라도 사.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1133">
+      <c r="A1133" t="inlineStr">
+        <is>
+          <t>choice.merchant.again2.0</t>
+        </is>
+      </c>
+      <c r="B1133" t="inlineStr">
+        <is>
+          <t>Back to spend, I hope. That I understand.</t>
+        </is>
+      </c>
+      <c r="C1133" t="inlineStr">
+        <is>
+          <t>돈 쓰러 왔길 바란다. 그거라면 내가 잘 알지.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1134">
+      <c r="A1134" t="inlineStr">
+        <is>
+          <t>choice.map_page.ask.0</t>
+        </is>
+      </c>
+      <c r="B1134" t="inlineStr">
+        <is>
+          <t>You read it twice.</t>
+        </is>
+      </c>
+      <c r="C1134" t="inlineStr">
+        <is>
+          <t>두 번 읽는다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1135">
+      <c r="A1135" t="inlineStr">
+        <is>
+          <t>choice.map_page.ask.1</t>
+        </is>
+      </c>
+      <c r="B1135" t="inlineStr">
+        <is>
+          <t>Whose hand is this?</t>
+        </is>
+      </c>
+      <c r="C1135" t="inlineStr">
+        <is>
+          <t>누구의 글씨일까?</t>
+        </is>
+      </c>
+    </row>
+    <row r="1136">
+      <c r="A1136" t="inlineStr">
+        <is>
+          <t>choice.map_page.label.0</t>
+        </is>
+      </c>
+      <c r="B1136" t="inlineStr">
+        <is>
+          <t>Mine.</t>
+        </is>
+      </c>
+      <c r="C1136" t="inlineStr">
+        <is>
+          <t>내 것.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1137">
+      <c r="A1137" t="inlineStr">
+        <is>
+          <t>choice.map_page.label.1</t>
+        </is>
+      </c>
+      <c r="B1137" t="inlineStr">
+        <is>
+          <t>Someone else's.</t>
+        </is>
+      </c>
+      <c r="C1137" t="inlineStr">
+        <is>
+          <t>남의 것.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1138">
+      <c r="A1138" t="inlineStr">
+        <is>
+          <t>choice.map_page.reply1.0</t>
+        </is>
+      </c>
+      <c r="B1138" t="inlineStr">
+        <is>
+          <t>Yours. You say it out loud.</t>
+        </is>
+      </c>
+      <c r="C1138" t="inlineStr">
+        <is>
+          <t>내 글씨다. 소리 내어 말해 본다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1139">
+      <c r="A1139" t="inlineStr">
+        <is>
+          <t>choice.map_page.reply1.1</t>
+        </is>
+      </c>
+      <c r="B1139" t="inlineStr">
+        <is>
+          <t>The ink seems to settle.</t>
+        </is>
+      </c>
+      <c r="C1139" t="inlineStr">
+        <is>
+          <t>잉크가 가라앉는 듯하다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1140">
+      <c r="A1140" t="inlineStr">
+        <is>
+          <t>choice.map_page.reply2.0</t>
+        </is>
+      </c>
+      <c r="B1140" t="inlineStr">
+        <is>
+          <t>Not yours. You say it out loud.</t>
+        </is>
+      </c>
+      <c r="C1140" t="inlineStr">
+        <is>
+          <t>내 글씨가 아니다. 소리 내어 말해 본다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1141">
+      <c r="A1141" t="inlineStr">
+        <is>
+          <t>choice.map_page.reply2.1</t>
+        </is>
+      </c>
+      <c r="B1141" t="inlineStr">
+        <is>
+          <t>The ink shivers.</t>
+        </is>
+      </c>
+      <c r="C1141" t="inlineStr">
+        <is>
+          <t>잉크가 떨리는 듯하다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1142">
+      <c r="A1142" t="inlineStr">
+        <is>
+          <t>choice.map_page.again1.0</t>
+        </is>
+      </c>
+      <c r="B1142" t="inlineStr">
+        <is>
+          <t>The ink is dry now. You've stopped doubting the hand.</t>
+        </is>
+      </c>
+      <c r="C1142" t="inlineStr">
+        <is>
+          <t>잉크가 말랐다. 이 글씨를 더는 의심하지 않는다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1143">
+      <c r="A1143" t="inlineStr">
+        <is>
+          <t>choice.map_page.again2.0</t>
+        </is>
+      </c>
+      <c r="B1143" t="inlineStr">
+        <is>
+          <t>The ink is dry now. You still say it isn't yours.</t>
+        </is>
+      </c>
+      <c r="C1143" t="inlineStr">
+        <is>
+          <t>잉크가 말랐다. 그래도 내 글씨가 아니라고 말한다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1144">
+      <c r="A1144" t="inlineStr">
+        <is>
+          <t>choice.wake.ask.0</t>
+        </is>
+      </c>
+      <c r="B1144" t="inlineStr">
+        <is>
+          <t>Your head swims.</t>
+        </is>
+      </c>
+      <c r="C1144" t="inlineStr">
+        <is>
+          <t>머리가 어지럽다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1145">
+      <c r="A1145" t="inlineStr">
+        <is>
+          <t>choice.wake.ask.1</t>
+        </is>
+      </c>
+      <c r="B1145" t="inlineStr">
+        <is>
+          <t>Your body waits for you to decide.</t>
+        </is>
+      </c>
+      <c r="C1145" t="inlineStr">
+        <is>
+          <t>몸이 당신의 결정을 기다린다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1146">
+      <c r="A1146" t="inlineStr">
+        <is>
+          <t>choice.wake.label.0</t>
+        </is>
+      </c>
+      <c r="B1146" t="inlineStr">
+        <is>
+          <t>Sit up.</t>
+        </is>
+      </c>
+      <c r="C1146" t="inlineStr">
+        <is>
+          <t>일어난다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1147">
+      <c r="A1147" t="inlineStr">
+        <is>
+          <t>choice.wake.label.1</t>
+        </is>
+      </c>
+      <c r="B1147" t="inlineStr">
+        <is>
+          <t>Lie still.</t>
+        </is>
+      </c>
+      <c r="C1147" t="inlineStr">
+        <is>
+          <t>가만히 있는다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1148">
+      <c r="A1148" t="inlineStr">
+        <is>
+          <t>choice.wake.reply1.0</t>
+        </is>
+      </c>
+      <c r="B1148" t="inlineStr">
+        <is>
+          <t>You push up. The stone lets go of your back slowly.</t>
+        </is>
+      </c>
+      <c r="C1148" t="inlineStr">
+        <is>
+          <t>몸을 일으킨다. 돌바닥이 등을 천천히 놓아 준다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1149">
+      <c r="A1149" t="inlineStr">
+        <is>
+          <t>choice.wake.reply2.0</t>
+        </is>
+      </c>
+      <c r="B1149" t="inlineStr">
+        <is>
+          <t>You lie still. The ceiling says nothing. Neither do you.</t>
+        </is>
+      </c>
+      <c r="C1149" t="inlineStr">
+        <is>
+          <t>가만히 누워 있다. 천장은 말이 없다. 당신도 그렇다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1150">
+      <c r="A1150" t="inlineStr">
+        <is>
+          <t>choice.wake.again1.0</t>
+        </is>
+      </c>
+      <c r="B1150" t="inlineStr">
+        <is>
+          <t>Your body already knows how to get up.</t>
+        </is>
+      </c>
+      <c r="C1150" t="inlineStr">
+        <is>
+          <t>몸은 이미 일어나는 법을 안다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1151">
+      <c r="A1151" t="inlineStr">
+        <is>
+          <t>choice.wake.again2.0</t>
+        </is>
+      </c>
+      <c r="B1151" t="inlineStr">
+        <is>
+          <t>You lie still a while first. You always do now.</t>
+        </is>
+      </c>
+      <c r="C1151" t="inlineStr">
+        <is>
+          <t>먼저 한참 누워 있는다. 이제는 늘 그렇다.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C678"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix(combat): read-only menu in a fight, save the pre-fight snapshot on close, Guard counts enemy turns, Take Aim / Muscle Up last their stated turns, the Stranger keeps loot after an escape (hunt 6, R-138 to R-142)
Changed assertion: BattleUi 'Brace fades after one more turn when nothing hit' now reads 'Brace fades after two enemy turns when nothing hit'; one assertion added beside it.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datafiles/localization/game_text.xlsx
+++ b/datafiles/localization/game_text.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1111"/>
+  <dimension ref="A1:C1113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -19310,6 +19310,40 @@
         </is>
       </c>
     </row>
+    <row r="1112">
+      <c r="A1112" t="inlineStr">
+        <is>
+          <t>menu.msg.items_in_fight</t>
+        </is>
+      </c>
+      <c r="B1112" t="inlineStr">
+        <is>
+          <t>In a fight, use ITEM in the battle menu.</t>
+        </is>
+      </c>
+      <c r="C1112" t="inlineStr">
+        <is>
+          <t>전투 중에는 전투 메뉴의 아이템을 사용하세요.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1113">
+      <c r="A1113" t="inlineStr">
+        <is>
+          <t>menu.msg.gear_in_fight</t>
+        </is>
+      </c>
+      <c r="B1113" t="inlineStr">
+        <is>
+          <t>You can't change gear in a fight.</t>
+        </is>
+      </c>
+      <c r="C1113" t="inlineStr">
+        <is>
+          <t>전투 중에는 장비를 바꿀 수 없습니다.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C678"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(text): story-side text rewritten to the style guide - dialogue, cutscenes, wake/death lines, Stranger, merchant, choices, notes (D155)
114 rows: 59 existing rows reworded (intro/ending/closing, wake t1-t3,
5 death lines, hero dialogue, interactables, graves, one note line, one
Stranger reply) and 55 new dialogue.<id>.<n> rows (en + ko) for the 8
DialogueDB_Init entries that only existed as English fallbacks. GML
fallbacks changed in the same commit. g4 test/scenario expectations for
sys_class_chest_guard updated (lookup, not wording).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datafiles/localization/game_text.xlsx
+++ b/datafiles/localization/game_text.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1151"/>
+  <dimension ref="A1:C1206"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -1026,12 +1026,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>How was that even alive?! I nearly died.</t>
+          <t>That thing was alive. And I nearly wasn't.</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>저게 어떻게 살아 있지?! 죽을 뻔했어.</t>
+          <t>저 녀석, 살아 있었어. 난 하마터면 죽을 뻔했고.</t>
         </is>
       </c>
     </row>
@@ -1043,12 +1043,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>God, I just need to get out of here.</t>
+          <t>Okay. Okay. I just need to get out of here.</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>맙소사... 어서 여기서 나가야 해.</t>
+          <t>좋아. 좋아. 어서 여기서 나가야 해.</t>
         </is>
       </c>
     </row>
@@ -1519,12 +1519,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Thank the Almighty...</t>
+          <t>Air. Actual air...</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>신이시여, 감사합니다...</t>
+          <t>공기다. 진짜 공기...</t>
         </is>
       </c>
     </row>
@@ -1553,12 +1553,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>I need to find out where I am.</t>
+          <t>First, I need to know where I am.</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>여기가 어딘지 알아내야 해.</t>
+          <t>먼저 여기가 어딘지 알아야 해.</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1604,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Isn't this the raid party?</t>
+          <t>Is that... the raid party?</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -1638,12 +1638,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>... What on earth...</t>
+          <t>...What happened out here?</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>...대체 이게 무슨...</t>
+          <t>...여기서 무슨 일이 있었던 거지?</t>
         </is>
       </c>
     </row>
@@ -1706,12 +1706,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>I wasn't so lucky after all.</t>
+          <t>So much for lucky.</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>결국 나는 운이 좋았던 게 아니었어.</t>
+          <t>운이 좋았다니, 웃기네.</t>
         </is>
       </c>
     </row>
@@ -1757,12 +1757,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>We're glad you made it all the way to the end.</t>
+          <t>You made it to the end. We're glad.</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>끝까지 함께해 주셔서 정말 기쁩니다.</t>
+          <t>끝까지 와 주셔서 기쁩니다.</t>
         </is>
       </c>
     </row>
@@ -1774,12 +1774,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>We're looking to use what we learned from this game for our next title.</t>
+          <t>What we learned here goes into our next game.</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>우리는 이 게임에서 배운 점들을 다음 작품에 담아낼 계획입니다.</t>
+          <t>이번에 배운 것은 다음 작품에 담겠습니다.</t>
         </is>
       </c>
     </row>
@@ -1791,12 +1791,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Please support our next development :)</t>
+          <t>Please support our next game.</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>다음 작품도 응원해 주세요 :)</t>
+          <t>다음 작품도 응원해 주세요.</t>
         </is>
       </c>
     </row>
@@ -1859,12 +1859,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>This is not a world of fantasy, magic, and dragons.</t>
+          <t>This is not a world of magic and dragons.</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>이곳은 환상과 마법, 용의 세계가 아니다.</t>
+          <t>이곳은 마법과 용의 세계가 아니다.</t>
         </is>
       </c>
     </row>
@@ -1893,12 +1893,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>It was worth it...</t>
+          <t>It seemed worth it...</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>그만한 가치는 있었다...</t>
+          <t>그만한 가치가 있어 보였다...</t>
         </is>
       </c>
     </row>
@@ -1944,12 +1944,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>This is a world of gritty medieval kingdoms and warring countries.</t>
+          <t>This is a world of mud, borders and kings.</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>이곳은 거칠고 투박한 중세 왕국과 전쟁 중인 나라들의 세계다.</t>
+          <t>이곳은 진흙과 국경, 그리고 왕들의 세계다.</t>
         </is>
       </c>
     </row>
@@ -2029,12 +2029,12 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>There were rumors of conscription for the war between two kingdoms.</t>
+          <t>Word came that the crown was drafting men for the war.</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>두 왕국의 전쟁을 위해 징집이 있을 거라는 소문이 돌았다.</t>
+          <t>전쟁에 나갈 사람들을 징집한다는 소문이 돌았다.</t>
         </is>
       </c>
     </row>
@@ -2046,12 +2046,12 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>The reward was enough to set you up for a year...</t>
+          <t>The pay would feed you for a year...</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>보수는 1년을 먹고살기에 충분했다...</t>
+          <t>보수면 1년은 먹고살 수 있었다...</t>
         </is>
       </c>
     </row>
@@ -2063,7 +2063,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>The plan was to ambush the enemy using a shortcut.</t>
+          <t>The plan was to ambush the enemy by a shortcut.</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -2080,12 +2080,12 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Good thing you grew up here and knew the forest.</t>
+          <t>You grew up in these woods. You knew every path.</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>이곳에서 자라 숲을 잘 아는 게 다행이었다.</t>
+          <t>당신은 이 숲에서 자랐다. 길이란 길은 다 알았다.</t>
         </is>
       </c>
     </row>
@@ -2097,12 +2097,12 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>You knew it was a mistake. You could feel it.</t>
+          <t>Your stomach knew it was a mistake.</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>잘못된 일이라는 걸 알았다. 느낄 수 있었다.</t>
+          <t>배 속이 먼저 알았다. 이건 잘못이라고.</t>
         </is>
       </c>
     </row>
@@ -2131,12 +2131,12 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>You hear cracking...</t>
+          <t>Stone cracks somewhere overhead...</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>갈라지는 소리가 들린다...</t>
+          <t>머리 위 어딘가에서 돌이 갈라진다...</t>
         </is>
       </c>
     </row>
@@ -2148,12 +2148,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Small tremors...</t>
+          <t>Dust sifts onto your shoulders...</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>작은 떨림...</t>
+          <t>어깨 위로 먼지가 내려앉는다...</t>
         </is>
       </c>
     </row>
@@ -2182,12 +2182,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>You'd never heard of such a tunnel in all your life.</t>
+          <t>You had never heard of a tunnel there. Not once.</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>평생 그런 터널은 들어 본 적이 없었다.</t>
+          <t>그곳에 터널이 있다는 말은 들어 본 적이 없었다. 한 번도.</t>
         </is>
       </c>
     </row>
@@ -2199,12 +2199,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>You couldn't help thinking it was a joke...</t>
+          <t>You took it for a joke...</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>농담이라고 생각할 수밖에 없었다...</t>
+          <t>농담인 줄 알았다...</t>
         </is>
       </c>
     </row>
@@ -2233,12 +2233,12 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>There really was a tunnel. You could hardly believe it.</t>
+          <t>The tunnel was real. None of your maps had room for it.</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>터널은 정말로 있었다. 믿기 어려웠다.</t>
+          <t>터널은 진짜였다. 당신의 어떤 지도에도 들어갈 자리가 없었다.</t>
         </is>
       </c>
     </row>
@@ -2250,12 +2250,12 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>The group ventured deep into the tunnel, heading toward the enemy castle...</t>
+          <t>The raid party went in, toward the enemy castle...</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>일행은 적의 성을 향해 터널 깊숙이 들어갔다...</t>
+          <t>토벌대는 적의 성을 향해 터널 안으로 들어갔다...</t>
         </is>
       </c>
     </row>
@@ -2267,12 +2267,12 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>You were just the navigator for this raid party.</t>
+          <t>You were only the navigator.</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>당신은 이 토벌대의 길잡이일 뿐이었다.</t>
+          <t>당신은 길잡이일 뿐이었다.</t>
         </is>
       </c>
     </row>
@@ -2284,12 +2284,12 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>And this place never existed before...</t>
+          <t>The day before, there was only hillside.</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>그리고 이곳은 전에는 없던 곳이었다...</t>
+          <t>전날까지만 해도 그곳엔 산비탈뿐이었다.</t>
         </is>
       </c>
     </row>
@@ -2369,12 +2369,12 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Like it was waiting here.</t>
+          <t>Like it was waiting for a hand like mine.</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>마치 여기서 기다리고 있었던 것처럼.</t>
+          <t>나 같은 손을 기다리고 있었던 것처럼.</t>
         </is>
       </c>
     </row>
@@ -2420,12 +2420,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>This chest shouldn't know me.</t>
+          <t>How does a chest know my size?</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>이 상자가 나를 알 리 없는데.</t>
+          <t>상자가 내 몸 치수를 어떻게 알지?</t>
         </is>
       </c>
     </row>
@@ -2590,12 +2590,12 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Somehow... my hands already know.</t>
+          <t>My hands already know it.</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>어쩐지... 손이 이미 알고 있어.</t>
+          <t>손이 이미 알고 있어.</t>
         </is>
       </c>
     </row>
@@ -2624,12 +2624,12 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>...The page is filled with symbols.</t>
+          <t>...Just symbols, page after page.</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>...페이지가 온통 기호투성이야.</t>
+          <t>...페이지마다 기호뿐이야.</t>
         </is>
       </c>
     </row>
@@ -2658,12 +2658,12 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>And I understand. It shows me where to place my hands.</t>
+          <t>Then I understand. It shows me where to put my hands.</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>그러자 이해가 된다. 손을 어디에 둬야 하는지 알려 준다.</t>
+          <t>그러자 이해가 돼. 손을 어디에 둬야 하는지 알려 줘.</t>
         </is>
       </c>
     </row>
@@ -2692,12 +2692,12 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>It's broken.</t>
+          <t>Splinters and a rusted hoop.</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>이미 부서졌다.</t>
+          <t>나뭇조각과 녹슨 쇠테.</t>
         </is>
       </c>
     </row>
@@ -2709,12 +2709,12 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>A pile of old bones.</t>
+          <t>A pile of bones. Old, and picked clean.</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>오래된 뼈 무더기.</t>
+          <t>오래된 뼈 무더기. 살점 하나 남지 않았다.</t>
         </is>
       </c>
     </row>
@@ -2811,12 +2811,12 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>How can such creatures exist?</t>
+          <t>I grew up in these hills. None of that lived here.</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>이런 생물이 어떻게 존재하지?</t>
+          <t>난 이 산골에서 자랐어. 저런 건 없었다고.</t>
         </is>
       </c>
     </row>
@@ -2828,12 +2828,12 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Some sort of mutated animals...</t>
+          <t>Sick animals, maybe. Something in the water...</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>돌연변이 짐승 같은 건가...</t>
+          <t>병든 짐승일지도. 물 때문인가...</t>
         </is>
       </c>
     </row>
@@ -2862,12 +2862,12 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>You extinguish the flame.</t>
+          <t>You put out the flame. The dark leans in.</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>불을 껐다.</t>
+          <t>불을 껐다. 어둠이 가까이 다가온다.</t>
         </is>
       </c>
     </row>
@@ -2879,12 +2879,12 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>The flame is out.</t>
+          <t>Only cold ash is left.</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>불이 꺼져 있다.</t>
+          <t>식은 재만 남아 있다.</t>
         </is>
       </c>
     </row>
@@ -3032,12 +3032,12 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Just what I need to get out of this place.</t>
+          <t>Something in there might get me out of here.</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>여기서 나가려면 꼭 필요한 것이다.</t>
+          <t>저 안에 여기서 나갈 방법이 있을지도 몰라.</t>
         </is>
       </c>
     </row>
@@ -3066,12 +3066,12 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Wha... What just happened?</t>
+          <t>Ugh... What just happened?</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>뭐... 방금 무슨 일이 일어난 거야?</t>
+          <t>으윽... 방금 무슨 일이야?</t>
         </is>
       </c>
     </row>
@@ -3117,12 +3117,12 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>I knew it. There's something wrong about this place.</t>
+          <t>I knew it. This tunnel was never right.</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>역시 그랬어. 이곳은 뭔가 이상해.</t>
+          <t>역시. 이 터널은 처음부터 이상했어.</t>
         </is>
       </c>
     </row>
@@ -3134,12 +3134,12 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>I need to get back.</t>
+          <t>I have to get back up.</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>돌아가야 해.</t>
+          <t>위로 돌아가야 해.</t>
         </is>
       </c>
     </row>
@@ -3219,12 +3219,12 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>You extinguish the torch.</t>
+          <t>You put out the torch. The corner goes black.</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>횃불을 껐다.</t>
+          <t>횃불을 껐다. 한쪽 구석이 까맣게 잠긴다.</t>
         </is>
       </c>
     </row>
@@ -3253,12 +3253,12 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>A sturdy tree.</t>
+          <t>A tree, growing where none should.</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>튼튼한 나무.</t>
+          <t>있을 리 없는 곳에 나무가 자라고 있다.</t>
         </is>
       </c>
     </row>
@@ -3270,12 +3270,12 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>A cut tree stump.</t>
+          <t>A stump, cut clean with a saw.</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>베어 낸 나무 그루터기.</t>
+          <t>톱으로 깨끗이 베어 낸 그루터기.</t>
         </is>
       </c>
     </row>
@@ -3542,12 +3542,12 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>You brush away dust from a weathered grave.</t>
+          <t>You brush the dust from the stone. No name under it.</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>비바람에 깎인 무덤의 먼지를 털어 낸다.</t>
+          <t>돌의 먼지를 털어 낸다. 그 밑에도 이름은 없다.</t>
         </is>
       </c>
     </row>
@@ -3593,12 +3593,12 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>The earth around this grave feels recently disturbed.</t>
+          <t>The earth is loose, as if turned this morning.</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>이 무덤 주위의 흙은 최근에 파헤쳐진 듯하다.</t>
+          <t>흙이 푹신하다. 오늘 아침에 파헤친 것처럼.</t>
         </is>
       </c>
     </row>
@@ -3627,12 +3627,12 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>This grave has been here for a long, long time.</t>
+          <t>Older than the tunnel, by the look of it.</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>이 무덤은 아주 오래전부터 여기 있었다.</t>
+          <t>생김새로 보아 터널보다 오래된 무덤이다.</t>
         </is>
       </c>
     </row>
@@ -11243,12 +11243,12 @@
       </c>
       <c r="B637" t="inlineStr">
         <is>
-          <t>So this is how it ends.</t>
+          <t>Is this it? It is so quiet.</t>
         </is>
       </c>
       <c r="C637" t="inlineStr">
         <is>
-          <t>결국 이렇게 끝나는구나.</t>
+          <t>이게 끝인가? 너무 조용하다.</t>
         </is>
       </c>
     </row>
@@ -11260,12 +11260,12 @@
       </c>
       <c r="B638" t="inlineStr">
         <is>
-          <t>The floor gives way beneath you.</t>
+          <t>Your own breath is the last thing you hear.</t>
         </is>
       </c>
       <c r="C638" t="inlineStr">
         <is>
-          <t>발밑의 바닥이 꺼진다.</t>
+          <t>마지막으로 들리는 건 자기 숨소리다.</t>
         </is>
       </c>
     </row>
@@ -11277,12 +11277,12 @@
       </c>
       <c r="B639" t="inlineStr">
         <is>
-          <t>You were sure that was the end.</t>
+          <t>You were sure that was it. You were wrong.</t>
         </is>
       </c>
       <c r="C639" t="inlineStr">
         <is>
-          <t>분명 이게 끝이라고 생각했다.</t>
+          <t>이게 끝이라고 확신했다. 틀렸다.</t>
         </is>
       </c>
     </row>
@@ -11362,12 +11362,12 @@
       </c>
       <c r="B644" t="inlineStr">
         <is>
-          <t>Dying is starting to feel like routine.</t>
+          <t>You know the ceiling before you open your eyes.</t>
         </is>
       </c>
       <c r="C644" t="inlineStr">
         <is>
-          <t>죽는 일이 일상처럼 느껴지기 시작한다.</t>
+          <t>눈을 뜨기도 전에 천장이 어떤지 안다.</t>
         </is>
       </c>
     </row>
@@ -11396,12 +11396,12 @@
       </c>
       <c r="B646" t="inlineStr">
         <is>
-          <t>{killer}. You don't even flinch anymore.</t>
+          <t>{killer}. Your hands don't even shake.</t>
         </is>
       </c>
       <c r="C646" t="inlineStr">
         <is>
-          <t>{killer}. 이제 놀라지도 않는다.</t>
+          <t>{killer}. 이제 손도 떨리지 않는다.</t>
         </is>
       </c>
     </row>
@@ -11736,12 +11736,12 @@
       </c>
       <c r="B666" t="inlineStr">
         <is>
-          <t>You wake where you first fell. Alive.</t>
+          <t>Cold stone under your cheek. You are where you fell. Alive, at least.</t>
         </is>
       </c>
       <c r="C666" t="inlineStr">
         <is>
-          <t>처음 떨어진 곳에서 눈을 뜬다. 살아 있다.</t>
+          <t>뺨에 차가운 돌이 닿는다. 떨어진 그 자리다. 적어도 살아 있다.</t>
         </is>
       </c>
     </row>
@@ -11753,12 +11753,12 @@
       </c>
       <c r="B667" t="inlineStr">
         <is>
-          <t>The same stone. The same cold. You wake again.</t>
+          <t>The same stone, the same cold. You almost expected it.</t>
         </is>
       </c>
       <c r="C667" t="inlineStr">
         <is>
-          <t>같은 돌바닥. 같은 냉기. 다시 눈을 뜬다.</t>
+          <t>같은 돌바닥, 같은 냉기. 어쩐지 예상했던 일이다.</t>
         </is>
       </c>
     </row>
@@ -11770,12 +11770,12 @@
       </c>
       <c r="B668" t="inlineStr">
         <is>
-          <t>You wake at the entrance. It almost feels like home.</t>
+          <t>The stone is almost warm now. It feels a little like home.</t>
         </is>
       </c>
       <c r="C668" t="inlineStr">
         <is>
-          <t>입구에서 눈을 뜬다. 어쩐지 집처럼 느껴진다.</t>
+          <t>돌바닥이 이제 거의 따뜻하다. 어쩐지 집 같다.</t>
         </is>
       </c>
     </row>
@@ -12195,12 +12195,12 @@
       </c>
       <c r="B693" t="inlineStr">
         <is>
-          <t>You made these. You don't remember making them.</t>
+          <t>Your thumb fits the groove exactly.</t>
         </is>
       </c>
       <c r="C693" t="inlineStr">
         <is>
-          <t>당신이 새긴 것이다. 새긴 기억은 없다.</t>
+          <t>당신의 엄지가 홈에 꼭 맞는다.</t>
         </is>
       </c>
     </row>
@@ -17805,12 +17805,12 @@
       </c>
       <c r="B1023" t="inlineStr">
         <is>
-          <t>Wait, there was a chest back there. I think I should open it...</t>
+          <t>Wait. There was a chest back there.</t>
         </is>
       </c>
       <c r="C1023" t="inlineStr">
         <is>
-          <t>잠깐, 저 뒤에 상자가 있었어. 열어 봐야겠어...</t>
+          <t>잠깐. 저 뒤에 상자가 있었어.</t>
         </is>
       </c>
     </row>
@@ -17822,12 +17822,12 @@
       </c>
       <c r="B1024" t="inlineStr">
         <is>
-          <t>...there might be something I can use to protect myself.</t>
+          <t>...Something in it might keep me alive.</t>
         </is>
       </c>
       <c r="C1024" t="inlineStr">
         <is>
-          <t>...나를 지킬 만한 뭔가가 들어 있을지도 몰라.</t>
+          <t>...안에 살아남는 데 쓸 만한 게 있을지도 몰라.</t>
         </is>
       </c>
     </row>
@@ -19403,12 +19403,12 @@
       </c>
       <c r="B1117" t="inlineStr">
         <is>
-          <t>Ask again when the tunnel has had you a few more times.</t>
+          <t>Ask again when the tunnel has had you a bit longer.</t>
         </is>
       </c>
       <c r="C1117" t="inlineStr">
         <is>
-          <t>터널이 널 몇 번 더 삼키면 다시 물어봐.</t>
+          <t>터널이 널 좀 더 삼키면 다시 물어봐.</t>
         </is>
       </c>
     </row>
@@ -19987,6 +19987,941 @@
       <c r="C1151" t="inlineStr">
         <is>
           <t>먼저 한참 누워 있는다. 이제는 늘 그렇다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1152">
+      <c r="A1152" t="inlineStr">
+        <is>
+          <t>dialogue.first_encounter_mini_boss.0</t>
+        </is>
+      </c>
+      <c r="B1152" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="C1152" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+    </row>
+    <row r="1153">
+      <c r="A1153" t="inlineStr">
+        <is>
+          <t>dialogue.first_encounter_mini_boss.1</t>
+        </is>
+      </c>
+      <c r="B1153" t="inlineStr">
+        <is>
+          <t>Oh, what the hell is that?</t>
+        </is>
+      </c>
+      <c r="C1153" t="inlineStr">
+        <is>
+          <t>아니, 저게 대체 뭐야?</t>
+        </is>
+      </c>
+    </row>
+    <row r="1154">
+      <c r="A1154" t="inlineStr">
+        <is>
+          <t>dialogue.first_encounter_mini_boss.2</t>
+        </is>
+      </c>
+      <c r="B1154" t="inlineStr">
+        <is>
+          <t>Half cow, half man?</t>
+        </is>
+      </c>
+      <c r="C1154" t="inlineStr">
+        <is>
+          <t>반은 소, 반은 사람?</t>
+        </is>
+      </c>
+    </row>
+    <row r="1155">
+      <c r="A1155" t="inlineStr">
+        <is>
+          <t>dialogue.first_encounter_mini_boss.3</t>
+        </is>
+      </c>
+      <c r="B1155" t="inlineStr">
+        <is>
+          <t>That breathing. Those horns...</t>
+        </is>
+      </c>
+      <c r="C1155" t="inlineStr">
+        <is>
+          <t>저 숨소리. 저 뿔...</t>
+        </is>
+      </c>
+    </row>
+    <row r="1156">
+      <c r="A1156" t="inlineStr">
+        <is>
+          <t>dialogue.first_encounter_mini_boss.4</t>
+        </is>
+      </c>
+      <c r="B1156" t="inlineStr">
+        <is>
+          <t>And he's blocking the only way forward.</t>
+        </is>
+      </c>
+      <c r="C1156" t="inlineStr">
+        <is>
+          <t>하필 하나뿐인 길을 막고 서 있어.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1157">
+      <c r="A1157" t="inlineStr">
+        <is>
+          <t>dialogue.first_encounter_mini_boss.5</t>
+        </is>
+      </c>
+      <c r="B1157" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="C1157" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+    </row>
+    <row r="1158">
+      <c r="A1158" t="inlineStr">
+        <is>
+          <t>dialogue.first_encounter_mini_boss.6</t>
+        </is>
+      </c>
+      <c r="B1158" t="inlineStr">
+        <is>
+          <t>Fuck.</t>
+        </is>
+      </c>
+      <c r="C1158" t="inlineStr">
+        <is>
+          <t>젠장.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1159">
+      <c r="A1159" t="inlineStr">
+        <is>
+          <t>dialogue.first_encounter_final_boss.0</t>
+        </is>
+      </c>
+      <c r="B1159" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="C1159" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+    </row>
+    <row r="1160">
+      <c r="A1160" t="inlineStr">
+        <is>
+          <t>dialogue.first_encounter_final_boss.1</t>
+        </is>
+      </c>
+      <c r="B1160" t="inlineStr">
+        <is>
+          <t>Another demon.</t>
+        </is>
+      </c>
+      <c r="C1160" t="inlineStr">
+        <is>
+          <t>또 악마인가.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1161">
+      <c r="A1161" t="inlineStr">
+        <is>
+          <t>dialogue.first_encounter_final_boss.2</t>
+        </is>
+      </c>
+      <c r="B1161" t="inlineStr">
+        <is>
+          <t>This one is different.</t>
+        </is>
+      </c>
+      <c r="C1161" t="inlineStr">
+        <is>
+          <t>이번 놈은 달라.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1162">
+      <c r="A1162" t="inlineStr">
+        <is>
+          <t>dialogue.first_encounter_final_boss.3</t>
+        </is>
+      </c>
+      <c r="B1162" t="inlineStr">
+        <is>
+          <t>As if it's looking for something...</t>
+        </is>
+      </c>
+      <c r="C1162" t="inlineStr">
+        <is>
+          <t>무언가를 찾는 것 같아...</t>
+        </is>
+      </c>
+    </row>
+    <row r="1163">
+      <c r="A1163" t="inlineStr">
+        <is>
+          <t>dialogue.first_encounter_final_boss.4</t>
+        </is>
+      </c>
+      <c r="B1163" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="C1163" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+    </row>
+    <row r="1164">
+      <c r="A1164" t="inlineStr">
+        <is>
+          <t>dialogue.first_encounter_final_boss.5</t>
+        </is>
+      </c>
+      <c r="B1164" t="inlineStr">
+        <is>
+          <t>...someone.</t>
+        </is>
+      </c>
+      <c r="C1164" t="inlineStr">
+        <is>
+          <t>...누군가를.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1165">
+      <c r="A1165" t="inlineStr">
+        <is>
+          <t>dialogue.sys_floor2_dire_wolf_reaction.0</t>
+        </is>
+      </c>
+      <c r="B1165" t="inlineStr">
+        <is>
+          <t>*Pant*... Whew.</t>
+        </is>
+      </c>
+      <c r="C1165" t="inlineStr">
+        <is>
+          <t>*헉*... 휴.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1166">
+      <c r="A1166" t="inlineStr">
+        <is>
+          <t>dialogue.sys_floor2_dire_wolf_reaction.1</t>
+        </is>
+      </c>
+      <c r="B1166" t="inlineStr">
+        <is>
+          <t>A wolf now? Seriously?</t>
+        </is>
+      </c>
+      <c r="C1166" t="inlineStr">
+        <is>
+          <t>이번엔 늑대라고? 진짜로?</t>
+        </is>
+      </c>
+    </row>
+    <row r="1167">
+      <c r="A1167" t="inlineStr">
+        <is>
+          <t>dialogue.sys_floor2_dire_wolf_reaction.2</t>
+        </is>
+      </c>
+      <c r="B1167" t="inlineStr">
+        <is>
+          <t>Where do these things come from?</t>
+        </is>
+      </c>
+      <c r="C1167" t="inlineStr">
+        <is>
+          <t>이것들은 다 어디서 나오는 거야?</t>
+        </is>
+      </c>
+    </row>
+    <row r="1168">
+      <c r="A1168" t="inlineStr">
+        <is>
+          <t>dialogue.sys_floor2_dire_wolf_reaction.3</t>
+        </is>
+      </c>
+      <c r="B1168" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="C1168" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+    </row>
+    <row r="1169">
+      <c r="A1169" t="inlineStr">
+        <is>
+          <t>dialogue.sys_floor2_dire_wolf_reaction.4</t>
+        </is>
+      </c>
+      <c r="B1169" t="inlineStr">
+        <is>
+          <t>Standing here won't answer that.</t>
+        </is>
+      </c>
+      <c r="C1169" t="inlineStr">
+        <is>
+          <t>여기 서 있어도 답은 안 나와.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1170">
+      <c r="A1170" t="inlineStr">
+        <is>
+          <t>dialogue.sys_floor2_dire_wolf_reaction.5</t>
+        </is>
+      </c>
+      <c r="B1170" t="inlineStr">
+        <is>
+          <t>Keep moving.</t>
+        </is>
+      </c>
+      <c r="C1170" t="inlineStr">
+        <is>
+          <t>계속 가자.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1171">
+      <c r="A1171" t="inlineStr">
+        <is>
+          <t>dialogue.sys_first_stranger_encounter_reaction.0</t>
+        </is>
+      </c>
+      <c r="B1171" t="inlineStr">
+        <is>
+          <t>Get your hands off me...</t>
+        </is>
+      </c>
+      <c r="C1171" t="inlineStr">
+        <is>
+          <t>손 치워...</t>
+        </is>
+      </c>
+    </row>
+    <row r="1172">
+      <c r="A1172" t="inlineStr">
+        <is>
+          <t>dialogue.sys_first_stranger_encounter_reaction.1</t>
+        </is>
+      </c>
+      <c r="B1172" t="inlineStr">
+        <is>
+          <t>He smiled the whole time.</t>
+        </is>
+      </c>
+      <c r="C1172" t="inlineStr">
+        <is>
+          <t>그 녀석, 내내 웃고 있었어.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1173">
+      <c r="A1173" t="inlineStr">
+        <is>
+          <t>dialogue.sys_first_stranger_encounter_reaction.2</t>
+        </is>
+      </c>
+      <c r="B1173" t="inlineStr">
+        <is>
+          <t>Are they all demons down here?</t>
+        </is>
+      </c>
+      <c r="C1173" t="inlineStr">
+        <is>
+          <t>여기 있는 건 전부 악마야?</t>
+        </is>
+      </c>
+    </row>
+    <row r="1174">
+      <c r="A1174" t="inlineStr">
+        <is>
+          <t>dialogue.sys_first_stranger_encounter_reaction.3</t>
+        </is>
+      </c>
+      <c r="B1174" t="inlineStr">
+        <is>
+          <t>What else would they be.</t>
+        </is>
+      </c>
+      <c r="C1174" t="inlineStr">
+        <is>
+          <t>달리 뭐겠어.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1175">
+      <c r="A1175" t="inlineStr">
+        <is>
+          <t>dialogue.sys_first_stranger_encounter_reaction.4</t>
+        </is>
+      </c>
+      <c r="B1175" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="C1175" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+    </row>
+    <row r="1176">
+      <c r="A1176" t="inlineStr">
+        <is>
+          <t>dialogue.sys_first_stranger_encounter_reaction.5</t>
+        </is>
+      </c>
+      <c r="B1176" t="inlineStr">
+        <is>
+          <t>I have to keep moving.</t>
+        </is>
+      </c>
+      <c r="C1176" t="inlineStr">
+        <is>
+          <t>계속 움직여야 해.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1177">
+      <c r="A1177" t="inlineStr">
+        <is>
+          <t>dialogue.sys_first_level_up_reaction.0</t>
+        </is>
+      </c>
+      <c r="B1177" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="C1177" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+    </row>
+    <row r="1178">
+      <c r="A1178" t="inlineStr">
+        <is>
+          <t>dialogue.sys_first_level_up_reaction.1</t>
+        </is>
+      </c>
+      <c r="B1178" t="inlineStr">
+        <is>
+          <t>The walls tilt. Easy... easy.</t>
+        </is>
+      </c>
+      <c r="C1178" t="inlineStr">
+        <is>
+          <t>벽이 기운다. 진정해... 진정해.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1179">
+      <c r="A1179" t="inlineStr">
+        <is>
+          <t>dialogue.sys_first_level_up_reaction.2</t>
+        </is>
+      </c>
+      <c r="B1179" t="inlineStr">
+        <is>
+          <t>I think I'm going to be sick...</t>
+        </is>
+      </c>
+      <c r="C1179" t="inlineStr">
+        <is>
+          <t>토할 것 같아...</t>
+        </is>
+      </c>
+    </row>
+    <row r="1180">
+      <c r="A1180" t="inlineStr">
+        <is>
+          <t>dialogue.sys_first_level_up_reaction.3</t>
+        </is>
+      </c>
+      <c r="B1180" t="inlineStr">
+        <is>
+          <t>Why does it feel like I've been training for years?</t>
+        </is>
+      </c>
+      <c r="C1180" t="inlineStr">
+        <is>
+          <t>왜 몇 년 동안 훈련한 것처럼 몸이 쑤시지?</t>
+        </is>
+      </c>
+    </row>
+    <row r="1181">
+      <c r="A1181" t="inlineStr">
+        <is>
+          <t>dialogue.sys_first_level_up_reaction.4</t>
+        </is>
+      </c>
+      <c r="B1181" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="C1181" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+    </row>
+    <row r="1182">
+      <c r="A1182" t="inlineStr">
+        <is>
+          <t>dialogue.sys_first_level_up_reaction.5</t>
+        </is>
+      </c>
+      <c r="B1182" t="inlineStr">
+        <is>
+          <t>...and different.</t>
+        </is>
+      </c>
+      <c r="C1182" t="inlineStr">
+        <is>
+          <t>...그리고 달라졌어.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1183">
+      <c r="A1183" t="inlineStr">
+        <is>
+          <t>dialogue.sys_first_equippable_item_reaction.0</t>
+        </is>
+      </c>
+      <c r="B1183" t="inlineStr">
+        <is>
+          <t>This might come in handy.</t>
+        </is>
+      </c>
+      <c r="C1183" t="inlineStr">
+        <is>
+          <t>쓸모가 있겠는걸.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1184">
+      <c r="A1184" t="inlineStr">
+        <is>
+          <t>dialogue.sys_first_equippable_item_reaction.1</t>
+        </is>
+      </c>
+      <c r="B1184" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="C1184" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+    </row>
+    <row r="1185">
+      <c r="A1185" t="inlineStr">
+        <is>
+          <t>dialogue.sys_first_equippable_item_reaction.2</t>
+        </is>
+      </c>
+      <c r="B1185" t="inlineStr">
+        <is>
+          <t>Chests every few steps.</t>
+        </is>
+      </c>
+      <c r="C1185" t="inlineStr">
+        <is>
+          <t>몇 걸음마다 상자가 있어.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1186">
+      <c r="A1186" t="inlineStr">
+        <is>
+          <t>dialogue.sys_first_equippable_item_reaction.3</t>
+        </is>
+      </c>
+      <c r="B1186" t="inlineStr">
+        <is>
+          <t>Gear that fits like it was made for me.</t>
+        </is>
+      </c>
+      <c r="C1186" t="inlineStr">
+        <is>
+          <t>내 몸에 맞춘 듯한 장비들.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1187">
+      <c r="A1187" t="inlineStr">
+        <is>
+          <t>dialogue.sys_first_equippable_item_reaction.4</t>
+        </is>
+      </c>
+      <c r="B1187" t="inlineStr">
+        <is>
+          <t>Somebody wants me armed.</t>
+        </is>
+      </c>
+      <c r="C1187" t="inlineStr">
+        <is>
+          <t>누군가 내가 무장하길 바라는 거야.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1188">
+      <c r="A1188" t="inlineStr">
+        <is>
+          <t>dialogue.sys_first_equippable_item_reaction.5</t>
+        </is>
+      </c>
+      <c r="B1188" t="inlineStr">
+        <is>
+          <t>But why arm us, if they wanted us dead?</t>
+        </is>
+      </c>
+      <c r="C1188" t="inlineStr">
+        <is>
+          <t>우리를 죽일 셈이면 왜 무기를 쥐여 주지?</t>
+        </is>
+      </c>
+    </row>
+    <row r="1189">
+      <c r="A1189" t="inlineStr">
+        <is>
+          <t>dialogue.sys_final_boss_defeated_reaction.0</t>
+        </is>
+      </c>
+      <c r="B1189" t="inlineStr">
+        <is>
+          <t>*Huff*... *Wheeze*... Fuck.</t>
+        </is>
+      </c>
+      <c r="C1189" t="inlineStr">
+        <is>
+          <t>*헉*... *쌕*... 젠장.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1190">
+      <c r="A1190" t="inlineStr">
+        <is>
+          <t>dialogue.sys_final_boss_defeated_reaction.1</t>
+        </is>
+      </c>
+      <c r="B1190" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="C1190" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+    </row>
+    <row r="1191">
+      <c r="A1191" t="inlineStr">
+        <is>
+          <t>dialogue.sys_final_boss_defeated_reaction.2</t>
+        </is>
+      </c>
+      <c r="B1191" t="inlineStr">
+        <is>
+          <t>I did it. I actually did it.</t>
+        </is>
+      </c>
+      <c r="C1191" t="inlineStr">
+        <is>
+          <t>해냈어. 정말 해냈어.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1192">
+      <c r="A1192" t="inlineStr">
+        <is>
+          <t>dialogue.sys_final_boss_defeated_reaction.3</t>
+        </is>
+      </c>
+      <c r="B1192" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="C1192" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+    </row>
+    <row r="1193">
+      <c r="A1193" t="inlineStr">
+        <is>
+          <t>dialogue.sys_final_boss_defeated_reaction.4</t>
+        </is>
+      </c>
+      <c r="B1193" t="inlineStr">
+        <is>
+          <t>Still...</t>
+        </is>
+      </c>
+      <c r="C1193" t="inlineStr">
+        <is>
+          <t>그런데...</t>
+        </is>
+      </c>
+    </row>
+    <row r="1194">
+      <c r="A1194" t="inlineStr">
+        <is>
+          <t>dialogue.sys_final_boss_defeated_reaction.5</t>
+        </is>
+      </c>
+      <c r="B1194" t="inlineStr">
+        <is>
+          <t>Nothing here makes sense.</t>
+        </is>
+      </c>
+      <c r="C1194" t="inlineStr">
+        <is>
+          <t>여긴 아무것도 말이 안 돼.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1195">
+      <c r="A1195" t="inlineStr">
+        <is>
+          <t>dialogue.sys_final_boss_defeated_reaction.6</t>
+        </is>
+      </c>
+      <c r="B1195" t="inlineStr">
+        <is>
+          <t>Am I the only one seeing this?</t>
+        </is>
+      </c>
+      <c r="C1195" t="inlineStr">
+        <is>
+          <t>이걸 보는 게 나뿐인가?</t>
+        </is>
+      </c>
+    </row>
+    <row r="1196">
+      <c r="A1196" t="inlineStr">
+        <is>
+          <t>dialogue.sys_final_boss_defeated_reaction.7</t>
+        </is>
+      </c>
+      <c r="B1196" t="inlineStr">
+        <is>
+          <t>Who cares. The exit is right there.</t>
+        </is>
+      </c>
+      <c r="C1196" t="inlineStr">
+        <is>
+          <t>아무렴 어때. 출구가 바로 저기야.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1197">
+      <c r="A1197" t="inlineStr">
+        <is>
+          <t>dialogue.sys_final_boss_defeated_reaction.8</t>
+        </is>
+      </c>
+      <c r="B1197" t="inlineStr">
+        <is>
+          <t>Time to find the others, and a way home.</t>
+        </is>
+      </c>
+      <c r="C1197" t="inlineStr">
+        <is>
+          <t>동료들을 찾아서 집으로 가는 길을 찾자.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1198">
+      <c r="A1198" t="inlineStr">
+        <is>
+          <t>dialogue.sys_floor9_5_exit_reaction.0</t>
+        </is>
+      </c>
+      <c r="B1198" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="C1198" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+    </row>
+    <row r="1199">
+      <c r="A1199" t="inlineStr">
+        <is>
+          <t>dialogue.sys_floor9_5_exit_reaction.1</t>
+        </is>
+      </c>
+      <c r="B1199" t="inlineStr">
+        <is>
+          <t>(Colors flood in, far too bright.)</t>
+        </is>
+      </c>
+      <c r="C1199" t="inlineStr">
+        <is>
+          <t>(색이 쏟아져 들어온다. 너무 밝다.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1200">
+      <c r="A1200" t="inlineStr">
+        <is>
+          <t>dialogue.sys_floor9_5_exit_reaction.2</t>
+        </is>
+      </c>
+      <c r="B1200" t="inlineStr">
+        <is>
+          <t>(Black threads curl through your sight, then vanish.)</t>
+        </is>
+      </c>
+      <c r="C1200" t="inlineStr">
+        <is>
+          <t>(검은 실 같은 것이 시야를 휘감았다가 사라진다.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1201">
+      <c r="A1201" t="inlineStr">
+        <is>
+          <t>dialogue.sys_floor9_5_exit_reaction.3</t>
+        </is>
+      </c>
+      <c r="B1201" t="inlineStr">
+        <is>
+          <t>(The tunnel snaps back around you.)</t>
+        </is>
+      </c>
+      <c r="C1201" t="inlineStr">
+        <is>
+          <t>(터널이 다시 당신을 에워싼다.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1202">
+      <c r="A1202" t="inlineStr">
+        <is>
+          <t>dialogue.sys_floor9_5_exit_reaction.4</t>
+        </is>
+      </c>
+      <c r="B1202" t="inlineStr">
+        <is>
+          <t>Huh?</t>
+        </is>
+      </c>
+      <c r="C1202" t="inlineStr">
+        <is>
+          <t>응?</t>
+        </is>
+      </c>
+    </row>
+    <row r="1203">
+      <c r="A1203" t="inlineStr">
+        <is>
+          <t>dialogue.sys_floor9_5_exit_reaction.5</t>
+        </is>
+      </c>
+      <c r="B1203" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="C1203" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+    </row>
+    <row r="1204">
+      <c r="A1204" t="inlineStr">
+        <is>
+          <t>dialogue.sys_floor9_5_exit_reaction.6</t>
+        </is>
+      </c>
+      <c r="B1204" t="inlineStr">
+        <is>
+          <t>My head...</t>
+        </is>
+      </c>
+      <c r="C1204" t="inlineStr">
+        <is>
+          <t>머리가...</t>
+        </is>
+      </c>
+    </row>
+    <row r="1205">
+      <c r="A1205" t="inlineStr">
+        <is>
+          <t>dialogue.sys_floor9_5_exit_reaction.7</t>
+        </is>
+      </c>
+      <c r="B1205" t="inlineStr">
+        <is>
+          <t>It feels like it's about to split.</t>
+        </is>
+      </c>
+      <c r="C1205" t="inlineStr">
+        <is>
+          <t>쪼개질 것 같아.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1206">
+      <c r="A1206" t="inlineStr">
+        <is>
+          <t>dialogue.sys_floor9_5_exit_reaction.8</t>
+        </is>
+      </c>
+      <c r="B1206" t="inlineStr">
+        <is>
+          <t>(You clutch your head while walking toward the exit.)</t>
+        </is>
+      </c>
+      <c r="C1206" t="inlineStr">
+        <is>
+          <t>(머리를 부여잡고 출구를 향해 걷는다.)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(text): game-side text rewritten to the style guide - classes, items, skills, statuses, tutorials, help, battle and menu lines (D155)
Class lines (lore + playstyle, kept to the class panel's five lines), throwable and
accessory sentences, passive effect lines, status descriptions, tutorials, Help page
lines, two settings help lines, one battle buff line and one Korean label fix.
Numbers, rules and placeholders unchanged; GML fallbacks match the sheet.
One scenario check follows the new Guard wording (next hit).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datafiles/localization/game_text.xlsx
+++ b/datafiles/localization/game_text.xlsx
@@ -4902,12 +4902,12 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>First hit: -1 [t]DEF[/t] for 2 turns</t>
+          <t>Your first hit cuts the enemy's [t]DEF[/t] by 1 for 2 turns</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>첫 타격: 2턴 동안 [t]DEF[/t] -1</t>
+          <t>첫 타격이 적의 [t]DEF[/t]를 2턴 동안 1 낮춘다</t>
         </is>
       </c>
     </row>
@@ -4919,7 +4919,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>First hit -3 damage (once per battle)</t>
+          <t>The first hit you take deals 3 less damage (once per battle)</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
@@ -4936,7 +4936,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>After a hit: next hit -40% (2-turn cooldown)</t>
+          <t>After you are hit, the next hit deals 40% less (2-turn cooldown)</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
@@ -4953,7 +4953,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>-30% damage from big hits</t>
+          <t>Big hits deal 30% less damage</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
@@ -4970,7 +4970,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>+1 [t]MP[/t] every 2 turns, +1 physical damage taken</t>
+          <t>+1 [t]MP[/t] every 2 turns, but physical hits deal 1 more damage</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
@@ -4987,7 +4987,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>+10% skill damage, +1 status turn</t>
+          <t>Skills deal +10% damage; your statuses last 1 turn longer</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
@@ -5004,12 +5004,12 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>Reflects the first status (costs 1 [t]MP[/t])</t>
+          <t>Reflects the first status cast on you (once per battle, costs 1 [t]MP[/t])</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>첫 상태 이상을 반사 ([t]MP[/t] 1 소모)</t>
+          <t>첫 상태 이상을 반사 (전투마다 1회, [t]MP[/t] 1 소모)</t>
         </is>
       </c>
     </row>
@@ -5021,7 +5021,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>+35% damage to foes below 35% [t]HP[/t]</t>
+          <t>+35% damage to enemies under 35% [t]HP[/t]</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
@@ -5055,12 +5055,12 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>[t]Good[/t] or [a]Perfect[/a]: may [t]Stun[/t] (3-turn cooldown)</t>
+          <t>A [t]Good[/t] or [a]Perfect[/a] press may [t]Stun[/t] the enemy (3-turn cooldown)</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>[t]좋음[/t] 또는 [a]완벽[/a]: [t]기절[/t]시킬 수 있음 (재사용 3턴)</t>
+          <t>[t]좋음[/t] 또는 [a]완벽[/a] 판정 시 적을 [t]기절[/t]시킬 수 있음 (재사용 3턴)</t>
         </is>
       </c>
     </row>
@@ -5072,7 +5072,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>+30% damage to foes with a status</t>
+          <t>+30% damage to enemies with a status</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
@@ -5106,7 +5106,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>+15% skill damage, +1 status turn</t>
+          <t>Skills deal +15% damage; your statuses last 1 turn longer</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
@@ -5123,7 +5123,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>+25% skill damage, [a]Perfect[/a] +1 [t]MP[/t]</t>
+          <t>Skills deal +25% damage; a [a]Perfect[/a] press gives +1 [t]MP[/t]</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
@@ -8421,7 +8421,7 @@
       </c>
       <c r="B471" t="inlineStr">
         <is>
-          <t>Turns the screen shake on hits on or off.</t>
+          <t>Screen shake when a hit lands: on or off.</t>
         </is>
       </c>
       <c r="C471" t="inlineStr">
@@ -8472,7 +8472,7 @@
       </c>
       <c r="B474" t="inlineStr">
         <is>
-          <t>How many times the picture is enlarged in a window. Only used when windowed. You are asked to keep a change.</t>
+          <t>How many times the picture is enlarged. Windowed mode only. You are asked to keep a change.</t>
         </is>
       </c>
       <c r="C474" t="inlineStr">
@@ -8659,7 +8659,7 @@
       </c>
       <c r="B485" t="inlineStr">
         <is>
-          <t>Pushed back on the turn bar. Then [t]Steadfast[/t]: cannot be stunned for 2 turns.</t>
+          <t>Pushed back on the turn strip. Then [t]Steadfast[/t]: cannot be stunned for 2 turns.</t>
         </is>
       </c>
       <c r="C485" t="inlineStr">
@@ -8676,7 +8676,7 @@
       </c>
       <c r="B486" t="inlineStr">
         <is>
-          <t>Blocks the next incoming hit.</t>
+          <t>Blocks the next hit.</t>
         </is>
       </c>
       <c r="C486" t="inlineStr">
@@ -8710,7 +8710,7 @@
       </c>
       <c r="B488" t="inlineStr">
         <is>
-          <t>Dodges the next incoming attack.</t>
+          <t>Dodges the next attack.</t>
         </is>
       </c>
       <c r="C488" t="inlineStr">
@@ -8795,7 +8795,7 @@
       </c>
       <c r="B493" t="inlineStr">
         <is>
-          <t>Until hit: take {take}% less, deal {deal}% more damage.</t>
+          <t>Until you are hit: take {take}% less damage, deal {deal}% more.</t>
         </is>
       </c>
       <c r="C493" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="B494" t="inlineStr">
         <is>
-          <t>Next incoming hit deals {pct}% less damage.</t>
+          <t>The next hit you take deals {pct}% less damage.</t>
         </is>
       </c>
       <c r="C494" t="inlineStr">
@@ -8829,12 +8829,12 @@
       </c>
       <c r="B495" t="inlineStr">
         <is>
-          <t>Lose defense.{mods}</t>
+          <t>Lowers [t]DEF[/t].{mods}</t>
         </is>
       </c>
       <c r="C495" t="inlineStr">
         <is>
-          <t>방어력이 떨어집니다.{mods}</t>
+          <t>[t]DEF[/t]가 떨어집니다.{mods}</t>
         </is>
       </c>
     </row>
@@ -10291,12 +10291,12 @@
       </c>
       <c r="B581" t="inlineStr">
         <is>
-          <t>A scout of the dark tunnels. Quick and sharp: poison and double shots.</t>
+          <t>A scout of the dark. Quick, with [t]Poison[/t] and double shots.</t>
         </is>
       </c>
       <c r="C581" t="inlineStr">
         <is>
-          <t>어두운 터널의 척후병. 빠르고 날카롭습니다. 독과 연속 사격.</t>
+          <t>어둠 속의 척후병. 빠르고, [t]독[/t]과 연속 사격을 쓴다.</t>
         </is>
       </c>
     </row>
@@ -10308,12 +10308,12 @@
       </c>
       <c r="B582" t="inlineStr">
         <is>
-          <t>Guard of the fallen keep. Hits hard, takes hits harder. Stands firm.</t>
+          <t>Guard of a keep that fell. Hits hard, slow to be hurt.</t>
         </is>
       </c>
       <c r="C582" t="inlineStr">
         <is>
-          <t>무너진 보루의 수호병. 강하게 치고 더 단단히 버팁니다.</t>
+          <t>무너진 보루의 수호병. 세게 치고 좀처럼 다치지 않는다.</t>
         </is>
       </c>
     </row>
@@ -10325,12 +10325,12 @@
       </c>
       <c r="B583" t="inlineStr">
         <is>
-          <t>A scholar who heard the dark. Frail, but great magic and mana.</t>
+          <t>A scholar the dark read back. Frail; spells hit hard.</t>
         </is>
       </c>
       <c r="C583" t="inlineStr">
         <is>
-          <t>어둠의 소리를 들은 학자. 약하지만 마법과 마나가 대단합니다.</t>
+          <t>어둠이 읽어 낸 학자. 약하지만 마법이 강하다.</t>
         </is>
       </c>
     </row>
@@ -10342,12 +10342,12 @@
       </c>
       <c r="B584" t="inlineStr">
         <is>
-          <t>No name, no past, no skills. Only blade, passives and items.</t>
+          <t>No name, no past, no skills. A blade and your pockets.</t>
         </is>
       </c>
       <c r="C584" t="inlineStr">
         <is>
-          <t>이름도 과거도 스킬도 없습니다. 칼과 패시브와 아이템뿐.</t>
+          <t>이름도 과거도 스킬도 없다. 칼 한 자루와 주머니뿐이다.</t>
         </is>
       </c>
     </row>
@@ -10495,7 +10495,7 @@
       </c>
       <c r="B593" t="inlineStr">
         <is>
-          <t>[t]Poison[/t] you apply adds {n} extra stack.</t>
+          <t>[t]Poison[/t] you inflict adds {n} extra stack.</t>
         </is>
       </c>
       <c r="C593" t="inlineStr">
@@ -12858,12 +12858,12 @@
       </c>
       <c r="B732" t="inlineStr">
         <is>
-          <t>Your enchantments are snuffed out!</t>
+          <t>Your buffs are snuffed out!</t>
         </is>
       </c>
       <c r="C732" t="inlineStr">
         <is>
-          <t>당신의 강화 효과가 꺼졌습니다!</t>
+          <t>당신의 버프가 꺼졌습니다!</t>
         </is>
       </c>
     </row>
@@ -13011,12 +13011,12 @@
       </c>
       <c r="B741" t="inlineStr">
         <is>
-          <t>Throw it for {power} power of damage; it burns for {turns} turns. Costs your turn.</t>
+          <t>Hits for {power} power and inflicts [t]Burn[/t] for {turns} turns. Costs your turn.</t>
         </is>
       </c>
       <c r="C741" t="inlineStr">
         <is>
-          <t>위력 {power}의 피해를 주고 {turns}턴 동안 불탑니다. 턴을 소모합니다.</t>
+          <t>위력 {power}의 피해를 주고 {turns}턴 동안 [t]화상[/t]을 입힙니다. 턴을 소모합니다.</t>
         </is>
       </c>
     </row>
@@ -13028,7 +13028,7 @@
       </c>
       <c r="B742" t="inlineStr">
         <is>
-          <t>Throw it to poison the enemy with {n} stacks. Costs your turn.</t>
+          <t>Inflicts {n} stacks of [t]Poison[/t]. Costs your turn.</t>
         </is>
       </c>
       <c r="C742" t="inlineStr">
@@ -13045,7 +13045,7 @@
       </c>
       <c r="B743" t="inlineStr">
         <is>
-          <t>Throw it for {power} power of damage and a stun that pushes the enemy back. Costs your turn.</t>
+          <t>Hits for {power} power and inflicts [t]Stun[/t], pushing the enemy back. Costs your turn.</t>
         </is>
       </c>
       <c r="C743" t="inlineStr">
@@ -13062,7 +13062,7 @@
       </c>
       <c r="B744" t="inlineStr">
         <is>
-          <t>Throw it to dodge the next attack ({turns} turns); a [a]Perfect[/a] throw lets you slip away. Costs your turn.</t>
+          <t>Dodge the next attack ({turns} turns). A [a]Perfect[/a] throw lets you slip away. Costs your turn.</t>
         </is>
       </c>
       <c r="C744" t="inlineStr">
@@ -13096,7 +13096,7 @@
       </c>
       <c r="B746" t="inlineStr">
         <is>
-          <t>Wear it for {bonus}.</t>
+          <t>Gives {bonus} while equipped.</t>
         </is>
       </c>
       <c r="C746" t="inlineStr">
@@ -13113,7 +13113,7 @@
       </c>
       <c r="B747" t="inlineStr">
         <is>
-          <t>Wear it: {line}.</t>
+          <t>While equipped: {line}.</t>
         </is>
       </c>
       <c r="C747" t="inlineStr">
@@ -13130,7 +13130,7 @@
       </c>
       <c r="B748" t="inlineStr">
         <is>
-          <t>A ring or charm worn in the accessory slot.</t>
+          <t>A ring or charm for the accessory slot.</t>
         </is>
       </c>
       <c r="C748" t="inlineStr">
@@ -14439,12 +14439,12 @@
       </c>
       <c r="B825" t="inlineStr">
         <is>
-          <t>The strip at the top shows who acts next. Faster fighters act more often, and some skills push an enemy back a turn.</t>
+          <t>The top strip shows who acts next. Faster fighters act more often, and some skills push an enemy back a turn.</t>
         </is>
       </c>
       <c r="C825" t="inlineStr">
         <is>
-          <t>위쪽 띠는 다음에 행동할 상대를 보여 줍니다. 빠른 쪽이 더 자주 행동하고, 어떤 스킬은 적을 한 턴 뒤로 밀어냅니다.</t>
+          <t>위쪽 띠가 다음에 행동할 차례를 보여 줍니다. 빠른 쪽이 더 자주 행동하고, 일부 스킬은 적을 한 턴 뒤로 밉니다.</t>
         </is>
       </c>
     </row>
@@ -14456,12 +14456,12 @@
       </c>
       <c r="B826" t="inlineStr">
         <is>
-          <t>The sliding bar</t>
+          <t>Timing bar</t>
         </is>
       </c>
       <c r="C826" t="inlineStr">
         <is>
-          <t>움직이는 막대</t>
+          <t>타이밍 막대</t>
         </is>
       </c>
     </row>
@@ -14473,12 +14473,12 @@
       </c>
       <c r="B827" t="inlineStr">
         <is>
-          <t>A cursor slides along the bar. Press [k:confirm] when it is over the bright zone. The closer to the middle, the harder you hit.</t>
+          <t>Press [k:confirm] when the cursor is on the bright zone. The closer to the middle, the harder the hit.</t>
         </is>
       </c>
       <c r="C827" t="inlineStr">
         <is>
-          <t>커서가 막대를 따라 움직입니다. 밝은 구간 위에 왔을 때 [k:confirm]을(를) 누르세요. 가운데에 가까울수록 더 세게 때립니다.</t>
+          <t>커서가 밝은 구간에 있을 때 [k:confirm]을(를) 누르세요. 가운데에 가까울수록 더 세게 때립니다.</t>
         </is>
       </c>
     </row>
@@ -14507,12 +14507,12 @@
       </c>
       <c r="B829" t="inlineStr">
         <is>
-          <t>Skills show a row of arrows. Press [k:up][k:down][k:left][k:right] in that order before the time bar runs out. A wrong press costs time.</t>
+          <t>Match the row of arrows with [k:up][k:down][k:left][k:right], in order, before the time bar empties. A wrong press costs time.</t>
         </is>
       </c>
       <c r="C829" t="inlineStr">
         <is>
-          <t>스킬을 쓰면 화살표 줄이 나옵니다. 시간 막대가 다 줄기 전에 [k:up][k:down][k:left][k:right]으로 순서대로 누르세요. 틀리면 시간이 깎입니다.</t>
+          <t>시간 막대가 비기 전에 [k:up][k:down][k:left][k:right]으로 화살표 줄을 순서대로 누르세요. 틀리면 시간이 깎입니다.</t>
         </is>
       </c>
     </row>
@@ -14558,12 +14558,12 @@
       </c>
       <c r="B832" t="inlineStr">
         <is>
-          <t>Stagger and BREAK</t>
+          <t>Stagger</t>
         </is>
       </c>
       <c r="C832" t="inlineStr">
         <is>
-          <t>경직과 브레이크</t>
+          <t>경직</t>
         </is>
       </c>
     </row>
@@ -14575,12 +14575,12 @@
       </c>
       <c r="B833" t="inlineStr">
         <is>
-          <t>[t]Good[/t] hits fill the enemy's [t]stagger[/t] meter. When it is full the enemy goes into [a]BREAK[/a]: it loses a turn and takes +50% damage.</t>
+          <t>[t]Good[/t] hits fill the enemy's [t]stagger[/t] meter. When it is full: [a]BREAK[/a]. The enemy loses a turn and takes +50% damage.</t>
         </is>
       </c>
       <c r="C833" t="inlineStr">
         <is>
-          <t>좋은 공격은 적의 [t]경직[/t] 게이지를 채웁니다. 가득 차면 적이 [a]브레이크[/a] 상태가 되어 한 턴을 잃고 피해를 50% 더 받습니다.</t>
+          <t>[t]좋음[/t] 판정 공격은 적의 [t]경직[/t] 게이지를 채웁니다. 가득 차면 [a]브레이크[/a]. 적은 한 턴을 잃고 피해를 50% 더 받습니다.</t>
         </is>
       </c>
     </row>
@@ -14609,7 +14609,7 @@
       </c>
       <c r="B835" t="inlineStr">
         <is>
-          <t>Level-ups and skill chests offer 3 cards: a new skill, an upgrade or a passive. Take one, or skip for a little gold.</t>
+          <t>Level-ups and skill chests offer 3 cards: a skill, an upgrade or a passive. Take one, or skip for a little gold.</t>
         </is>
       </c>
       <c r="C835" t="inlineStr">
@@ -14643,7 +14643,7 @@
       </c>
       <c r="B837" t="inlineStr">
         <is>
-          <t>The merchant sells potions and gear. Gold is kept for the whole run, and the stock changes with every run.</t>
+          <t>The merchant sells potions and gear. Gold lasts the whole run; the stock changes every run.</t>
         </is>
       </c>
       <c r="C837" t="inlineStr">
@@ -14677,7 +14677,7 @@
       </c>
       <c r="B839" t="inlineStr">
         <is>
-          <t>Throwable items hurt an enemy straight from the item menu. Each one is used up when thrown, so save them for hard fights.</t>
+          <t>Throw them from the item menu to hurt an enemy. Each is used up, so save them for hard fights.</t>
         </is>
       </c>
       <c r="C839" t="inlineStr">
@@ -14711,7 +14711,7 @@
       </c>
       <c r="B841" t="inlineStr">
         <is>
-          <t>Each bed can be used once per run. Rest to restore all your [t]HP[/t] and [t]MP[/t], or use it to upgrade one of your skills.</t>
+          <t>Each bed works once per run. Rest to restore all your [t]HP[/t] and [t]MP[/t], or upgrade one skill.</t>
         </is>
       </c>
       <c r="C841" t="inlineStr">
@@ -14745,7 +14745,7 @@
       </c>
       <c r="B843" t="inlineStr">
         <is>
-          <t>Marked enemies are [t]Elites[/t]. They are tougher than normal ones, but their rewards are better.</t>
+          <t>Marked enemies are [t]Elites[/t]: tougher than the rest, with better rewards.</t>
         </is>
       </c>
       <c r="C843" t="inlineStr">
@@ -14779,12 +14779,12 @@
       </c>
       <c r="B845" t="inlineStr">
         <is>
-          <t>[t]Poison[/t], [t]Burn[/t], [t]Bleed[/t] and [t]Stun[/t] last a few turns. The icons under a name show which ones a fighter has.</t>
+          <t>Icons under a name show a fighter's statuses, like [t]Poison[/t] or [t]Burn[/t]. They last a few turns.</t>
         </is>
       </c>
       <c r="C845" t="inlineStr">
         <is>
-          <t>[t]독[/t], [t]화상[/t], [t]출혈[/t], [t]기절[/t]은 몇 턴 동안 이어집니다. 이름 아래 아이콘이 걸려 있는 상태를 보여 줍니다.</t>
+          <t>이름 아래 아이콘은 [t]독[/t]이나 [t]화상[/t] 같은 상태 이상을 보여 줍니다. 몇 턴 동안 이어집니다.</t>
         </is>
       </c>
     </row>
@@ -17997,7 +17997,7 @@
       </c>
       <c r="C1034" t="inlineStr">
         <is>
-          <t>퍼펙트 비율</t>
+          <t>완벽 비율</t>
         </is>
       </c>
     </row>
@@ -19199,12 +19199,12 @@
       </c>
       <c r="B1105" t="inlineStr">
         <is>
-          <t>A critical hit deals {mult} times the damage. Take Aim and some gear raise the odds.</t>
+          <t>A critical hit deals {mult} times the damage. [t]Take Aim[/t] and some gear raise the odds.</t>
         </is>
       </c>
       <c r="C1105" t="inlineStr">
         <is>
-          <t>치명타는 피해를 {mult}배로 줍니다. 조준과 일부 장비가 확률을 높입니다.</t>
+          <t>치명타는 피해를 {mult}배로 줍니다. [t]조준[/t]과 일부 장비가 확률을 높입니다.</t>
         </is>
       </c>
     </row>
@@ -19250,7 +19250,7 @@
       </c>
       <c r="B1108" t="inlineStr">
         <is>
-          <t>Press on the bar but off the middle for normal damage.</t>
+          <t>Press on the bar, off the middle, for normal damage.</t>
         </is>
       </c>
       <c r="C1108" t="inlineStr">
@@ -19284,12 +19284,12 @@
       </c>
       <c r="B1110" t="inlineStr">
         <is>
-          <t>Good hits fill the stagger meter. When it is full the enemy loses a turn and takes +{pct}% damage.</t>
+          <t>Good hits fill the [t]stagger[/t] meter. When it is full the enemy loses a turn and takes +{pct}% damage.</t>
         </is>
       </c>
       <c r="C1110" t="inlineStr">
         <is>
-          <t>좋은 공격은 경직 게이지를 채웁니다. 가득 차면 적이 한 턴을 잃고 피해를 {pct}% 더 받습니다.</t>
+          <t>좋은 공격은 [t]경직[/t] 게이지를 채웁니다. 가득 차면 적이 한 턴을 잃고 피해를 {pct}% 더 받습니다.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(ui): menu press mid-step is kept and opens on the next settled frame, a pad leaves Press a key, Y is Back in the menu and Esc stays Back, Keep this? ignores the second click of a double click, Items in a fight say read-only
New string controls.waiting_pad (en + ko). Replaces the stubs of the check commit.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datafiles/localization/game_text.xlsx
+++ b/datafiles/localization/game_text.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1153"/>
+  <dimension ref="A1:C1154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -20024,6 +20024,23 @@
         </is>
       </c>
     </row>
+    <row r="1154">
+      <c r="A1154" t="inlineStr">
+        <is>
+          <t>controls.waiting_pad</t>
+        </is>
+      </c>
+      <c r="B1154" t="inlineStr">
+        <is>
+          <t>Press the new key for {action}. [k:back] cancels.</t>
+        </is>
+      </c>
+      <c r="C1154" t="inlineStr">
+        <is>
+          <t>{action}에 쓸 새 키를 누르세요. [k:back] 버튼으로 취소합니다.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C678"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(text): one word per meaning and Title Case labels across the UI (D133); ui_deny refuse sound key
159 workbook cells (en and ko) and their GML fallbacks: Enemy (not foe), battle (not fight), Quit (not Exit), Equipped / Unequip / 장착, Choose, Take, Abandon, EXP, Evasion, Bag, Status tab, Title Case labels and battle commands. Refusals call SFX_PlayUI("ui_deny") (plays the back asset until the owner picks one by ear). Exact-text assertions updated to the new words; purposes unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datafiles/localization/game_text.xlsx
+++ b/datafiles/localization/game_text.xlsx
@@ -448,7 +448,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ATTACK</t>
+          <t>Attack</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -465,7 +465,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ITEM</t>
+          <t>Item</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -482,7 +482,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>RUN</t>
+          <t>Run</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -499,7 +499,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SKILL</t>
+          <t>Skill</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -516,7 +516,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>GOOD</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -550,7 +550,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>PERFECT</t>
+          <t>Perfect</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -567,7 +567,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>WEAK</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -839,7 +839,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Select class</t>
+          <t>Choose Class</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -5446,7 +5446,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Select difficulty</t>
+          <t>Choose Difficulty</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -5497,7 +5497,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>New game</t>
+          <t>New Game</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -5514,7 +5514,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Load game</t>
+          <t>Load Game</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -5548,7 +5548,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Exit game</t>
+          <t>Quit Game</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -5667,7 +5667,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Item not in inventory.</t>
+          <t>Item not in bag.</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -5701,7 +5701,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Learn a skill</t>
+          <t>Learn a Skill</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -5718,7 +5718,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Available points: {points}</t>
+          <t>Available Points: {points}</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -5752,7 +5752,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Level cap</t>
+          <t>Level Cap</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -5803,7 +5803,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Inventory</t>
+          <t>Bag</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -5854,7 +5854,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>All classes</t>
+          <t>All Classes</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -5871,7 +5871,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>{classes} only</t>
+          <t>{classes} Only</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -5990,7 +5990,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>Effect: Multiple statuses</t>
+          <t>Effect: Multiple Statuses</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -6041,7 +6041,7 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Effect: Steal one random item</t>
+          <t>Effect: Steal One Random Item</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -6160,7 +6160,7 @@
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Teaches: Unknown skill</t>
+          <t>Teaches: Unknown Skill</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>Key item</t>
+          <t>Key Item</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
@@ -6483,7 +6483,7 @@
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>Affects combat performance.</t>
+          <t>Affects battle performance.</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
@@ -6653,7 +6653,7 @@
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>All allies</t>
+          <t>All Allies</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
@@ -6670,7 +6670,7 @@
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>All enemies</t>
+          <t>All Enemies</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
@@ -6738,12 +6738,12 @@
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>Exit to main menu</t>
+          <t>Quit to Title</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>메인 메뉴로 나가기</t>
+          <t>타이틀로 나가기</t>
         </is>
       </c>
     </row>
@@ -6959,7 +6959,7 @@
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t>Load game</t>
+          <t>Load Game</t>
         </is>
       </c>
       <c r="C385" t="inlineStr">
@@ -6976,7 +6976,7 @@
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t>Save game</t>
+          <t>Save Game</t>
         </is>
       </c>
       <c r="C386" t="inlineStr">
@@ -8149,7 +8149,7 @@
       </c>
       <c r="B455" t="inlineStr">
         <is>
-          <t>Hold to skip</t>
+          <t>Hold to Skip</t>
         </is>
       </c>
       <c r="C455" t="inlineStr">
@@ -8166,7 +8166,7 @@
       </c>
       <c r="B456" t="inlineStr">
         <is>
-          <t>Text speed</t>
+          <t>Text Speed</t>
         </is>
       </c>
       <c r="C456" t="inlineStr">
@@ -8183,7 +8183,7 @@
       </c>
       <c r="B457" t="inlineStr">
         <is>
-          <t>Screen shake</t>
+          <t>Screen Shake</t>
         </is>
       </c>
       <c r="C457" t="inlineStr">
@@ -8200,7 +8200,7 @@
       </c>
       <c r="B458" t="inlineStr">
         <is>
-          <t>Timing assist</t>
+          <t>Timing Assist</t>
         </is>
       </c>
       <c r="C458" t="inlineStr">
@@ -8302,7 +8302,7 @@
       </c>
       <c r="B464" t="inlineStr">
         <is>
-          <t>Chars per sec</t>
+          <t>Chars per Sec</t>
         </is>
       </c>
       <c r="C464" t="inlineStr">
@@ -8336,7 +8336,7 @@
       </c>
       <c r="B466" t="inlineStr">
         <is>
-          <t>Window size</t>
+          <t>Window Size</t>
         </is>
       </c>
       <c r="C466" t="inlineStr">
@@ -8664,7 +8664,7 @@
       </c>
       <c r="C485" t="inlineStr">
         <is>
-          <t>차례가 뒤로 밀립니다. 이후 2턴간 [t]버티기[/t] 상태가 되어 [t]기절[/t]하지 않습니다.</t>
+          <t>턴이 뒤로 밀립니다. 이후 2턴간 [t]버티기[/t] 상태가 되어 [t]기절[/t]하지 않습니다.</t>
         </is>
       </c>
     </row>
@@ -8761,7 +8761,7 @@
       </c>
       <c r="B491" t="inlineStr">
         <is>
-          <t>Recover {n} [t]MP[/t] each turn.</t>
+          <t>Restore {n} [t]MP[/t] each turn.</t>
         </is>
       </c>
       <c r="C491" t="inlineStr">
@@ -8965,7 +8965,7 @@
       </c>
       <c r="B503" t="inlineStr">
         <is>
-          <t>Abandon run</t>
+          <t>Abandon Run</t>
         </is>
       </c>
       <c r="C503" t="inlineStr">
@@ -9067,7 +9067,7 @@
       </c>
       <c r="B509" t="inlineStr">
         <is>
-          <t>You gave up the run.</t>
+          <t>You abandoned the run.</t>
         </is>
       </c>
       <c r="C509" t="inlineStr">
@@ -9089,7 +9089,7 @@
       </c>
       <c r="C510" t="inlineStr">
         <is>
-          <t>쓰러뜨린 상대: {name}</t>
+          <t>쓰러진 원인: {name}</t>
         </is>
       </c>
     </row>
@@ -9135,7 +9135,7 @@
       </c>
       <c r="B513" t="inlineStr">
         <is>
-          <t>Press [k:confirm] to go on</t>
+          <t>Press [k:confirm] to continue</t>
         </is>
       </c>
       <c r="C513" t="inlineStr">
@@ -9152,12 +9152,12 @@
       </c>
       <c r="B514" t="inlineStr">
         <is>
-          <t>[k:up][k:down] Choose   [k:confirm] Take it</t>
+          <t>[k:up][k:down] Choose   [k:confirm] Take</t>
         </is>
       </c>
       <c r="C514" t="inlineStr">
         <is>
-          <t>[k:up][k:down] 고르기   [k:confirm] 가져가기</t>
+          <t>[k:up][k:down] 선택   [k:confirm] 받기</t>
         </is>
       </c>
     </row>
@@ -9203,7 +9203,7 @@
       </c>
       <c r="B517" t="inlineStr">
         <is>
-          <t>Carry one echo into the next fall</t>
+          <t>Carry One Echo into the Next Fall</t>
         </is>
       </c>
       <c r="C517" t="inlineStr">
@@ -9220,7 +9220,7 @@
       </c>
       <c r="B518" t="inlineStr">
         <is>
-          <t>Falls so far: {n}</t>
+          <t>Falls So Far: {n}</t>
         </is>
       </c>
       <c r="C518" t="inlineStr">
@@ -9237,7 +9237,7 @@
       </c>
       <c r="B519" t="inlineStr">
         <is>
-          <t>Floor reached: {n}</t>
+          <t>Floor Reached: {n}</t>
         </is>
       </c>
       <c r="C519" t="inlineStr">
@@ -9293,7 +9293,7 @@
       </c>
       <c r="C522" t="inlineStr">
         <is>
-          <t>{name}의 차례가 뒤로 밀렸습니다!</t>
+          <t>{name}의 턴이 뒤로 밀렸습니다!</t>
         </is>
       </c>
     </row>
@@ -9310,7 +9310,7 @@
       </c>
       <c r="C523" t="inlineStr">
         <is>
-          <t>차례가 뒤로 밀렸습니다!</t>
+          <t>턴이 뒤로 밀렸습니다!</t>
         </is>
       </c>
     </row>
@@ -9560,7 +9560,7 @@
       </c>
       <c r="B538" t="inlineStr">
         <is>
-          <t>Main stat</t>
+          <t>Main Stat</t>
         </is>
       </c>
       <c r="C538" t="inlineStr">
@@ -9577,7 +9577,7 @@
       </c>
       <c r="B539" t="inlineStr">
         <is>
-          <t>Poison stacks</t>
+          <t>Poison Stacks</t>
         </is>
       </c>
       <c r="C539" t="inlineStr">
@@ -9594,7 +9594,7 @@
       </c>
       <c r="B540" t="inlineStr">
         <is>
-          <t>After fight</t>
+          <t>After Battle</t>
         </is>
       </c>
       <c r="C540" t="inlineStr">
@@ -9611,7 +9611,7 @@
       </c>
       <c r="B541" t="inlineStr">
         <is>
-          <t>Potion find</t>
+          <t>Potion Find</t>
         </is>
       </c>
       <c r="C541" t="inlineStr">
@@ -9628,7 +9628,7 @@
       </c>
       <c r="B542" t="inlineStr">
         <is>
-          <t>Perfect zone</t>
+          <t>Perfect Zone</t>
         </is>
       </c>
       <c r="C542" t="inlineStr">
@@ -9662,7 +9662,7 @@
       </c>
       <c r="B544" t="inlineStr">
         <is>
-          <t>Each turn</t>
+          <t>Each Turn</t>
         </is>
       </c>
       <c r="C544" t="inlineStr">
@@ -9713,7 +9713,7 @@
       </c>
       <c r="B547" t="inlineStr">
         <is>
-          <t>Skill power</t>
+          <t>Skill Power</t>
         </is>
       </c>
       <c r="C547" t="inlineStr">
@@ -9747,7 +9747,7 @@
       </c>
       <c r="B549" t="inlineStr">
         <is>
-          <t>Status turns</t>
+          <t>Status Turns</t>
         </is>
       </c>
       <c r="C549" t="inlineStr">
@@ -10019,7 +10019,7 @@
       </c>
       <c r="B565" t="inlineStr">
         <is>
-          <t>Class passive</t>
+          <t>Class Passive</t>
         </is>
       </c>
       <c r="C565" t="inlineStr">
@@ -10092,7 +10092,7 @@
       </c>
       <c r="C569" t="inlineStr">
         <is>
-          <t>[k:left][k:right] 고르기   [k:confirm] 받기</t>
+          <t>[k:left][k:right] 선택   [k:confirm] 받기</t>
         </is>
       </c>
     </row>
@@ -10121,7 +10121,7 @@
       </c>
       <c r="B571" t="inlineStr">
         <is>
-          <t>Skip: +{gold} gold</t>
+          <t>Skip: +{gold} Gold</t>
         </is>
       </c>
       <c r="C571" t="inlineStr">
@@ -10138,7 +10138,7 @@
       </c>
       <c r="B572" t="inlineStr">
         <is>
-          <t>Choose a card</t>
+          <t>Choose a Card</t>
         </is>
       </c>
       <c r="C572" t="inlineStr">
@@ -10155,7 +10155,7 @@
       </c>
       <c r="B573" t="inlineStr">
         <is>
-          <t>Keep my skills</t>
+          <t>Keep My Skills</t>
         </is>
       </c>
       <c r="C573" t="inlineStr">
@@ -10172,7 +10172,7 @@
       </c>
       <c r="B574" t="inlineStr">
         <is>
-          <t>Gives up: {line}</t>
+          <t>Loses: {line}</t>
         </is>
       </c>
       <c r="C574" t="inlineStr">
@@ -10206,7 +10206,7 @@
       </c>
       <c r="B576" t="inlineStr">
         <is>
-          <t>Learn {skill}: replace which?</t>
+          <t>Learn {skill}: Replace Which?</t>
         </is>
       </c>
       <c r="C576" t="inlineStr">
@@ -10257,7 +10257,7 @@
       </c>
       <c r="B579" t="inlineStr">
         <is>
-          <t>Level {lvl}: place 1 point</t>
+          <t>Level {lvl}: Place 1 Point</t>
         </is>
       </c>
       <c r="C579" t="inlineStr">
@@ -10529,7 +10529,7 @@
       </c>
       <c r="B595" t="inlineStr">
         <is>
-          <t>Restore {n} [t]HP[/t] after each fight you win.</t>
+          <t>Restore {n} [t]HP[/t] after each battle you win.</t>
         </is>
       </c>
       <c r="C595" t="inlineStr">
@@ -10699,7 +10699,7 @@
       </c>
       <c r="B605" t="inlineStr">
         <is>
-          <t>Enemies start each fight with {n} [t]stagger[/t].</t>
+          <t>Enemies start each battle with {n} [t]stagger[/t].</t>
         </is>
       </c>
       <c r="C605" t="inlineStr">
@@ -10903,7 +10903,7 @@
       </c>
       <c r="B617" t="inlineStr">
         <is>
-          <t>Regain {n} [t]MP[/t] after each fight you win.</t>
+          <t>Regain {n} [t]MP[/t] after each battle you win.</t>
         </is>
       </c>
       <c r="C617" t="inlineStr">
@@ -11107,7 +11107,7 @@
       </c>
       <c r="B629" t="inlineStr">
         <is>
-          <t>{n}% chance to find a potion after each fight you win.</t>
+          <t>{n}% chance to find a potion after each battle you win.</t>
         </is>
       </c>
       <c r="C629" t="inlineStr">
@@ -11804,7 +11804,7 @@
       </c>
       <c r="B670" t="inlineStr">
         <is>
-          <t>Floor reached</t>
+          <t>Floor Reached</t>
         </is>
       </c>
       <c r="C670" t="inlineStr">
@@ -11855,12 +11855,12 @@
       </c>
       <c r="B673" t="inlineStr">
         <is>
-          <t>Foes beaten</t>
+          <t>Enemies Beaten</t>
         </is>
       </c>
       <c r="C673" t="inlineStr">
         <is>
-          <t>쓰러뜨린 적</t>
+          <t>처치한 적</t>
         </is>
       </c>
     </row>
@@ -11872,7 +11872,7 @@
       </c>
       <c r="B674" t="inlineStr">
         <is>
-          <t>Falls so far</t>
+          <t>Falls So Far</t>
         </is>
       </c>
       <c r="C674" t="inlineStr">
@@ -12875,7 +12875,7 @@
       </c>
       <c r="B733" t="inlineStr">
         <is>
-          <t>ELITE</t>
+          <t>Elite</t>
         </is>
       </c>
       <c r="C733" t="inlineStr">
@@ -13101,7 +13101,7 @@
       </c>
       <c r="C746" t="inlineStr">
         <is>
-          <t>착용 효과: {bonus}.</t>
+          <t>장착 효과: {bonus}.</t>
         </is>
       </c>
     </row>
@@ -13118,7 +13118,7 @@
       </c>
       <c r="C747" t="inlineStr">
         <is>
-          <t>착용 효과: {line}.</t>
+          <t>장착 효과: {line}.</t>
         </is>
       </c>
     </row>
@@ -13135,7 +13135,7 @@
       </c>
       <c r="C748" t="inlineStr">
         <is>
-          <t>장신구 칸에 착용하는 반지나 부적입니다.</t>
+          <t>장신구 칸에 장착하는 반지나 부적입니다.</t>
         </is>
       </c>
     </row>
@@ -13300,7 +13300,7 @@
       </c>
       <c r="B758" t="inlineStr">
         <is>
-          <t>Push back</t>
+          <t>Push Back</t>
         </is>
       </c>
       <c r="C758" t="inlineStr">
@@ -13317,7 +13317,7 @@
       </c>
       <c r="B759" t="inlineStr">
         <is>
-          <t>Dodge</t>
+          <t>Evasion</t>
         </is>
       </c>
       <c r="C759" t="inlineStr">
@@ -13402,7 +13402,7 @@
       </c>
       <c r="B764" t="inlineStr">
         <is>
-          <t>Carry up to</t>
+          <t>Carry Limit</t>
         </is>
       </c>
       <c r="C764" t="inlineStr">
@@ -13419,7 +13419,7 @@
       </c>
       <c r="B765" t="inlineStr">
         <is>
-          <t>Damage taken</t>
+          <t>Damage Taken</t>
         </is>
       </c>
       <c r="C765" t="inlineStr">
@@ -13742,7 +13742,7 @@
       </c>
       <c r="B784" t="inlineStr">
         <is>
-          <t>Regenerating: heals {pct}% of its HP each turn.</t>
+          <t>Regenerating: restores {pct}% of its HP each turn.</t>
         </is>
       </c>
       <c r="C784" t="inlineStr">
@@ -13793,7 +13793,7 @@
       </c>
       <c r="B787" t="inlineStr">
         <is>
-          <t>Sold out</t>
+          <t>Sold Out</t>
         </is>
       </c>
       <c r="C787" t="inlineStr">
@@ -13810,7 +13810,7 @@
       </c>
       <c r="B788" t="inlineStr">
         <is>
-          <t>You have</t>
+          <t>You Have</t>
         </is>
       </c>
       <c r="C788" t="inlineStr">
@@ -13827,7 +13827,7 @@
       </c>
       <c r="B789" t="inlineStr">
         <is>
-          <t>In stock</t>
+          <t>In Stock</t>
         </is>
       </c>
       <c r="C789" t="inlineStr">
@@ -13844,7 +13844,7 @@
       </c>
       <c r="B790" t="inlineStr">
         <is>
-          <t>Sells for</t>
+          <t>Sells For</t>
         </is>
       </c>
       <c r="C790" t="inlineStr">
@@ -13866,7 +13866,7 @@
       </c>
       <c r="C791" t="inlineStr">
         <is>
-          <t>착용 중</t>
+          <t>장착 중</t>
         </is>
       </c>
     </row>
@@ -13878,7 +13878,7 @@
       </c>
       <c r="B792" t="inlineStr">
         <is>
-          <t>Nothing to sell</t>
+          <t>Nothing to Sell</t>
         </is>
       </c>
       <c r="C792" t="inlineStr">
@@ -13895,12 +13895,12 @@
       </c>
       <c r="B793" t="inlineStr">
         <is>
-          <t>Gold {n}</t>
+          <t>Gold: {n}</t>
         </is>
       </c>
       <c r="C793" t="inlineStr">
         <is>
-          <t>골드 {n}</t>
+          <t>골드: {n}</t>
         </is>
       </c>
     </row>
@@ -14065,7 +14065,7 @@
       </c>
       <c r="B803" t="inlineStr">
         <is>
-          <t>Take it off first.</t>
+          <t>Unequip it first.</t>
         </is>
       </c>
       <c r="C803" t="inlineStr">
@@ -14422,7 +14422,7 @@
       </c>
       <c r="B824" t="inlineStr">
         <is>
-          <t>Turn order</t>
+          <t>Turn Order</t>
         </is>
       </c>
       <c r="C824" t="inlineStr">
@@ -14444,7 +14444,7 @@
       </c>
       <c r="C825" t="inlineStr">
         <is>
-          <t>위쪽 띠가 다음에 행동할 차례를 보여 줍니다. 빠른 쪽이 더 자주 행동하고, 일부 스킬은 적을 한 턴 뒤로 밉니다.</t>
+          <t>위쪽 띠가 다음에 행동할 턴을 보여 줍니다. 빠른 쪽이 더 자주 행동하고, 일부 스킬은 적을 한 턴 뒤로 밉니다.</t>
         </is>
       </c>
     </row>
@@ -14456,7 +14456,7 @@
       </c>
       <c r="B826" t="inlineStr">
         <is>
-          <t>Timing bar</t>
+          <t>Timing Bar</t>
         </is>
       </c>
       <c r="C826" t="inlineStr">
@@ -14490,7 +14490,7 @@
       </c>
       <c r="B828" t="inlineStr">
         <is>
-          <t>Arrow skills</t>
+          <t>Arrow Skills</t>
         </is>
       </c>
       <c r="C828" t="inlineStr">
@@ -14626,7 +14626,7 @@
       </c>
       <c r="B836" t="inlineStr">
         <is>
-          <t>The shop</t>
+          <t>The Shop</t>
         </is>
       </c>
       <c r="C836" t="inlineStr">
@@ -14677,12 +14677,12 @@
       </c>
       <c r="B839" t="inlineStr">
         <is>
-          <t>Throw them from the item menu to hurt an enemy. Each is used up, so save them for hard fights.</t>
+          <t>Throw them from the item menu to hurt an enemy. Each is used up, so save them for hard battles.</t>
         </is>
       </c>
       <c r="C839" t="inlineStr">
         <is>
-          <t>투척 도구는 아이템 메뉴에서 바로 적에게 피해를 줍니다. 던지면 사라지니 어려운 싸움을 위해 아껴 두세요.</t>
+          <t>투척 도구는 아이템 메뉴에서 바로 적에게 피해를 줍니다. 던지면 사라지니 어려운 전투를 위해 아껴 두세요.</t>
         </is>
       </c>
     </row>
@@ -14886,7 +14886,7 @@
       </c>
       <c r="C851" t="inlineStr">
         <is>
-          <t>쉬기</t>
+          <t>휴식</t>
         </is>
       </c>
     </row>
@@ -14898,7 +14898,7 @@
       </c>
       <c r="B852" t="inlineStr">
         <is>
-          <t>Upgrade a skill</t>
+          <t>Upgrade a Skill</t>
         </is>
       </c>
       <c r="C852" t="inlineStr">
@@ -14920,7 +14920,7 @@
       </c>
       <c r="C853" t="inlineStr">
         <is>
-          <t>떠나기</t>
+          <t>나가기</t>
         </is>
       </c>
     </row>
@@ -15051,7 +15051,7 @@
       </c>
       <c r="B861" t="inlineStr">
         <is>
-          <t>Upgrade which skill?</t>
+          <t>Upgrade Which Skill?</t>
         </is>
       </c>
       <c r="C861" t="inlineStr">
@@ -15289,7 +15289,7 @@
       </c>
       <c r="B875" t="inlineStr">
         <is>
-          <t>Previous tab</t>
+          <t>Previous Tab</t>
         </is>
       </c>
       <c r="C875" t="inlineStr">
@@ -15306,7 +15306,7 @@
       </c>
       <c r="B876" t="inlineStr">
         <is>
-          <t>Next tab</t>
+          <t>Next Tab</t>
         </is>
       </c>
       <c r="C876" t="inlineStr">
@@ -15340,7 +15340,7 @@
       </c>
       <c r="B878" t="inlineStr">
         <is>
-          <t>Reset to defaults</t>
+          <t>Reset to Defaults</t>
         </is>
       </c>
       <c r="C878" t="inlineStr">
@@ -15510,7 +15510,7 @@
       </c>
       <c r="B888" t="inlineStr">
         <is>
-          <t>GUARD</t>
+          <t>Guard</t>
         </is>
       </c>
       <c r="C888" t="inlineStr">
@@ -15753,7 +15753,7 @@
       </c>
       <c r="C902" t="inlineStr">
         <is>
-          <t>다음 차례까지 받는 피해가 50% 늘어납니다.</t>
+          <t>다음 턴까지 받는 피해가 50% 늘어납니다.</t>
         </is>
       </c>
     </row>
@@ -16110,7 +16110,7 @@
       </c>
       <c r="C923" t="inlineStr">
         <is>
-          <t>이 상대에게서는 도망칠 수 없습니다.</t>
+          <t>이 적에게서는 도망칠 수 없습니다.</t>
         </is>
       </c>
     </row>
@@ -16241,7 +16241,7 @@
       </c>
       <c r="B931" t="inlineStr">
         <is>
-          <t>Quit to title</t>
+          <t>Quit to Title</t>
         </is>
       </c>
       <c r="C931" t="inlineStr">
@@ -16411,7 +16411,7 @@
       </c>
       <c r="B941" t="inlineStr">
         <is>
-          <t>Run history</t>
+          <t>Run History</t>
         </is>
       </c>
       <c r="C941" t="inlineStr">
@@ -16479,7 +16479,7 @@
       </c>
       <c r="B945" t="inlineStr">
         <is>
-          <t>Notes found {n}/{max}</t>
+          <t>Notes Found {n}/{max}</t>
         </is>
       </c>
       <c r="C945" t="inlineStr">
@@ -16552,7 +16552,7 @@
       </c>
       <c r="C949" t="inlineStr">
         <is>
-          <t>가방</t>
+          <t>소지품</t>
         </is>
       </c>
     </row>
@@ -16564,12 +16564,12 @@
       </c>
       <c r="B950" t="inlineStr">
         <is>
-          <t>Nothing equipped</t>
+          <t>Nothing Equipped</t>
         </is>
       </c>
       <c r="C950" t="inlineStr">
         <is>
-          <t>착용 없음</t>
+          <t>장착 없음</t>
         </is>
       </c>
     </row>
@@ -16586,7 +16586,7 @@
       </c>
       <c r="C951" t="inlineStr">
         <is>
-          <t>이 칸에는 아무것도 착용하지 않았습니다.</t>
+          <t>이 칸에는 아무것도 장착하지 않았습니다.</t>
         </is>
       </c>
     </row>
@@ -16598,7 +16598,7 @@
       </c>
       <c r="B952" t="inlineStr">
         <is>
-          <t>No accessory</t>
+          <t>No Accessory</t>
         </is>
       </c>
       <c r="C952" t="inlineStr">
@@ -16615,7 +16615,7 @@
       </c>
       <c r="B953" t="inlineStr">
         <is>
-          <t>No armor</t>
+          <t>No Armor</t>
         </is>
       </c>
       <c r="C953" t="inlineStr">
@@ -16632,7 +16632,7 @@
       </c>
       <c r="B954" t="inlineStr">
         <is>
-          <t>No weapon</t>
+          <t>No Weapon</t>
         </is>
       </c>
       <c r="C954" t="inlineStr">
@@ -16671,7 +16671,7 @@
       </c>
       <c r="C956" t="inlineStr">
         <is>
-          <t>착용 중</t>
+          <t>장착 중</t>
         </is>
       </c>
     </row>
@@ -16739,7 +16739,7 @@
       </c>
       <c r="C960" t="inlineStr">
         <is>
-          <t>[k:confirm] 착용</t>
+          <t>[k:confirm] 장착</t>
         </is>
       </c>
     </row>
@@ -16768,7 +16768,7 @@
       </c>
       <c r="B962" t="inlineStr">
         <is>
-          <t>[k:confirm] Select</t>
+          <t>[k:confirm] Choose</t>
         </is>
       </c>
       <c r="C962" t="inlineStr">
@@ -16785,7 +16785,7 @@
       </c>
       <c r="B963" t="inlineStr">
         <is>
-          <t>[k:confirm] Take off</t>
+          <t>[k:confirm] Unequip</t>
         </is>
       </c>
       <c r="C963" t="inlineStr">
@@ -16819,7 +16819,7 @@
       </c>
       <c r="B965" t="inlineStr">
         <is>
-          <t>You gave this run up on floor {n}.</t>
+          <t>You abandoned this run on floor {n}.</t>
         </is>
       </c>
       <c r="C965" t="inlineStr">
@@ -16938,7 +16938,7 @@
       </c>
       <c r="B972" t="inlineStr">
         <is>
-          <t>Nothing in your bag</t>
+          <t>Nothing in Your Bag</t>
         </is>
       </c>
       <c r="C972" t="inlineStr">
@@ -16989,7 +16989,7 @@
       </c>
       <c r="B975" t="inlineStr">
         <is>
-          <t>Best floor</t>
+          <t>Best Floor</t>
         </is>
       </c>
       <c r="C975" t="inlineStr">
@@ -17125,7 +17125,7 @@
       </c>
       <c r="B983" t="inlineStr">
         <is>
-          <t>Foes beaten</t>
+          <t>Enemies Beaten</t>
         </is>
       </c>
       <c r="C983" t="inlineStr">
@@ -17261,7 +17261,7 @@
       </c>
       <c r="B991" t="inlineStr">
         <is>
-          <t>XP</t>
+          <t>EXP</t>
         </is>
       </c>
       <c r="C991" t="inlineStr">
@@ -17329,7 +17329,7 @@
       </c>
       <c r="B995" t="inlineStr">
         <is>
-          <t>No skills yet</t>
+          <t>No Skills Yet</t>
         </is>
       </c>
       <c r="C995" t="inlineStr">
@@ -17465,12 +17465,12 @@
       </c>
       <c r="B1003" t="inlineStr">
         <is>
-          <t>Stats</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="C1003" t="inlineStr">
         <is>
-          <t>능력치</t>
+          <t>상태</t>
         </is>
       </c>
     </row>
@@ -17533,7 +17533,7 @@
       </c>
       <c r="B1007" t="inlineStr">
         <is>
-          <t>Gave up</t>
+          <t>Abandoned</t>
         </is>
       </c>
       <c r="C1007" t="inlineStr">
@@ -17703,7 +17703,7 @@
       </c>
       <c r="B1017" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>No</t>
         </is>
       </c>
       <c r="C1017" t="inlineStr">
@@ -17737,7 +17737,7 @@
       </c>
       <c r="B1019" t="inlineStr">
         <is>
-          <t>Press any key</t>
+          <t>Press Any Key</t>
         </is>
       </c>
       <c r="C1019" t="inlineStr">
@@ -17754,7 +17754,7 @@
       </c>
       <c r="B1020" t="inlineStr">
         <is>
-          <t>Press any button</t>
+          <t>Press Any Button</t>
         </is>
       </c>
       <c r="C1020" t="inlineStr">
@@ -17771,7 +17771,7 @@
       </c>
       <c r="B1021" t="inlineStr">
         <is>
-          <t>Can't continue</t>
+          <t>Can't Continue</t>
         </is>
       </c>
       <c r="C1021" t="inlineStr">
@@ -17873,7 +17873,7 @@
       </c>
       <c r="B1027" t="inlineStr">
         <is>
-          <t>Keep one skill you remember</t>
+          <t>Keep One Skill You Remember</t>
         </is>
       </c>
       <c r="C1027" t="inlineStr">
@@ -17992,7 +17992,7 @@
       </c>
       <c r="B1034" t="inlineStr">
         <is>
-          <t>Perfect rate</t>
+          <t>Perfect Rate</t>
         </is>
       </c>
       <c r="C1034" t="inlineStr">
@@ -18009,7 +18009,7 @@
       </c>
       <c r="B1035" t="inlineStr">
         <is>
-          <t>Crits landed</t>
+          <t>Crits Landed</t>
         </is>
       </c>
       <c r="C1035" t="inlineStr">
@@ -18026,7 +18026,7 @@
       </c>
       <c r="B1036" t="inlineStr">
         <is>
-          <t>Damage dealt</t>
+          <t>Damage Dealt</t>
         </is>
       </c>
       <c r="C1036" t="inlineStr">
@@ -18043,7 +18043,7 @@
       </c>
       <c r="B1037" t="inlineStr">
         <is>
-          <t>Damage taken</t>
+          <t>Damage Taken</t>
         </is>
       </c>
       <c r="C1037" t="inlineStr">
@@ -18060,7 +18060,7 @@
       </c>
       <c r="B1038" t="inlineStr">
         <is>
-          <t>Fights won</t>
+          <t>Battles Won</t>
         </is>
       </c>
       <c r="C1038" t="inlineStr">
@@ -18077,7 +18077,7 @@
       </c>
       <c r="B1039" t="inlineStr">
         <is>
-          <t>Run time</t>
+          <t>Run Time</t>
         </is>
       </c>
       <c r="C1039" t="inlineStr">
@@ -18162,7 +18162,7 @@
       </c>
       <c r="B1044" t="inlineStr">
         <is>
-          <t>Raises your max [t]HP[/t] by {n} and heals {n} [t]HP[/t].</t>
+          <t>Raises your max [t]HP[/t] by {n} and restores {n} [t]HP[/t].</t>
         </is>
       </c>
       <c r="C1044" t="inlineStr">
@@ -18230,7 +18230,7 @@
       </c>
       <c r="B1048" t="inlineStr">
         <is>
-          <t>Goes back to the title. Continue puts you back just before this fight.</t>
+          <t>Goes back to the title. Continue puts you back just before this battle.</t>
         </is>
       </c>
       <c r="C1048" t="inlineStr">
@@ -18247,7 +18247,7 @@
       </c>
       <c r="B1049" t="inlineStr">
         <is>
-          <t>Keep this setting?</t>
+          <t>Keep This Setting?</t>
         </is>
       </c>
       <c r="C1049" t="inlineStr">
@@ -18298,7 +18298,7 @@
       </c>
       <c r="B1052" t="inlineStr">
         <is>
-          <t>Choose a seed</t>
+          <t>Choose a Seed</t>
         </is>
       </c>
       <c r="C1052" t="inlineStr">
@@ -18315,7 +18315,7 @@
       </c>
       <c r="B1053" t="inlineStr">
         <is>
-          <t>Random seed</t>
+          <t>Random Seed</t>
         </is>
       </c>
       <c r="C1053" t="inlineStr">
@@ -18332,7 +18332,7 @@
       </c>
       <c r="B1054" t="inlineStr">
         <is>
-          <t>Enter seed</t>
+          <t>Enter Seed</t>
         </is>
       </c>
       <c r="C1054" t="inlineStr">
@@ -18349,7 +18349,7 @@
       </c>
       <c r="B1055" t="inlineStr">
         <is>
-          <t>Enter seed</t>
+          <t>Enter Seed</t>
         </is>
       </c>
       <c r="C1055" t="inlineStr">
@@ -18371,7 +18371,7 @@
       </c>
       <c r="C1056" t="inlineStr">
         <is>
-          <t>최대 9자리. 같은 시드, 같은 모험.</t>
+          <t>최대 9자리. 같은 시드, 같은 도전.</t>
         </is>
       </c>
     </row>
@@ -18439,7 +18439,7 @@
       </c>
       <c r="C1060" t="inlineStr">
         <is>
-          <t>[k:back] 뒤로   [k:tab_prev] 지우기</t>
+          <t>[k:back] 뒤로   [k:tab_prev] 삭제</t>
         </is>
       </c>
     </row>
@@ -18485,7 +18485,7 @@
       </c>
       <c r="B1063" t="inlineStr">
         <is>
-          <t>Quit to title? Continue puts you back just before this fight.</t>
+          <t>Quit to title? Continue puts you back just before this battle.</t>
         </is>
       </c>
       <c r="C1063" t="inlineStr">
@@ -19029,7 +19029,7 @@
       </c>
       <c r="B1095" t="inlineStr">
         <is>
-          <t>Stats &amp; terms</t>
+          <t>Stats &amp; Terms</t>
         </is>
       </c>
       <c r="C1095" t="inlineStr">
@@ -19998,7 +19998,7 @@
       </c>
       <c r="B1152" t="inlineStr">
         <is>
-          <t>In a fight, use ITEM in the battle menu.</t>
+          <t>In a battle, use Item in the battle menu.</t>
         </is>
       </c>
       <c r="C1152" t="inlineStr">
@@ -20015,7 +20015,7 @@
       </c>
       <c r="B1153" t="inlineStr">
         <is>
-          <t>You can't change gear in a fight.</t>
+          <t>You can't change gear during a battle.</t>
         </is>
       </c>
       <c r="C1153" t="inlineStr">

</xml_diff>

<commit_message>
feat(text): rows that did not fit their panels shortened; TextFit_Known down to the names (D156)
Throwable sentences (Firebomb, Ice Flask, Smoke Bomb, en + ko), the card sentences
("Hit for 5 power. 75% Poison."), Scrounger, and the Korean Codex Met / Seen lines
were shortened and their GML fallbacks matched. Their entries are removed from
TextFit_Known; what is left are names (skills, passives, "The Pale Choirbeast"),
which are the owner's call.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datafiles/localization/game_text.xlsx
+++ b/datafiles/localization/game_text.xlsx
@@ -9934,7 +9934,7 @@
       </c>
       <c r="B560" t="inlineStr">
         <is>
-          <t>Strike for {power} power.</t>
+          <t>Hit for {power} power.</t>
         </is>
       </c>
       <c r="C560" t="inlineStr">
@@ -9951,7 +9951,7 @@
       </c>
       <c r="B561" t="inlineStr">
         <is>
-          <t>{chance}% to inflict [t]{status}[/t].</t>
+          <t>{chance}% [t]{status}[/t].</t>
         </is>
       </c>
       <c r="C561" t="inlineStr">
@@ -9968,7 +9968,7 @@
       </c>
       <c r="B562" t="inlineStr">
         <is>
-          <t>Strike {hits} times for {power} power each.</t>
+          <t>Hit {hits} times for {power} power each.</t>
         </is>
       </c>
       <c r="C562" t="inlineStr">
@@ -11107,7 +11107,7 @@
       </c>
       <c r="B629" t="inlineStr">
         <is>
-          <t>{n}% chance to find a potion after each battle you win.</t>
+          <t>After each win, {n}% to find a potion.</t>
         </is>
       </c>
       <c r="C629" t="inlineStr">
@@ -13011,7 +13011,7 @@
       </c>
       <c r="B741" t="inlineStr">
         <is>
-          <t>Hits for {power} power and inflicts [t]Burn[/t] for {turns} turns. Costs your turn.</t>
+          <t>Hits for {power} power. Inflicts [t]Burn[/t] for {turns} turns. Costs your turn.</t>
         </is>
       </c>
       <c r="C741" t="inlineStr">
@@ -13045,7 +13045,7 @@
       </c>
       <c r="B743" t="inlineStr">
         <is>
-          <t>Hits for {power} power and inflicts [t]Stun[/t], pushing the enemy back. Costs your turn.</t>
+          <t>Hits for {power} power. [t]Stun[/t] and push back. Costs your turn.</t>
         </is>
       </c>
       <c r="C743" t="inlineStr">
@@ -13062,12 +13062,12 @@
       </c>
       <c r="B744" t="inlineStr">
         <is>
-          <t>Dodge the next attack ({turns} turns). A [a]Perfect[/a] throw lets you slip away. Costs your turn.</t>
+          <t>Dodge for {turns} turns. [a]Perfect[/a]: escape. Costs your turn.</t>
         </is>
       </c>
       <c r="C744" t="inlineStr">
         <is>
-          <t>다음 공격을 피합니다({turns}턴). [a]완벽[/a]하게 던지면 도망칩니다. 턴을 소모합니다.</t>
+          <t>{turns}턴 회피. [a]완벽[/a]하면 도망. 턴을 소모합니다.</t>
         </is>
       </c>
     </row>
@@ -17164,7 +17164,7 @@
       </c>
       <c r="C985" t="inlineStr">
         <is>
-          <t>만난 횟수</t>
+          <t>만남</t>
         </is>
       </c>
     </row>
@@ -17640,7 +17640,7 @@
       </c>
       <c r="C1013" t="inlineStr">
         <is>
-          <t>목격</t>
+          <t>봄</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(hunt7feel): alt-tab freezes the QTE clocks, ko loot/victory text, refusal sound, BREAK layer, world sounds on the SFX bus (R-080..R-084)
- Qte_StepMs adds nothing while the window is out of focus (bar, arrows, defence bar + telegraph, grade word, hit freeze).
- Loot lines get a space after a prefix that ends in a colon; the auto-resolve victory line is the localized row combat.msg.overpower_prefix and its loot line uses combat.msg.loot_prefix.
- Menus take an optional refuse callback: a skill with too little MP, Skill/Item with nothing in the list play ui_deny, not ui_confirm.
- A Perfect BREAK layers sword_impact (lower, softer) under qte_perfect instead of the same sample twice.
- chest, barrel and torch sounds and the new alert_spotted / alert_lost keys (the "!" and "?") are on the SFX bus.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datafiles/localization/game_text.xlsx
+++ b/datafiles/localization/game_text.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1209"/>
+  <dimension ref="A1:C1210"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -20976,6 +20976,23 @@
         </is>
       </c>
     </row>
+    <row r="1210">
+      <c r="A1210" t="inlineStr">
+        <is>
+          <t>combat.msg.overpower_prefix</t>
+        </is>
+      </c>
+      <c r="B1210" t="inlineStr">
+        <is>
+          <t>You overpower {enemy}.</t>
+        </is>
+      </c>
+      <c r="C1210" t="inlineStr">
+        <is>
+          <t>{enemy}을(를) 가볍게 쓰러뜨렸습니다.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C678"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(r3menus): section headers as dark strips, QTE grade words in capitals, Controls reset asks and shows what it changed (R-096, R-097)
Headers (Equipped, Bag, Passives) share one draw: dark strip, pale text, gap above, line under. Reset to Defaults opens the Yes/No confirm, then a notice, then the changed rows blink. Grade words PERFECT/GOOD/OK/WEAK (en), held inside the screen.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datafiles/localization/game_text.xlsx
+++ b/datafiles/localization/game_text.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1210"/>
+  <dimension ref="A1:C1212"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -516,7 +516,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>GOOD</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -550,7 +550,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Perfect</t>
+          <t>PERFECT</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -567,7 +567,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>WEAK</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -20990,6 +20990,40 @@
       <c r="C1210" t="inlineStr">
         <is>
           <t>{enemy}을(를) 가볍게 쓰러뜨렸습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1211">
+      <c r="A1211" t="inlineStr">
+        <is>
+          <t>controls.reset_ask</t>
+        </is>
+      </c>
+      <c r="B1211" t="inlineStr">
+        <is>
+          <t>Reset every key to its default?</t>
+        </is>
+      </c>
+      <c r="C1211" t="inlineStr">
+        <is>
+          <t>모든 키를 기본값으로 되돌릴까요?</t>
+        </is>
+      </c>
+    </row>
+    <row r="1212">
+      <c r="A1212" t="inlineStr">
+        <is>
+          <t>controls.reset_same</t>
+        </is>
+      </c>
+      <c r="B1212" t="inlineStr">
+        <is>
+          <t>Keys were already the defaults.</t>
+        </is>
+      </c>
+      <c r="C1212" t="inlineStr">
+        <is>
+          <t>키가 이미 기본값입니다.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(r3saves1): D175 data layer: profiles index, 3 save files per profile, migration
profiles.sav index (own validator, rebuild + quarantine), profile_<id>.sav and
run_<id>_<slot>.sav; Profile_Path/RunSave_Path follow the active profile and slot.
Profiles_* and Slot(s)_* API, Slots_Summary, Continue target. PROFILE_VERSION 3
(name), RUN_SAVE_VERSION 3 (summary block; v2 loads and migrates in memory).
First launch moves profile.sav/run.sav to profile 1 / save file 1 and keeps the
originals as *.pre-profiles.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datafiles/localization/game_text.xlsx
+++ b/datafiles/localization/game_text.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1211"/>
+  <dimension ref="A1:C1212"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -21010,6 +21010,23 @@
         </is>
       </c>
     </row>
+    <row r="1212">
+      <c r="A1212" t="inlineStr">
+        <is>
+          <t>profile.default_name</t>
+        </is>
+      </c>
+      <c r="B1212" t="inlineStr">
+        <is>
+          <t>Profile</t>
+        </is>
+      </c>
+      <c r="C1212" t="inlineStr">
+        <is>
+          <t>프로필</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C678"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(r3saves2): title model, New Game / Continue / Load Game over three save files (D175, R-107)
Title rows are Continue, New Game, Load Game, Settings, Quit; Continue follows the active profile's last played save file, New Game takes the first empty file (picker + Yes/No when all three are used), Load Game is a three-file picker with a delete key. Old title checks updated to the new row order.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datafiles/localization/game_text.xlsx
+++ b/datafiles/localization/game_text.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1212"/>
+  <dimension ref="A1:C1225"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -21027,6 +21027,227 @@
         </is>
       </c>
     </row>
+    <row r="1213">
+      <c r="A1213" t="inlineStr">
+        <is>
+          <t>save.slot.name</t>
+        </is>
+      </c>
+      <c r="B1213" t="inlineStr">
+        <is>
+          <t>Save {n}</t>
+        </is>
+      </c>
+      <c r="C1213" t="inlineStr">
+        <is>
+          <t>저장 {n}</t>
+        </is>
+      </c>
+    </row>
+    <row r="1214">
+      <c r="A1214" t="inlineStr">
+        <is>
+          <t>save.slot.empty</t>
+        </is>
+      </c>
+      <c r="B1214" t="inlineStr">
+        <is>
+          <t>Empty</t>
+        </is>
+      </c>
+      <c r="C1214" t="inlineStr">
+        <is>
+          <t>비어 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="1215">
+      <c r="A1215" t="inlineStr">
+        <is>
+          <t>save.slot.cant</t>
+        </is>
+      </c>
+      <c r="B1215" t="inlineStr">
+        <is>
+          <t>Cannot load</t>
+        </is>
+      </c>
+      <c r="C1215" t="inlineStr">
+        <is>
+          <t>불러올 수 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="1216">
+      <c r="A1216" t="inlineStr">
+        <is>
+          <t>save.lbl.saved</t>
+        </is>
+      </c>
+      <c r="B1216" t="inlineStr">
+        <is>
+          <t>Last Saved</t>
+        </is>
+      </c>
+      <c r="C1216" t="inlineStr">
+        <is>
+          <t>마지막 저장</t>
+        </is>
+      </c>
+    </row>
+    <row r="1217">
+      <c r="A1217" t="inlineStr">
+        <is>
+          <t>save.slot.help_load</t>
+        </is>
+      </c>
+      <c r="B1217" t="inlineStr">
+        <is>
+          <t>Pick up this run where you left it.</t>
+        </is>
+      </c>
+      <c r="C1217" t="inlineStr">
+        <is>
+          <t>중단한 곳에서 이 도전을 이어갑니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1218">
+      <c r="A1218" t="inlineStr">
+        <is>
+          <t>save.slot.help_over</t>
+        </is>
+      </c>
+      <c r="B1218" t="inlineStr">
+        <is>
+          <t>A new game here replaces this run.</t>
+        </is>
+      </c>
+      <c r="C1218" t="inlineStr">
+        <is>
+          <t>여기서 새 게임을 시작하면 이 도전은 사라집니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1219">
+      <c r="A1219" t="inlineStr">
+        <is>
+          <t>save.slot.help_empty</t>
+        </is>
+      </c>
+      <c r="B1219" t="inlineStr">
+        <is>
+          <t>No run is saved in this file.</t>
+        </is>
+      </c>
+      <c r="C1219" t="inlineStr">
+        <is>
+          <t>이 파일에는 저장된 도전이 없습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1220">
+      <c r="A1220" t="inlineStr">
+        <is>
+          <t>save.overwrite.title</t>
+        </is>
+      </c>
+      <c r="B1220" t="inlineStr">
+        <is>
+          <t>Overwrite which save file?</t>
+        </is>
+      </c>
+      <c r="C1220" t="inlineStr">
+        <is>
+          <t>어느 저장 파일을 덮어쓸까요?</t>
+        </is>
+      </c>
+    </row>
+    <row r="1221">
+      <c r="A1221" t="inlineStr">
+        <is>
+          <t>save.overwrite.ask</t>
+        </is>
+      </c>
+      <c r="B1221" t="inlineStr">
+        <is>
+          <t>Overwrite Save {n}? The run in it will be lost.</t>
+        </is>
+      </c>
+      <c r="C1221" t="inlineStr">
+        <is>
+          <t>저장 {n}을(를) 덮어쓸까요? 그 안의 도전은 사라집니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1222">
+      <c r="A1222" t="inlineStr">
+        <is>
+          <t>save.delete.ask</t>
+        </is>
+      </c>
+      <c r="B1222" t="inlineStr">
+        <is>
+          <t>Delete Save {n}? The run in it will be lost.</t>
+        </is>
+      </c>
+      <c r="C1222" t="inlineStr">
+        <is>
+          <t>저장 {n}을(를) 삭제할까요? 그 안의 도전은 사라집니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1223">
+      <c r="A1223" t="inlineStr">
+        <is>
+          <t>save.hint.load</t>
+        </is>
+      </c>
+      <c r="B1223" t="inlineStr">
+        <is>
+          <t>[k:confirm] Load</t>
+        </is>
+      </c>
+      <c r="C1223" t="inlineStr">
+        <is>
+          <t>[k:confirm] 불러오기</t>
+        </is>
+      </c>
+    </row>
+    <row r="1224">
+      <c r="A1224" t="inlineStr">
+        <is>
+          <t>save.hint.overwrite</t>
+        </is>
+      </c>
+      <c r="B1224" t="inlineStr">
+        <is>
+          <t>[k:confirm] Overwrite</t>
+        </is>
+      </c>
+      <c r="C1224" t="inlineStr">
+        <is>
+          <t>[k:confirm] 덮어쓰기</t>
+        </is>
+      </c>
+    </row>
+    <row r="1225">
+      <c r="A1225" t="inlineStr">
+        <is>
+          <t>save.hint.delete</t>
+        </is>
+      </c>
+      <c r="B1225" t="inlineStr">
+        <is>
+          <t>[k:tab_prev] Delete</t>
+        </is>
+      </c>
+      <c r="C1225" t="inlineStr">
+        <is>
+          <t>[k:tab_prev] 삭제</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C678"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(r3saves2): profile screen, name entry and the title's Profile button (D175)
Q (pad LB) or a click on the lower-left Profile button opens the profile screen: up to four profiles with runs / wins / best floor, switch on confirm, delete after Yes/No, New Profile while fewer than four. The name entry types with the keyboard (letters, digits, space; Backspace, Enter, Esc) and has an on-screen grid for pad and mouse. Pickers fall back to a side-by-side layout when the stacked one would not fit.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datafiles/localization/game_text.xlsx
+++ b/datafiles/localization/game_text.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1225"/>
+  <dimension ref="A1:C1244"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -21248,6 +21248,329 @@
         </is>
       </c>
     </row>
+    <row r="1226">
+      <c r="A1226" t="inlineStr">
+        <is>
+          <t>profile.btn</t>
+        </is>
+      </c>
+      <c r="B1226" t="inlineStr">
+        <is>
+          <t>[k:tab_prev] Profile</t>
+        </is>
+      </c>
+      <c r="C1226" t="inlineStr">
+        <is>
+          <t>[k:tab_prev] 프로필</t>
+        </is>
+      </c>
+    </row>
+    <row r="1227">
+      <c r="A1227" t="inlineStr">
+        <is>
+          <t>profile.title</t>
+        </is>
+      </c>
+      <c r="B1227" t="inlineStr">
+        <is>
+          <t>Profiles</t>
+        </is>
+      </c>
+      <c r="C1227" t="inlineStr">
+        <is>
+          <t>프로필</t>
+        </is>
+      </c>
+    </row>
+    <row r="1228">
+      <c r="A1228" t="inlineStr">
+        <is>
+          <t>profile.row.new</t>
+        </is>
+      </c>
+      <c r="B1228" t="inlineStr">
+        <is>
+          <t>New Profile</t>
+        </is>
+      </c>
+      <c r="C1228" t="inlineStr">
+        <is>
+          <t>새 프로필</t>
+        </is>
+      </c>
+    </row>
+    <row r="1229">
+      <c r="A1229" t="inlineStr">
+        <is>
+          <t>profile.val.active</t>
+        </is>
+      </c>
+      <c r="B1229" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="C1229" t="inlineStr">
+        <is>
+          <t>사용 중</t>
+        </is>
+      </c>
+    </row>
+    <row r="1230">
+      <c r="A1230" t="inlineStr">
+        <is>
+          <t>profile.lbl.runs</t>
+        </is>
+      </c>
+      <c r="B1230" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="C1230" t="inlineStr">
+        <is>
+          <t>도전 횟수</t>
+        </is>
+      </c>
+    </row>
+    <row r="1231">
+      <c r="A1231" t="inlineStr">
+        <is>
+          <t>profile.help.active</t>
+        </is>
+      </c>
+      <c r="B1231" t="inlineStr">
+        <is>
+          <t>The profile in use. Its Codex, run history and story are the ones you see.</t>
+        </is>
+      </c>
+      <c r="C1231" t="inlineStr">
+        <is>
+          <t>지금 쓰는 프로필입니다. 도감, 도전 기록, 이야기는 이 프로필의 것입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1232">
+      <c r="A1232" t="inlineStr">
+        <is>
+          <t>profile.help.other</t>
+        </is>
+      </c>
+      <c r="B1232" t="inlineStr">
+        <is>
+          <t>Switch to this profile. Its Codex, run history, story and save files come with it.</t>
+        </is>
+      </c>
+      <c r="C1232" t="inlineStr">
+        <is>
+          <t>이 프로필로 바꿉니다. 도감, 도전 기록, 이야기, 저장 파일도 함께 바뀝니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1233">
+      <c r="A1233" t="inlineStr">
+        <is>
+          <t>profile.help.new</t>
+        </is>
+      </c>
+      <c r="B1233" t="inlineStr">
+        <is>
+          <t>Start a new profile. Its Codex and run history are empty and the story begins again.</t>
+        </is>
+      </c>
+      <c r="C1233" t="inlineStr">
+        <is>
+          <t>새 프로필을 만듭니다. 도감과 도전 기록은 비어 있고 이야기는 처음부터 시작합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1234">
+      <c r="A1234" t="inlineStr">
+        <is>
+          <t>profile.hint.switch</t>
+        </is>
+      </c>
+      <c r="B1234" t="inlineStr">
+        <is>
+          <t>[k:confirm] Switch</t>
+        </is>
+      </c>
+      <c r="C1234" t="inlineStr">
+        <is>
+          <t>[k:confirm] 바꾸기</t>
+        </is>
+      </c>
+    </row>
+    <row r="1235">
+      <c r="A1235" t="inlineStr">
+        <is>
+          <t>profile.hint.create</t>
+        </is>
+      </c>
+      <c r="B1235" t="inlineStr">
+        <is>
+          <t>[k:confirm] Create</t>
+        </is>
+      </c>
+      <c r="C1235" t="inlineStr">
+        <is>
+          <t>[k:confirm] 만들기</t>
+        </is>
+      </c>
+    </row>
+    <row r="1236">
+      <c r="A1236" t="inlineStr">
+        <is>
+          <t>profile.delete.ask</t>
+        </is>
+      </c>
+      <c r="B1236" t="inlineStr">
+        <is>
+          <t>Delete profile {name}? Its Codex, history and save files are lost.</t>
+        </is>
+      </c>
+      <c r="C1236" t="inlineStr">
+        <is>
+          <t>프로필 {name}을(를) 삭제할까요? 도감, 기록, 저장 파일이 모두 사라집니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1237">
+      <c r="A1237" t="inlineStr">
+        <is>
+          <t>profile.name.need</t>
+        </is>
+      </c>
+      <c r="B1237" t="inlineStr">
+        <is>
+          <t>Enter a name.</t>
+        </is>
+      </c>
+      <c r="C1237" t="inlineStr">
+        <is>
+          <t>이름을 입력하세요.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1238">
+      <c r="A1238" t="inlineStr">
+        <is>
+          <t>profile.name.key_space</t>
+        </is>
+      </c>
+      <c r="B1238" t="inlineStr">
+        <is>
+          <t>Space</t>
+        </is>
+      </c>
+      <c r="C1238" t="inlineStr">
+        <is>
+          <t>띄어쓰기</t>
+        </is>
+      </c>
+    </row>
+    <row r="1239">
+      <c r="A1239" t="inlineStr">
+        <is>
+          <t>profile.name.key_delete</t>
+        </is>
+      </c>
+      <c r="B1239" t="inlineStr">
+        <is>
+          <t>Delete</t>
+        </is>
+      </c>
+      <c r="C1239" t="inlineStr">
+        <is>
+          <t>삭제</t>
+        </is>
+      </c>
+    </row>
+    <row r="1240">
+      <c r="A1240" t="inlineStr">
+        <is>
+          <t>profile.name.key_ok</t>
+        </is>
+      </c>
+      <c r="B1240" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="C1240" t="inlineStr">
+        <is>
+          <t>확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="1241">
+      <c r="A1241" t="inlineStr">
+        <is>
+          <t>profile.name.hint_pick</t>
+        </is>
+      </c>
+      <c r="B1241" t="inlineStr">
+        <is>
+          <t>[k:confirm] Pick</t>
+        </is>
+      </c>
+      <c r="C1241" t="inlineStr">
+        <is>
+          <t>[k:confirm] 선택</t>
+        </is>
+      </c>
+    </row>
+    <row r="1242">
+      <c r="A1242" t="inlineStr">
+        <is>
+          <t>profile.name.hint_cancel</t>
+        </is>
+      </c>
+      <c r="B1242" t="inlineStr">
+        <is>
+          <t>[k:back] Cancel</t>
+        </is>
+      </c>
+      <c r="C1242" t="inlineStr">
+        <is>
+          <t>[k:back] 취소</t>
+        </is>
+      </c>
+    </row>
+    <row r="1243">
+      <c r="A1243" t="inlineStr">
+        <is>
+          <t>profile.name.info_kb</t>
+        </is>
+      </c>
+      <c r="B1243" t="inlineStr">
+        <is>
+          <t>Up to 12 letters. Backspace deletes, Enter finishes.</t>
+        </is>
+      </c>
+      <c r="C1243" t="inlineStr">
+        <is>
+          <t>최대 12자. Backspace로 지우고 Enter로 끝냅니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1244">
+      <c r="A1244" t="inlineStr">
+        <is>
+          <t>profile.name.info_pad</t>
+        </is>
+      </c>
+      <c r="B1244" t="inlineStr">
+        <is>
+          <t>Up to 12 letters. Pick them on the grid.</t>
+        </is>
+      </c>
+      <c r="C1244" t="inlineStr">
+        <is>
+          <t>최대 12자. 칸에서 골라 입력하세요.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C678"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(r3saves2): Codex and Run History button on the title (D175)
E (pad RB, or a click on the button above Profile) opens the active profile's Codex read-only: Bestiary, Notes, Run History, Unlocks with the Tab menu's own rows, pages and fit; Back goes up one level, Back at the list closes it. Corner buttons are hit-tested from the rectangles the draw keeps. Shots 361, shots timeout 700, frame caps raised.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datafiles/localization/game_text.xlsx
+++ b/datafiles/localization/game_text.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1244"/>
+  <dimension ref="A1:C1245"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -21571,6 +21571,23 @@
         </is>
       </c>
     </row>
+    <row r="1245">
+      <c r="A1245" t="inlineStr">
+        <is>
+          <t>codex.btn</t>
+        </is>
+      </c>
+      <c r="B1245" t="inlineStr">
+        <is>
+          <t>[k:tab_next] Codex</t>
+        </is>
+      </c>
+      <c r="C1245" t="inlineStr">
+        <is>
+          <t>[k:tab_next] 도감</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C678"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix(r3guardsmall): Guard halves every hit until the player's next turn starts and restores 25% of max MP, min 2 (D180, R-102)
The Brace is no longer used up by a hit and no longer counts enemy turns: it ends as the
player's next turn starts, once the enemy has had a turn. Guard gives back floor(25% of
max MP), at least 2, capped at max MP; the log and a popup show '+N MP'. Old assertions
that expected one-hit or two-enemy-turn Braces were updated.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datafiles/localization/game_text.xlsx
+++ b/datafiles/localization/game_text.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1212"/>
+  <dimension ref="A1:C1214"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -15782,12 +15782,12 @@
       </c>
       <c r="B904" t="inlineStr">
         <is>
-          <t>Braced for the next hit: it deals {pct}% less damage.</t>
+          <t>Until your next turn every hit you take deals {pct}% less damage.</t>
         </is>
       </c>
       <c r="C904" t="inlineStr">
         <is>
-          <t>다음 공격에 대비합니다. 피해가 {pct}% 줄어듭니다.</t>
+          <t>내 다음 턴까지 받는 모든 공격의 피해가 {pct}% 줄어듭니다.</t>
         </is>
       </c>
     </row>
@@ -21024,6 +21024,40 @@
       <c r="C1212" t="inlineStr">
         <is>
           <t>프로필</t>
+        </is>
+      </c>
+    </row>
+    <row r="1213">
+      <c r="A1213" t="inlineStr">
+        <is>
+          <t>combat.msg.guard_mp</t>
+        </is>
+      </c>
+      <c r="B1213" t="inlineStr">
+        <is>
+          <t>You brace yourself. +{mp} MP</t>
+        </is>
+      </c>
+      <c r="C1213" t="inlineStr">
+        <is>
+          <t>몸을 웅크립니다. MP +{mp}</t>
+        </is>
+      </c>
+    </row>
+    <row r="1214">
+      <c r="A1214" t="inlineStr">
+        <is>
+          <t>combat.pop.guard_mp</t>
+        </is>
+      </c>
+      <c r="B1214" t="inlineStr">
+        <is>
+          <t>+{mp} MP</t>
+        </is>
+      </c>
+      <c r="C1214" t="inlineStr">
+        <is>
+          <t>MP +{mp}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(r3guardsmall): shop rows the bag would refuse (full throwables, gear already owned) are dimmed and say why (R-104)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datafiles/localization/game_text.xlsx
+++ b/datafiles/localization/game_text.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1214"/>
+  <dimension ref="A1:C1216"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -21061,6 +21061,40 @@
         </is>
       </c>
     </row>
+    <row r="1215">
+      <c r="A1215" t="inlineStr">
+        <is>
+          <t>shop.reason.full</t>
+        </is>
+      </c>
+      <c r="B1215" t="inlineStr">
+        <is>
+          <t>Bag full for this item</t>
+        </is>
+      </c>
+      <c r="C1215" t="inlineStr">
+        <is>
+          <t>이 아이템은 더 들 수 없습니다</t>
+        </is>
+      </c>
+    </row>
+    <row r="1216">
+      <c r="A1216" t="inlineStr">
+        <is>
+          <t>shop.reason.owned</t>
+        </is>
+      </c>
+      <c r="B1216" t="inlineStr">
+        <is>
+          <t>Already owned</t>
+        </is>
+      </c>
+      <c r="C1216" t="inlineStr">
+        <is>
+          <t>이미 가지고 있습니다</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C678"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(r3guardsmall): the run-end title varies by death tier, with its own titles for a win and an abandoned run, never the same twice running (D183, R-105)
Three titles per death tier (same tiers and tone as the death lines), three for a win, three
for an abandoned run, en + ko. The profile keeps the key of the last title (last_title).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datafiles/localization/game_text.xlsx
+++ b/datafiles/localization/game_text.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1216"/>
+  <dimension ref="A1:C1236"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -21095,6 +21095,346 @@
         </is>
       </c>
     </row>
+    <row r="1217">
+      <c r="A1217" t="inlineStr">
+        <is>
+          <t>runflow.title.t1.1</t>
+        </is>
+      </c>
+      <c r="B1217" t="inlineStr">
+        <is>
+          <t>The dark closes over you.</t>
+        </is>
+      </c>
+      <c r="C1217" t="inlineStr">
+        <is>
+          <t>어둠이 당신을 덮는다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1218">
+      <c r="A1218" t="inlineStr">
+        <is>
+          <t>runflow.title.t1.2</t>
+        </is>
+      </c>
+      <c r="B1218" t="inlineStr">
+        <is>
+          <t>Is this the end?</t>
+        </is>
+      </c>
+      <c r="C1218" t="inlineStr">
+        <is>
+          <t>이게 끝일까?</t>
+        </is>
+      </c>
+    </row>
+    <row r="1219">
+      <c r="A1219" t="inlineStr">
+        <is>
+          <t>runflow.title.t2.0</t>
+        </is>
+      </c>
+      <c r="B1219" t="inlineStr">
+        <is>
+          <t>Not the end.</t>
+        </is>
+      </c>
+      <c r="C1219" t="inlineStr">
+        <is>
+          <t>끝이 아니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1220">
+      <c r="A1220" t="inlineStr">
+        <is>
+          <t>runflow.title.t2.1</t>
+        </is>
+      </c>
+      <c r="B1220" t="inlineStr">
+        <is>
+          <t>It begins again.</t>
+        </is>
+      </c>
+      <c r="C1220" t="inlineStr">
+        <is>
+          <t>다시 시작된다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1221">
+      <c r="A1221" t="inlineStr">
+        <is>
+          <t>runflow.title.t2.2</t>
+        </is>
+      </c>
+      <c r="B1221" t="inlineStr">
+        <is>
+          <t>Back so soon.</t>
+        </is>
+      </c>
+      <c r="C1221" t="inlineStr">
+        <is>
+          <t>벌써 돌아왔다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1222">
+      <c r="A1222" t="inlineStr">
+        <is>
+          <t>runflow.title.t3.0</t>
+        </is>
+      </c>
+      <c r="B1222" t="inlineStr">
+        <is>
+          <t>You know the way.</t>
+        </is>
+      </c>
+      <c r="C1222" t="inlineStr">
+        <is>
+          <t>길을 안다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1223">
+      <c r="A1223" t="inlineStr">
+        <is>
+          <t>runflow.title.t3.1</t>
+        </is>
+      </c>
+      <c r="B1223" t="inlineStr">
+        <is>
+          <t>The same fall.</t>
+        </is>
+      </c>
+      <c r="C1223" t="inlineStr">
+        <is>
+          <t>같은 추락.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1224">
+      <c r="A1224" t="inlineStr">
+        <is>
+          <t>runflow.title.t3.2</t>
+        </is>
+      </c>
+      <c r="B1224" t="inlineStr">
+        <is>
+          <t>Down, once more.</t>
+        </is>
+      </c>
+      <c r="C1224" t="inlineStr">
+        <is>
+          <t>다시, 아래로.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1225">
+      <c r="A1225" t="inlineStr">
+        <is>
+          <t>runflow.title.t4.0</t>
+        </is>
+      </c>
+      <c r="B1225" t="inlineStr">
+        <is>
+          <t>Nothing new.</t>
+        </is>
+      </c>
+      <c r="C1225" t="inlineStr">
+        <is>
+          <t>새로울 것 없다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1226">
+      <c r="A1226" t="inlineStr">
+        <is>
+          <t>runflow.title.t4.1</t>
+        </is>
+      </c>
+      <c r="B1226" t="inlineStr">
+        <is>
+          <t>Quiet again.</t>
+        </is>
+      </c>
+      <c r="C1226" t="inlineStr">
+        <is>
+          <t>다시 고요하다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1227">
+      <c r="A1227" t="inlineStr">
+        <is>
+          <t>runflow.title.t4.2</t>
+        </is>
+      </c>
+      <c r="B1227" t="inlineStr">
+        <is>
+          <t>No one came.</t>
+        </is>
+      </c>
+      <c r="C1227" t="inlineStr">
+        <is>
+          <t>아무도 오지 않았다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1228">
+      <c r="A1228" t="inlineStr">
+        <is>
+          <t>runflow.title.t5.0</t>
+        </is>
+      </c>
+      <c r="B1228" t="inlineStr">
+        <is>
+          <t>Home again.</t>
+        </is>
+      </c>
+      <c r="C1228" t="inlineStr">
+        <is>
+          <t>다시 집이다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1229">
+      <c r="A1229" t="inlineStr">
+        <is>
+          <t>runflow.title.t5.1</t>
+        </is>
+      </c>
+      <c r="B1229" t="inlineStr">
+        <is>
+          <t>As expected.</t>
+        </is>
+      </c>
+      <c r="C1229" t="inlineStr">
+        <is>
+          <t>짐작대로다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1230">
+      <c r="A1230" t="inlineStr">
+        <is>
+          <t>runflow.title.t5.2</t>
+        </is>
+      </c>
+      <c r="B1230" t="inlineStr">
+        <is>
+          <t>You stay.</t>
+        </is>
+      </c>
+      <c r="C1230" t="inlineStr">
+        <is>
+          <t>당신은 남는다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1231">
+      <c r="A1231" t="inlineStr">
+        <is>
+          <t>runflow.title.won.0</t>
+        </is>
+      </c>
+      <c r="B1231" t="inlineStr">
+        <is>
+          <t>The choir falls silent.</t>
+        </is>
+      </c>
+      <c r="C1231" t="inlineStr">
+        <is>
+          <t>성가대가 침묵한다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1232">
+      <c r="A1232" t="inlineStr">
+        <is>
+          <t>runflow.title.won.1</t>
+        </is>
+      </c>
+      <c r="B1232" t="inlineStr">
+        <is>
+          <t>The tunnel lets go.</t>
+        </is>
+      </c>
+      <c r="C1232" t="inlineStr">
+        <is>
+          <t>터널이 당신을 놓아준다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1233">
+      <c r="A1233" t="inlineStr">
+        <is>
+          <t>runflow.title.won.2</t>
+        </is>
+      </c>
+      <c r="B1233" t="inlineStr">
+        <is>
+          <t>The way is open.</t>
+        </is>
+      </c>
+      <c r="C1233" t="inlineStr">
+        <is>
+          <t>길이 열렸다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1234">
+      <c r="A1234" t="inlineStr">
+        <is>
+          <t>runflow.title.abandoned.0</t>
+        </is>
+      </c>
+      <c r="B1234" t="inlineStr">
+        <is>
+          <t>You let go.</t>
+        </is>
+      </c>
+      <c r="C1234" t="inlineStr">
+        <is>
+          <t>당신은 손을 놓았다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1235">
+      <c r="A1235" t="inlineStr">
+        <is>
+          <t>runflow.title.abandoned.1</t>
+        </is>
+      </c>
+      <c r="B1235" t="inlineStr">
+        <is>
+          <t>The tunnel waits.</t>
+        </is>
+      </c>
+      <c r="C1235" t="inlineStr">
+        <is>
+          <t>터널은 기다린다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1236">
+      <c r="A1236" t="inlineStr">
+        <is>
+          <t>runflow.title.abandoned.2</t>
+        </is>
+      </c>
+      <c r="B1236" t="inlineStr">
+        <is>
+          <t>You turned back.</t>
+        </is>
+      </c>
+      <c r="C1236" t="inlineStr">
+        <is>
+          <t>당신은 돌아섰다.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C678"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(r3rarity): item rarity colours and gems: Item_Rarity, [r1]/[r2]/[r3] name markup, every item message via Item_NameMarked, rarity row colours, icon gems (R-110)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datafiles/localization/game_text.xlsx
+++ b/datafiles/localization/game_text.xlsx
@@ -2964,12 +2964,12 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Received [a]{item}[/a] x{qty}.</t>
+          <t>Received {item} x{qty}.</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>[a]{item}[/a] x{qty}을(를) 받았습니다.</t>
+          <t>{item} x{qty}을(를) 받았습니다.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(r3levelup): VIG and MND stats make Max HP and Max MP; run save version 4 (D176, D184)
Max HP comes from VIG (3 per point, then 2, then 1) and Max MP from MND (1 per point, then 1/2,
then 1/4); every class starts at VIG 10 and MND 11/12/16/11. Class growth lists VIG and MND, tuned
to stay within 10% of the old HP/MP at every level, the Mage the most fragile. MAG no longer adds
MP. The free point may go to VIG or MND (the Max HP +3 / Max MP +2 rows are gone). A run save of
version 2 or 3 migrates in place: hp_bonus/3 and mp_bonus/2 become VIG/MND points on top of the
class's own growth. Status tab, Help and the stat prompt show VIG and MND with one-line texts.
Old-behaviour assertions updated (Status row counts, growth lines, free-point rows, save version).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datafiles/localization/game_text.xlsx
+++ b/datafiles/localization/game_text.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1245"/>
+  <dimension ref="A1:C1249"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -6500,12 +6500,12 @@
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>Increases spell damage and max [t]MP[/t].</t>
+          <t>Increases spell damage.</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>마법 피해와 최대 [t]MP[/t]를 늘립니다.</t>
+          <t>마법 피해를 늘립니다.</t>
         </is>
       </c>
     </row>
@@ -19029,12 +19029,12 @@
       </c>
       <c r="B1095" t="inlineStr">
         <is>
-          <t>What Power, ATK, DEF, MAG, SPD, Crit, the grades, BREAK and every status mean.</t>
+          <t>What Power, ATK, DEF, MAG, SPD, VIG, MND, Crit, the grades, BREAK and every status mean.</t>
         </is>
       </c>
       <c r="C1095" t="inlineStr">
         <is>
-          <t>위력, ATK, DEF, MAG, SPD, 치명타, 등급, 브레이크와 모든 상태 이상의 뜻입니다.</t>
+          <t>위력, ATK, DEF, MAG, SPD, VIG, MND, 치명타, 등급, 브레이크와 모든 상태 이상의 뜻입니다.</t>
         </is>
       </c>
     </row>
@@ -21585,6 +21585,74 @@
       <c r="C1245" t="inlineStr">
         <is>
           <t>[k:tab_next] 도감</t>
+        </is>
+      </c>
+    </row>
+    <row r="1246">
+      <c r="A1246" t="inlineStr">
+        <is>
+          <t>menu.tooltip.stat.vig.desc</t>
+        </is>
+      </c>
+      <c r="B1246" t="inlineStr">
+        <is>
+          <t>Raises max [t]HP[/t]. The more you add, the less each point gives.</t>
+        </is>
+      </c>
+      <c r="C1246" t="inlineStr">
+        <is>
+          <t>최대 [t]HP[/t]를 늘립니다. 많이 올릴수록 포인트 하나의 효과는 줄어듭니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1247">
+      <c r="A1247" t="inlineStr">
+        <is>
+          <t>menu.tooltip.stat.mnd.desc</t>
+        </is>
+      </c>
+      <c r="B1247" t="inlineStr">
+        <is>
+          <t>Raises max [t]MP[/t]. The more you add, the less each point gives.</t>
+        </is>
+      </c>
+      <c r="C1247" t="inlineStr">
+        <is>
+          <t>최대 [t]MP[/t]를 늘립니다. 많이 올릴수록 포인트 하나의 효과는 줄어듭니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1248">
+      <c r="A1248" t="inlineStr">
+        <is>
+          <t>tab.lbl.max_hp</t>
+        </is>
+      </c>
+      <c r="B1248" t="inlineStr">
+        <is>
+          <t>Max HP</t>
+        </is>
+      </c>
+      <c r="C1248" t="inlineStr">
+        <is>
+          <t>최대 HP</t>
+        </is>
+      </c>
+    </row>
+    <row r="1249">
+      <c r="A1249" t="inlineStr">
+        <is>
+          <t>tab.lbl.max_mp</t>
+        </is>
+      </c>
+      <c r="B1249" t="inlineStr">
+        <is>
+          <t>Max MP</t>
+        </is>
+      </c>
+      <c r="C1249" t="inlineStr">
+        <is>
+          <t>최대 MP</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(r3levelup): level gains wait for the level-up screen; the confirm gives level + growth + the point (D177, note 14)
Winning a fight in a run only owes levels (ch.levels_owed): level, stats, Max HP/MP, banked points
and card picks stay as they were; the EXP bar fills and says Level Up. The screen is for the next
owed level (one screen per level); Cards_PlaceStat applies it on confirm (class growth, one free
point, one card pick) and raises the current HP/MP by what VIG/MND added. Outside a run EXP still
levels at once. A death before the screen, the history and the save summary count the owed levels
(Player_EffLevel); a load, a class change and the cap keep the debt. last_stat_points_gained is
set (R-113). tools/balance: sim.py plays VIG/MND (constants.vigmnd), vig_mnd.py is the reference.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datafiles/localization/game_text.xlsx
+++ b/datafiles/localization/game_text.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1249"/>
+  <dimension ref="A1:C1250"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -21656,6 +21656,23 @@
         </is>
       </c>
     </row>
+    <row r="1250">
+      <c r="A1250" t="inlineStr">
+        <is>
+          <t>tab.val.level_up</t>
+        </is>
+      </c>
+      <c r="B1250" t="inlineStr">
+        <is>
+          <t>Level Up</t>
+        </is>
+      </c>
+      <c r="C1250" t="inlineStr">
+        <is>
+          <t>레벨 업</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C678"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(r3levelup): the level-up screen: gold growth rows, +1 on the hovered row, VIG/MND details (D177, note 15)
Rows ATK DEF SPD MAG VIG MND. The class's growth rows are gold and read now > now+growth (Mage:
MAG, VIG, MND; Knight: ATK, DEF, VIG, MND ...); the others read only the number; the row under the
cursor (keys or mouse) adds its +1 (a growth row now > now+growth+1). The 'Knight growth' line is a
gold legend. Details: what the stat does, Now / After (VIG: Max HP, MND: Max MP), class growth and
the point counted. Fits at 480/640/800 in en and ko (TextFit + pictures 1100..1103). The growth
text function and the Max HP/MP row strings are gone. The simulator snapshot is re-exported
(VIG/MND by_level, parity with the vectors); the combat spec says Max HP/MP are VIG/MND.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datafiles/localization/game_text.xlsx
+++ b/datafiles/localization/game_text.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1250"/>
+  <dimension ref="A1:C1249"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -18072,2030 +18072,2030 @@
     <row r="1039">
       <c r="A1039" t="inlineStr">
         <is>
-          <t>levelup.gain</t>
+          <t>tab.system</t>
         </is>
       </c>
       <c r="B1039" t="inlineStr">
         <is>
-          <t>{stat} +{n}</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C1039" t="inlineStr">
         <is>
-          <t>{stat} +{n}</t>
+          <t>시스템</t>
         </is>
       </c>
     </row>
     <row r="1040">
       <c r="A1040" t="inlineStr">
         <is>
-          <t>levelup.growth</t>
+          <t>tab.title.system</t>
         </is>
       </c>
       <c r="B1040" t="inlineStr">
         <is>
-          <t>{name} growth: {gains}</t>
+          <t>System</t>
         </is>
       </c>
       <c r="C1040" t="inlineStr">
         <is>
-          <t>{name} 성장: {gains}</t>
+          <t>시스템</t>
         </is>
       </c>
     </row>
     <row r="1041">
       <c r="A1041" t="inlineStr">
         <is>
-          <t>cards.stat.maxhp</t>
+          <t>tab.system.quit_battle_help</t>
         </is>
       </c>
       <c r="B1041" t="inlineStr">
         <is>
-          <t>Max HP +{n}</t>
+          <t>Goes back to the title. Continue puts you back just before this battle.</t>
         </is>
       </c>
       <c r="C1041" t="inlineStr">
         <is>
-          <t>최대 HP +{n}</t>
+          <t>타이틀로 나갑니다. 이어하기를 하면 이 전투 직전부터 다시 시작합니다.</t>
         </is>
       </c>
     </row>
     <row r="1042">
       <c r="A1042" t="inlineStr">
         <is>
-          <t>cards.stat.maxmp</t>
+          <t>settings.keep.title</t>
         </is>
       </c>
       <c r="B1042" t="inlineStr">
         <is>
-          <t>Max MP +{n}</t>
+          <t>Keep This Setting?</t>
         </is>
       </c>
       <c r="C1042" t="inlineStr">
         <is>
-          <t>최대 MP +{n}</t>
+          <t>이 설정을 유지할까요?</t>
         </is>
       </c>
     </row>
     <row r="1043">
       <c r="A1043" t="inlineStr">
         <is>
-          <t>cards.stat.maxhp.desc</t>
+          <t>settings.keep.body</t>
         </is>
       </c>
       <c r="B1043" t="inlineStr">
         <is>
-          <t>Raises your max [t]HP[/t] by {n} and restores {n} [t]HP[/t].</t>
+          <t>It goes back by itself in {n} s.</t>
         </is>
       </c>
       <c r="C1043" t="inlineStr">
         <is>
-          <t>최대 [t]HP[/t]가 {n} 오르고 [t]HP[/t]를 {n} 회복합니다.</t>
+          <t>{n}초 뒤에 자동으로 원래대로 돌아갑니다.</t>
         </is>
       </c>
     </row>
     <row r="1044">
       <c r="A1044" t="inlineStr">
         <is>
-          <t>cards.stat.maxmp.desc</t>
+          <t>settings.keep.hint</t>
         </is>
       </c>
       <c r="B1044" t="inlineStr">
         <is>
-          <t>Raises your max [t]MP[/t] by {n} and restores {n} [t]MP[/t].</t>
+          <t>[k:confirm] Keep   [k:back] Revert</t>
         </is>
       </c>
       <c r="C1044" t="inlineStr">
         <is>
-          <t>최대 [t]MP[/t]가 {n} 오르고 [t]MP[/t]를 {n} 회복합니다.</t>
+          <t>[k:confirm] 유지   [k:back] 되돌리기</t>
         </is>
       </c>
     </row>
     <row r="1045">
       <c r="A1045" t="inlineStr">
         <is>
-          <t>tab.system</t>
+          <t>seed.choice.title</t>
         </is>
       </c>
       <c r="B1045" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>Choose a Seed</t>
         </is>
       </c>
       <c r="C1045" t="inlineStr">
         <is>
-          <t>시스템</t>
+          <t>시드 선택</t>
         </is>
       </c>
     </row>
     <row r="1046">
       <c r="A1046" t="inlineStr">
         <is>
-          <t>tab.title.system</t>
+          <t>seed.choice.random</t>
         </is>
       </c>
       <c r="B1046" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>Random Seed</t>
         </is>
       </c>
       <c r="C1046" t="inlineStr">
         <is>
-          <t>시스템</t>
+          <t>무작위 시드</t>
         </is>
       </c>
     </row>
     <row r="1047">
       <c r="A1047" t="inlineStr">
         <is>
-          <t>tab.system.quit_battle_help</t>
+          <t>seed.choice.enter</t>
         </is>
       </c>
       <c r="B1047" t="inlineStr">
         <is>
-          <t>Goes back to the title. Continue puts you back just before this battle.</t>
+          <t>Enter Seed</t>
         </is>
       </c>
       <c r="C1047" t="inlineStr">
         <is>
-          <t>타이틀로 나갑니다. 이어하기를 하면 이 전투 직전부터 다시 시작합니다.</t>
+          <t>시드 입력</t>
         </is>
       </c>
     </row>
     <row r="1048">
       <c r="A1048" t="inlineStr">
         <is>
-          <t>settings.keep.title</t>
+          <t>seed.entry.title</t>
         </is>
       </c>
       <c r="B1048" t="inlineStr">
         <is>
-          <t>Keep This Setting?</t>
+          <t>Enter Seed</t>
         </is>
       </c>
       <c r="C1048" t="inlineStr">
         <is>
-          <t>이 설정을 유지할까요?</t>
+          <t>시드 입력</t>
         </is>
       </c>
     </row>
     <row r="1049">
       <c r="A1049" t="inlineStr">
         <is>
-          <t>settings.keep.body</t>
+          <t>seed.entry.info</t>
         </is>
       </c>
       <c r="B1049" t="inlineStr">
         <is>
-          <t>It goes back by itself in {n} s.</t>
+          <t>Up to 9 digits. Same seed, same run.</t>
         </is>
       </c>
       <c r="C1049" t="inlineStr">
         <is>
-          <t>{n}초 뒤에 자동으로 원래대로 돌아갑니다.</t>
+          <t>최대 9자리. 같은 시드, 같은 도전.</t>
         </is>
       </c>
     </row>
     <row r="1050">
       <c r="A1050" t="inlineStr">
         <is>
-          <t>settings.keep.hint</t>
+          <t>seed.entry.need</t>
         </is>
       </c>
       <c r="B1050" t="inlineStr">
         <is>
-          <t>[k:confirm] Keep   [k:back] Revert</t>
+          <t>Enter a seed above zero.</t>
         </is>
       </c>
       <c r="C1050" t="inlineStr">
         <is>
-          <t>[k:confirm] 유지   [k:back] 되돌리기</t>
+          <t>0보다 큰 시드를 입력하세요.</t>
         </is>
       </c>
     </row>
     <row r="1051">
       <c r="A1051" t="inlineStr">
         <is>
-          <t>seed.choice.title</t>
+          <t>seed.entry.hint</t>
         </is>
       </c>
       <c r="B1051" t="inlineStr">
         <is>
-          <t>Choose a Seed</t>
+          <t>[k:up][k:down] Digit   [k:left][k:right] Move</t>
         </is>
       </c>
       <c r="C1051" t="inlineStr">
         <is>
-          <t>시드 선택</t>
+          <t>[k:up][k:down] 숫자   [k:left][k:right] 이동</t>
         </is>
       </c>
     </row>
     <row r="1052">
       <c r="A1052" t="inlineStr">
         <is>
-          <t>seed.choice.random</t>
+          <t>seed.entry.hint2</t>
         </is>
       </c>
       <c r="B1052" t="inlineStr">
         <is>
-          <t>Random Seed</t>
+          <t>[k:confirm] Start</t>
         </is>
       </c>
       <c r="C1052" t="inlineStr">
         <is>
-          <t>무작위 시드</t>
+          <t>[k:confirm] 시작</t>
         </is>
       </c>
     </row>
     <row r="1053">
       <c r="A1053" t="inlineStr">
         <is>
-          <t>seed.choice.enter</t>
+          <t>seed.entry.hint3</t>
         </is>
       </c>
       <c r="B1053" t="inlineStr">
         <is>
-          <t>Enter Seed</t>
+          <t>[k:back] Back   [k:tab_prev] Delete</t>
         </is>
       </c>
       <c r="C1053" t="inlineStr">
         <is>
-          <t>시드 입력</t>
+          <t>[k:back] 뒤로   [k:tab_prev] 삭제</t>
         </is>
       </c>
     </row>
     <row r="1054">
       <c r="A1054" t="inlineStr">
         <is>
-          <t>seed.entry.title</t>
+          <t>confirm.abandon</t>
         </is>
       </c>
       <c r="B1054" t="inlineStr">
         <is>
-          <t>Enter Seed</t>
+          <t>Abandon this run? It counts as a death, but you keep the echo.</t>
         </is>
       </c>
       <c r="C1054" t="inlineStr">
         <is>
-          <t>시드 입력</t>
+          <t>이번 도전을 포기할까요? 죽은 것으로 기록되지만 메아리는 남습니다.</t>
         </is>
       </c>
     </row>
     <row r="1055">
       <c r="A1055" t="inlineStr">
         <is>
-          <t>seed.entry.info</t>
+          <t>confirm.quit</t>
         </is>
       </c>
       <c r="B1055" t="inlineStr">
         <is>
-          <t>Up to 9 digits. Same seed, same run.</t>
+          <t>Quit to title? The run is saved and Continue picks it up again.</t>
         </is>
       </c>
       <c r="C1055" t="inlineStr">
         <is>
-          <t>최대 9자리. 같은 시드, 같은 도전.</t>
+          <t>타이틀로 나갈까요? 도전은 저장되며 이어하기로 계속할 수 있습니다.</t>
         </is>
       </c>
     </row>
     <row r="1056">
       <c r="A1056" t="inlineStr">
         <is>
-          <t>seed.entry.need</t>
+          <t>confirm.quit_battle</t>
         </is>
       </c>
       <c r="B1056" t="inlineStr">
         <is>
-          <t>Enter a seed above zero.</t>
+          <t>Quit to title? Continue puts you back just before this battle.</t>
         </is>
       </c>
       <c r="C1056" t="inlineStr">
         <is>
-          <t>0보다 큰 시드를 입력하세요.</t>
+          <t>타이틀로 나갈까요? 이어하기를 하면 이 전투 직전으로 돌아옵니다.</t>
         </is>
       </c>
     </row>
     <row r="1057">
       <c r="A1057" t="inlineStr">
         <is>
-          <t>seed.entry.hint</t>
+          <t>confirm.new_game</t>
         </is>
       </c>
       <c r="B1057" t="inlineStr">
         <is>
-          <t>[k:up][k:down] Digit   [k:left][k:right] Move</t>
+          <t>Start a new game? The saved run will be abandoned.</t>
         </is>
       </c>
       <c r="C1057" t="inlineStr">
         <is>
-          <t>[k:up][k:down] 숫자   [k:left][k:right] 이동</t>
+          <t>새 게임을 시작할까요? 저장된 도전은 사라집니다.</t>
         </is>
       </c>
     </row>
     <row r="1058">
       <c r="A1058" t="inlineStr">
         <is>
-          <t>seed.entry.hint2</t>
+          <t>confirm.echo</t>
         </is>
       </c>
       <c r="B1058" t="inlineStr">
         <is>
-          <t>[k:confirm] Start</t>
+          <t>Keep {name} as your echo?</t>
         </is>
       </c>
       <c r="C1058" t="inlineStr">
         <is>
-          <t>[k:confirm] 시작</t>
+          <t>{name}을(를) 메아리로 남길까요?</t>
         </is>
       </c>
     </row>
     <row r="1059">
       <c r="A1059" t="inlineStr">
         <is>
-          <t>seed.entry.hint3</t>
+          <t>confirm.replace</t>
         </is>
       </c>
       <c r="B1059" t="inlineStr">
         <is>
-          <t>[k:back] Back   [k:tab_prev] Delete</t>
+          <t>Forget {forget} and learn {learn}?</t>
         </is>
       </c>
       <c r="C1059" t="inlineStr">
         <is>
-          <t>[k:back] 뒤로   [k:tab_prev] 삭제</t>
+          <t>{forget}을(를) 잊고 {learn}을(를) 배울까요?</t>
         </is>
       </c>
     </row>
     <row r="1060">
       <c r="A1060" t="inlineStr">
         <is>
-          <t>confirm.abandon</t>
+          <t>confirm.sell</t>
         </is>
       </c>
       <c r="B1060" t="inlineStr">
         <is>
-          <t>Abandon this run? It counts as a death, but you keep the echo.</t>
+          <t>Sell {name} for {price}?</t>
         </is>
       </c>
       <c r="C1060" t="inlineStr">
         <is>
-          <t>이번 도전을 포기할까요? 죽은 것으로 기록되지만 메아리는 남습니다.</t>
+          <t>{name}을(를) {price}에 팔까요?</t>
         </is>
       </c>
     </row>
     <row r="1061">
       <c r="A1061" t="inlineStr">
         <is>
-          <t>confirm.quit</t>
+          <t>tab.hint.read</t>
         </is>
       </c>
       <c r="B1061" t="inlineStr">
         <is>
-          <t>Quit to title? The run is saved and Continue picks it up again.</t>
+          <t>[k:confirm] Read</t>
         </is>
       </c>
       <c r="C1061" t="inlineStr">
         <is>
-          <t>타이틀로 나갈까요? 도전은 저장되며 이어하기로 계속할 수 있습니다.</t>
+          <t>[k:confirm] 읽기</t>
         </is>
       </c>
     </row>
     <row r="1062">
       <c r="A1062" t="inlineStr">
         <is>
-          <t>confirm.quit_battle</t>
+          <t>tab.hint.scroll</t>
         </is>
       </c>
       <c r="B1062" t="inlineStr">
         <is>
-          <t>Quit to title? Continue puts you back just before this battle.</t>
+          <t>[k:up][k:down] Scroll</t>
         </is>
       </c>
       <c r="C1062" t="inlineStr">
         <is>
-          <t>타이틀로 나갈까요? 이어하기를 하면 이 전투 직전으로 돌아옵니다.</t>
+          <t>[k:up][k:down] 넘기기</t>
         </is>
       </c>
     </row>
     <row r="1063">
       <c r="A1063" t="inlineStr">
         <is>
-          <t>confirm.new_game</t>
+          <t>note.found</t>
         </is>
       </c>
       <c r="B1063" t="inlineStr">
         <is>
-          <t>Start a new game? The saved run will be abandoned.</t>
+          <t>Note found: {title}</t>
         </is>
       </c>
       <c r="C1063" t="inlineStr">
         <is>
-          <t>새 게임을 시작할까요? 저장된 도전은 사라집니다.</t>
+          <t>쪽지를 찾았다: {title}</t>
         </is>
       </c>
     </row>
     <row r="1064">
       <c r="A1064" t="inlineStr">
         <is>
-          <t>confirm.echo</t>
+          <t>class.skill.unknown</t>
         </is>
       </c>
       <c r="B1064" t="inlineStr">
         <is>
-          <t>Keep {name} as your echo?</t>
+          <t>???</t>
         </is>
       </c>
       <c r="C1064" t="inlineStr">
         <is>
-          <t>{name}을(를) 메아리로 남길까요?</t>
+          <t>???</t>
         </is>
       </c>
     </row>
     <row r="1065">
       <c r="A1065" t="inlineStr">
         <is>
-          <t>confirm.replace</t>
+          <t>status.short.status_poison</t>
         </is>
       </c>
       <c r="B1065" t="inlineStr">
         <is>
-          <t>Forget {forget} and learn {learn}?</t>
+          <t>PSN</t>
         </is>
       </c>
       <c r="C1065" t="inlineStr">
         <is>
-          <t>{forget}을(를) 잊고 {learn}을(를) 배울까요?</t>
+          <t>독</t>
         </is>
       </c>
     </row>
     <row r="1066">
       <c r="A1066" t="inlineStr">
         <is>
-          <t>confirm.sell</t>
+          <t>status.short.status_bleed</t>
         </is>
       </c>
       <c r="B1066" t="inlineStr">
         <is>
-          <t>Sell {name} for {price}?</t>
+          <t>BLD</t>
         </is>
       </c>
       <c r="C1066" t="inlineStr">
         <is>
-          <t>{name}을(를) {price}에 팔까요?</t>
+          <t>출혈</t>
         </is>
       </c>
     </row>
     <row r="1067">
       <c r="A1067" t="inlineStr">
         <is>
-          <t>tab.hint.read</t>
+          <t>status.short.status_burn</t>
         </is>
       </c>
       <c r="B1067" t="inlineStr">
         <is>
-          <t>[k:confirm] Read</t>
+          <t>BRN</t>
         </is>
       </c>
       <c r="C1067" t="inlineStr">
         <is>
-          <t>[k:confirm] 읽기</t>
+          <t>화상</t>
         </is>
       </c>
     </row>
     <row r="1068">
       <c r="A1068" t="inlineStr">
         <is>
-          <t>tab.hint.scroll</t>
+          <t>status.short.status_stun</t>
         </is>
       </c>
       <c r="B1068" t="inlineStr">
         <is>
-          <t>[k:up][k:down] Scroll</t>
+          <t>STN</t>
         </is>
       </c>
       <c r="C1068" t="inlineStr">
         <is>
-          <t>[k:up][k:down] 넘기기</t>
+          <t>기절</t>
         </is>
       </c>
     </row>
     <row r="1069">
       <c r="A1069" t="inlineStr">
         <is>
-          <t>note.found</t>
+          <t>status.short.status_guard</t>
         </is>
       </c>
       <c r="B1069" t="inlineStr">
         <is>
-          <t>Note found: {title}</t>
+          <t>GRD</t>
         </is>
       </c>
       <c r="C1069" t="inlineStr">
         <is>
-          <t>쪽지를 찾았다: {title}</t>
+          <t>방어</t>
         </is>
       </c>
     </row>
     <row r="1070">
       <c r="A1070" t="inlineStr">
         <is>
-          <t>class.skill.unknown</t>
+          <t>status.short.status_dmg_up</t>
         </is>
       </c>
       <c r="B1070" t="inlineStr">
         <is>
-          <t>???</t>
+          <t>REV</t>
         </is>
       </c>
       <c r="C1070" t="inlineStr">
         <is>
-          <t>???</t>
+          <t>기세</t>
         </is>
       </c>
     </row>
     <row r="1071">
       <c r="A1071" t="inlineStr">
         <is>
-          <t>status.short.status_poison</t>
+          <t>status.short.status_evasion</t>
         </is>
       </c>
       <c r="B1071" t="inlineStr">
         <is>
-          <t>PSN</t>
+          <t>EVA</t>
         </is>
       </c>
       <c r="C1071" t="inlineStr">
         <is>
-          <t>독</t>
+          <t>회피</t>
         </is>
       </c>
     </row>
     <row r="1072">
       <c r="A1072" t="inlineStr">
         <is>
-          <t>status.short.status_bleed</t>
+          <t>status.short.status_crit_up</t>
         </is>
       </c>
       <c r="B1072" t="inlineStr">
         <is>
-          <t>BLD</t>
+          <t>AIM</t>
         </is>
       </c>
       <c r="C1072" t="inlineStr">
         <is>
-          <t>출혈</t>
+          <t>조준</t>
         </is>
       </c>
     </row>
     <row r="1073">
       <c r="A1073" t="inlineStr">
         <is>
-          <t>status.short.status_burn</t>
+          <t>status.short.status_hit_up</t>
         </is>
       </c>
       <c r="B1073" t="inlineStr">
         <is>
-          <t>BRN</t>
+          <t>FORE</t>
         </is>
       </c>
       <c r="C1073" t="inlineStr">
         <is>
-          <t>화상</t>
+          <t>선견</t>
         </is>
       </c>
     </row>
     <row r="1074">
       <c r="A1074" t="inlineStr">
         <is>
-          <t>status.short.status_stun</t>
+          <t>status.short.status_meditation</t>
         </is>
       </c>
       <c r="B1074" t="inlineStr">
         <is>
-          <t>STN</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="C1074" t="inlineStr">
         <is>
-          <t>기절</t>
+          <t>명상</t>
         </is>
       </c>
     </row>
     <row r="1075">
       <c r="A1075" t="inlineStr">
         <is>
-          <t>status.short.status_guard</t>
+          <t>status.short.status_solidify</t>
         </is>
       </c>
       <c r="B1075" t="inlineStr">
         <is>
-          <t>GRD</t>
+          <t>Solid</t>
         </is>
       </c>
       <c r="C1075" t="inlineStr">
         <is>
-          <t>방어</t>
+          <t>굳힘</t>
         </is>
       </c>
     </row>
     <row r="1076">
       <c r="A1076" t="inlineStr">
         <is>
-          <t>status.short.status_dmg_up</t>
+          <t>status.short.status_bloodthirsty</t>
         </is>
       </c>
       <c r="B1076" t="inlineStr">
         <is>
-          <t>REV</t>
+          <t>Thirst</t>
         </is>
       </c>
       <c r="C1076" t="inlineStr">
         <is>
-          <t>기세</t>
+          <t>갈증</t>
         </is>
       </c>
     </row>
     <row r="1077">
       <c r="A1077" t="inlineStr">
         <is>
-          <t>status.short.status_evasion</t>
+          <t>status.short.status_blessing</t>
         </is>
       </c>
       <c r="B1077" t="inlineStr">
         <is>
-          <t>EVA</t>
+          <t>Bless</t>
         </is>
       </c>
       <c r="C1077" t="inlineStr">
         <is>
-          <t>회피</t>
+          <t>축복</t>
         </is>
       </c>
     </row>
     <row r="1078">
       <c r="A1078" t="inlineStr">
         <is>
-          <t>status.short.status_crit_up</t>
+          <t>status.short.status_sunder</t>
         </is>
       </c>
       <c r="B1078" t="inlineStr">
         <is>
-          <t>AIM</t>
+          <t>Sunder</t>
         </is>
       </c>
       <c r="C1078" t="inlineStr">
         <is>
-          <t>조준</t>
+          <t>분쇄</t>
         </is>
       </c>
     </row>
     <row r="1079">
       <c r="A1079" t="inlineStr">
         <is>
-          <t>status.short.status_hit_up</t>
+          <t>status.short.status_brace</t>
         </is>
       </c>
       <c r="B1079" t="inlineStr">
         <is>
-          <t>FORE</t>
+          <t>Brace</t>
         </is>
       </c>
       <c r="C1079" t="inlineStr">
         <is>
-          <t>선견</t>
+          <t>태세</t>
         </is>
       </c>
     </row>
     <row r="1080">
       <c r="A1080" t="inlineStr">
         <is>
-          <t>status.short.status_meditation</t>
+          <t>battle.chip.steadfast.short</t>
         </is>
       </c>
       <c r="B1080" t="inlineStr">
         <is>
-          <t>MED</t>
+          <t>Steady</t>
         </is>
       </c>
       <c r="C1080" t="inlineStr">
         <is>
-          <t>명상</t>
+          <t>버티기</t>
         </is>
       </c>
     </row>
     <row r="1081">
       <c r="A1081" t="inlineStr">
         <is>
-          <t>status.short.status_solidify</t>
+          <t>battle.chip.break.short</t>
         </is>
       </c>
       <c r="B1081" t="inlineStr">
         <is>
-          <t>Solid</t>
+          <t>BREAK</t>
         </is>
       </c>
       <c r="C1081" t="inlineStr">
         <is>
-          <t>굳힘</t>
+          <t>브레이크</t>
         </is>
       </c>
     </row>
     <row r="1082">
       <c r="A1082" t="inlineStr">
         <is>
-          <t>status.short.status_bloodthirsty</t>
+          <t>status.turns_left</t>
         </is>
       </c>
       <c r="B1082" t="inlineStr">
         <is>
-          <t>Thirst</t>
+          <t>{turns} turns left.</t>
         </is>
       </c>
       <c r="C1082" t="inlineStr">
         <is>
-          <t>갈증</t>
+          <t>{turns}턴 남았습니다.</t>
         </is>
       </c>
     </row>
     <row r="1083">
       <c r="A1083" t="inlineStr">
         <is>
-          <t>status.short.status_blessing</t>
+          <t>status.turn_left</t>
         </is>
       </c>
       <c r="B1083" t="inlineStr">
         <is>
-          <t>Bless</t>
+          <t>1 turn left.</t>
         </is>
       </c>
       <c r="C1083" t="inlineStr">
         <is>
-          <t>축복</t>
+          <t>1턴 남았습니다.</t>
         </is>
       </c>
     </row>
     <row r="1084">
       <c r="A1084" t="inlineStr">
         <is>
-          <t>status.short.status_sunder</t>
+          <t>bed.msg.rested</t>
         </is>
       </c>
       <c r="B1084" t="inlineStr">
         <is>
-          <t>Sunder</t>
+          <t>You are already rested.</t>
         </is>
       </c>
       <c r="C1084" t="inlineStr">
         <is>
-          <t>분쇄</t>
+          <t>이미 충분히 쉬었습니다.</t>
         </is>
       </c>
     </row>
     <row r="1085">
       <c r="A1085" t="inlineStr">
         <is>
-          <t>status.short.status_brace</t>
+          <t>bed.msg.nothing_to_upgrade</t>
         </is>
       </c>
       <c r="B1085" t="inlineStr">
         <is>
-          <t>Brace</t>
+          <t>Nothing to upgrade there.</t>
         </is>
       </c>
       <c r="C1085" t="inlineStr">
         <is>
-          <t>태세</t>
+          <t>강화할 수 있는 것이 없습니다.</t>
         </is>
       </c>
     </row>
     <row r="1086">
       <c r="A1086" t="inlineStr">
         <is>
-          <t>battle.chip.steadfast.short</t>
+          <t>bed.help.heal_rested</t>
         </is>
       </c>
       <c r="B1086" t="inlineStr">
         <is>
-          <t>Steady</t>
+          <t>You are already rested. Come back when HP or MP is missing.</t>
         </is>
       </c>
       <c r="C1086" t="inlineStr">
         <is>
-          <t>버티기</t>
+          <t>이미 충분히 쉬었습니다. HP나 MP가 줄었을 때 다시 오세요.</t>
         </is>
       </c>
     </row>
     <row r="1087">
       <c r="A1087" t="inlineStr">
         <is>
-          <t>battle.chip.break.short</t>
+          <t>item.msg.nothing_happens</t>
         </is>
       </c>
       <c r="B1087" t="inlineStr">
         <is>
-          <t>BREAK</t>
+          <t>Nothing happens.</t>
         </is>
       </c>
       <c r="C1087" t="inlineStr">
         <is>
-          <t>브레이크</t>
+          <t>아무 일도 일어나지 않았습니다.</t>
         </is>
       </c>
     </row>
     <row r="1088">
       <c r="A1088" t="inlineStr">
         <is>
-          <t>status.turns_left</t>
+          <t>help.stats.title</t>
         </is>
       </c>
       <c r="B1088" t="inlineStr">
         <is>
-          <t>{turns} turns left.</t>
+          <t>Stats &amp; Terms</t>
         </is>
       </c>
       <c r="C1088" t="inlineStr">
         <is>
-          <t>{turns}턴 남았습니다.</t>
+          <t>능력치와 용어</t>
         </is>
       </c>
     </row>
     <row r="1089">
       <c r="A1089" t="inlineStr">
         <is>
-          <t>status.turn_left</t>
+          <t>help.stats.help</t>
         </is>
       </c>
       <c r="B1089" t="inlineStr">
         <is>
-          <t>1 turn left.</t>
+          <t>What Power, ATK, DEF, MAG, SPD, VIG, MND, Crit, the grades, BREAK and every status mean.</t>
         </is>
       </c>
       <c r="C1089" t="inlineStr">
         <is>
-          <t>1턴 남았습니다.</t>
+          <t>위력, ATK, DEF, MAG, SPD, VIG, MND, 치명타, 등급, 브레이크와 모든 상태 이상의 뜻입니다.</t>
         </is>
       </c>
     </row>
     <row r="1090">
       <c r="A1090" t="inlineStr">
         <is>
-          <t>bed.msg.rested</t>
+          <t>help.term.crit</t>
         </is>
       </c>
       <c r="B1090" t="inlineStr">
         <is>
-          <t>You are already rested.</t>
+          <t>Crit</t>
         </is>
       </c>
       <c r="C1090" t="inlineStr">
         <is>
-          <t>이미 충분히 쉬었습니다.</t>
+          <t>치명타</t>
         </is>
       </c>
     </row>
     <row r="1091">
       <c r="A1091" t="inlineStr">
         <is>
-          <t>bed.msg.nothing_to_upgrade</t>
+          <t>help.term.good</t>
         </is>
       </c>
       <c r="B1091" t="inlineStr">
         <is>
-          <t>Nothing to upgrade there.</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="C1091" t="inlineStr">
         <is>
-          <t>강화할 수 있는 것이 없습니다.</t>
+          <t>좋음</t>
         </is>
       </c>
     </row>
     <row r="1092">
       <c r="A1092" t="inlineStr">
         <is>
-          <t>bed.help.heal_rested</t>
+          <t>help.term.ok</t>
         </is>
       </c>
       <c r="B1092" t="inlineStr">
         <is>
-          <t>You are already rested. Come back when HP or MP is missing.</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="C1092" t="inlineStr">
         <is>
-          <t>이미 충분히 쉬었습니다. HP나 MP가 줄었을 때 다시 오세요.</t>
+          <t>무난</t>
         </is>
       </c>
     </row>
     <row r="1093">
       <c r="A1093" t="inlineStr">
         <is>
-          <t>item.msg.nothing_happens</t>
+          <t>help.term.weak</t>
         </is>
       </c>
       <c r="B1093" t="inlineStr">
         <is>
-          <t>Nothing happens.</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="C1093" t="inlineStr">
         <is>
-          <t>아무 일도 일어나지 않았습니다.</t>
+          <t>약함</t>
         </is>
       </c>
     </row>
     <row r="1094">
       <c r="A1094" t="inlineStr">
         <is>
-          <t>help.stats.title</t>
+          <t>help.term.break</t>
         </is>
       </c>
       <c r="B1094" t="inlineStr">
         <is>
-          <t>Stats &amp; Terms</t>
+          <t>BREAK</t>
         </is>
       </c>
       <c r="C1094" t="inlineStr">
         <is>
-          <t>능력치와 용어</t>
+          <t>브레이크</t>
         </is>
       </c>
     </row>
     <row r="1095">
       <c r="A1095" t="inlineStr">
         <is>
-          <t>help.stats.help</t>
+          <t>help.line.power</t>
         </is>
       </c>
       <c r="B1095" t="inlineStr">
         <is>
-          <t>What Power, ATK, DEF, MAG, SPD, VIG, MND, Crit, the grades, BREAK and every status mean.</t>
+          <t>How hard a weapon or skill hits. More Power means more damage.</t>
         </is>
       </c>
       <c r="C1095" t="inlineStr">
         <is>
-          <t>위력, ATK, DEF, MAG, SPD, VIG, MND, 치명타, 등급, 브레이크와 모든 상태 이상의 뜻입니다.</t>
+          <t>무기나 스킬의 타격 세기입니다. 위력이 높을수록 피해가 커집니다.</t>
         </is>
       </c>
     </row>
     <row r="1096">
       <c r="A1096" t="inlineStr">
         <is>
-          <t>help.term.crit</t>
+          <t>help.line.hp</t>
         </is>
       </c>
       <c r="B1096" t="inlineStr">
         <is>
-          <t>Crit</t>
+          <t>Health. At 0 HP you fall.</t>
         </is>
       </c>
       <c r="C1096" t="inlineStr">
         <is>
-          <t>치명타</t>
+          <t>체력입니다. HP가 0이 되면 쓰러집니다.</t>
         </is>
       </c>
     </row>
     <row r="1097">
       <c r="A1097" t="inlineStr">
         <is>
-          <t>help.term.good</t>
+          <t>help.line.mp</t>
         </is>
       </c>
       <c r="B1097" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Magic points. Skills spend them; potions and rest restore them.</t>
         </is>
       </c>
       <c r="C1097" t="inlineStr">
         <is>
-          <t>좋음</t>
+          <t>스킬을 쓰면 줄어드는 마력입니다. 물약과 휴식으로 회복합니다.</t>
         </is>
       </c>
     </row>
     <row r="1098">
       <c r="A1098" t="inlineStr">
         <is>
-          <t>help.term.ok</t>
+          <t>help.line.crit</t>
         </is>
       </c>
       <c r="B1098" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>A critical hit deals {mult} times the damage. [t]Take Aim[/t] and some gear raise the odds.</t>
         </is>
       </c>
       <c r="C1098" t="inlineStr">
         <is>
-          <t>무난</t>
+          <t>치명타는 피해를 {mult}배로 줍니다. [t]조준[/t]과 일부 장비가 확률을 높입니다.</t>
         </is>
       </c>
     </row>
     <row r="1099">
       <c r="A1099" t="inlineStr">
         <is>
-          <t>help.term.weak</t>
+          <t>help.line.perfect</t>
         </is>
       </c>
       <c r="B1099" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>Press in the bright zone of the bar for +{pct}% damage.</t>
         </is>
       </c>
       <c r="C1099" t="inlineStr">
         <is>
-          <t>약함</t>
+          <t>막대의 밝은 구간에서 누르면 피해가 {pct}% 늘어납니다.</t>
         </is>
       </c>
     </row>
     <row r="1100">
       <c r="A1100" t="inlineStr">
         <is>
-          <t>help.term.break</t>
+          <t>help.line.good</t>
         </is>
       </c>
       <c r="B1100" t="inlineStr">
         <is>
-          <t>BREAK</t>
+          <t>Press near the middle for +{pct}% damage.</t>
         </is>
       </c>
       <c r="C1100" t="inlineStr">
         <is>
-          <t>브레이크</t>
+          <t>가운데 근처에서 누르면 피해가 {pct}% 늘어납니다.</t>
         </is>
       </c>
     </row>
     <row r="1101">
       <c r="A1101" t="inlineStr">
         <is>
-          <t>help.line.power</t>
+          <t>help.line.ok</t>
         </is>
       </c>
       <c r="B1101" t="inlineStr">
         <is>
-          <t>How hard a weapon or skill hits. More Power means more damage.</t>
+          <t>Press on the bar, off the middle, for normal damage.</t>
         </is>
       </c>
       <c r="C1101" t="inlineStr">
         <is>
-          <t>무기나 스킬의 타격 세기입니다. 위력이 높을수록 피해가 커집니다.</t>
+          <t>막대 위에서 가운데를 벗어나 누르면 보통 피해를 줍니다.</t>
         </is>
       </c>
     </row>
     <row r="1102">
       <c r="A1102" t="inlineStr">
         <is>
-          <t>help.line.hp</t>
+          <t>help.line.weak</t>
         </is>
       </c>
       <c r="B1102" t="inlineStr">
         <is>
-          <t>Health. At 0 HP you fall.</t>
+          <t>Miss the zone and the hit deals {pct}% less damage.</t>
         </is>
       </c>
       <c r="C1102" t="inlineStr">
         <is>
-          <t>체력입니다. HP가 0이 되면 쓰러집니다.</t>
+          <t>구간을 놓치면 피해가 {pct}% 줄어듭니다.</t>
         </is>
       </c>
     </row>
     <row r="1103">
       <c r="A1103" t="inlineStr">
         <is>
-          <t>help.line.mp</t>
+          <t>help.line.break</t>
         </is>
       </c>
       <c r="B1103" t="inlineStr">
         <is>
-          <t>Magic points. Skills spend them; potions and rest restore them.</t>
+          <t>Good hits fill the [t]stagger[/t] meter. When it is full the enemy loses a turn and takes +{pct}% damage.</t>
         </is>
       </c>
       <c r="C1103" t="inlineStr">
         <is>
-          <t>스킬을 쓰면 줄어드는 마력입니다. 물약과 휴식으로 회복합니다.</t>
+          <t>좋은 공격은 [t]경직[/t] 게이지를 채웁니다. 가득 차면 적이 한 턴을 잃고 피해를 {pct}% 더 받습니다.</t>
         </is>
       </c>
     </row>
     <row r="1104">
       <c r="A1104" t="inlineStr">
         <is>
-          <t>help.line.crit</t>
+          <t>help.line.elite</t>
         </is>
       </c>
       <c r="B1104" t="inlineStr">
         <is>
-          <t>A critical hit deals {mult} times the damage. [t]Take Aim[/t] and some gear raise the odds.</t>
+          <t>A marked, tougher enemy with a special trait. Its rewards are better.</t>
         </is>
       </c>
       <c r="C1104" t="inlineStr">
         <is>
-          <t>치명타는 피해를 {mult}배로 줍니다. [t]조준[/t]과 일부 장비가 확률을 높입니다.</t>
+          <t>표시가 붙은 더 강한 적으로, 특별한 특성이 있습니다. 보상이 더 좋습니다.</t>
         </is>
       </c>
     </row>
     <row r="1105">
       <c r="A1105" t="inlineStr">
         <is>
-          <t>help.line.perfect</t>
+          <t>choice.stranger.ask.0</t>
         </is>
       </c>
       <c r="B1105" t="inlineStr">
         <is>
-          <t>Press in the bright zone of the bar for +{pct}% damage.</t>
+          <t>There you are.</t>
         </is>
       </c>
       <c r="C1105" t="inlineStr">
         <is>
-          <t>막대의 밝은 구간에서 누르면 피해가 {pct}% 늘어납니다.</t>
+          <t>거기 있었군.</t>
         </is>
       </c>
     </row>
     <row r="1106">
       <c r="A1106" t="inlineStr">
         <is>
-          <t>help.line.good</t>
+          <t>choice.stranger.ask.1</t>
         </is>
       </c>
       <c r="B1106" t="inlineStr">
         <is>
-          <t>Press near the middle for +{pct}% damage.</t>
+          <t>Do you remember me?</t>
         </is>
       </c>
       <c r="C1106" t="inlineStr">
         <is>
-          <t>가운데 근처에서 누르면 피해가 {pct}% 늘어납니다.</t>
+          <t>나를 기억해?</t>
         </is>
       </c>
     </row>
     <row r="1107">
       <c r="A1107" t="inlineStr">
         <is>
-          <t>help.line.ok</t>
+          <t>choice.stranger.label.0</t>
         </is>
       </c>
       <c r="B1107" t="inlineStr">
         <is>
-          <t>Press on the bar, off the middle, for normal damage.</t>
+          <t>Should I?</t>
         </is>
       </c>
       <c r="C1107" t="inlineStr">
         <is>
-          <t>막대 위에서 가운데를 벗어나 누르면 보통 피해를 줍니다.</t>
+          <t>기억해야 해?</t>
         </is>
       </c>
     </row>
     <row r="1108">
       <c r="A1108" t="inlineStr">
         <is>
-          <t>help.line.weak</t>
+          <t>choice.stranger.label.1</t>
         </is>
       </c>
       <c r="B1108" t="inlineStr">
         <is>
-          <t>Miss the zone and the hit deals {pct}% less damage.</t>
+          <t>Back off.</t>
         </is>
       </c>
       <c r="C1108" t="inlineStr">
         <is>
-          <t>구간을 놓치면 피해가 {pct}% 줄어듭니다.</t>
+          <t>저리 가.</t>
         </is>
       </c>
     </row>
     <row r="1109">
       <c r="A1109" t="inlineStr">
         <is>
-          <t>help.line.break</t>
+          <t>choice.stranger.reply1.0</t>
         </is>
       </c>
       <c r="B1109" t="inlineStr">
         <is>
-          <t>Good hits fill the [t]stagger[/t] meter. When it is full the enemy loses a turn and takes +{pct}% damage.</t>
+          <t>Not yet.</t>
         </is>
       </c>
       <c r="C1109" t="inlineStr">
         <is>
-          <t>좋은 공격은 [t]경직[/t] 게이지를 채웁니다. 가득 차면 적이 한 턴을 잃고 피해를 {pct}% 더 받습니다.</t>
+          <t>아직은 아니야.</t>
         </is>
       </c>
     </row>
     <row r="1110">
       <c r="A1110" t="inlineStr">
         <is>
-          <t>help.line.elite</t>
+          <t>choice.stranger.reply1.1</t>
         </is>
       </c>
       <c r="B1110" t="inlineStr">
         <is>
-          <t>A marked, tougher enemy with a special trait. Its rewards are better.</t>
+          <t>Ask again when the tunnel has had you a bit longer.</t>
         </is>
       </c>
       <c r="C1110" t="inlineStr">
         <is>
-          <t>표시가 붙은 더 강한 적으로, 특별한 특성이 있습니다. 보상이 더 좋습니다.</t>
+          <t>터널이 널 좀 더 삼키면 다시 물어봐.</t>
         </is>
       </c>
     </row>
     <row r="1111">
       <c r="A1111" t="inlineStr">
         <is>
-          <t>choice.stranger.ask.0</t>
+          <t>choice.stranger.reply2.0</t>
         </is>
       </c>
       <c r="B1111" t="inlineStr">
         <is>
-          <t>There you are.</t>
+          <t>Ha. Fair.</t>
         </is>
       </c>
       <c r="C1111" t="inlineStr">
         <is>
-          <t>거기 있었군.</t>
+          <t>하하, 그렇겠지.</t>
         </is>
       </c>
     </row>
     <row r="1112">
       <c r="A1112" t="inlineStr">
         <is>
-          <t>choice.stranger.ask.1</t>
+          <t>choice.stranger.reply2.1</t>
         </is>
       </c>
       <c r="B1112" t="inlineStr">
         <is>
-          <t>Do you remember me?</t>
+          <t>Nobody does, at first.</t>
         </is>
       </c>
       <c r="C1112" t="inlineStr">
         <is>
-          <t>나를 기억해?</t>
+          <t>처음엔 다들 그래.</t>
         </is>
       </c>
     </row>
     <row r="1113">
       <c r="A1113" t="inlineStr">
         <is>
-          <t>choice.stranger.label.0</t>
+          <t>choice.stranger.again1.0</t>
         </is>
       </c>
       <c r="B1113" t="inlineStr">
         <is>
-          <t>Should I?</t>
+          <t>Still asking if you should?</t>
         </is>
       </c>
       <c r="C1113" t="inlineStr">
         <is>
-          <t>기억해야 해?</t>
+          <t>아직도 기억해야 하는지 묻는군?</t>
         </is>
       </c>
     </row>
     <row r="1114">
       <c r="A1114" t="inlineStr">
         <is>
-          <t>choice.stranger.label.1</t>
+          <t>choice.stranger.again1.1</t>
         </is>
       </c>
       <c r="B1114" t="inlineStr">
         <is>
-          <t>Back off.</t>
+          <t>You'll know me when you stop asking.</t>
         </is>
       </c>
       <c r="C1114" t="inlineStr">
         <is>
-          <t>저리 가.</t>
+          <t>묻기를 그만두면 알게 될 거야.</t>
         </is>
       </c>
     </row>
     <row r="1115">
       <c r="A1115" t="inlineStr">
         <is>
-          <t>choice.stranger.reply1.0</t>
+          <t>choice.stranger.again2.0</t>
         </is>
       </c>
       <c r="B1115" t="inlineStr">
         <is>
-          <t>Not yet.</t>
+          <t>Still telling me to back off?</t>
         </is>
       </c>
       <c r="C1115" t="inlineStr">
         <is>
-          <t>아직은 아니야.</t>
+          <t>아직도 저리 가라고 하는군?</t>
         </is>
       </c>
     </row>
     <row r="1116">
       <c r="A1116" t="inlineStr">
         <is>
-          <t>choice.stranger.reply1.1</t>
+          <t>choice.stranger.again2.1</t>
         </is>
       </c>
       <c r="B1116" t="inlineStr">
         <is>
-          <t>Ask again when the tunnel has had you a bit longer.</t>
+          <t>I'm patient. I've had practice.</t>
         </is>
       </c>
       <c r="C1116" t="inlineStr">
         <is>
-          <t>터널이 널 좀 더 삼키면 다시 물어봐.</t>
+          <t>난 참을성이 있어. 연습을 많이 했거든.</t>
         </is>
       </c>
     </row>
     <row r="1117">
       <c r="A1117" t="inlineStr">
         <is>
-          <t>choice.stranger.reply2.0</t>
+          <t>choice.merchant.ask.0</t>
         </is>
       </c>
       <c r="B1117" t="inlineStr">
         <is>
-          <t>Ha. Fair.</t>
+          <t>Tell me, friend.</t>
         </is>
       </c>
       <c r="C1117" t="inlineStr">
         <is>
-          <t>하하, 그렇겠지.</t>
+          <t>말해 봐, 친구.</t>
         </is>
       </c>
     </row>
     <row r="1118">
       <c r="A1118" t="inlineStr">
         <is>
-          <t>choice.stranger.reply2.1</t>
+          <t>choice.merchant.ask.1</t>
         </is>
       </c>
       <c r="B1118" t="inlineStr">
         <is>
-          <t>Nobody does, at first.</t>
+          <t>Looking for a way out, or something to buy?</t>
         </is>
       </c>
       <c r="C1118" t="inlineStr">
         <is>
-          <t>처음엔 다들 그래.</t>
+          <t>나갈 길을 찾는 거야, 아니면 살 게 있는 거야?</t>
         </is>
       </c>
     </row>
     <row r="1119">
       <c r="A1119" t="inlineStr">
         <is>
-          <t>choice.stranger.again1.0</t>
+          <t>choice.merchant.label.0</t>
         </is>
       </c>
       <c r="B1119" t="inlineStr">
         <is>
-          <t>Still asking if you should?</t>
+          <t>A way out.</t>
         </is>
       </c>
       <c r="C1119" t="inlineStr">
         <is>
-          <t>아직도 기억해야 하는지 묻는군?</t>
+          <t>나갈 길.</t>
         </is>
       </c>
     </row>
     <row r="1120">
       <c r="A1120" t="inlineStr">
         <is>
-          <t>choice.stranger.again1.1</t>
+          <t>choice.merchant.label.1</t>
         </is>
       </c>
       <c r="B1120" t="inlineStr">
         <is>
-          <t>You'll know me when you stop asking.</t>
+          <t>Something to buy.</t>
         </is>
       </c>
       <c r="C1120" t="inlineStr">
         <is>
-          <t>묻기를 그만두면 알게 될 거야.</t>
+          <t>살 물건.</t>
         </is>
       </c>
     </row>
     <row r="1121">
       <c r="A1121" t="inlineStr">
         <is>
-          <t>choice.stranger.again2.0</t>
+          <t>choice.merchant.reply1.0</t>
         </is>
       </c>
       <c r="B1121" t="inlineStr">
         <is>
-          <t>Still telling me to back off?</t>
+          <t>Ha. They all say that.</t>
         </is>
       </c>
       <c r="C1121" t="inlineStr">
         <is>
-          <t>아직도 저리 가라고 하는군?</t>
+          <t>하하, 다들 그렇게 말하지.</t>
         </is>
       </c>
     </row>
     <row r="1122">
       <c r="A1122" t="inlineStr">
         <is>
-          <t>choice.stranger.again2.1</t>
+          <t>choice.merchant.reply1.1</t>
         </is>
       </c>
       <c r="B1122" t="inlineStr">
         <is>
-          <t>I'm patient. I've had practice.</t>
+          <t>Shop first. Hope walks better with a full pack.</t>
         </is>
       </c>
       <c r="C1122" t="inlineStr">
         <is>
-          <t>난 참을성이 있어. 연습을 많이 했거든.</t>
+          <t>일단 사. 짐이 든든해야 희망도 잘 걷거든.</t>
         </is>
       </c>
     </row>
     <row r="1123">
       <c r="A1123" t="inlineStr">
         <is>
-          <t>choice.merchant.ask.0</t>
+          <t>choice.merchant.reply2.0</t>
         </is>
       </c>
       <c r="B1123" t="inlineStr">
         <is>
-          <t>Tell me, friend.</t>
+          <t>Good. Buying I understand.</t>
         </is>
       </c>
       <c r="C1123" t="inlineStr">
         <is>
-          <t>말해 봐, 친구.</t>
+          <t>좋아. 장사라면 내가 잘 알지.</t>
         </is>
       </c>
     </row>
     <row r="1124">
       <c r="A1124" t="inlineStr">
         <is>
-          <t>choice.merchant.ask.1</t>
+          <t>choice.merchant.reply2.1</t>
         </is>
       </c>
       <c r="B1124" t="inlineStr">
         <is>
-          <t>Looking for a way out, or something to buy?</t>
+          <t>Asking after exits gets people killed.</t>
         </is>
       </c>
       <c r="C1124" t="inlineStr">
         <is>
-          <t>나갈 길을 찾는 거야, 아니면 살 게 있는 거야?</t>
+          <t>출구를 캐묻다 죽은 사람이 한둘이 아니야.</t>
         </is>
       </c>
     </row>
     <row r="1125">
       <c r="A1125" t="inlineStr">
         <is>
-          <t>choice.merchant.label.0</t>
+          <t>choice.merchant.again1.0</t>
         </is>
       </c>
       <c r="B1125" t="inlineStr">
         <is>
-          <t>A way out.</t>
+          <t>Found your way out yet? No? Then buy something.</t>
         </is>
       </c>
       <c r="C1125" t="inlineStr">
         <is>
-          <t>나갈 길.</t>
+          <t>나갈 길은 찾았어? 아직이면 뭐라도 사.</t>
         </is>
       </c>
     </row>
     <row r="1126">
       <c r="A1126" t="inlineStr">
         <is>
-          <t>choice.merchant.label.1</t>
+          <t>choice.merchant.again2.0</t>
         </is>
       </c>
       <c r="B1126" t="inlineStr">
         <is>
-          <t>Something to buy.</t>
+          <t>Back to spend, I hope. That I understand.</t>
         </is>
       </c>
       <c r="C1126" t="inlineStr">
         <is>
-          <t>살 물건.</t>
+          <t>돈 쓰러 왔길 바란다. 그거라면 내가 잘 알지.</t>
         </is>
       </c>
     </row>
     <row r="1127">
       <c r="A1127" t="inlineStr">
         <is>
-          <t>choice.merchant.reply1.0</t>
+          <t>choice.map_page.ask.0</t>
         </is>
       </c>
       <c r="B1127" t="inlineStr">
         <is>
-          <t>Ha. They all say that.</t>
+          <t>You read it twice.</t>
         </is>
       </c>
       <c r="C1127" t="inlineStr">
         <is>
-          <t>하하, 다들 그렇게 말하지.</t>
+          <t>두 번 읽는다.</t>
         </is>
       </c>
     </row>
     <row r="1128">
       <c r="A1128" t="inlineStr">
         <is>
-          <t>choice.merchant.reply1.1</t>
+          <t>choice.map_page.ask.1</t>
         </is>
       </c>
       <c r="B1128" t="inlineStr">
         <is>
-          <t>Shop first. Hope walks better with a full pack.</t>
+          <t>Whose hand is this?</t>
         </is>
       </c>
       <c r="C1128" t="inlineStr">
         <is>
-          <t>일단 사. 짐이 든든해야 희망도 잘 걷거든.</t>
+          <t>누구의 글씨일까?</t>
         </is>
       </c>
     </row>
     <row r="1129">
       <c r="A1129" t="inlineStr">
         <is>
-          <t>choice.merchant.reply2.0</t>
+          <t>choice.map_page.label.0</t>
         </is>
       </c>
       <c r="B1129" t="inlineStr">
         <is>
-          <t>Good. Buying I understand.</t>
+          <t>Mine.</t>
         </is>
       </c>
       <c r="C1129" t="inlineStr">
         <is>
-          <t>좋아. 장사라면 내가 잘 알지.</t>
+          <t>내 것.</t>
         </is>
       </c>
     </row>
     <row r="1130">
       <c r="A1130" t="inlineStr">
         <is>
-          <t>choice.merchant.reply2.1</t>
+          <t>choice.map_page.label.1</t>
         </is>
       </c>
       <c r="B1130" t="inlineStr">
         <is>
-          <t>Asking after exits gets people killed.</t>
+          <t>Someone else's.</t>
         </is>
       </c>
       <c r="C1130" t="inlineStr">
         <is>
-          <t>출구를 캐묻다 죽은 사람이 한둘이 아니야.</t>
+          <t>남의 것.</t>
         </is>
       </c>
     </row>
     <row r="1131">
       <c r="A1131" t="inlineStr">
         <is>
-          <t>choice.merchant.again1.0</t>
+          <t>choice.map_page.reply1.0</t>
         </is>
       </c>
       <c r="B1131" t="inlineStr">
         <is>
-          <t>Found your way out yet? No? Then buy something.</t>
+          <t>Yours. You say it out loud.</t>
         </is>
       </c>
       <c r="C1131" t="inlineStr">
         <is>
-          <t>나갈 길은 찾았어? 아직이면 뭐라도 사.</t>
+          <t>내 글씨다. 소리 내어 말해 본다.</t>
         </is>
       </c>
     </row>
     <row r="1132">
       <c r="A1132" t="inlineStr">
         <is>
-          <t>choice.merchant.again2.0</t>
+          <t>choice.map_page.reply1.1</t>
         </is>
       </c>
       <c r="B1132" t="inlineStr">
         <is>
-          <t>Back to spend, I hope. That I understand.</t>
+          <t>The ink seems to settle.</t>
         </is>
       </c>
       <c r="C1132" t="inlineStr">
         <is>
-          <t>돈 쓰러 왔길 바란다. 그거라면 내가 잘 알지.</t>
+          <t>잉크가 가라앉는 듯하다.</t>
         </is>
       </c>
     </row>
     <row r="1133">
       <c r="A1133" t="inlineStr">
         <is>
-          <t>choice.map_page.ask.0</t>
+          <t>choice.map_page.reply2.0</t>
         </is>
       </c>
       <c r="B1133" t="inlineStr">
         <is>
-          <t>You read it twice.</t>
+          <t>Not yours. You say it out loud.</t>
         </is>
       </c>
       <c r="C1133" t="inlineStr">
         <is>
-          <t>두 번 읽는다.</t>
+          <t>내 글씨가 아니다. 소리 내어 말해 본다.</t>
         </is>
       </c>
     </row>
     <row r="1134">
       <c r="A1134" t="inlineStr">
         <is>
-          <t>choice.map_page.ask.1</t>
+          <t>choice.map_page.reply2.1</t>
         </is>
       </c>
       <c r="B1134" t="inlineStr">
         <is>
-          <t>Whose hand is this?</t>
+          <t>The ink shivers.</t>
         </is>
       </c>
       <c r="C1134" t="inlineStr">
         <is>
-          <t>누구의 글씨일까?</t>
+          <t>잉크가 떨리는 듯하다.</t>
         </is>
       </c>
     </row>
     <row r="1135">
       <c r="A1135" t="inlineStr">
         <is>
-          <t>choice.map_page.label.0</t>
+          <t>choice.map_page.again1.0</t>
         </is>
       </c>
       <c r="B1135" t="inlineStr">
         <is>
-          <t>Mine.</t>
+          <t>The ink is dry now. You've stopped doubting the hand.</t>
         </is>
       </c>
       <c r="C1135" t="inlineStr">
         <is>
-          <t>내 것.</t>
+          <t>잉크가 말랐다. 이 글씨를 더는 의심하지 않는다.</t>
         </is>
       </c>
     </row>
     <row r="1136">
       <c r="A1136" t="inlineStr">
         <is>
-          <t>choice.map_page.label.1</t>
+          <t>choice.map_page.again2.0</t>
         </is>
       </c>
       <c r="B1136" t="inlineStr">
         <is>
-          <t>Someone else's.</t>
+          <t>The ink is dry now. You still say it isn't yours.</t>
         </is>
       </c>
       <c r="C1136" t="inlineStr">
         <is>
-          <t>남의 것.</t>
+          <t>잉크가 말랐다. 그래도 내 글씨가 아니라고 말한다.</t>
         </is>
       </c>
     </row>
     <row r="1137">
       <c r="A1137" t="inlineStr">
         <is>
-          <t>choice.map_page.reply1.0</t>
+          <t>choice.wake.ask.0</t>
         </is>
       </c>
       <c r="B1137" t="inlineStr">
         <is>
-          <t>Yours. You say it out loud.</t>
+          <t>Your head swims.</t>
         </is>
       </c>
       <c r="C1137" t="inlineStr">
         <is>
-          <t>내 글씨다. 소리 내어 말해 본다.</t>
+          <t>머리가 어지럽다.</t>
         </is>
       </c>
     </row>
     <row r="1138">
       <c r="A1138" t="inlineStr">
         <is>
-          <t>choice.map_page.reply1.1</t>
+          <t>choice.wake.ask.1</t>
         </is>
       </c>
       <c r="B1138" t="inlineStr">
         <is>
-          <t>The ink seems to settle.</t>
+          <t>Your body waits for you to decide.</t>
         </is>
       </c>
       <c r="C1138" t="inlineStr">
         <is>
-          <t>잉크가 가라앉는 듯하다.</t>
+          <t>몸이 당신의 결정을 기다린다.</t>
         </is>
       </c>
     </row>
     <row r="1139">
       <c r="A1139" t="inlineStr">
         <is>
-          <t>choice.map_page.reply2.0</t>
+          <t>choice.wake.label.0</t>
         </is>
       </c>
       <c r="B1139" t="inlineStr">
         <is>
-          <t>Not yours. You say it out loud.</t>
+          <t>Sit up.</t>
         </is>
       </c>
       <c r="C1139" t="inlineStr">
         <is>
-          <t>내 글씨가 아니다. 소리 내어 말해 본다.</t>
+          <t>일어난다.</t>
         </is>
       </c>
     </row>
     <row r="1140">
       <c r="A1140" t="inlineStr">
         <is>
-          <t>choice.map_page.reply2.1</t>
+          <t>choice.wake.label.1</t>
         </is>
       </c>
       <c r="B1140" t="inlineStr">
         <is>
-          <t>The ink shivers.</t>
+          <t>Lie still.</t>
         </is>
       </c>
       <c r="C1140" t="inlineStr">
         <is>
-          <t>잉크가 떨리는 듯하다.</t>
+          <t>가만히 있는다.</t>
         </is>
       </c>
     </row>
     <row r="1141">
       <c r="A1141" t="inlineStr">
         <is>
-          <t>choice.map_page.again1.0</t>
+          <t>choice.wake.reply1.0</t>
         </is>
       </c>
       <c r="B1141" t="inlineStr">
         <is>
-          <t>The ink is dry now. You've stopped doubting the hand.</t>
+          <t>You push up. The stone lets go of your back slowly.</t>
         </is>
       </c>
       <c r="C1141" t="inlineStr">
         <is>
-          <t>잉크가 말랐다. 이 글씨를 더는 의심하지 않는다.</t>
+          <t>몸을 일으킨다. 돌바닥이 등을 천천히 놓아 준다.</t>
         </is>
       </c>
     </row>
     <row r="1142">
       <c r="A1142" t="inlineStr">
         <is>
-          <t>choice.map_page.again2.0</t>
+          <t>choice.wake.reply2.0</t>
         </is>
       </c>
       <c r="B1142" t="inlineStr">
         <is>
-          <t>The ink is dry now. You still say it isn't yours.</t>
+          <t>You lie still. The ceiling says nothing. Neither do you.</t>
         </is>
       </c>
       <c r="C1142" t="inlineStr">
         <is>
-          <t>잉크가 말랐다. 그래도 내 글씨가 아니라고 말한다.</t>
+          <t>가만히 누워 있다. 천장은 말이 없다. 당신도 그렇다.</t>
         </is>
       </c>
     </row>
     <row r="1143">
       <c r="A1143" t="inlineStr">
         <is>
-          <t>choice.wake.ask.0</t>
+          <t>choice.wake.again1.0</t>
         </is>
       </c>
       <c r="B1143" t="inlineStr">
         <is>
-          <t>Your head swims.</t>
+          <t>Your body already knows how to get up.</t>
         </is>
       </c>
       <c r="C1143" t="inlineStr">
         <is>
-          <t>머리가 어지럽다.</t>
+          <t>몸은 이미 일어나는 법을 안다.</t>
         </is>
       </c>
     </row>
     <row r="1144">
       <c r="A1144" t="inlineStr">
         <is>
-          <t>choice.wake.ask.1</t>
+          <t>choice.wake.again2.0</t>
         </is>
       </c>
       <c r="B1144" t="inlineStr">
         <is>
-          <t>Your body waits for you to decide.</t>
+          <t>You lie still a while first. You always do now.</t>
         </is>
       </c>
       <c r="C1144" t="inlineStr">
         <is>
-          <t>몸이 당신의 결정을 기다린다.</t>
+          <t>먼저 한참 누워 있는다. 이제는 늘 그렇다.</t>
         </is>
       </c>
     </row>
     <row r="1145">
       <c r="A1145" t="inlineStr">
         <is>
-          <t>choice.wake.label.0</t>
+          <t>menu.msg.items_in_fight</t>
         </is>
       </c>
       <c r="B1145" t="inlineStr">
         <is>
-          <t>Sit up.</t>
+          <t>In a battle, use Item in the battle menu.</t>
         </is>
       </c>
       <c r="C1145" t="inlineStr">
         <is>
-          <t>일어난다.</t>
+          <t>전투 중에는 전투 메뉴의 아이템을 사용하세요.</t>
         </is>
       </c>
     </row>
     <row r="1146">
       <c r="A1146" t="inlineStr">
         <is>
-          <t>choice.wake.label.1</t>
+          <t>menu.msg.gear_in_fight</t>
         </is>
       </c>
       <c r="B1146" t="inlineStr">
         <is>
-          <t>Lie still.</t>
+          <t>You can't change gear during a battle.</t>
         </is>
       </c>
       <c r="C1146" t="inlineStr">
         <is>
-          <t>가만히 있는다.</t>
+          <t>전투 중에는 장비를 바꿀 수 없습니다.</t>
         </is>
       </c>
     </row>
     <row r="1147">
       <c r="A1147" t="inlineStr">
         <is>
-          <t>choice.wake.reply1.0</t>
+          <t>dialogue.first_encounter_mini_boss.0</t>
         </is>
       </c>
       <c r="B1147" t="inlineStr">
         <is>
-          <t>You push up. The stone lets go of your back slowly.</t>
+          <t>...</t>
         </is>
       </c>
       <c r="C1147" t="inlineStr">
         <is>
-          <t>몸을 일으킨다. 돌바닥이 등을 천천히 놓아 준다.</t>
+          <t>...</t>
         </is>
       </c>
     </row>
     <row r="1148">
       <c r="A1148" t="inlineStr">
         <is>
-          <t>choice.wake.reply2.0</t>
+          <t>dialogue.first_encounter_mini_boss.1</t>
         </is>
       </c>
       <c r="B1148" t="inlineStr">
         <is>
-          <t>You lie still. The ceiling says nothing. Neither do you.</t>
+          <t>Oh, what the hell is that?</t>
         </is>
       </c>
       <c r="C1148" t="inlineStr">
         <is>
-          <t>가만히 누워 있다. 천장은 말이 없다. 당신도 그렇다.</t>
+          <t>아니, 저게 대체 뭐야?</t>
         </is>
       </c>
     </row>
     <row r="1149">
       <c r="A1149" t="inlineStr">
         <is>
-          <t>choice.wake.again1.0</t>
+          <t>dialogue.first_encounter_mini_boss.2</t>
         </is>
       </c>
       <c r="B1149" t="inlineStr">
         <is>
-          <t>Your body already knows how to get up.</t>
+          <t>Half cow, half man?</t>
         </is>
       </c>
       <c r="C1149" t="inlineStr">
         <is>
-          <t>몸은 이미 일어나는 법을 안다.</t>
+          <t>반은 소, 반은 사람?</t>
         </is>
       </c>
     </row>
     <row r="1150">
       <c r="A1150" t="inlineStr">
         <is>
-          <t>choice.wake.again2.0</t>
+          <t>dialogue.first_encounter_mini_boss.3</t>
         </is>
       </c>
       <c r="B1150" t="inlineStr">
         <is>
-          <t>You lie still a while first. You always do now.</t>
+          <t>That breathing. Those horns...</t>
         </is>
       </c>
       <c r="C1150" t="inlineStr">
         <is>
-          <t>먼저 한참 누워 있는다. 이제는 늘 그렇다.</t>
+          <t>저 숨소리. 저 뿔...</t>
         </is>
       </c>
     </row>
     <row r="1151">
       <c r="A1151" t="inlineStr">
         <is>
-          <t>menu.msg.items_in_fight</t>
+          <t>dialogue.first_encounter_mini_boss.4</t>
         </is>
       </c>
       <c r="B1151" t="inlineStr">
         <is>
-          <t>In a battle, use Item in the battle menu.</t>
+          <t>And he's blocking the only way forward.</t>
         </is>
       </c>
       <c r="C1151" t="inlineStr">
         <is>
-          <t>전투 중에는 전투 메뉴의 아이템을 사용하세요.</t>
+          <t>하필 하나뿐인 길을 막고 서 있어.</t>
         </is>
       </c>
     </row>
     <row r="1152">
       <c r="A1152" t="inlineStr">
         <is>
-          <t>menu.msg.gear_in_fight</t>
+          <t>dialogue.first_encounter_mini_boss.5</t>
         </is>
       </c>
       <c r="B1152" t="inlineStr">
         <is>
-          <t>You can't change gear during a battle.</t>
+          <t>...</t>
         </is>
       </c>
       <c r="C1152" t="inlineStr">
         <is>
-          <t>전투 중에는 장비를 바꿀 수 없습니다.</t>
+          <t>...</t>
         </is>
       </c>
     </row>
     <row r="1153">
       <c r="A1153" t="inlineStr">
         <is>
-          <t>dialogue.first_encounter_mini_boss.0</t>
+          <t>dialogue.first_encounter_mini_boss.6</t>
         </is>
       </c>
       <c r="B1153" t="inlineStr">
         <is>
-          <t>...</t>
+          <t>Fuck.</t>
         </is>
       </c>
       <c r="C1153" t="inlineStr">
         <is>
-          <t>...</t>
+          <t>젠장.</t>
         </is>
       </c>
     </row>
     <row r="1154">
       <c r="A1154" t="inlineStr">
         <is>
-          <t>dialogue.first_encounter_mini_boss.1</t>
+          <t>dialogue.first_encounter_final_boss.0</t>
         </is>
       </c>
       <c r="B1154" t="inlineStr">
         <is>
-          <t>Oh, what the hell is that?</t>
+          <t>...</t>
         </is>
       </c>
       <c r="C1154" t="inlineStr">
         <is>
-          <t>아니, 저게 대체 뭐야?</t>
+          <t>...</t>
         </is>
       </c>
     </row>
     <row r="1155">
       <c r="A1155" t="inlineStr">
         <is>
-          <t>dialogue.first_encounter_mini_boss.2</t>
+          <t>dialogue.first_encounter_final_boss.1</t>
         </is>
       </c>
       <c r="B1155" t="inlineStr">
         <is>
-          <t>Half cow, half man?</t>
+          <t>Another demon.</t>
         </is>
       </c>
       <c r="C1155" t="inlineStr">
         <is>
-          <t>반은 소, 반은 사람?</t>
+          <t>또 악마인가.</t>
         </is>
       </c>
     </row>
     <row r="1156">
       <c r="A1156" t="inlineStr">
         <is>
-          <t>dialogue.first_encounter_mini_boss.3</t>
+          <t>dialogue.first_encounter_final_boss.2</t>
         </is>
       </c>
       <c r="B1156" t="inlineStr">
         <is>
-          <t>That breathing. Those horns...</t>
+          <t>This one is different.</t>
         </is>
       </c>
       <c r="C1156" t="inlineStr">
         <is>
-          <t>저 숨소리. 저 뿔...</t>
+          <t>이번 놈은 달라.</t>
         </is>
       </c>
     </row>
     <row r="1157">
       <c r="A1157" t="inlineStr">
         <is>
-          <t>dialogue.first_encounter_mini_boss.4</t>
+          <t>dialogue.first_encounter_final_boss.3</t>
         </is>
       </c>
       <c r="B1157" t="inlineStr">
         <is>
-          <t>And he's blocking the only way forward.</t>
+          <t>As if it's looking for something...</t>
         </is>
       </c>
       <c r="C1157" t="inlineStr">
         <is>
-          <t>하필 하나뿐인 길을 막고 서 있어.</t>
+          <t>무언가를 찾는 것 같아...</t>
         </is>
       </c>
     </row>
     <row r="1158">
       <c r="A1158" t="inlineStr">
         <is>
-          <t>dialogue.first_encounter_mini_boss.5</t>
+          <t>dialogue.first_encounter_final_boss.4</t>
         </is>
       </c>
       <c r="B1158" t="inlineStr">
@@ -20112,296 +20112,296 @@
     <row r="1159">
       <c r="A1159" t="inlineStr">
         <is>
-          <t>dialogue.first_encounter_mini_boss.6</t>
+          <t>dialogue.first_encounter_final_boss.5</t>
         </is>
       </c>
       <c r="B1159" t="inlineStr">
         <is>
-          <t>Fuck.</t>
+          <t>...someone.</t>
         </is>
       </c>
       <c r="C1159" t="inlineStr">
         <is>
-          <t>젠장.</t>
+          <t>...누군가를.</t>
         </is>
       </c>
     </row>
     <row r="1160">
       <c r="A1160" t="inlineStr">
         <is>
-          <t>dialogue.first_encounter_final_boss.0</t>
+          <t>dialogue.sys_floor2_dire_wolf_reaction.0</t>
         </is>
       </c>
       <c r="B1160" t="inlineStr">
         <is>
-          <t>...</t>
+          <t>*Pant*... Whew.</t>
         </is>
       </c>
       <c r="C1160" t="inlineStr">
         <is>
-          <t>...</t>
+          <t>*헉*... 휴.</t>
         </is>
       </c>
     </row>
     <row r="1161">
       <c r="A1161" t="inlineStr">
         <is>
-          <t>dialogue.first_encounter_final_boss.1</t>
+          <t>dialogue.sys_floor2_dire_wolf_reaction.1</t>
         </is>
       </c>
       <c r="B1161" t="inlineStr">
         <is>
-          <t>Another demon.</t>
+          <t>A wolf now? Seriously?</t>
         </is>
       </c>
       <c r="C1161" t="inlineStr">
         <is>
-          <t>또 악마인가.</t>
+          <t>이번엔 늑대라고? 진짜로?</t>
         </is>
       </c>
     </row>
     <row r="1162">
       <c r="A1162" t="inlineStr">
         <is>
-          <t>dialogue.first_encounter_final_boss.2</t>
+          <t>dialogue.sys_floor2_dire_wolf_reaction.2</t>
         </is>
       </c>
       <c r="B1162" t="inlineStr">
         <is>
-          <t>This one is different.</t>
+          <t>Where do these things come from?</t>
         </is>
       </c>
       <c r="C1162" t="inlineStr">
         <is>
-          <t>이번 놈은 달라.</t>
+          <t>이것들은 다 어디서 나오는 거야?</t>
         </is>
       </c>
     </row>
     <row r="1163">
       <c r="A1163" t="inlineStr">
         <is>
-          <t>dialogue.first_encounter_final_boss.3</t>
+          <t>dialogue.sys_floor2_dire_wolf_reaction.3</t>
         </is>
       </c>
       <c r="B1163" t="inlineStr">
         <is>
-          <t>As if it's looking for something...</t>
+          <t>...</t>
         </is>
       </c>
       <c r="C1163" t="inlineStr">
         <is>
-          <t>무언가를 찾는 것 같아...</t>
+          <t>...</t>
         </is>
       </c>
     </row>
     <row r="1164">
       <c r="A1164" t="inlineStr">
         <is>
-          <t>dialogue.first_encounter_final_boss.4</t>
+          <t>dialogue.sys_floor2_dire_wolf_reaction.4</t>
         </is>
       </c>
       <c r="B1164" t="inlineStr">
         <is>
-          <t>...</t>
+          <t>Standing here won't answer that.</t>
         </is>
       </c>
       <c r="C1164" t="inlineStr">
         <is>
-          <t>...</t>
+          <t>여기 서 있어도 답은 안 나와.</t>
         </is>
       </c>
     </row>
     <row r="1165">
       <c r="A1165" t="inlineStr">
         <is>
-          <t>dialogue.first_encounter_final_boss.5</t>
+          <t>dialogue.sys_floor2_dire_wolf_reaction.5</t>
         </is>
       </c>
       <c r="B1165" t="inlineStr">
         <is>
-          <t>...someone.</t>
+          <t>Keep moving.</t>
         </is>
       </c>
       <c r="C1165" t="inlineStr">
         <is>
-          <t>...누군가를.</t>
+          <t>계속 가자.</t>
         </is>
       </c>
     </row>
     <row r="1166">
       <c r="A1166" t="inlineStr">
         <is>
-          <t>dialogue.sys_floor2_dire_wolf_reaction.0</t>
+          <t>dialogue.sys_first_stranger_encounter_reaction.0</t>
         </is>
       </c>
       <c r="B1166" t="inlineStr">
         <is>
-          <t>*Pant*... Whew.</t>
+          <t>Get your hands off me...</t>
         </is>
       </c>
       <c r="C1166" t="inlineStr">
         <is>
-          <t>*헉*... 휴.</t>
+          <t>손 치워...</t>
         </is>
       </c>
     </row>
     <row r="1167">
       <c r="A1167" t="inlineStr">
         <is>
-          <t>dialogue.sys_floor2_dire_wolf_reaction.1</t>
+          <t>dialogue.sys_first_stranger_encounter_reaction.1</t>
         </is>
       </c>
       <c r="B1167" t="inlineStr">
         <is>
-          <t>A wolf now? Seriously?</t>
+          <t>He smiled the whole time.</t>
         </is>
       </c>
       <c r="C1167" t="inlineStr">
         <is>
-          <t>이번엔 늑대라고? 진짜로?</t>
+          <t>그 녀석, 내내 웃고 있었어.</t>
         </is>
       </c>
     </row>
     <row r="1168">
       <c r="A1168" t="inlineStr">
         <is>
-          <t>dialogue.sys_floor2_dire_wolf_reaction.2</t>
+          <t>dialogue.sys_first_stranger_encounter_reaction.2</t>
         </is>
       </c>
       <c r="B1168" t="inlineStr">
         <is>
-          <t>Where do these things come from?</t>
+          <t>Are they all demons down here?</t>
         </is>
       </c>
       <c r="C1168" t="inlineStr">
         <is>
-          <t>이것들은 다 어디서 나오는 거야?</t>
+          <t>여기 있는 건 전부 악마야?</t>
         </is>
       </c>
     </row>
     <row r="1169">
       <c r="A1169" t="inlineStr">
         <is>
-          <t>dialogue.sys_floor2_dire_wolf_reaction.3</t>
+          <t>dialogue.sys_first_stranger_encounter_reaction.3</t>
         </is>
       </c>
       <c r="B1169" t="inlineStr">
         <is>
-          <t>...</t>
+          <t>What else would they be.</t>
         </is>
       </c>
       <c r="C1169" t="inlineStr">
         <is>
-          <t>...</t>
+          <t>달리 뭐겠어.</t>
         </is>
       </c>
     </row>
     <row r="1170">
       <c r="A1170" t="inlineStr">
         <is>
-          <t>dialogue.sys_floor2_dire_wolf_reaction.4</t>
+          <t>dialogue.sys_first_stranger_encounter_reaction.4</t>
         </is>
       </c>
       <c r="B1170" t="inlineStr">
         <is>
-          <t>Standing here won't answer that.</t>
+          <t>...</t>
         </is>
       </c>
       <c r="C1170" t="inlineStr">
         <is>
-          <t>여기 서 있어도 답은 안 나와.</t>
+          <t>...</t>
         </is>
       </c>
     </row>
     <row r="1171">
       <c r="A1171" t="inlineStr">
         <is>
-          <t>dialogue.sys_floor2_dire_wolf_reaction.5</t>
+          <t>dialogue.sys_first_stranger_encounter_reaction.5</t>
         </is>
       </c>
       <c r="B1171" t="inlineStr">
         <is>
-          <t>Keep moving.</t>
+          <t>I have to keep moving.</t>
         </is>
       </c>
       <c r="C1171" t="inlineStr">
         <is>
-          <t>계속 가자.</t>
+          <t>계속 움직여야 해.</t>
         </is>
       </c>
     </row>
     <row r="1172">
       <c r="A1172" t="inlineStr">
         <is>
-          <t>dialogue.sys_first_stranger_encounter_reaction.0</t>
+          <t>dialogue.sys_first_level_up_reaction.0</t>
         </is>
       </c>
       <c r="B1172" t="inlineStr">
         <is>
-          <t>Get your hands off me...</t>
+          <t>...</t>
         </is>
       </c>
       <c r="C1172" t="inlineStr">
         <is>
-          <t>손 치워...</t>
+          <t>...</t>
         </is>
       </c>
     </row>
     <row r="1173">
       <c r="A1173" t="inlineStr">
         <is>
-          <t>dialogue.sys_first_stranger_encounter_reaction.1</t>
+          <t>dialogue.sys_first_level_up_reaction.1</t>
         </is>
       </c>
       <c r="B1173" t="inlineStr">
         <is>
-          <t>He smiled the whole time.</t>
+          <t>The walls tilt. Easy... easy.</t>
         </is>
       </c>
       <c r="C1173" t="inlineStr">
         <is>
-          <t>그 녀석, 내내 웃고 있었어.</t>
+          <t>벽이 기운다. 진정해... 진정해.</t>
         </is>
       </c>
     </row>
     <row r="1174">
       <c r="A1174" t="inlineStr">
         <is>
-          <t>dialogue.sys_first_stranger_encounter_reaction.2</t>
+          <t>dialogue.sys_first_level_up_reaction.2</t>
         </is>
       </c>
       <c r="B1174" t="inlineStr">
         <is>
-          <t>Are they all demons down here?</t>
+          <t>I think I'm going to be sick...</t>
         </is>
       </c>
       <c r="C1174" t="inlineStr">
         <is>
-          <t>여기 있는 건 전부 악마야?</t>
+          <t>토할 것 같아...</t>
         </is>
       </c>
     </row>
     <row r="1175">
       <c r="A1175" t="inlineStr">
         <is>
-          <t>dialogue.sys_first_stranger_encounter_reaction.3</t>
+          <t>dialogue.sys_first_level_up_reaction.3</t>
         </is>
       </c>
       <c r="B1175" t="inlineStr">
         <is>
-          <t>What else would they be.</t>
+          <t>Why does it feel like I've been training for years?</t>
         </is>
       </c>
       <c r="C1175" t="inlineStr">
         <is>
-          <t>달리 뭐겠어.</t>
+          <t>왜 몇 년 동안 훈련한 것처럼 몸이 쑤시지?</t>
         </is>
       </c>
     </row>
     <row r="1176">
       <c r="A1176" t="inlineStr">
         <is>
-          <t>dialogue.sys_first_stranger_encounter_reaction.4</t>
+          <t>dialogue.sys_first_level_up_reaction.4</t>
         </is>
       </c>
       <c r="B1176" t="inlineStr">
@@ -20418,143 +20418,143 @@
     <row r="1177">
       <c r="A1177" t="inlineStr">
         <is>
-          <t>dialogue.sys_first_stranger_encounter_reaction.5</t>
+          <t>dialogue.sys_first_level_up_reaction.5</t>
         </is>
       </c>
       <c r="B1177" t="inlineStr">
         <is>
-          <t>I have to keep moving.</t>
+          <t>...and different.</t>
         </is>
       </c>
       <c r="C1177" t="inlineStr">
         <is>
-          <t>계속 움직여야 해.</t>
+          <t>...그리고 달라졌어.</t>
         </is>
       </c>
     </row>
     <row r="1178">
       <c r="A1178" t="inlineStr">
         <is>
-          <t>dialogue.sys_first_level_up_reaction.0</t>
+          <t>dialogue.sys_first_equippable_item_reaction.0</t>
         </is>
       </c>
       <c r="B1178" t="inlineStr">
         <is>
-          <t>...</t>
+          <t>This might come in handy.</t>
         </is>
       </c>
       <c r="C1178" t="inlineStr">
         <is>
-          <t>...</t>
+          <t>쓸모가 있겠는걸.</t>
         </is>
       </c>
     </row>
     <row r="1179">
       <c r="A1179" t="inlineStr">
         <is>
-          <t>dialogue.sys_first_level_up_reaction.1</t>
+          <t>dialogue.sys_first_equippable_item_reaction.1</t>
         </is>
       </c>
       <c r="B1179" t="inlineStr">
         <is>
-          <t>The walls tilt. Easy... easy.</t>
+          <t>...</t>
         </is>
       </c>
       <c r="C1179" t="inlineStr">
         <is>
-          <t>벽이 기운다. 진정해... 진정해.</t>
+          <t>...</t>
         </is>
       </c>
     </row>
     <row r="1180">
       <c r="A1180" t="inlineStr">
         <is>
-          <t>dialogue.sys_first_level_up_reaction.2</t>
+          <t>dialogue.sys_first_equippable_item_reaction.2</t>
         </is>
       </c>
       <c r="B1180" t="inlineStr">
         <is>
-          <t>I think I'm going to be sick...</t>
+          <t>Chests every few steps.</t>
         </is>
       </c>
       <c r="C1180" t="inlineStr">
         <is>
-          <t>토할 것 같아...</t>
+          <t>몇 걸음마다 상자가 있어.</t>
         </is>
       </c>
     </row>
     <row r="1181">
       <c r="A1181" t="inlineStr">
         <is>
-          <t>dialogue.sys_first_level_up_reaction.3</t>
+          <t>dialogue.sys_first_equippable_item_reaction.3</t>
         </is>
       </c>
       <c r="B1181" t="inlineStr">
         <is>
-          <t>Why does it feel like I've been training for years?</t>
+          <t>Gear that fits like it was made for me.</t>
         </is>
       </c>
       <c r="C1181" t="inlineStr">
         <is>
-          <t>왜 몇 년 동안 훈련한 것처럼 몸이 쑤시지?</t>
+          <t>내 몸에 맞춘 듯한 장비들.</t>
         </is>
       </c>
     </row>
     <row r="1182">
       <c r="A1182" t="inlineStr">
         <is>
-          <t>dialogue.sys_first_level_up_reaction.4</t>
+          <t>dialogue.sys_first_equippable_item_reaction.4</t>
         </is>
       </c>
       <c r="B1182" t="inlineStr">
         <is>
-          <t>...</t>
+          <t>Somebody wants me armed.</t>
         </is>
       </c>
       <c r="C1182" t="inlineStr">
         <is>
-          <t>...</t>
+          <t>누군가 내가 무장하길 바라는 거야.</t>
         </is>
       </c>
     </row>
     <row r="1183">
       <c r="A1183" t="inlineStr">
         <is>
-          <t>dialogue.sys_first_level_up_reaction.5</t>
+          <t>dialogue.sys_first_equippable_item_reaction.5</t>
         </is>
       </c>
       <c r="B1183" t="inlineStr">
         <is>
-          <t>...and different.</t>
+          <t>But why arm us, if they wanted us dead?</t>
         </is>
       </c>
       <c r="C1183" t="inlineStr">
         <is>
-          <t>...그리고 달라졌어.</t>
+          <t>우리를 죽일 셈이면 왜 무기를 쥐여 주지?</t>
         </is>
       </c>
     </row>
     <row r="1184">
       <c r="A1184" t="inlineStr">
         <is>
-          <t>dialogue.sys_first_equippable_item_reaction.0</t>
+          <t>dialogue.sys_final_boss_defeated_reaction.0</t>
         </is>
       </c>
       <c r="B1184" t="inlineStr">
         <is>
-          <t>This might come in handy.</t>
+          <t>*Huff*... *Wheeze*... Fuck.</t>
         </is>
       </c>
       <c r="C1184" t="inlineStr">
         <is>
-          <t>쓸모가 있겠는걸.</t>
+          <t>*헉*... *쌕*... 젠장.</t>
         </is>
       </c>
     </row>
     <row r="1185">
       <c r="A1185" t="inlineStr">
         <is>
-          <t>dialogue.sys_first_equippable_item_reaction.1</t>
+          <t>dialogue.sys_final_boss_defeated_reaction.1</t>
         </is>
       </c>
       <c r="B1185" t="inlineStr">
@@ -20571,126 +20571,126 @@
     <row r="1186">
       <c r="A1186" t="inlineStr">
         <is>
-          <t>dialogue.sys_first_equippable_item_reaction.2</t>
+          <t>dialogue.sys_final_boss_defeated_reaction.2</t>
         </is>
       </c>
       <c r="B1186" t="inlineStr">
         <is>
-          <t>Chests every few steps.</t>
+          <t>I did it. I actually did it.</t>
         </is>
       </c>
       <c r="C1186" t="inlineStr">
         <is>
-          <t>몇 걸음마다 상자가 있어.</t>
+          <t>해냈어. 정말 해냈어.</t>
         </is>
       </c>
     </row>
     <row r="1187">
       <c r="A1187" t="inlineStr">
         <is>
-          <t>dialogue.sys_first_equippable_item_reaction.3</t>
+          <t>dialogue.sys_final_boss_defeated_reaction.3</t>
         </is>
       </c>
       <c r="B1187" t="inlineStr">
         <is>
-          <t>Gear that fits like it was made for me.</t>
+          <t>...</t>
         </is>
       </c>
       <c r="C1187" t="inlineStr">
         <is>
-          <t>내 몸에 맞춘 듯한 장비들.</t>
+          <t>...</t>
         </is>
       </c>
     </row>
     <row r="1188">
       <c r="A1188" t="inlineStr">
         <is>
-          <t>dialogue.sys_first_equippable_item_reaction.4</t>
+          <t>dialogue.sys_final_boss_defeated_reaction.4</t>
         </is>
       </c>
       <c r="B1188" t="inlineStr">
         <is>
-          <t>Somebody wants me armed.</t>
+          <t>Still...</t>
         </is>
       </c>
       <c r="C1188" t="inlineStr">
         <is>
-          <t>누군가 내가 무장하길 바라는 거야.</t>
+          <t>그런데...</t>
         </is>
       </c>
     </row>
     <row r="1189">
       <c r="A1189" t="inlineStr">
         <is>
-          <t>dialogue.sys_first_equippable_item_reaction.5</t>
+          <t>dialogue.sys_final_boss_defeated_reaction.5</t>
         </is>
       </c>
       <c r="B1189" t="inlineStr">
         <is>
-          <t>But why arm us, if they wanted us dead?</t>
+          <t>Nothing here makes sense.</t>
         </is>
       </c>
       <c r="C1189" t="inlineStr">
         <is>
-          <t>우리를 죽일 셈이면 왜 무기를 쥐여 주지?</t>
+          <t>여긴 아무것도 말이 안 돼.</t>
         </is>
       </c>
     </row>
     <row r="1190">
       <c r="A1190" t="inlineStr">
         <is>
-          <t>dialogue.sys_final_boss_defeated_reaction.0</t>
+          <t>dialogue.sys_final_boss_defeated_reaction.6</t>
         </is>
       </c>
       <c r="B1190" t="inlineStr">
         <is>
-          <t>*Huff*... *Wheeze*... Fuck.</t>
+          <t>Am I the only one seeing this?</t>
         </is>
       </c>
       <c r="C1190" t="inlineStr">
         <is>
-          <t>*헉*... *쌕*... 젠장.</t>
+          <t>이걸 보는 게 나뿐인가?</t>
         </is>
       </c>
     </row>
     <row r="1191">
       <c r="A1191" t="inlineStr">
         <is>
-          <t>dialogue.sys_final_boss_defeated_reaction.1</t>
+          <t>dialogue.sys_final_boss_defeated_reaction.7</t>
         </is>
       </c>
       <c r="B1191" t="inlineStr">
         <is>
-          <t>...</t>
+          <t>Who cares. The exit is right there.</t>
         </is>
       </c>
       <c r="C1191" t="inlineStr">
         <is>
-          <t>...</t>
+          <t>아무렴 어때. 출구가 바로 저기야.</t>
         </is>
       </c>
     </row>
     <row r="1192">
       <c r="A1192" t="inlineStr">
         <is>
-          <t>dialogue.sys_final_boss_defeated_reaction.2</t>
+          <t>dialogue.sys_final_boss_defeated_reaction.8</t>
         </is>
       </c>
       <c r="B1192" t="inlineStr">
         <is>
-          <t>I did it. I actually did it.</t>
+          <t>Time to find the others, and a way home.</t>
         </is>
       </c>
       <c r="C1192" t="inlineStr">
         <is>
-          <t>해냈어. 정말 해냈어.</t>
+          <t>동료들을 찾아서 집으로 가는 길을 찾자.</t>
         </is>
       </c>
     </row>
     <row r="1193">
       <c r="A1193" t="inlineStr">
         <is>
-          <t>dialogue.sys_final_boss_defeated_reaction.3</t>
+          <t>dialogue.sys_floor9_5_exit_reaction.0</t>
         </is>
       </c>
       <c r="B1193" t="inlineStr">
@@ -20707,969 +20707,952 @@
     <row r="1194">
       <c r="A1194" t="inlineStr">
         <is>
-          <t>dialogue.sys_final_boss_defeated_reaction.4</t>
+          <t>dialogue.sys_floor9_5_exit_reaction.1</t>
         </is>
       </c>
       <c r="B1194" t="inlineStr">
         <is>
-          <t>Still...</t>
+          <t>(Colors flood in, far too bright.)</t>
         </is>
       </c>
       <c r="C1194" t="inlineStr">
         <is>
-          <t>그런데...</t>
+          <t>(색이 쏟아져 들어온다. 너무 밝다.)</t>
         </is>
       </c>
     </row>
     <row r="1195">
       <c r="A1195" t="inlineStr">
         <is>
-          <t>dialogue.sys_final_boss_defeated_reaction.5</t>
+          <t>dialogue.sys_floor9_5_exit_reaction.2</t>
         </is>
       </c>
       <c r="B1195" t="inlineStr">
         <is>
-          <t>Nothing here makes sense.</t>
+          <t>(Black threads curl through your sight, then vanish.)</t>
         </is>
       </c>
       <c r="C1195" t="inlineStr">
         <is>
-          <t>여긴 아무것도 말이 안 돼.</t>
+          <t>(검은 실 같은 것이 시야를 휘감았다가 사라진다.)</t>
         </is>
       </c>
     </row>
     <row r="1196">
       <c r="A1196" t="inlineStr">
         <is>
-          <t>dialogue.sys_final_boss_defeated_reaction.6</t>
+          <t>dialogue.sys_floor9_5_exit_reaction.3</t>
         </is>
       </c>
       <c r="B1196" t="inlineStr">
         <is>
-          <t>Am I the only one seeing this?</t>
+          <t>(The tunnel snaps back around you.)</t>
         </is>
       </c>
       <c r="C1196" t="inlineStr">
         <is>
-          <t>이걸 보는 게 나뿐인가?</t>
+          <t>(터널이 다시 당신을 에워싼다.)</t>
         </is>
       </c>
     </row>
     <row r="1197">
       <c r="A1197" t="inlineStr">
         <is>
-          <t>dialogue.sys_final_boss_defeated_reaction.7</t>
+          <t>dialogue.sys_floor9_5_exit_reaction.4</t>
         </is>
       </c>
       <c r="B1197" t="inlineStr">
         <is>
-          <t>Who cares. The exit is right there.</t>
+          <t>Huh?</t>
         </is>
       </c>
       <c r="C1197" t="inlineStr">
         <is>
-          <t>아무렴 어때. 출구가 바로 저기야.</t>
+          <t>응?</t>
         </is>
       </c>
     </row>
     <row r="1198">
       <c r="A1198" t="inlineStr">
         <is>
-          <t>dialogue.sys_final_boss_defeated_reaction.8</t>
+          <t>dialogue.sys_floor9_5_exit_reaction.5</t>
         </is>
       </c>
       <c r="B1198" t="inlineStr">
         <is>
-          <t>Time to find the others, and a way home.</t>
+          <t>...</t>
         </is>
       </c>
       <c r="C1198" t="inlineStr">
         <is>
-          <t>동료들을 찾아서 집으로 가는 길을 찾자.</t>
+          <t>...</t>
         </is>
       </c>
     </row>
     <row r="1199">
       <c r="A1199" t="inlineStr">
         <is>
-          <t>dialogue.sys_floor9_5_exit_reaction.0</t>
+          <t>dialogue.sys_floor9_5_exit_reaction.6</t>
         </is>
       </c>
       <c r="B1199" t="inlineStr">
         <is>
-          <t>...</t>
+          <t>My head...</t>
         </is>
       </c>
       <c r="C1199" t="inlineStr">
         <is>
-          <t>...</t>
+          <t>머리가...</t>
         </is>
       </c>
     </row>
     <row r="1200">
       <c r="A1200" t="inlineStr">
         <is>
-          <t>dialogue.sys_floor9_5_exit_reaction.1</t>
+          <t>dialogue.sys_floor9_5_exit_reaction.7</t>
         </is>
       </c>
       <c r="B1200" t="inlineStr">
         <is>
-          <t>(Colors flood in, far too bright.)</t>
+          <t>It feels like it's about to split.</t>
         </is>
       </c>
       <c r="C1200" t="inlineStr">
         <is>
-          <t>(색이 쏟아져 들어온다. 너무 밝다.)</t>
+          <t>쪼개질 것 같아.</t>
         </is>
       </c>
     </row>
     <row r="1201">
       <c r="A1201" t="inlineStr">
         <is>
-          <t>dialogue.sys_floor9_5_exit_reaction.2</t>
+          <t>dialogue.sys_floor9_5_exit_reaction.8</t>
         </is>
       </c>
       <c r="B1201" t="inlineStr">
         <is>
-          <t>(Black threads curl through your sight, then vanish.)</t>
+          <t>(You clutch your head while walking toward the exit.)</t>
         </is>
       </c>
       <c r="C1201" t="inlineStr">
         <is>
-          <t>(검은 실 같은 것이 시야를 휘감았다가 사라진다.)</t>
+          <t>(머리를 부여잡고 출구를 향해 걷는다.)</t>
         </is>
       </c>
     </row>
     <row r="1202">
       <c r="A1202" t="inlineStr">
         <is>
-          <t>dialogue.sys_floor9_5_exit_reaction.3</t>
+          <t>controls.waiting_pad</t>
         </is>
       </c>
       <c r="B1202" t="inlineStr">
         <is>
-          <t>(The tunnel snaps back around you.)</t>
+          <t>Press the new key for {action}. [k:back] cancels.</t>
         </is>
       </c>
       <c r="C1202" t="inlineStr">
         <is>
-          <t>(터널이 다시 당신을 에워싼다.)</t>
+          <t>{action}에 쓸 새 키를 누르세요. [k:back] 버튼으로 취소합니다.</t>
         </is>
       </c>
     </row>
     <row r="1203">
       <c r="A1203" t="inlineStr">
         <is>
-          <t>dialogue.sys_floor9_5_exit_reaction.4</t>
+          <t>combat.msg.overpower_prefix</t>
         </is>
       </c>
       <c r="B1203" t="inlineStr">
         <is>
-          <t>Huh?</t>
+          <t>You overpower {enemy}.</t>
         </is>
       </c>
       <c r="C1203" t="inlineStr">
         <is>
-          <t>응?</t>
+          <t>{enemy}을(를) 가볍게 쓰러뜨렸습니다.</t>
         </is>
       </c>
     </row>
     <row r="1204">
       <c r="A1204" t="inlineStr">
         <is>
-          <t>dialogue.sys_floor9_5_exit_reaction.5</t>
+          <t>controls.reset_ask</t>
         </is>
       </c>
       <c r="B1204" t="inlineStr">
         <is>
-          <t>...</t>
+          <t>Reset every key to its default?</t>
         </is>
       </c>
       <c r="C1204" t="inlineStr">
         <is>
-          <t>...</t>
+          <t>모든 키를 기본값으로 되돌릴까요?</t>
         </is>
       </c>
     </row>
     <row r="1205">
       <c r="A1205" t="inlineStr">
         <is>
-          <t>dialogue.sys_floor9_5_exit_reaction.6</t>
+          <t>controls.reset_same</t>
         </is>
       </c>
       <c r="B1205" t="inlineStr">
         <is>
-          <t>My head...</t>
+          <t>Keys were already the defaults.</t>
         </is>
       </c>
       <c r="C1205" t="inlineStr">
         <is>
-          <t>머리가...</t>
+          <t>키가 이미 기본값입니다.</t>
         </is>
       </c>
     </row>
     <row r="1206">
       <c r="A1206" t="inlineStr">
         <is>
-          <t>dialogue.sys_floor9_5_exit_reaction.7</t>
+          <t>profile.default_name</t>
         </is>
       </c>
       <c r="B1206" t="inlineStr">
         <is>
-          <t>It feels like it's about to split.</t>
+          <t>Profile</t>
         </is>
       </c>
       <c r="C1206" t="inlineStr">
         <is>
-          <t>쪼개질 것 같아.</t>
+          <t>프로필</t>
         </is>
       </c>
     </row>
     <row r="1207">
       <c r="A1207" t="inlineStr">
         <is>
-          <t>dialogue.sys_floor9_5_exit_reaction.8</t>
+          <t>save.slot.name</t>
         </is>
       </c>
       <c r="B1207" t="inlineStr">
         <is>
-          <t>(You clutch your head while walking toward the exit.)</t>
+          <t>Save {n}</t>
         </is>
       </c>
       <c r="C1207" t="inlineStr">
         <is>
-          <t>(머리를 부여잡고 출구를 향해 걷는다.)</t>
+          <t>저장 {n}</t>
         </is>
       </c>
     </row>
     <row r="1208">
       <c r="A1208" t="inlineStr">
         <is>
-          <t>controls.waiting_pad</t>
+          <t>save.slot.empty</t>
         </is>
       </c>
       <c r="B1208" t="inlineStr">
         <is>
-          <t>Press the new key for {action}. [k:back] cancels.</t>
+          <t>Empty</t>
         </is>
       </c>
       <c r="C1208" t="inlineStr">
         <is>
-          <t>{action}에 쓸 새 키를 누르세요. [k:back] 버튼으로 취소합니다.</t>
+          <t>비어 있음</t>
         </is>
       </c>
     </row>
     <row r="1209">
       <c r="A1209" t="inlineStr">
         <is>
-          <t>combat.msg.overpower_prefix</t>
+          <t>save.slot.cant</t>
         </is>
       </c>
       <c r="B1209" t="inlineStr">
         <is>
-          <t>You overpower {enemy}.</t>
+          <t>Cannot load</t>
         </is>
       </c>
       <c r="C1209" t="inlineStr">
         <is>
-          <t>{enemy}을(를) 가볍게 쓰러뜨렸습니다.</t>
+          <t>불러올 수 없음</t>
         </is>
       </c>
     </row>
     <row r="1210">
       <c r="A1210" t="inlineStr">
         <is>
-          <t>controls.reset_ask</t>
+          <t>save.lbl.saved</t>
         </is>
       </c>
       <c r="B1210" t="inlineStr">
         <is>
-          <t>Reset every key to its default?</t>
+          <t>Last Saved</t>
         </is>
       </c>
       <c r="C1210" t="inlineStr">
         <is>
-          <t>모든 키를 기본값으로 되돌릴까요?</t>
+          <t>마지막 저장</t>
         </is>
       </c>
     </row>
     <row r="1211">
       <c r="A1211" t="inlineStr">
         <is>
-          <t>controls.reset_same</t>
+          <t>save.slot.help_load</t>
         </is>
       </c>
       <c r="B1211" t="inlineStr">
         <is>
-          <t>Keys were already the defaults.</t>
+          <t>Pick up this run where you left it.</t>
         </is>
       </c>
       <c r="C1211" t="inlineStr">
         <is>
-          <t>키가 이미 기본값입니다.</t>
+          <t>중단한 곳에서 이 도전을 이어갑니다.</t>
         </is>
       </c>
     </row>
     <row r="1212">
       <c r="A1212" t="inlineStr">
         <is>
-          <t>profile.default_name</t>
+          <t>save.slot.help_over</t>
         </is>
       </c>
       <c r="B1212" t="inlineStr">
         <is>
-          <t>Profile</t>
+          <t>A new game here replaces this run.</t>
         </is>
       </c>
       <c r="C1212" t="inlineStr">
         <is>
-          <t>프로필</t>
+          <t>여기서 새 게임을 시작하면 이 도전은 사라집니다.</t>
         </is>
       </c>
     </row>
     <row r="1213">
       <c r="A1213" t="inlineStr">
         <is>
-          <t>save.slot.name</t>
+          <t>save.slot.help_empty</t>
         </is>
       </c>
       <c r="B1213" t="inlineStr">
         <is>
-          <t>Save {n}</t>
+          <t>No run is saved in this file.</t>
         </is>
       </c>
       <c r="C1213" t="inlineStr">
         <is>
-          <t>저장 {n}</t>
+          <t>이 파일에는 저장된 도전이 없습니다.</t>
         </is>
       </c>
     </row>
     <row r="1214">
       <c r="A1214" t="inlineStr">
         <is>
-          <t>save.slot.empty</t>
+          <t>save.overwrite.title</t>
         </is>
       </c>
       <c r="B1214" t="inlineStr">
         <is>
-          <t>Empty</t>
+          <t>Overwrite which save file?</t>
         </is>
       </c>
       <c r="C1214" t="inlineStr">
         <is>
-          <t>비어 있음</t>
+          <t>어느 저장 파일을 덮어쓸까요?</t>
         </is>
       </c>
     </row>
     <row r="1215">
       <c r="A1215" t="inlineStr">
         <is>
-          <t>save.slot.cant</t>
+          <t>save.overwrite.ask</t>
         </is>
       </c>
       <c r="B1215" t="inlineStr">
         <is>
-          <t>Cannot load</t>
+          <t>Overwrite Save {n}? The run in it will be lost.</t>
         </is>
       </c>
       <c r="C1215" t="inlineStr">
         <is>
-          <t>불러올 수 없음</t>
+          <t>저장 {n}을(를) 덮어쓸까요? 그 안의 도전은 사라집니다.</t>
         </is>
       </c>
     </row>
     <row r="1216">
       <c r="A1216" t="inlineStr">
         <is>
-          <t>save.lbl.saved</t>
+          <t>save.delete.ask</t>
         </is>
       </c>
       <c r="B1216" t="inlineStr">
         <is>
-          <t>Last Saved</t>
+          <t>Delete Save {n}? The run in it will be lost.</t>
         </is>
       </c>
       <c r="C1216" t="inlineStr">
         <is>
-          <t>마지막 저장</t>
+          <t>저장 {n}을(를) 삭제할까요? 그 안의 도전은 사라집니다.</t>
         </is>
       </c>
     </row>
     <row r="1217">
       <c r="A1217" t="inlineStr">
         <is>
-          <t>save.slot.help_load</t>
+          <t>save.hint.load</t>
         </is>
       </c>
       <c r="B1217" t="inlineStr">
         <is>
-          <t>Pick up this run where you left it.</t>
+          <t>[k:confirm] Load</t>
         </is>
       </c>
       <c r="C1217" t="inlineStr">
         <is>
-          <t>중단한 곳에서 이 도전을 이어갑니다.</t>
+          <t>[k:confirm] 불러오기</t>
         </is>
       </c>
     </row>
     <row r="1218">
       <c r="A1218" t="inlineStr">
         <is>
-          <t>save.slot.help_over</t>
+          <t>save.hint.overwrite</t>
         </is>
       </c>
       <c r="B1218" t="inlineStr">
         <is>
-          <t>A new game here replaces this run.</t>
+          <t>[k:confirm] Overwrite</t>
         </is>
       </c>
       <c r="C1218" t="inlineStr">
         <is>
-          <t>여기서 새 게임을 시작하면 이 도전은 사라집니다.</t>
+          <t>[k:confirm] 덮어쓰기</t>
         </is>
       </c>
     </row>
     <row r="1219">
       <c r="A1219" t="inlineStr">
         <is>
-          <t>save.slot.help_empty</t>
+          <t>save.hint.delete</t>
         </is>
       </c>
       <c r="B1219" t="inlineStr">
         <is>
-          <t>No run is saved in this file.</t>
+          <t>[k:tab_prev] Delete</t>
         </is>
       </c>
       <c r="C1219" t="inlineStr">
         <is>
-          <t>이 파일에는 저장된 도전이 없습니다.</t>
+          <t>[k:tab_prev] 삭제</t>
         </is>
       </c>
     </row>
     <row r="1220">
       <c r="A1220" t="inlineStr">
         <is>
-          <t>save.overwrite.title</t>
+          <t>profile.btn</t>
         </is>
       </c>
       <c r="B1220" t="inlineStr">
         <is>
-          <t>Overwrite which save file?</t>
+          <t>[k:tab_prev] Profile</t>
         </is>
       </c>
       <c r="C1220" t="inlineStr">
         <is>
-          <t>어느 저장 파일을 덮어쓸까요?</t>
+          <t>[k:tab_prev] 프로필</t>
         </is>
       </c>
     </row>
     <row r="1221">
       <c r="A1221" t="inlineStr">
         <is>
-          <t>save.overwrite.ask</t>
+          <t>profile.title</t>
         </is>
       </c>
       <c r="B1221" t="inlineStr">
         <is>
-          <t>Overwrite Save {n}? The run in it will be lost.</t>
+          <t>Profiles</t>
         </is>
       </c>
       <c r="C1221" t="inlineStr">
         <is>
-          <t>저장 {n}을(를) 덮어쓸까요? 그 안의 도전은 사라집니다.</t>
+          <t>프로필</t>
         </is>
       </c>
     </row>
     <row r="1222">
       <c r="A1222" t="inlineStr">
         <is>
-          <t>save.delete.ask</t>
+          <t>profile.row.new</t>
         </is>
       </c>
       <c r="B1222" t="inlineStr">
         <is>
-          <t>Delete Save {n}? The run in it will be lost.</t>
+          <t>New Profile</t>
         </is>
       </c>
       <c r="C1222" t="inlineStr">
         <is>
-          <t>저장 {n}을(를) 삭제할까요? 그 안의 도전은 사라집니다.</t>
+          <t>새 프로필</t>
         </is>
       </c>
     </row>
     <row r="1223">
       <c r="A1223" t="inlineStr">
         <is>
-          <t>save.hint.load</t>
+          <t>profile.val.active</t>
         </is>
       </c>
       <c r="B1223" t="inlineStr">
         <is>
-          <t>[k:confirm] Load</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="C1223" t="inlineStr">
         <is>
-          <t>[k:confirm] 불러오기</t>
+          <t>사용 중</t>
         </is>
       </c>
     </row>
     <row r="1224">
       <c r="A1224" t="inlineStr">
         <is>
-          <t>save.hint.overwrite</t>
+          <t>profile.lbl.runs</t>
         </is>
       </c>
       <c r="B1224" t="inlineStr">
         <is>
-          <t>[k:confirm] Overwrite</t>
+          <t>Runs</t>
         </is>
       </c>
       <c r="C1224" t="inlineStr">
         <is>
-          <t>[k:confirm] 덮어쓰기</t>
+          <t>도전 횟수</t>
         </is>
       </c>
     </row>
     <row r="1225">
       <c r="A1225" t="inlineStr">
         <is>
-          <t>save.hint.delete</t>
+          <t>profile.help.active</t>
         </is>
       </c>
       <c r="B1225" t="inlineStr">
         <is>
-          <t>[k:tab_prev] Delete</t>
+          <t>The profile in use. Its Codex, run history and story are the ones you see.</t>
         </is>
       </c>
       <c r="C1225" t="inlineStr">
         <is>
-          <t>[k:tab_prev] 삭제</t>
+          <t>지금 쓰는 프로필입니다. 도감, 도전 기록, 이야기는 이 프로필의 것입니다.</t>
         </is>
       </c>
     </row>
     <row r="1226">
       <c r="A1226" t="inlineStr">
         <is>
-          <t>profile.btn</t>
+          <t>profile.help.other</t>
         </is>
       </c>
       <c r="B1226" t="inlineStr">
         <is>
-          <t>[k:tab_prev] Profile</t>
+          <t>Switch to this profile. Its Codex, run history, story and save files come with it.</t>
         </is>
       </c>
       <c r="C1226" t="inlineStr">
         <is>
-          <t>[k:tab_prev] 프로필</t>
+          <t>이 프로필로 바꿉니다. 도감, 도전 기록, 이야기, 저장 파일도 함께 바뀝니다.</t>
         </is>
       </c>
     </row>
     <row r="1227">
       <c r="A1227" t="inlineStr">
         <is>
-          <t>profile.title</t>
+          <t>profile.help.new</t>
         </is>
       </c>
       <c r="B1227" t="inlineStr">
         <is>
-          <t>Profiles</t>
+          <t>Start a new profile. Its Codex and run history are empty and the story begins again.</t>
         </is>
       </c>
       <c r="C1227" t="inlineStr">
         <is>
-          <t>프로필</t>
+          <t>새 프로필을 만듭니다. 도감과 도전 기록은 비어 있고 이야기는 처음부터 시작합니다.</t>
         </is>
       </c>
     </row>
     <row r="1228">
       <c r="A1228" t="inlineStr">
         <is>
-          <t>profile.row.new</t>
+          <t>profile.hint.switch</t>
         </is>
       </c>
       <c r="B1228" t="inlineStr">
         <is>
-          <t>New Profile</t>
+          <t>[k:confirm] Switch</t>
         </is>
       </c>
       <c r="C1228" t="inlineStr">
         <is>
-          <t>새 프로필</t>
+          <t>[k:confirm] 바꾸기</t>
         </is>
       </c>
     </row>
     <row r="1229">
       <c r="A1229" t="inlineStr">
         <is>
-          <t>profile.val.active</t>
+          <t>profile.hint.create</t>
         </is>
       </c>
       <c r="B1229" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>[k:confirm] Create</t>
         </is>
       </c>
       <c r="C1229" t="inlineStr">
         <is>
-          <t>사용 중</t>
+          <t>[k:confirm] 만들기</t>
         </is>
       </c>
     </row>
     <row r="1230">
       <c r="A1230" t="inlineStr">
         <is>
-          <t>profile.lbl.runs</t>
+          <t>profile.delete.ask</t>
         </is>
       </c>
       <c r="B1230" t="inlineStr">
         <is>
-          <t>Runs</t>
+          <t>Delete profile {name}? Its Codex, history and save files are lost.</t>
         </is>
       </c>
       <c r="C1230" t="inlineStr">
         <is>
-          <t>도전 횟수</t>
+          <t>프로필 {name}을(를) 삭제할까요? 도감, 기록, 저장 파일이 모두 사라집니다.</t>
         </is>
       </c>
     </row>
     <row r="1231">
       <c r="A1231" t="inlineStr">
         <is>
-          <t>profile.help.active</t>
+          <t>profile.name.need</t>
         </is>
       </c>
       <c r="B1231" t="inlineStr">
         <is>
-          <t>The profile in use. Its Codex, run history and story are the ones you see.</t>
+          <t>Enter a name.</t>
         </is>
       </c>
       <c r="C1231" t="inlineStr">
         <is>
-          <t>지금 쓰는 프로필입니다. 도감, 도전 기록, 이야기는 이 프로필의 것입니다.</t>
+          <t>이름을 입력하세요.</t>
         </is>
       </c>
     </row>
     <row r="1232">
       <c r="A1232" t="inlineStr">
         <is>
-          <t>profile.help.other</t>
+          <t>profile.name.key_space</t>
         </is>
       </c>
       <c r="B1232" t="inlineStr">
         <is>
-          <t>Switch to this profile. Its Codex, run history, story and save files come with it.</t>
+          <t>Space</t>
         </is>
       </c>
       <c r="C1232" t="inlineStr">
         <is>
-          <t>이 프로필로 바꿉니다. 도감, 도전 기록, 이야기, 저장 파일도 함께 바뀝니다.</t>
+          <t>띄어쓰기</t>
         </is>
       </c>
     </row>
     <row r="1233">
       <c r="A1233" t="inlineStr">
         <is>
-          <t>profile.help.new</t>
+          <t>profile.name.key_delete</t>
         </is>
       </c>
       <c r="B1233" t="inlineStr">
         <is>
-          <t>Start a new profile. Its Codex and run history are empty and the story begins again.</t>
+          <t>Delete</t>
         </is>
       </c>
       <c r="C1233" t="inlineStr">
         <is>
-          <t>새 프로필을 만듭니다. 도감과 도전 기록은 비어 있고 이야기는 처음부터 시작합니다.</t>
+          <t>삭제</t>
         </is>
       </c>
     </row>
     <row r="1234">
       <c r="A1234" t="inlineStr">
         <is>
-          <t>profile.hint.switch</t>
+          <t>profile.name.key_ok</t>
         </is>
       </c>
       <c r="B1234" t="inlineStr">
         <is>
-          <t>[k:confirm] Switch</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="C1234" t="inlineStr">
         <is>
-          <t>[k:confirm] 바꾸기</t>
+          <t>확인</t>
         </is>
       </c>
     </row>
     <row r="1235">
       <c r="A1235" t="inlineStr">
         <is>
-          <t>profile.hint.create</t>
+          <t>profile.name.hint_pick</t>
         </is>
       </c>
       <c r="B1235" t="inlineStr">
         <is>
-          <t>[k:confirm] Create</t>
+          <t>[k:confirm] Pick</t>
         </is>
       </c>
       <c r="C1235" t="inlineStr">
         <is>
-          <t>[k:confirm] 만들기</t>
+          <t>[k:confirm] 선택</t>
         </is>
       </c>
     </row>
     <row r="1236">
       <c r="A1236" t="inlineStr">
         <is>
-          <t>profile.delete.ask</t>
+          <t>profile.name.hint_cancel</t>
         </is>
       </c>
       <c r="B1236" t="inlineStr">
         <is>
-          <t>Delete profile {name}? Its Codex, history and save files are lost.</t>
+          <t>[k:back] Cancel</t>
         </is>
       </c>
       <c r="C1236" t="inlineStr">
         <is>
-          <t>프로필 {name}을(를) 삭제할까요? 도감, 기록, 저장 파일이 모두 사라집니다.</t>
+          <t>[k:back] 취소</t>
         </is>
       </c>
     </row>
     <row r="1237">
       <c r="A1237" t="inlineStr">
         <is>
-          <t>profile.name.need</t>
+          <t>profile.name.info_kb</t>
         </is>
       </c>
       <c r="B1237" t="inlineStr">
         <is>
-          <t>Enter a name.</t>
+          <t>Up to 12 letters. Backspace deletes, Enter finishes.</t>
         </is>
       </c>
       <c r="C1237" t="inlineStr">
         <is>
-          <t>이름을 입력하세요.</t>
+          <t>최대 12자. Backspace로 지우고 Enter로 끝냅니다.</t>
         </is>
       </c>
     </row>
     <row r="1238">
       <c r="A1238" t="inlineStr">
         <is>
-          <t>profile.name.key_space</t>
+          <t>profile.name.info_pad</t>
         </is>
       </c>
       <c r="B1238" t="inlineStr">
         <is>
-          <t>Space</t>
+          <t>Up to 12 letters. Pick them on the grid.</t>
         </is>
       </c>
       <c r="C1238" t="inlineStr">
         <is>
-          <t>띄어쓰기</t>
+          <t>최대 12자. 칸에서 골라 입력하세요.</t>
         </is>
       </c>
     </row>
     <row r="1239">
       <c r="A1239" t="inlineStr">
         <is>
-          <t>profile.name.key_delete</t>
+          <t>codex.btn</t>
         </is>
       </c>
       <c r="B1239" t="inlineStr">
         <is>
-          <t>Delete</t>
+          <t>[k:tab_next] Codex</t>
         </is>
       </c>
       <c r="C1239" t="inlineStr">
         <is>
-          <t>삭제</t>
+          <t>[k:tab_next] 도감</t>
         </is>
       </c>
     </row>
     <row r="1240">
       <c r="A1240" t="inlineStr">
         <is>
-          <t>profile.name.key_ok</t>
+          <t>menu.tooltip.stat.vig.desc</t>
         </is>
       </c>
       <c r="B1240" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Raises max [t]HP[/t]. The more you add, the less each point gives.</t>
         </is>
       </c>
       <c r="C1240" t="inlineStr">
         <is>
-          <t>확인</t>
+          <t>최대 [t]HP[/t]를 늘립니다. 많이 올릴수록 포인트 하나의 효과는 줄어듭니다.</t>
         </is>
       </c>
     </row>
     <row r="1241">
       <c r="A1241" t="inlineStr">
         <is>
-          <t>profile.name.hint_pick</t>
+          <t>menu.tooltip.stat.mnd.desc</t>
         </is>
       </c>
       <c r="B1241" t="inlineStr">
         <is>
-          <t>[k:confirm] Pick</t>
+          <t>Raises max [t]MP[/t]. The more you add, the less each point gives.</t>
         </is>
       </c>
       <c r="C1241" t="inlineStr">
         <is>
-          <t>[k:confirm] 선택</t>
+          <t>최대 [t]MP[/t]를 늘립니다. 많이 올릴수록 포인트 하나의 효과는 줄어듭니다.</t>
         </is>
       </c>
     </row>
     <row r="1242">
       <c r="A1242" t="inlineStr">
         <is>
-          <t>profile.name.hint_cancel</t>
+          <t>tab.lbl.max_hp</t>
         </is>
       </c>
       <c r="B1242" t="inlineStr">
         <is>
-          <t>[k:back] Cancel</t>
+          <t>Max HP</t>
         </is>
       </c>
       <c r="C1242" t="inlineStr">
         <is>
-          <t>[k:back] 취소</t>
+          <t>최대 HP</t>
         </is>
       </c>
     </row>
     <row r="1243">
       <c r="A1243" t="inlineStr">
         <is>
-          <t>profile.name.info_kb</t>
+          <t>tab.lbl.max_mp</t>
         </is>
       </c>
       <c r="B1243" t="inlineStr">
         <is>
-          <t>Up to 12 letters. Backspace deletes, Enter finishes.</t>
+          <t>Max MP</t>
         </is>
       </c>
       <c r="C1243" t="inlineStr">
         <is>
-          <t>최대 12자. Backspace로 지우고 Enter로 끝냅니다.</t>
+          <t>최대 MP</t>
         </is>
       </c>
     </row>
     <row r="1244">
       <c r="A1244" t="inlineStr">
         <is>
-          <t>profile.name.info_pad</t>
+          <t>tab.val.level_up</t>
         </is>
       </c>
       <c r="B1244" t="inlineStr">
         <is>
-          <t>Up to 12 letters. Pick them on the grid.</t>
+          <t>Level Up</t>
         </is>
       </c>
       <c r="C1244" t="inlineStr">
         <is>
-          <t>최대 12자. 칸에서 골라 입력하세요.</t>
+          <t>레벨 업</t>
         </is>
       </c>
     </row>
     <row r="1245">
       <c r="A1245" t="inlineStr">
         <is>
-          <t>codex.btn</t>
+          <t>levelup.legend</t>
         </is>
       </c>
       <c r="B1245" t="inlineStr">
         <is>
-          <t>[k:tab_next] Codex</t>
+          <t>Gold = your class grows these</t>
         </is>
       </c>
       <c r="C1245" t="inlineStr">
         <is>
-          <t>[k:tab_next] 도감</t>
+          <t>금색 = 직업이 성장시키는 능력치</t>
         </is>
       </c>
     </row>
     <row r="1246">
       <c r="A1246" t="inlineStr">
         <is>
-          <t>menu.tooltip.stat.vig.desc</t>
+          <t>cards.stat.hp_now</t>
         </is>
       </c>
       <c r="B1246" t="inlineStr">
         <is>
-          <t>Raises max [t]HP[/t]. The more you add, the less each point gives.</t>
+          <t>Max HP Now</t>
         </is>
       </c>
       <c r="C1246" t="inlineStr">
         <is>
-          <t>최대 [t]HP[/t]를 늘립니다. 많이 올릴수록 포인트 하나의 효과는 줄어듭니다.</t>
+          <t>최대 HP 현재</t>
         </is>
       </c>
     </row>
     <row r="1247">
       <c r="A1247" t="inlineStr">
         <is>
-          <t>menu.tooltip.stat.mnd.desc</t>
+          <t>cards.stat.hp_after</t>
         </is>
       </c>
       <c r="B1247" t="inlineStr">
         <is>
-          <t>Raises max [t]MP[/t]. The more you add, the less each point gives.</t>
+          <t>Max HP After</t>
         </is>
       </c>
       <c r="C1247" t="inlineStr">
         <is>
-          <t>최대 [t]MP[/t]를 늘립니다. 많이 올릴수록 포인트 하나의 효과는 줄어듭니다.</t>
+          <t>최대 HP 이후</t>
         </is>
       </c>
     </row>
     <row r="1248">
       <c r="A1248" t="inlineStr">
         <is>
-          <t>tab.lbl.max_hp</t>
+          <t>cards.stat.mp_now</t>
         </is>
       </c>
       <c r="B1248" t="inlineStr">
         <is>
-          <t>Max HP</t>
+          <t>Max MP Now</t>
         </is>
       </c>
       <c r="C1248" t="inlineStr">
         <is>
-          <t>최대 HP</t>
+          <t>최대 MP 현재</t>
         </is>
       </c>
     </row>
     <row r="1249">
       <c r="A1249" t="inlineStr">
         <is>
-          <t>tab.lbl.max_mp</t>
+          <t>cards.stat.mp_after</t>
         </is>
       </c>
       <c r="B1249" t="inlineStr">
         <is>
-          <t>Max MP</t>
+          <t>Max MP After</t>
         </is>
       </c>
       <c r="C1249" t="inlineStr">
         <is>
-          <t>최대 MP</t>
-        </is>
-      </c>
-    </row>
-    <row r="1250">
-      <c r="A1250" t="inlineStr">
-        <is>
-          <t>tab.val.level_up</t>
-        </is>
-      </c>
-      <c r="B1250" t="inlineStr">
-        <is>
-          <t>Level Up</t>
-        </is>
-      </c>
-      <c r="C1250" t="inlineStr">
-        <is>
-          <t>레벨 업</t>
+          <t>최대 MP 이후</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(r3ideas1): weak points and resistances (D173, R-114), the death-screen tip (D185, R-115)
IDEA-07: every enemy has weak / resist (scr_db_enemy); a weak enemy takes +1 Burning turn (cap 4) or +1 Poison / Bleeding stack (D78 caps), a resisting one a halved chance
(rounded down, a sure 100% -> 50%) through Skill_StatusApplyArgs / Skill_StatusTry and Throw_Resolve; the log says "is weak to" once per fight and "resists" each time; the
Codex bestiary shows Weak / Resists as ? until a fight showed each (profile flags). One table of numbers: WeakPoint_Table. Balance sim plays the rule.
IDEA-25: the death scene adds one tip under the line from the killer status, then the last enemy move, then a generic pool that never repeats back to back (profile last_tip).
Existing assertions that asserted the old behaviour were updated (Slime Firebomb 3 turns, Fireball / Wound target a neutral enemy, the death scene lasts the line plus the tip).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datafiles/localization/game_text.xlsx
+++ b/datafiles/localization/game_text.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1269"/>
+  <dimension ref="A1:C1285"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -21996,6 +21996,278 @@
         </is>
       </c>
     </row>
+    <row r="1270">
+      <c r="A1270" t="inlineStr">
+        <is>
+          <t>combat.msg.weak_to</t>
+        </is>
+      </c>
+      <c r="B1270" t="inlineStr">
+        <is>
+          <t>{enemy} is weak to [t]{status}[/t]!</t>
+        </is>
+      </c>
+      <c r="C1270" t="inlineStr">
+        <is>
+          <t>{enemy}은(는) [t]{status}[/t]에 약합니다!</t>
+        </is>
+      </c>
+    </row>
+    <row r="1271">
+      <c r="A1271" t="inlineStr">
+        <is>
+          <t>combat.msg.resists</t>
+        </is>
+      </c>
+      <c r="B1271" t="inlineStr">
+        <is>
+          <t>{enemy} resists [t]{status}[/t].</t>
+        </is>
+      </c>
+      <c r="C1271" t="inlineStr">
+        <is>
+          <t>{enemy}은(는) [t]{status}[/t]에 저항합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1272">
+      <c r="A1272" t="inlineStr">
+        <is>
+          <t>tab.lbl.weak</t>
+        </is>
+      </c>
+      <c r="B1272" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="C1272" t="inlineStr">
+        <is>
+          <t>약점</t>
+        </is>
+      </c>
+    </row>
+    <row r="1273">
+      <c r="A1273" t="inlineStr">
+        <is>
+          <t>tab.lbl.resists</t>
+        </is>
+      </c>
+      <c r="B1273" t="inlineStr">
+        <is>
+          <t>Resists</t>
+        </is>
+      </c>
+      <c r="C1273" t="inlineStr">
+        <is>
+          <t>저항</t>
+        </is>
+      </c>
+    </row>
+    <row r="1274">
+      <c r="A1274" t="inlineStr">
+        <is>
+          <t>death.tip.status_poison</t>
+        </is>
+      </c>
+      <c r="B1274" t="inlineStr">
+        <is>
+          <t>Poison killed you: an Antidote cures it.</t>
+        </is>
+      </c>
+      <c r="C1274" t="inlineStr">
+        <is>
+          <t>독에 쓰러졌습니다. 해독제로 치료할 수 있습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1275">
+      <c r="A1275" t="inlineStr">
+        <is>
+          <t>death.tip.status_bleed</t>
+        </is>
+      </c>
+      <c r="B1275" t="inlineStr">
+        <is>
+          <t>Bleeding hurts when you act: a Bandage stops it.</t>
+        </is>
+      </c>
+      <c r="C1275" t="inlineStr">
+        <is>
+          <t>출혈은 행동할 때 피해를 줍니다. 붕대로 멈출 수 있습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1276">
+      <c r="A1276" t="inlineStr">
+        <is>
+          <t>death.tip.status_burn</t>
+        </is>
+      </c>
+      <c r="B1276" t="inlineStr">
+        <is>
+          <t>Burn lowers your DEF while it lasts: Guard to halve the hits.</t>
+        </is>
+      </c>
+      <c r="C1276" t="inlineStr">
+        <is>
+          <t>화상이 지속되는 동안 DEF가 낮아집니다. 방어로 피해를 반으로 줄이세요.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1277">
+      <c r="A1277" t="inlineStr">
+        <is>
+          <t>death.tip.skill_pale_hymn</t>
+        </is>
+      </c>
+      <c r="B1277" t="inlineStr">
+        <is>
+          <t>{skill}: [a]BREAK[/a] it before it lands.</t>
+        </is>
+      </c>
+      <c r="C1277" t="inlineStr">
+        <is>
+          <t>{skill}: 공격이 닿기 전에 [a]브레이크[/a]시키세요.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1278">
+      <c r="A1278" t="inlineStr">
+        <is>
+          <t>death.tip.skill_ramming</t>
+        </is>
+      </c>
+      <c r="B1278" t="inlineStr">
+        <is>
+          <t>{skill}: [a]BREAK[/a] it first, or Guard and time the defence bar.</t>
+        </is>
+      </c>
+      <c r="C1278" t="inlineStr">
+        <is>
+          <t>{skill}: 먼저 [a]브레이크[/a]시키거나, 방어하고 막대의 타이밍을 맞추세요.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1279">
+      <c r="A1279" t="inlineStr">
+        <is>
+          <t>death.tip.skill_windup</t>
+        </is>
+      </c>
+      <c r="B1279" t="inlineStr">
+        <is>
+          <t>{skill} comes after a wind-up: [a]BREAK[/a] it first, or Guard.</t>
+        </is>
+      </c>
+      <c r="C1279" t="inlineStr">
+        <is>
+          <t>{skill}은(는) 준비 동작 뒤에 옵니다. 먼저 [a]브레이크[/a]시키거나 방어하세요.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1280">
+      <c r="A1280" t="inlineStr">
+        <is>
+          <t>death.tip.gen_guard</t>
+        </is>
+      </c>
+      <c r="B1280" t="inlineStr">
+        <is>
+          <t>Guard halves all hits until your next turn and restores {pct}% of max MP.</t>
+        </is>
+      </c>
+      <c r="C1280" t="inlineStr">
+        <is>
+          <t>방어는 다음 턴까지 모든 피해를 반으로 줄이고 최대 MP의 {pct}%를 회복합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1281">
+      <c r="A1281" t="inlineStr">
+        <is>
+          <t>death.tip.gen_weak</t>
+        </is>
+      </c>
+      <c r="B1281" t="inlineStr">
+        <is>
+          <t>Every enemy has a weak point and a resistance. The Codex remembers them.</t>
+        </is>
+      </c>
+      <c r="C1281" t="inlineStr">
+        <is>
+          <t>모든 적에게는 약점과 저항이 있습니다. 도감이 기억해 줍니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1282">
+      <c r="A1282" t="inlineStr">
+        <is>
+          <t>death.tip.gen_bed</t>
+        </is>
+      </c>
+      <c r="B1282" t="inlineStr">
+        <is>
+          <t>Each bed restores all your HP and MP, once per run.</t>
+        </is>
+      </c>
+      <c r="C1282" t="inlineStr">
+        <is>
+          <t>침대는 도전마다 한 번, HP와 MP를 모두 회복해 줍니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1283">
+      <c r="A1283" t="inlineStr">
+        <is>
+          <t>death.tip.gen_break</t>
+        </is>
+      </c>
+      <c r="B1283" t="inlineStr">
+        <is>
+          <t>When an enemy hits [a]BREAK[/a], it loses a turn and takes {pct}% more damage.</t>
+        </is>
+      </c>
+      <c r="C1283" t="inlineStr">
+        <is>
+          <t>적이 [a]브레이크[/a] 상태가 되면 한 턴을 잃고 피해를 {pct}% 더 받습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1284">
+      <c r="A1284" t="inlineStr">
+        <is>
+          <t>death.tip.gen_smoke</t>
+        </is>
+      </c>
+      <c r="B1284" t="inlineStr">
+        <is>
+          <t>A [a]Perfect[/a] Smoke Bomb throw gets you out of any battle but a boss.</t>
+        </is>
+      </c>
+      <c r="C1284" t="inlineStr">
+        <is>
+          <t>연막탄을 [a]완벽[/a]하게 던지면 보스 전투를 뺀 모든 전투에서 빠져나갑니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1285">
+      <c r="A1285" t="inlineStr">
+        <is>
+          <t>death.tip.gen_throw</t>
+        </is>
+      </c>
+      <c r="B1285" t="inlineStr">
+        <is>
+          <t>A thrown Firebomb or Poison Pot finds weak points like a skill does.</t>
+        </is>
+      </c>
+      <c r="C1285" t="inlineStr">
+        <is>
+          <t>던진 화염병이나 독 항아리도 스킬처럼 약점을 찌릅니다.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C678"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(r4final2): System tab gets Save (notice Game saved.) and Save & Quit to Title; greyed with a reason in a fight, a cutscene and with no run (I-112, R-127)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datafiles/localization/game_text.xlsx
+++ b/datafiles/localization/game_text.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1297"/>
+  <dimension ref="A1:C1308"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -22472,6 +22472,193 @@
         </is>
       </c>
     </row>
+    <row r="1298">
+      <c r="A1298" t="inlineStr">
+        <is>
+          <t>pause.option.save</t>
+        </is>
+      </c>
+      <c r="B1298" t="inlineStr">
+        <is>
+          <t>Save</t>
+        </is>
+      </c>
+      <c r="C1298" t="inlineStr">
+        <is>
+          <t>저장하기</t>
+        </is>
+      </c>
+    </row>
+    <row r="1299">
+      <c r="A1299" t="inlineStr">
+        <is>
+          <t>pause.option.save_quit</t>
+        </is>
+      </c>
+      <c r="B1299" t="inlineStr">
+        <is>
+          <t>Save &amp; Quit to Title</t>
+        </is>
+      </c>
+      <c r="C1299" t="inlineStr">
+        <is>
+          <t>저장하고 타이틀로 나가기</t>
+        </is>
+      </c>
+    </row>
+    <row r="1300">
+      <c r="A1300" t="inlineStr">
+        <is>
+          <t>pause.help.save</t>
+        </is>
+      </c>
+      <c r="B1300" t="inlineStr">
+        <is>
+          <t>Saves your run now. Continue picks it up from here.</t>
+        </is>
+      </c>
+      <c r="C1300" t="inlineStr">
+        <is>
+          <t>지금 도전을 저장합니다. 이어하기로 여기서부터 계속할 수 있습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1301">
+      <c r="A1301" t="inlineStr">
+        <is>
+          <t>pause.help.save_quit</t>
+        </is>
+      </c>
+      <c r="B1301" t="inlineStr">
+        <is>
+          <t>Saves your run, then goes to the title. Continue picks it up from here.</t>
+        </is>
+      </c>
+      <c r="C1301" t="inlineStr">
+        <is>
+          <t>도전을 저장하고 타이틀로 갑니다. 이어하기로 여기서부터 계속할 수 있습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1302">
+      <c r="A1302" t="inlineStr">
+        <is>
+          <t>tab.system.save_battle</t>
+        </is>
+      </c>
+      <c r="B1302" t="inlineStr">
+        <is>
+          <t>You cannot save during a battle.</t>
+        </is>
+      </c>
+      <c r="C1302" t="inlineStr">
+        <is>
+          <t>전투 중에는 저장할 수 없습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1303">
+      <c r="A1303" t="inlineStr">
+        <is>
+          <t>tab.system.save_cutscene</t>
+        </is>
+      </c>
+      <c r="B1303" t="inlineStr">
+        <is>
+          <t>You cannot save during a cutscene.</t>
+        </is>
+      </c>
+      <c r="C1303" t="inlineStr">
+        <is>
+          <t>컷신 중에는 저장할 수 없습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1304">
+      <c r="A1304" t="inlineStr">
+        <is>
+          <t>tab.system.save_none</t>
+        </is>
+      </c>
+      <c r="B1304" t="inlineStr">
+        <is>
+          <t>There is no run to save.</t>
+        </is>
+      </c>
+      <c r="C1304" t="inlineStr">
+        <is>
+          <t>저장할 도전이 없습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1305">
+      <c r="A1305" t="inlineStr">
+        <is>
+          <t>tab.system.save_busy</t>
+        </is>
+      </c>
+      <c r="B1305" t="inlineStr">
+        <is>
+          <t>You cannot save right now.</t>
+        </is>
+      </c>
+      <c r="C1305" t="inlineStr">
+        <is>
+          <t>지금은 저장할 수 없습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1306">
+      <c r="A1306" t="inlineStr">
+        <is>
+          <t>save.done</t>
+        </is>
+      </c>
+      <c r="B1306" t="inlineStr">
+        <is>
+          <t>Game saved.</t>
+        </is>
+      </c>
+      <c r="C1306" t="inlineStr">
+        <is>
+          <t>게임이 저장되었습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1307">
+      <c r="A1307" t="inlineStr">
+        <is>
+          <t>save.failed</t>
+        </is>
+      </c>
+      <c r="B1307" t="inlineStr">
+        <is>
+          <t>The game could not be saved.</t>
+        </is>
+      </c>
+      <c r="C1307" t="inlineStr">
+        <is>
+          <t>게임을 저장하지 못했습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1308">
+      <c r="A1308" t="inlineStr">
+        <is>
+          <t>confirm.save_quit</t>
+        </is>
+      </c>
+      <c r="B1308" t="inlineStr">
+        <is>
+          <t>Save and quit to title? Continue picks it up from here.</t>
+        </is>
+      </c>
+      <c r="C1308" t="inlineStr">
+        <is>
+          <t>저장하고 타이틀로 나갈까요? 이어하기로 여기서부터 계속할 수 있습니다.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C678"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix(r4polish): battle toast clear of the enemy, plate and chips (R-131); level-up legend says what gold is (R-132)
Toast: under the turn strip when it fits above the name plate, else over the HUD row's right column while no menu is up; not drawn with the menu up and no room. Legend: Gold numbers: your class's growth (en + ko). Shots +15 (500).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datafiles/localization/game_text.xlsx
+++ b/datafiles/localization/game_text.xlsx
@@ -21953,12 +21953,12 @@
       </c>
       <c r="B1267" t="inlineStr">
         <is>
-          <t>Gold = your class grows these</t>
+          <t>Gold numbers: your class's growth</t>
         </is>
       </c>
       <c r="C1267" t="inlineStr">
         <is>
-          <t>금색 = 직업이 성장시키는 능력치</t>
+          <t>금색 숫자: 직업의 성장</t>
         </is>
       </c>
     </row>

</xml_diff>